<commit_message>
feat(it): GR 타이틀 표시 교체 백포트 (v0.6.15)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -1465,7 +1465,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>W16 - CineBeam S PDP Video Update</t>
+          <t>GR26-W16-MS-ITB2C-CineBeam S PDP Video Update</t>
         </is>
       </c>
       <c r="C1" s="3" t="n"/>
@@ -2966,7 +2966,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -3482,7 +3481,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -4696,7 +4694,7 @@
       </c>
       <c r="B1" s="36" t="inlineStr">
         <is>
-          <t>W16 - Copilot+ Filter Creation</t>
+          <t>GR26-W16-MS-IT-PC Copilot+ Filter Creation</t>
         </is>
       </c>
       <c r="C1" s="37" t="n"/>
@@ -5667,7 +5665,7 @@
       </c>
       <c r="B1" s="125" t="inlineStr">
         <is>
-          <t>W16 - Microsoft PDP Gallery Card</t>
+          <t>GR26-W16-MS-IT-PC PDP Gallery Card Addition for JS Global</t>
         </is>
       </c>
       <c r="C1" s="126" t="n"/>
@@ -5733,7 +5731,6 @@
       <c r="G5" s="127" t="n"/>
     </row>
     <row r="6" ht="40.5" customHeight="1" s="203"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
@@ -6219,7 +6216,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>W17 - GNB Structure</t>
+          <t>GR26-W17-MS-IT-B2C GNB Structure Update 2026 – GP1</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>
@@ -7324,7 +7321,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>W18 - FAQ Request (UltraGear PLP)</t>
+          <t>GR26-W18-MS-IT UltraGear evo / Hyper Mini LED PLP FAQ Creation</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>
@@ -7360,10 +7357,6 @@
       <c r="E3" s="131" t="n"/>
       <c r="F3" s="127" t="n"/>
     </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -7726,7 +7719,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>W18 - UltraGear OLED FAQ Update</t>
+          <t>GR26-W18-MS-IT UltraGear / OLED Gaming Monitor PLP FAQ Update</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>
@@ -8157,7 +8150,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>W22 - UltraGear Buying Guide</t>
+          <t>GR26-W22-MS-IT UltraGear Bying Guide</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>
@@ -8216,7 +8209,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -9265,7 +9257,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -9815,7 +9806,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat(it): FAQ Creation Status 재편(완료/법인리뷰)·Status 2(GNB 미반영) 백포트 (v0.6.16)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -595,7 +595,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="287">
+  <cellXfs count="289">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1164,6 +1164,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7306,7 +7312,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="34.5" customWidth="1" style="203" min="3" max="3"/>
@@ -7326,8 +7332,8 @@
       </c>
       <c r="C1" s="164" t="n"/>
       <c r="D1" s="164" t="n"/>
-      <c r="E1" s="165" t="n"/>
-      <c r="F1" s="127" t="n"/>
+      <c r="F1" s="165" t="n"/>
+      <c r="G1" s="127" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -7342,8 +7348,8 @@
         </is>
       </c>
       <c r="D2" s="164" t="n"/>
-      <c r="E2" s="165" t="n"/>
-      <c r="F2" s="127" t="n"/>
+      <c r="F2" s="165" t="n"/>
+      <c r="G2" s="127" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="166" t="n"/>
@@ -7354,9 +7360,13 @@
       </c>
       <c r="C3" s="131" t="n"/>
       <c r="D3" s="131" t="n"/>
-      <c r="E3" s="131" t="n"/>
-      <c r="F3" s="127" t="n"/>
-    </row>
+      <c r="F3" s="131" t="n"/>
+      <c r="G3" s="127" t="n"/>
+    </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -7380,15 +7390,20 @@
       </c>
       <c r="E8" s="266" t="inlineStr">
         <is>
+          <t>Status 2</t>
+        </is>
+      </c>
+      <c r="F8" s="266" t="inlineStr">
+        <is>
           <t>완료일</t>
         </is>
       </c>
-      <c r="F8" s="266" t="inlineStr">
+      <c r="G8" s="266" t="inlineStr">
         <is>
           <t>Page#</t>
         </is>
       </c>
-      <c r="G8" s="266" t="inlineStr">
+      <c r="H8" s="266" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
@@ -7407,14 +7422,15 @@
       </c>
       <c r="D9" s="269" t="inlineStr">
         <is>
-          <t>미반영</t>
-        </is>
-      </c>
-      <c r="E9" s="270" t="n"/>
-      <c r="F9" s="177" t="n">
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E9" s="287" t="n"/>
+      <c r="F9" s="270" t="n"/>
+      <c r="G9" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="0" t="inlineStr">
+      <c r="H9" s="0" t="inlineStr">
         <is>
           <t>FAQ 미게시 (evo·Hyper)</t>
         </is>
@@ -7431,16 +7447,21 @@
           <t>https://www.lg.com/ca_en/monitors/hyper-mini-led-gaming-monitor/</t>
         </is>
       </c>
-      <c r="D10" s="286" t="inlineStr">
-        <is>
-          <t>부분반영</t>
-        </is>
-      </c>
-      <c r="E10" s="270" t="n"/>
-      <c r="F10" s="177" t="n">
+      <c r="D10" s="285" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" s="269" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F10" s="270" t="n"/>
+      <c r="G10" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="0" t="inlineStr">
+      <c r="H10" s="0" t="inlineStr">
         <is>
           <t>evo 반영 · Hyper GNB 미노출</t>
         </is>
@@ -7457,16 +7478,21 @@
           <t>https://www.lg.com/ca_fr/moniteurs/hyper-mini-led-gaming-monitor/</t>
         </is>
       </c>
-      <c r="D11" s="286" t="inlineStr">
-        <is>
-          <t>부분반영</t>
-        </is>
-      </c>
-      <c r="E11" s="270" t="n"/>
-      <c r="F11" s="177" t="n">
+      <c r="D11" s="285" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" s="269" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F11" s="270" t="n"/>
+      <c r="G11" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="0" t="inlineStr">
+      <c r="H11" s="0" t="inlineStr">
         <is>
           <t>evo 반영 · Hyper GNB 미노출</t>
         </is>
@@ -7485,14 +7511,15 @@
       </c>
       <c r="D12" s="273" t="inlineStr">
         <is>
-          <t>미반영</t>
-        </is>
-      </c>
-      <c r="E12" s="274" t="n"/>
-      <c r="F12" s="185" t="n">
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E12" s="288" t="n"/>
+      <c r="F12" s="274" t="n"/>
+      <c r="G12" s="185" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="0" t="inlineStr">
+      <c r="H12" s="0" t="inlineStr">
         <is>
           <t>FAQ 미게시 (evo·Hyper)</t>
         </is>
@@ -7511,14 +7538,15 @@
       </c>
       <c r="D13" s="273" t="inlineStr">
         <is>
-          <t>미반영</t>
-        </is>
-      </c>
-      <c r="E13" s="270" t="n"/>
-      <c r="F13" s="177" t="n">
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E13" s="288" t="n"/>
+      <c r="F13" s="270" t="n"/>
+      <c r="G13" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="0" t="inlineStr">
+      <c r="H13" s="0" t="inlineStr">
         <is>
           <t>evo FAQ 미게시 · Hyper 페이지/FAQ 게시 대기</t>
         </is>
@@ -7537,14 +7565,15 @@
       </c>
       <c r="D14" s="273" t="inlineStr">
         <is>
-          <t>미반영</t>
-        </is>
-      </c>
-      <c r="E14" s="270" t="n"/>
-      <c r="F14" s="177" t="n">
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E14" s="288" t="n"/>
+      <c r="F14" s="270" t="n"/>
+      <c r="G14" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="0" t="inlineStr">
+      <c r="H14" s="0" t="inlineStr">
         <is>
           <t>FAQ 미게시 (evo·Hyper)</t>
         </is>
@@ -7561,16 +7590,21 @@
           <t>https://www.lg.com/it/monitor/hyper-mini-led-gaming-monitor/</t>
         </is>
       </c>
-      <c r="D15" s="273" t="inlineStr">
-        <is>
-          <t>미반영</t>
-        </is>
-      </c>
-      <c r="E15" s="275" t="n"/>
-      <c r="F15" s="177" t="n">
+      <c r="D15" s="247" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E15" s="273" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F15" s="275" t="n"/>
+      <c r="G15" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="0" t="inlineStr">
+      <c r="H15" s="0" t="inlineStr">
         <is>
           <t>FAQ 라이브 but GNB 미노출 (evo·Hyper)</t>
         </is>
@@ -7589,14 +7623,15 @@
       </c>
       <c r="D16" s="273" t="inlineStr">
         <is>
-          <t>미반영</t>
-        </is>
-      </c>
-      <c r="E16" s="275" t="n"/>
-      <c r="F16" s="177" t="n">
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E16" s="288" t="n"/>
+      <c r="F16" s="275" t="n"/>
+      <c r="G16" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="0" t="inlineStr">
+      <c r="H16" s="0" t="inlineStr">
         <is>
           <t>페이지/FAQ 게시 대기 (evo·Hyper)</t>
         </is>
@@ -7615,18 +7650,19 @@
       </c>
       <c r="D17" s="247" t="inlineStr">
         <is>
-          <t>반영</t>
-        </is>
-      </c>
-      <c r="E17" s="270" t="inlineStr">
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E17" s="288" t="n"/>
+      <c r="F17" s="270" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="F17" s="177" t="n">
+      <c r="G17" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="0" t="n"/>
+      <c r="H17" s="0" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="267" t="inlineStr">
@@ -7639,16 +7675,21 @@
           <t>https://www.lg.com/se/monitor/hyper-mini-led-gaming-monitor/</t>
         </is>
       </c>
-      <c r="D18" s="273" t="inlineStr">
-        <is>
-          <t>미반영</t>
-        </is>
-      </c>
-      <c r="E18" s="275" t="n"/>
-      <c r="F18" s="177" t="n">
+      <c r="D18" s="247" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" s="273" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F18" s="275" t="n"/>
+      <c r="G18" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="0" t="inlineStr">
+      <c r="H18" s="0" t="inlineStr">
         <is>
           <t>FAQ 라이브 but GNB 미노출 (evo·Hyper)</t>
         </is>
@@ -7665,16 +7706,21 @@
           <t>https://www.lg.com/uk/monitors/ultragear-evo/</t>
         </is>
       </c>
-      <c r="D19" s="256" t="inlineStr">
-        <is>
-          <t>부분반영</t>
-        </is>
-      </c>
-      <c r="E19" s="275" t="n"/>
-      <c r="F19" s="177" t="n">
+      <c r="D19" s="247" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E19" s="273" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F19" s="275" t="n"/>
+      <c r="G19" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G19" s="0" t="inlineStr">
+      <c r="H19" s="0" t="inlineStr">
         <is>
           <t>evo 반영 · Hyper GNB 미노출</t>
         </is>

</xml_diff>

<commit_message>
fix(it): W22 Buying Guide·W23 27GM950B 금주 신규 표시 제거 — NEW 배지 63건·B2 목록 정리 (사용자 지시)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -7363,10 +7363,6 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -8211,37 +8207,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>AE_AR : 신규
-BD : 신규
-BE : 신규
-BR : 신규
-CAC : 신규
-CA_EN : 신규
-CA_FR : 신규
-CN : 신규
-CO : 신규
-CP : 신규
-CZ : 신규
-DK : 신규
-EC : 신규
-EE : 신규
-ES : 신규
-FI : 신규
-FR : 신규
-GR : 신규
-HK : 신규
-HK_EN : 신규
-HU : 신규
-ID : 신규
-IL : 신규
-IN : 신규
-IT : 신규
-JP : 신규
-KZ : 신규
-LT : 신규
-LV : 신규
-NL : 신규
-… 외 15건</t>
+          <t>금주 변경 없음</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -9272,24 +9238,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>AU : 신규
-CA_EN : 신규
-CA_FR : 신규
-CN : 신규
-DE : 신규
-FR : 신규
-HK : 신규
-HK_EN : 신규
-IL : 신규
-IT : 신규
-JP : 신규
-NL : 신규
-NZ : 신규
-SA : 신규
-SA_EN : 신규
-SE : 신규
-TW : 신규
-UK : 신규</t>
+          <t>금주 변경 없음</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>

</xml_diff>

<commit_message>
feat(it): W28 AI Upscaling Disclaimer GR 추가 (63 pages 작업중)
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -14,6 +14,7 @@
     <sheet name="W23 - 39GX950B 이미지 수정 2차" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="W23 - 52G930B Feature 수정 건" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="W23 - UL인증 feature 삭제 1차" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="W28 - AI Upscaling Disclaimer" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4678,6 +4679,1741 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G71"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="166" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="163" t="inlineStr">
+        <is>
+          <t>GR26-W28-IT-PDP-AI-Upscaling-Disclaimer-Update</t>
+        </is>
+      </c>
+      <c r="C1" s="164" t="n"/>
+      <c r="D1" s="164" t="n"/>
+      <c r="E1" s="165" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" s="163" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · AI Upscaling Disclaimer Update (63 pages / 31 sites)</t>
+        </is>
+      </c>
+      <c r="C2" s="164" t="n"/>
+      <c r="D2" s="164" t="n"/>
+      <c r="E2" s="165" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="166" t="n"/>
+      <c r="B3" s="163" t="n"/>
+      <c r="C3" s="164" t="n"/>
+      <c r="D3" s="164" t="n"/>
+      <c r="E3" s="165" t="n"/>
+    </row>
+    <row r="5">
+      <c r="E5" s="127" t="n"/>
+    </row>
+    <row r="6">
+      <c r="E6" s="127" t="n"/>
+    </row>
+    <row r="7">
+      <c r="E7" s="127" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="283" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B8" s="283" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C8" s="283" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D8" s="283" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E8" s="283" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F8" s="283" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G8" s="283" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" s="203">
+      <c r="B9" s="261" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C9" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-27gm950b-b</t>
+        </is>
+      </c>
+      <c r="D9" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E9" s="123" t="n"/>
+      <c r="F9" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="261" t="inlineStr">
+        <is>
+          <t>AE_AR : AE (ar)</t>
+        </is>
+      </c>
+      <c r="C10" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae_ar/consumer-monitors/lg-27gm950b-b</t>
+        </is>
+      </c>
+      <c r="D10" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E10" s="123" t="n"/>
+      <c r="F10" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="261" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C11" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/monitors/ultragear-gaming/27gm950b/</t>
+        </is>
+      </c>
+      <c r="D11" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E11" s="123" t="n"/>
+      <c r="F11" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="261" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C12" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/gaming/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D12" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E12" s="123" t="n"/>
+      <c r="F12" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="261" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C13" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/gaming/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D13" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E13" s="123" t="n"/>
+      <c r="F13" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="261" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C14" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27gm950b-b</t>
+        </is>
+      </c>
+      <c r="D14" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E14" s="123" t="n"/>
+      <c r="F14" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="261" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C15" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/monitore/gaming/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D15" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E15" s="123" t="n"/>
+      <c r="F15" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="261" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C16" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/gaming/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D16" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E16" s="123" t="n"/>
+      <c r="F16" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="261" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C17" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-27gm950b-b</t>
+        </is>
+      </c>
+      <c r="D17" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E17" s="123" t="n"/>
+      <c r="F17" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="261" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C18" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/monitor/gaming/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D18" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E18" s="123" t="n"/>
+      <c r="F18" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C19" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D19" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E19" s="123" t="n"/>
+      <c r="F19" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="261" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C20" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D20" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E20" s="123" t="n"/>
+      <c r="F20" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="261" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C21" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D21" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E21" s="123" t="n"/>
+      <c r="F21" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="261" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C22" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/gaming-monitor/27gm950b-b/</t>
+        </is>
+      </c>
+      <c r="D22" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E22" s="123" t="n"/>
+      <c r="F22" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>27GM950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="261" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C23" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-39gx950b-b</t>
+        </is>
+      </c>
+      <c r="D23" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E23" s="123" t="n"/>
+      <c r="F23" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="261" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C24" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/business/monitors/lg-39gx950b-b</t>
+        </is>
+      </c>
+      <c r="D24" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E24" s="123" t="n"/>
+      <c r="F24" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="261" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C25" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/monitors/ultragear-gaming/39gx950b/</t>
+        </is>
+      </c>
+      <c r="D25" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E25" s="123" t="n"/>
+      <c r="F25" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="261" t="inlineStr">
+        <is>
+          <t>BE : BE (nl)</t>
+        </is>
+      </c>
+      <c r="C26" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/be/monitoren/ultragear-gaming-monitoren/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D26" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E26" s="123" t="n"/>
+      <c r="F26" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="261" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C27" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D27" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E27" s="123" t="n"/>
+      <c r="F27" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="261" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C28" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D28" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E28" s="123" t="n"/>
+      <c r="F28" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="261" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C29" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-39gx950b-b</t>
+        </is>
+      </c>
+      <c r="D29" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E29" s="123" t="n"/>
+      <c r="F29" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="261" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C30" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/monitore/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D30" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E30" s="123" t="n"/>
+      <c r="F30" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="261" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C31" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-39gx950b-b</t>
+        </is>
+      </c>
+      <c r="D31" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E31" s="123" t="n"/>
+      <c r="F31" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="261" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C32" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/monitors/gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D32" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E32" s="123" t="n"/>
+      <c r="F32" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B · SUSPENDED</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="261" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C33" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-evo/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D33" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E33" s="123" t="n"/>
+      <c r="F33" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="261" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C34" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/outlet/outlet-informatica/monitores/39gx950b-b-outlet/</t>
+        </is>
+      </c>
+      <c r="D34" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E34" s="123" t="n"/>
+      <c r="F34" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="261" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C35" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/gaming/39GX950B-B/</t>
+        </is>
+      </c>
+      <c r="D35" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E35" s="123" t="n"/>
+      <c r="F35" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="261" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C36" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D36" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E36" s="123" t="n"/>
+      <c r="F36" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="261" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C37" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D37" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E37" s="123" t="n"/>
+      <c r="F37" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="261" t="inlineStr">
+        <is>
+          <t>HU : HU (hu)</t>
+        </is>
+      </c>
+      <c r="C38" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D38" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E38" s="123" t="n"/>
+      <c r="F38" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="261" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C39" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/gaming/39gx950b/</t>
+        </is>
+      </c>
+      <c r="D39" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E39" s="123" t="n"/>
+      <c r="F39" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="261" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C40" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D40" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E40" s="123" t="n"/>
+      <c r="F40" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C41" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D41" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E41" s="123" t="n"/>
+      <c r="F41" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C42" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-bajp/</t>
+        </is>
+      </c>
+      <c r="D42" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E42" s="123" t="n"/>
+      <c r="F42" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="261" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C43" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D43" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E43" s="123" t="n"/>
+      <c r="F43" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="261" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C44" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/gamer/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D44" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E44" s="123" t="n"/>
+      <c r="F44" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="261" t="inlineStr">
+        <is>
+          <t>PL : PL (pl)</t>
+        </is>
+      </c>
+      <c r="C45" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pl/monitory/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D45" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E45" s="123" t="n"/>
+      <c r="F45" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="261" t="inlineStr">
+        <is>
+          <t>SA : SA (ar)</t>
+        </is>
+      </c>
+      <c r="C46" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa/monitors/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D46" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E46" s="123" t="n"/>
+      <c r="F46" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="261" t="inlineStr">
+        <is>
+          <t>SA_EN : SA (en)</t>
+        </is>
+      </c>
+      <c r="C47" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa_en/monitors/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D47" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E47" s="123" t="n"/>
+      <c r="F47" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="261" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C48" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D48" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E48" s="123" t="n"/>
+      <c r="F48" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="261" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C49" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D49" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E49" s="123" t="n"/>
+      <c r="F49" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="261" t="inlineStr">
+        <is>
+          <t>TH : TH (th)</t>
+        </is>
+      </c>
+      <c r="C50" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/th/monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D50" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E50" s="123" t="n"/>
+      <c r="F50" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="261" t="inlineStr">
+        <is>
+          <t>TR : TR (tr)</t>
+        </is>
+      </c>
+      <c r="C51" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D51" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E51" s="123" t="n"/>
+      <c r="F51" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="261" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C52" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/monitors/ultragear-gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D52" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E52" s="123" t="n"/>
+      <c r="F52" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="261" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C53" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/gaming-monitor/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D53" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E53" s="123" t="n"/>
+      <c r="F53" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="261" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C54" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-32gx870b-b</t>
+        </is>
+      </c>
+      <c r="D54" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E54" s="123" t="n"/>
+      <c r="F54" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="261" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C55" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/gaming/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D55" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E55" s="123" t="n"/>
+      <c r="F55" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="261" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C56" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/gaming/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D56" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E56" s="123" t="n"/>
+      <c r="F56" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="261" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C57" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/gaming/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D57" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E57" s="123" t="n"/>
+      <c r="F57" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C58" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D58" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E58" s="123" t="n"/>
+      <c r="F58" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C59" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-bajp/</t>
+        </is>
+      </c>
+      <c r="D59" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E59" s="123" t="n"/>
+      <c r="F59" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="261" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C60" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/ultragear-gaming-oled/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D60" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E60" s="123" t="n"/>
+      <c r="F60" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="261" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C61" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D61" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E61" s="123" t="n"/>
+      <c r="F61" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="261" t="inlineStr">
+        <is>
+          <t>TR : TR (tr)</t>
+        </is>
+      </c>
+      <c r="C62" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/monitor/smart-monitorleri/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D62" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E62" s="123" t="n"/>
+      <c r="F62" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="261" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C63" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/gaming/45gx950b/</t>
+        </is>
+      </c>
+      <c r="D63" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E63" s="123" t="n"/>
+      <c r="F63" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="261" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C64" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/45gx950b/</t>
+        </is>
+      </c>
+      <c r="D64" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E64" s="123" t="n"/>
+      <c r="F64" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="261" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C65" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-45gx950b-b</t>
+        </is>
+      </c>
+      <c r="D65" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E65" s="123" t="n"/>
+      <c r="F65" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="261" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C66" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/gaming/45gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D66" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E66" s="123" t="n"/>
+      <c r="F66" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="261" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C67" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/gaming/45gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D67" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E67" s="123" t="n"/>
+      <c r="F67" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C68" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/45gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D68" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E68" s="123" t="n"/>
+      <c r="F68" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="261" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C69" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/45gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D69" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E69" s="123" t="n"/>
+      <c r="F69" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="261" t="inlineStr">
+        <is>
+          <t>TR : TR (tr)</t>
+        </is>
+      </c>
+      <c r="C70" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/45gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D70" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E70" s="123" t="n"/>
+      <c r="F70" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="261" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C71" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-gaming-ultragear/45gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D71" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E71" s="123" t="n"/>
+      <c r="F71" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="0" t="inlineStr">
+        <is>
+          <t>45GX950B</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(it): W28 UL Verified Eye Comfort GR 추가 (79 pages 작업중)
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -15,6 +15,7 @@
     <sheet name="W23 - 52G930B Feature 수정 건" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="W23 - UL인증 feature 삭제 1차" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="W28 - AI Upscaling Disclaimer" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="W28 - UL Verified Eye Comfort" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6414,6 +6415,2157 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G87"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="166" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="163" t="inlineStr">
+        <is>
+          <t>GR26-W28-IT-PDP-UL-Verified-Eye-Comfort-Feature-Upload</t>
+        </is>
+      </c>
+      <c r="C1" s="164" t="n"/>
+      <c r="D1" s="164" t="n"/>
+      <c r="E1" s="165" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" s="163" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · UL-Verified Eye Comfort Feature Upload (79 pages / 38 sites)</t>
+        </is>
+      </c>
+      <c r="C2" s="164" t="n"/>
+      <c r="D2" s="164" t="n"/>
+      <c r="E2" s="165" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="166" t="n"/>
+      <c r="B3" s="163" t="n"/>
+      <c r="C3" s="164" t="n"/>
+      <c r="D3" s="164" t="n"/>
+      <c r="E3" s="165" t="n"/>
+    </row>
+    <row r="5">
+      <c r="E5" s="127" t="n"/>
+    </row>
+    <row r="6">
+      <c r="E6" s="127" t="n"/>
+    </row>
+    <row r="7">
+      <c r="E7" s="127" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="283" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B8" s="283" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C8" s="283" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D8" s="283" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E8" s="283" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F8" s="283" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G8" s="283" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" s="203">
+      <c r="B9" s="261" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C9" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/monitors/ultragear-gaming/27gx700a-b-aau/</t>
+        </is>
+      </c>
+      <c r="D9" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E9" s="123" t="n"/>
+      <c r="F9" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="261" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C10" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D10" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E10" s="123" t="n"/>
+      <c r="F10" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="261" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C11" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D11" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E11" s="123" t="n"/>
+      <c r="F11" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="261" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C12" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/monitors/gaming-monitors/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D12" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E12" s="123" t="n"/>
+      <c r="F12" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="261" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C13" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D13" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E13" s="123" t="n"/>
+      <c r="F13" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="261" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C14" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/business/moniteurs/moniteurs-de-jeu/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D14" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E14" s="123" t="n"/>
+      <c r="F14" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="261" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C15" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D15" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E15" s="123" t="n"/>
+      <c r="F15" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="261" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C16" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/monitore/gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D16" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E16" s="123" t="n"/>
+      <c r="F16" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="261" t="inlineStr">
+        <is>
+          <t>DK : DK (da)</t>
+        </is>
+      </c>
+      <c r="C17" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/dk/skaerme/ultragear-gamerskaerme/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D17" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E17" s="123" t="n"/>
+      <c r="F17" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="261" t="inlineStr">
+        <is>
+          <t>FI : FI (fi)</t>
+        </is>
+      </c>
+      <c r="C18" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fi/naytot/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D18" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E18" s="123" t="n"/>
+      <c r="F18" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="261" t="inlineStr">
+        <is>
+          <t>GR : GR (el)</t>
+        </is>
+      </c>
+      <c r="C19" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/gr/othones/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D19" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E19" s="123" t="n"/>
+      <c r="F19" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="261" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C20" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D20" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E20" s="123" t="n"/>
+      <c r="F20" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="261" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C21" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D21" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E21" s="123" t="n"/>
+      <c r="F21" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="261" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C22" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D22" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E22" s="123" t="n"/>
+      <c r="F22" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="261" t="inlineStr">
+        <is>
+          <t>HU : HU (hu)</t>
+        </is>
+      </c>
+      <c r="C23" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-monitor/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D23" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E23" s="123" t="n"/>
+      <c r="F23" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="261" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C24" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D24" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E24" s="123" t="n"/>
+      <c r="F24" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="261" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C25" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D25" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E25" s="123" t="n"/>
+      <c r="F25" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="261" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C26" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/monitor/gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D26" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E26" s="123" t="n"/>
+      <c r="F26" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C27" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D27" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E27" s="123" t="n"/>
+      <c r="F27" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="261" t="inlineStr">
+        <is>
+          <t>KZ : KZ (ru)</t>
+        </is>
+      </c>
+      <c r="C28" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/kz/monitors/gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D28" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E28" s="123" t="n"/>
+      <c r="F28" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="261" t="inlineStr">
+        <is>
+          <t>NO : NO (no)</t>
+        </is>
+      </c>
+      <c r="C29" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/no/skjermer/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D29" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E29" s="123" t="n"/>
+      <c r="F29" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="261" t="inlineStr">
+        <is>
+          <t>PL : PL (pl)</t>
+        </is>
+      </c>
+      <c r="C30" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pl/monitory/ultragear-gaming/27gx700a/</t>
+        </is>
+      </c>
+      <c r="D30" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E30" s="123" t="n"/>
+      <c r="F30" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="261" t="inlineStr">
+        <is>
+          <t>RO : RO (ro)</t>
+        </is>
+      </c>
+      <c r="C31" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ro/monitoare/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D31" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E31" s="123" t="n"/>
+      <c r="F31" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="261" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C32" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D32" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E32" s="123" t="n"/>
+      <c r="F32" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="261" t="inlineStr">
+        <is>
+          <t>RU : RU (ru)</t>
+        </is>
+      </c>
+      <c r="C33" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ru/monitors/lg-27gx700a-b</t>
+        </is>
+      </c>
+      <c r="D33" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E33" s="123" t="n"/>
+      <c r="F33" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="261" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C34" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D34" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E34" s="123" t="n"/>
+      <c r="F34" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="261" t="inlineStr">
+        <is>
+          <t>TR : TR (tr)</t>
+        </is>
+      </c>
+      <c r="C35" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/monitor/oyun-monitorleri/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D35" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E35" s="123" t="n"/>
+      <c r="F35" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="261" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C36" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/gaming/27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D36" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E36" s="123" t="n"/>
+      <c r="F36" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="261" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C37" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/gaming/27gx700a-b-27gx001-pck-uk-c/</t>
+        </is>
+      </c>
+      <c r="D37" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E37" s="123" t="n"/>
+      <c r="F37" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="261" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C38" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/gaming/lg-27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D38" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E38" s="123" t="n"/>
+      <c r="F38" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>27GX700A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="261" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C39" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-27gx790b-b</t>
+        </is>
+      </c>
+      <c r="D39" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E39" s="123" t="n"/>
+      <c r="F39" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="261" t="inlineStr">
+        <is>
+          <t>AE_AR : AE (ar)</t>
+        </is>
+      </c>
+      <c r="C40" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae_ar/consumer-monitors/lg-27gx790b-b</t>
+        </is>
+      </c>
+      <c r="D40" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E40" s="123" t="n"/>
+      <c r="F40" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="261" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C41" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/monitors/ultragear-gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D41" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E41" s="123" t="n"/>
+      <c r="F41" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="261" t="inlineStr">
+        <is>
+          <t>BE_FR : BE (fr)</t>
+        </is>
+      </c>
+      <c r="C42" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/be_fr/moniteurs/lg-27gx790b-b</t>
+        </is>
+      </c>
+      <c r="D42" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E42" s="123" t="n"/>
+      <c r="F42" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="261" t="inlineStr">
+        <is>
+          <t>BR : BR (pt)</t>
+        </is>
+      </c>
+      <c r="C43" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/br/monitores/monitores-ultragear-oled/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D43" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E43" s="123" t="n"/>
+      <c r="F43" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="261" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C44" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D44" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E44" s="123" t="n"/>
+      <c r="F44" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="261" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C45" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D45" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E45" s="123" t="n"/>
+      <c r="F45" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="261" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C46" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27gx790b-b</t>
+        </is>
+      </c>
+      <c r="D46" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E46" s="123" t="n"/>
+      <c r="F46" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="261" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C47" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/monitore/gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D47" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E47" s="123" t="n"/>
+      <c r="F47" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="261" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C48" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-oled-gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D48" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E48" s="123" t="n"/>
+      <c r="F48" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="261" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C49" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/gaming/lg-27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D49" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E49" s="123" t="n"/>
+      <c r="F49" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="261" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C50" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/lg-27gx790b-b-27g411a-bundle/</t>
+        </is>
+      </c>
+      <c r="D50" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E50" s="123" t="n"/>
+      <c r="F50" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="261" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C51" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D51" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E51" s="123" t="n"/>
+      <c r="F51" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="261" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C52" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D52" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E52" s="123" t="n"/>
+      <c r="F52" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C53" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D53" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E53" s="123" t="n"/>
+      <c r="F53" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="261" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C54" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-oled/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D54" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E54" s="123" t="n"/>
+      <c r="F54" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="261" t="inlineStr">
+        <is>
+          <t>PL : PL (pl)</t>
+        </is>
+      </c>
+      <c r="C55" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pl/monitory/ultragear-gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D55" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E55" s="123" t="n"/>
+      <c r="F55" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="261" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C56" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D56" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E56" s="123" t="n"/>
+      <c r="F56" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="261" t="inlineStr">
+        <is>
+          <t>TR : TR (tr)</t>
+        </is>
+      </c>
+      <c r="C57" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D57" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E57" s="123" t="n"/>
+      <c r="F57" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="261" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C58" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D58" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E58" s="123" t="n"/>
+      <c r="F58" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="261" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C59" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/gaming/27gx790b-b-27g640a/</t>
+        </is>
+      </c>
+      <c r="D59" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E59" s="123" t="n"/>
+      <c r="F59" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="261" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C60" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-gaming-oled-ultragear-oled/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D60" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E60" s="123" t="n"/>
+      <c r="F60" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="261" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C61" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/gamer/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D61" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E61" s="123" t="n"/>
+      <c r="F61" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="0" t="inlineStr">
+        <is>
+          <t>27GX790B</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="261" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C62" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-32gx870b-b</t>
+        </is>
+      </c>
+      <c r="D62" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E62" s="123" t="n"/>
+      <c r="F62" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C63" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D63" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E63" s="123" t="n"/>
+      <c r="F63" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="261" t="inlineStr">
+        <is>
+          <t>TR : TR (tr)</t>
+        </is>
+      </c>
+      <c r="C64" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/monitors/32gx870b-b/</t>
+        </is>
+      </c>
+      <c r="D64" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E64" s="123" t="n"/>
+      <c r="F64" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C65" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-bajp/</t>
+        </is>
+      </c>
+      <c r="D65" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E65" s="123" t="n"/>
+      <c r="F65" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="0" t="inlineStr">
+        <is>
+          <t>32GX870B</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="261" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C66" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/monitors/ultragear-gaming/39gx950b/</t>
+        </is>
+      </c>
+      <c r="D66" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E66" s="123" t="n"/>
+      <c r="F66" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="261" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C67" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D67" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E67" s="123" t="n"/>
+      <c r="F67" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="261" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C68" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D68" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E68" s="123" t="n"/>
+      <c r="F68" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="261" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C69" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-39gx950b-b</t>
+        </is>
+      </c>
+      <c r="D69" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E69" s="123" t="n"/>
+      <c r="F69" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="261" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C70" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/monitore/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D70" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E70" s="123" t="n"/>
+      <c r="F70" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="261" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C71" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-evo/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D71" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E71" s="123" t="n"/>
+      <c r="F71" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="261" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C72" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/gaming/39GX950B-B/</t>
+        </is>
+      </c>
+      <c r="D72" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E72" s="123" t="n"/>
+      <c r="F72" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="261" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C73" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D73" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E73" s="123" t="n"/>
+      <c r="F73" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="261" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C74" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D74" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E74" s="123" t="n"/>
+      <c r="F74" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="261" t="inlineStr">
+        <is>
+          <t>HU : HU (hu)</t>
+        </is>
+      </c>
+      <c r="C75" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D75" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E75" s="123" t="n"/>
+      <c r="F75" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="261" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C76" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D76" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E76" s="123" t="n"/>
+      <c r="F76" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C77" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D77" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E77" s="123" t="n"/>
+      <c r="F77" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C78" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-bajp/</t>
+        </is>
+      </c>
+      <c r="D78" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E78" s="123" t="n"/>
+      <c r="F78" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="261" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C79" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D79" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E79" s="123" t="n"/>
+      <c r="F79" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="261" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C80" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D80" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E80" s="123" t="n"/>
+      <c r="F80" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="261" t="inlineStr">
+        <is>
+          <t>PL : PL (pl)</t>
+        </is>
+      </c>
+      <c r="C81" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pl/monitory/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D81" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E81" s="123" t="n"/>
+      <c r="F81" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="261" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C82" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D82" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E82" s="123" t="n"/>
+      <c r="F82" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="261" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C83" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D83" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E83" s="123" t="n"/>
+      <c r="F83" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="261" t="inlineStr">
+        <is>
+          <t>TH : TH (th)</t>
+        </is>
+      </c>
+      <c r="C84" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/th/monitors/gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D84" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E84" s="123" t="n"/>
+      <c r="F84" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="261" t="inlineStr">
+        <is>
+          <t>TR : TR (tr)</t>
+        </is>
+      </c>
+      <c r="C85" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D85" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E85" s="123" t="n"/>
+      <c r="F85" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="261" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C86" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/monitors/ultragear-gaming/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D86" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E86" s="123" t="n"/>
+      <c r="F86" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="261" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C87" s="261" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/gaming-monitor/39gx950b-b/</t>
+        </is>
+      </c>
+      <c r="D87" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E87" s="123" t="n"/>
+      <c r="F87" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="0" t="inlineStr">
+        <is>
+          <t>39GX950B</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(it): Readiness Ready/Not Ready 표기·W28 중복행 Remark 구분 백포트 (v0.6.36)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -5158,7 +5158,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>39GX950B · Consumer (URL 404 — 재확인 필요)</t>
         </is>
       </c>
     </row>
@@ -5184,7 +5184,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>39GX950B · Business (URL 404 — 재확인 필요)</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>39GX950B · Outlet</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>39GX950B (B)</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5652,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>39GX950B (BAJP)</t>
         </is>
       </c>
     </row>
@@ -6068,7 +6068,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>32GX870B</t>
+          <t>32GX870B (B)</t>
         </is>
       </c>
     </row>
@@ -6094,7 +6094,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>32GX870B</t>
+          <t>32GX870B (BAJP)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): GR26-W25 Copilot+ Hero Banner 신규 등록 — B2C 14·B2B 7 (완료 10·작업중 11)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -14,8 +14,9 @@
     <sheet name="W23 - 39GX950B 이미지 수정 2차" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="W23 - 52G930B Feature 수정 건" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="W23 - UL인증 feature 삭제 1차" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="W28 - AI Upscaling Disclaimer" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="W28 - UL Verified Eye Comfort" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="W25 - Copilot+ Hero Banner" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="W28 - AI Upscaling Disclaimer" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="W28 - UL Verified Eye Comfort" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4683,6 +4684,606 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GR26-W25-Request to add Copilot+ Hero Banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · Copilot+ Hero Banner (B2C 완료 10 · 작업중 4 · B2B 작업중 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/ordinateurs-portables/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/laptops</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/laptops/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/pc-portables/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/laptop/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/pcs/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/business/san-pham-tin-hoc/laptop</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/business/computers/laptops/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/business/informatique/pc-portables-professionnels/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -6415,7 +7016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>

</xml_diff>

<commit_message>
data(it): W28 AI Upscaling — EE(Estonia) 행 삭제·ES(SUSPENDED) 완료 처리, 잔여 작업중 0
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -4691,586 +4691,586 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>GR26-W25-Request to add Copilot+ Hero Banner</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>이번주 추가</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>금주 신규 등록 · Copilot+ Hero Banner (B2C 완료 10 · 작업중 4 · B2B 작업중 7)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>완료일</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="0" t="inlineStr">
         <is>
           <t>Page#</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="0" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/laptops/</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>CA_FR : CA (fr)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_fr/ordinateurs-portables/</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/laptops</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="F6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/notebook/</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="F7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>UK : GB (en)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/uk/laptops/</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/notebooks</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>FR : FR (fr)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/fr/pc-portables/</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>AU : AU (en)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/au/laptops/</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>IN : IN (en)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/in/laptop/</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>JP : JP (ja)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/jp/mobile-pc/</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>CN : CN (zh)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/cn/notebooks</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="F14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/laptops/</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>VN : VN (vi)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/vn/laptop-lg-gram/</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="F16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>TW : TW (zh)</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/tw/laptops/</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>GLOBAL : GLOBAL (en)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/global/business/monitors-pcs/pcs/</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="F18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/business/it-products/lg-gram/</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="F19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>VN : VN (vi)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/vn/business/san-pham-tin-hoc/laptop</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="F20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>IN : IN (en)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/in/business/computers/laptops/</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="F21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="F22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="F23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>FR : FR (fr)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/fr/business/informatique/pc-portables-professionnels/</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="F24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
@@ -5287,7 +5287,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -5313,7 +5313,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>W29 신규 완료(27GM950B·39GX950B·32GX870B·45GX950B 로케일 다수) · AE 39GX950B(Consumer/Business) URL 404 취소</t>
+          <t>W29 신규 완료(27GM950B·39GX950B·32GX870B·45GX950B) · AE 4건 URL 404 취소 · EE 대상 제외 · ES(SUSPENDED 포함) 완료 — 잔여 작업중 0</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -5948,17 +5948,17 @@
     <row r="31">
       <c r="B31" s="261" t="inlineStr">
         <is>
-          <t>EE : EE (et)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C31" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ee/monitorid/lg-39gx950b-b</t>
+          <t>https://www.lg.com/es/monitors/gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D31" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E31" s="123" t="n"/>
@@ -5967,7 +5967,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>39GX950B · SUSPENDED</t>
         </is>
       </c>
     </row>
@@ -5979,12 +5979,12 @@
       </c>
       <c r="C32" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/monitors/gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-evo/39gx950b-b/</t>
         </is>
       </c>
       <c r="D32" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E32" s="123" t="n"/>
@@ -5993,7 +5993,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>39GX950B · SUSPENDED</t>
+          <t>39GX950B</t>
         </is>
       </c>
     </row>
@@ -6005,7 +6005,7 @@
       </c>
       <c r="C33" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/monitores/monitores-ultragear-evo/39gx950b-b/</t>
+          <t>https://www.lg.com/es/outlet/outlet-informatica/monitores/39gx950b-b-outlet/</t>
         </is>
       </c>
       <c r="D33" s="264" t="inlineStr">
@@ -6019,19 +6019,19 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>39GX950B · Outlet</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="261" t="inlineStr">
         <is>
-          <t>ES : ES (es)</t>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C34" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/outlet/outlet-informatica/monitores/39gx950b-b-outlet/</t>
+          <t>https://www.lg.com/fr/moniteurs/gaming/39GX950B-B/</t>
         </is>
       </c>
       <c r="D34" s="264" t="inlineStr">
@@ -6045,19 +6045,19 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>39GX950B · Outlet</t>
+          <t>39GX950B</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="261" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C35" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr/moniteurs/gaming/39GX950B-B/</t>
+          <t>https://www.lg.com/hk/monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D35" s="264" t="inlineStr">
@@ -6078,12 +6078,12 @@
     <row r="36">
       <c r="B36" s="261" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C36" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/hk_en/monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D36" s="264" t="inlineStr">
@@ -6104,12 +6104,12 @@
     <row r="37">
       <c r="B37" s="261" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>HU : HU (hu)</t>
         </is>
       </c>
       <c r="C37" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D37" s="264" t="inlineStr">
@@ -6130,12 +6130,12 @@
     <row r="38">
       <c r="B38" s="261" t="inlineStr">
         <is>
-          <t>HU : HU (hu)</t>
+          <t>ID : ID (in)</t>
         </is>
       </c>
       <c r="C38" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/id/monitor/gaming/39gx950b/</t>
         </is>
       </c>
       <c r="D38" s="264" t="inlineStr">
@@ -6156,12 +6156,12 @@
     <row r="39">
       <c r="B39" s="261" t="inlineStr">
         <is>
-          <t>ID : ID (in)</t>
+          <t>IT : IT (it)</t>
         </is>
       </c>
       <c r="C39" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/id/monitor/gaming/39gx950b/</t>
+          <t>https://www.lg.com/it/monitor/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D39" s="264" t="inlineStr">
@@ -6182,12 +6182,12 @@
     <row r="40">
       <c r="B40" s="261" t="inlineStr">
         <is>
-          <t>IT : IT (it)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C40" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/it/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-b/</t>
         </is>
       </c>
       <c r="D40" s="264" t="inlineStr">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>39GX950B (B)</t>
         </is>
       </c>
     </row>
@@ -6213,7 +6213,7 @@
       </c>
       <c r="C41" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-bajp/</t>
         </is>
       </c>
       <c r="D41" s="264" t="inlineStr">
@@ -6227,19 +6227,19 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>39GX950B (B)</t>
+          <t>39GX950B (BAJP)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>NL : NL (nl)</t>
         </is>
       </c>
       <c r="C42" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-bajp/</t>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/39gx950b-b/</t>
         </is>
       </c>
       <c r="D42" s="264" t="inlineStr">
@@ -6253,19 +6253,19 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>39GX950B (BAJP)</t>
+          <t>39GX950B</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="261" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
+          <t>PE : PE (es)</t>
         </is>
       </c>
       <c r="C43" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/39gx950b-b/</t>
+          <t>https://www.lg.com/pe/monitores/gamer/39gx950b-b/</t>
         </is>
       </c>
       <c r="D43" s="264" t="inlineStr">
@@ -6286,12 +6286,12 @@
     <row r="44">
       <c r="B44" s="261" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>PL : PL (pl)</t>
         </is>
       </c>
       <c r="C44" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe/monitores/gamer/39gx950b-b/</t>
+          <t>https://www.lg.com/pl/monitory/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D44" s="264" t="inlineStr">
@@ -6312,12 +6312,12 @@
     <row r="45">
       <c r="B45" s="261" t="inlineStr">
         <is>
-          <t>PL : PL (pl)</t>
+          <t>SA : SA (ar)</t>
         </is>
       </c>
       <c r="C45" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pl/monitory/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/sa/monitors/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D45" s="264" t="inlineStr">
@@ -6338,12 +6338,12 @@
     <row r="46">
       <c r="B46" s="261" t="inlineStr">
         <is>
-          <t>SA : SA (ar)</t>
+          <t>SA_EN : SA (en)</t>
         </is>
       </c>
       <c r="C46" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa/monitors/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/sa_en/monitors/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D46" s="264" t="inlineStr">
@@ -6364,12 +6364,12 @@
     <row r="47">
       <c r="B47" s="261" t="inlineStr">
         <is>
-          <t>SA_EN : SA (en)</t>
+          <t>SE : SE (sv)</t>
         </is>
       </c>
       <c r="C47" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa_en/monitors/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D47" s="264" t="inlineStr">
@@ -6390,12 +6390,12 @@
     <row r="48">
       <c r="B48" s="261" t="inlineStr">
         <is>
-          <t>SE : SE (sv)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C48" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/se/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D48" s="264" t="inlineStr">
@@ -6416,12 +6416,12 @@
     <row r="49">
       <c r="B49" s="261" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>TH : TH (th)</t>
         </is>
       </c>
       <c r="C49" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/consumer-monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/th/monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D49" s="264" t="inlineStr">
@@ -6442,12 +6442,12 @@
     <row r="50">
       <c r="B50" s="261" t="inlineStr">
         <is>
-          <t>TH : TH (th)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C50" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/th/monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D50" s="264" t="inlineStr">
@@ -6468,12 +6468,12 @@
     <row r="51">
       <c r="B51" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>TW : TW (zh)</t>
         </is>
       </c>
       <c r="C51" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/tw/monitors/ultragear-gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D51" s="264" t="inlineStr">
@@ -6494,12 +6494,12 @@
     <row r="52">
       <c r="B52" s="261" t="inlineStr">
         <is>
-          <t>TW : TW (zh)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C52" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tw/monitors/ultragear-gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/uk/monitors/gaming-monitor/39gx950b-b/</t>
         </is>
       </c>
       <c r="D52" s="264" t="inlineStr">
@@ -6520,12 +6520,12 @@
     <row r="53">
       <c r="B53" s="261" t="inlineStr">
         <is>
-          <t>UK : GB (en)</t>
+          <t>CN : CN (zh)</t>
         </is>
       </c>
       <c r="C53" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/monitors/gaming-monitor/39gx950b-b/</t>
+          <t>https://www.lg.com/cn/monitors/lg-32gx870b-b</t>
         </is>
       </c>
       <c r="D53" s="264" t="inlineStr">
@@ -6539,19 +6539,19 @@
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>39GX950B</t>
+          <t>32GX870B</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="261" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>CO : CO (es)</t>
         </is>
       </c>
       <c r="C54" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/monitors/lg-32gx870b-b</t>
+          <t>https://www.lg.com/co/monitores/gaming/32gx870b-b/</t>
         </is>
       </c>
       <c r="D54" s="264" t="inlineStr">
@@ -6572,12 +6572,12 @@
     <row r="55">
       <c r="B55" s="261" t="inlineStr">
         <is>
-          <t>CO : CO (es)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C55" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/co/monitores/gaming/32gx870b-b/</t>
+          <t>https://www.lg.com/hk/monitors/gaming/32gx870b-b/</t>
         </is>
       </c>
       <c r="D55" s="264" t="inlineStr">
@@ -6598,12 +6598,12 @@
     <row r="56">
       <c r="B56" s="261" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C56" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/monitors/gaming/32gx870b-b/</t>
+          <t>https://www.lg.com/hk_en/monitors/gaming/32gx870b-b/</t>
         </is>
       </c>
       <c r="D56" s="264" t="inlineStr">
@@ -6624,12 +6624,12 @@
     <row r="57">
       <c r="B57" s="261" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C57" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/monitors/gaming/32gx870b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-b/</t>
         </is>
       </c>
       <c r="D57" s="264" t="inlineStr">
@@ -6643,7 +6643,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>32GX870B</t>
+          <t>32GX870B (B)</t>
         </is>
       </c>
     </row>
@@ -6655,7 +6655,7 @@
       </c>
       <c r="C58" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-bajp/</t>
         </is>
       </c>
       <c r="D58" s="264" t="inlineStr">
@@ -6669,19 +6669,19 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>32GX870B (B)</t>
+          <t>32GX870B (BAJP)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>PE : PE (es)</t>
         </is>
       </c>
       <c r="C59" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-bajp/</t>
+          <t>https://www.lg.com/pe/monitores/ultragear-gaming-oled/32gx870b-b/</t>
         </is>
       </c>
       <c r="D59" s="264" t="inlineStr">
@@ -6695,19 +6695,19 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>32GX870B (BAJP)</t>
+          <t>32GX870B</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="261" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C60" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe/monitores/ultragear-gaming-oled/32gx870b-b/</t>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/32gx870b-b/</t>
         </is>
       </c>
       <c r="D60" s="264" t="inlineStr">
@@ -6728,12 +6728,12 @@
     <row r="61">
       <c r="B61" s="261" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C61" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/consumer-monitors/gaming/32gx870b-b/</t>
+          <t>https://www.lg.com/tr/monitor/smart-monitorleri/32gx870b-b/</t>
         </is>
       </c>
       <c r="D61" s="264" t="inlineStr">
@@ -6754,12 +6754,12 @@
     <row r="62">
       <c r="B62" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C62" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/monitor/smart-monitorleri/32gx870b-b/</t>
+          <t>https://www.lg.com/ca_en/monitors/gaming/45gx950b/</t>
         </is>
       </c>
       <c r="D62" s="264" t="inlineStr">
@@ -6773,19 +6773,19 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>32GX870B</t>
+          <t>45GX950B</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" s="261" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C63" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/monitors/gaming/45gx950b/</t>
+          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/45gx950b/</t>
         </is>
       </c>
       <c r="D63" s="264" t="inlineStr">
@@ -6806,12 +6806,12 @@
     <row r="64">
       <c r="B64" s="261" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>CN : CN (zh)</t>
         </is>
       </c>
       <c r="C64" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/45gx950b/</t>
+          <t>https://www.lg.com/cn/monitors/lg-45gx950b-b</t>
         </is>
       </c>
       <c r="D64" s="264" t="inlineStr">
@@ -6832,12 +6832,12 @@
     <row r="65">
       <c r="B65" s="261" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C65" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/monitors/lg-45gx950b-b</t>
+          <t>https://www.lg.com/hk/monitors/gaming/45gx950b-b/</t>
         </is>
       </c>
       <c r="D65" s="264" t="inlineStr">
@@ -6858,12 +6858,12 @@
     <row r="66">
       <c r="B66" s="261" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C66" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/monitors/gaming/45gx950b-b/</t>
+          <t>https://www.lg.com/hk_en/monitors/gaming/45gx950b-b/</t>
         </is>
       </c>
       <c r="D66" s="264" t="inlineStr">
@@ -6884,12 +6884,12 @@
     <row r="67">
       <c r="B67" s="261" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C67" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/monitors/gaming/45gx950b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/45gx950b-b/</t>
         </is>
       </c>
       <c r="D67" s="264" t="inlineStr">
@@ -6910,12 +6910,12 @@
     <row r="68">
       <c r="B68" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C68" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/45gx950b-b/</t>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/45gx950b-b/</t>
         </is>
       </c>
       <c r="D68" s="264" t="inlineStr">
@@ -6936,12 +6936,12 @@
     <row r="69">
       <c r="B69" s="261" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C69" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/consumer-monitors/gaming/45gx950b-b/</t>
+          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/45gx950b-b/</t>
         </is>
       </c>
       <c r="D69" s="264" t="inlineStr">
@@ -6962,12 +6962,12 @@
     <row r="70">
       <c r="B70" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>VN : VN (vi)</t>
         </is>
       </c>
       <c r="C70" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/45gx950b-b/</t>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-gaming-ultragear/45gx950b-b/</t>
         </is>
       </c>
       <c r="D70" s="264" t="inlineStr">
@@ -6980,32 +6980,6 @@
         <v>1</v>
       </c>
       <c r="G70" s="0" t="inlineStr">
-        <is>
-          <t>45GX950B</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="261" t="inlineStr">
-        <is>
-          <t>VN : VN (vi)</t>
-        </is>
-      </c>
-      <c r="C71" s="261" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-gaming-ultragear/45gx950b-b/</t>
-        </is>
-      </c>
-      <c r="D71" s="264" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E71" s="123" t="n"/>
-      <c r="F71" s="123" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" s="0" t="inlineStr">
         <is>
           <t>45GX950B</t>
         </is>

</xml_diff>

<commit_message>
data(it): W17 GNB Structure — IN(인도) 법인리뷰→완료 (7/16 게시 7건, PTT 0721 확인)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -10701,7 +10701,8 @@
       <c r="B2" s="163" t="inlineStr">
         <is>
           <t>CZ : 작업중 → 완료
-TR : 법인리뷰 → 작업중</t>
+TR : 법인리뷰 → 작업중
+IN : 법인리뷰 → 완료 (7/16 게시, PTT 확인)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -11241,10 +11242,14 @@
       </c>
       <c r="D29" s="263" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E29" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E29" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
       <c r="F29" s="123" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
data(it): W28 UL Verified 전건 완료(작업중 40→완료) + CA business 2행 삭제 — 75완료·2취소, 100%
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -6996,7 +6996,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -7022,7 +7022,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>W29 신규 완료 35건(27GX700A·27GX790B 로케일 다수) · URL 404·에러 2건 취소(27GX790B PE, 32GX870B TR)</t>
+          <t>W30 전건 작업 완료 — 잔여 작업중 0 · 취소 2건(27GX790B PE 404·32GX870B TR 에러) 유지 · CA business 2행 대상 제외(삭제)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -7036,6 +7036,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -7121,7 +7122,7 @@
       </c>
       <c r="D10" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E10" s="123" t="n"/>
@@ -7163,17 +7164,17 @@
     <row r="12">
       <c r="B12" s="261" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C12" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/business/monitors/gaming-monitors/27gx700a-b/</t>
+          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/27gx700a-b/</t>
         </is>
       </c>
       <c r="D12" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E12" s="123" t="n"/>
@@ -7189,12 +7190,12 @@
     <row r="13">
       <c r="B13" s="261" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>CN : CN (zh)</t>
         </is>
       </c>
       <c r="C13" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/27gx700a-b/</t>
+          <t>https://www.lg.com/cn/monitors/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D13" s="264" t="inlineStr">
@@ -7215,17 +7216,17 @@
     <row r="14">
       <c r="B14" s="261" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C14" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/business/moniteurs/moniteurs-de-jeu/27gx700a-b/</t>
+          <t>https://www.lg.com/de/monitore/gaming/27gx700a-b/</t>
         </is>
       </c>
       <c r="D14" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E14" s="123" t="n"/>
@@ -7241,17 +7242,17 @@
     <row r="15">
       <c r="B15" s="261" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>DK : DK (da)</t>
         </is>
       </c>
       <c r="C15" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/monitors/lg-27gx700a-b</t>
+          <t>https://www.lg.com/dk/skaerme/ultragear-gamerskaerme/27gx700a-b/</t>
         </is>
       </c>
       <c r="D15" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E15" s="123" t="n"/>
@@ -7267,12 +7268,12 @@
     <row r="16">
       <c r="B16" s="261" t="inlineStr">
         <is>
-          <t>DE : DE (de)</t>
+          <t>FI : FI (fi)</t>
         </is>
       </c>
       <c r="C16" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de/monitore/gaming/27gx700a-b/</t>
+          <t>https://www.lg.com/fi/naytot/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D16" s="264" t="inlineStr">
@@ -7293,12 +7294,12 @@
     <row r="17">
       <c r="B17" s="261" t="inlineStr">
         <is>
-          <t>DK : DK (da)</t>
+          <t>GR : GR (el)</t>
         </is>
       </c>
       <c r="C17" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/dk/skaerme/ultragear-gamerskaerme/27gx700a-b/</t>
+          <t>https://www.lg.com/gr/othones/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D17" s="264" t="inlineStr">
@@ -7319,17 +7320,17 @@
     <row r="18">
       <c r="B18" s="261" t="inlineStr">
         <is>
-          <t>FI : FI (fi)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C18" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fi/naytot/lg-27gx700a-b</t>
+          <t>https://www.lg.com/hk/monitors/gaming/27gx700a-b/</t>
         </is>
       </c>
       <c r="D18" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E18" s="123" t="n"/>
@@ -7345,17 +7346,17 @@
     <row r="19">
       <c r="B19" s="261" t="inlineStr">
         <is>
-          <t>GR : GR (el)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C19" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/gr/othones/lg-27gx700a-b</t>
+          <t>https://www.lg.com/hk_en/monitors/gaming/27gx700a-b/</t>
         </is>
       </c>
       <c r="D19" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E19" s="123" t="n"/>
@@ -7371,12 +7372,12 @@
     <row r="20">
       <c r="B20" s="261" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>HR : HR (hr)</t>
         </is>
       </c>
       <c r="C20" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/monitors/gaming/27gx700a-b/</t>
+          <t>https://www.lg.com/hr/monitori/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D20" s="264" t="inlineStr">
@@ -7397,12 +7398,12 @@
     <row r="21">
       <c r="B21" s="261" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>HU : HU (hu)</t>
         </is>
       </c>
       <c r="C21" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/monitors/gaming/27gx700a-b/</t>
+          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-monitor/27gx700a-b/</t>
         </is>
       </c>
       <c r="D21" s="264" t="inlineStr">
@@ -7423,17 +7424,17 @@
     <row r="22">
       <c r="B22" s="261" t="inlineStr">
         <is>
-          <t>HR : HR (hr)</t>
+          <t>ID : ID (in)</t>
         </is>
       </c>
       <c r="C22" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hr/monitori/lg-27gx700a-b</t>
+          <t>https://www.lg.com/id/monitor/gaming/27gx700a-b/</t>
         </is>
       </c>
       <c r="D22" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E22" s="123" t="n"/>
@@ -7449,12 +7450,12 @@
     <row r="23">
       <c r="B23" s="261" t="inlineStr">
         <is>
-          <t>HU : HU (hu)</t>
+          <t>IL : IL (iw)</t>
         </is>
       </c>
       <c r="C23" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-monitor/27gx700a-b/</t>
+          <t>https://www.lg.com/il/monitors/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D23" s="264" t="inlineStr">
@@ -7475,12 +7476,12 @@
     <row r="24">
       <c r="B24" s="261" t="inlineStr">
         <is>
-          <t>ID : ID (in)</t>
+          <t>IT : IT (it)</t>
         </is>
       </c>
       <c r="C24" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/id/monitor/gaming/27gx700a-b/</t>
+          <t>https://www.lg.com/it/monitor/gaming/27gx700a-b/</t>
         </is>
       </c>
       <c r="D24" s="264" t="inlineStr">
@@ -7501,17 +7502,17 @@
     <row r="25">
       <c r="B25" s="261" t="inlineStr">
         <is>
-          <t>IL : IL (iw)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C25" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/il/monitors/lg-27gx700a-b</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/27gx700a-b/</t>
         </is>
       </c>
       <c r="D25" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E25" s="123" t="n"/>
@@ -7527,12 +7528,12 @@
     <row r="26">
       <c r="B26" s="261" t="inlineStr">
         <is>
-          <t>IT : IT (it)</t>
+          <t>KZ : KZ (ru)</t>
         </is>
       </c>
       <c r="C26" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/it/monitor/gaming/27gx700a-b/</t>
+          <t>https://www.lg.com/kz/monitors/gaming/27gx700a-b/</t>
         </is>
       </c>
       <c r="D26" s="264" t="inlineStr">
@@ -7553,17 +7554,17 @@
     <row r="27">
       <c r="B27" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>NO : NO (no)</t>
         </is>
       </c>
       <c r="C27" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/27gx700a-b/</t>
+          <t>https://www.lg.com/no/skjermer/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D27" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E27" s="123" t="n"/>
@@ -7579,12 +7580,12 @@
     <row r="28">
       <c r="B28" s="261" t="inlineStr">
         <is>
-          <t>KZ : KZ (ru)</t>
+          <t>PL : PL (pl)</t>
         </is>
       </c>
       <c r="C28" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/kz/monitors/gaming/27gx700a-b/</t>
+          <t>https://www.lg.com/pl/monitory/ultragear-gaming/27gx700a/</t>
         </is>
       </c>
       <c r="D28" s="264" t="inlineStr">
@@ -7605,17 +7606,17 @@
     <row r="29">
       <c r="B29" s="261" t="inlineStr">
         <is>
-          <t>NO : NO (no)</t>
+          <t>RO : RO (ro)</t>
         </is>
       </c>
       <c r="C29" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/no/skjermer/lg-27gx700a-b</t>
+          <t>https://www.lg.com/ro/monitoare/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D29" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E29" s="123" t="n"/>
@@ -7631,12 +7632,12 @@
     <row r="30">
       <c r="B30" s="261" t="inlineStr">
         <is>
-          <t>PL : PL (pl)</t>
+          <t>RS : RS (sr)</t>
         </is>
       </c>
       <c r="C30" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pl/monitory/ultragear-gaming/27gx700a/</t>
+          <t>https://www.lg.com/rs/monitori/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D30" s="264" t="inlineStr">
@@ -7657,17 +7658,17 @@
     <row r="31">
       <c r="B31" s="261" t="inlineStr">
         <is>
-          <t>RO : RO (ro)</t>
+          <t>RU : RU (ru)</t>
         </is>
       </c>
       <c r="C31" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ro/monitoare/lg-27gx700a-b</t>
+          <t>https://www.lg.com/ru/monitors/lg-27gx700a-b</t>
         </is>
       </c>
       <c r="D31" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E31" s="123" t="n"/>
@@ -7683,17 +7684,17 @@
     <row r="32">
       <c r="B32" s="261" t="inlineStr">
         <is>
-          <t>RS : RS (sr)</t>
+          <t>SE : SE (sv)</t>
         </is>
       </c>
       <c r="C32" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/rs/monitori/lg-27gx700a-b</t>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming/27gx700a-b/</t>
         </is>
       </c>
       <c r="D32" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E32" s="123" t="n"/>
@@ -7709,17 +7710,17 @@
     <row r="33">
       <c r="B33" s="261" t="inlineStr">
         <is>
-          <t>RU : RU (ru)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C33" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ru/monitors/lg-27gx700a-b</t>
+          <t>https://www.lg.com/tr/monitor/oyun-monitorleri/27gx700a-b/</t>
         </is>
       </c>
       <c r="D33" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E33" s="123" t="n"/>
@@ -7735,12 +7736,12 @@
     <row r="34">
       <c r="B34" s="261" t="inlineStr">
         <is>
-          <t>SE : SE (sv)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C34" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/se/monitor/ultragear-gaming/27gx700a-b/</t>
+          <t>https://www.lg.com/uk/monitors/gaming/27gx700a-b/</t>
         </is>
       </c>
       <c r="D34" s="264" t="inlineStr">
@@ -7761,12 +7762,12 @@
     <row r="35">
       <c r="B35" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C35" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/monitor/oyun-monitorleri/27gx700a-b/</t>
+          <t>https://www.lg.com/uk/monitors/gaming/27gx700a-b-27gx001-pck-uk-c/</t>
         </is>
       </c>
       <c r="D35" s="264" t="inlineStr">
@@ -7787,12 +7788,12 @@
     <row r="36">
       <c r="B36" s="261" t="inlineStr">
         <is>
-          <t>UK : GB (en)</t>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C36" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/monitors/gaming/27gx700a-b/</t>
+          <t>https://www.lg.com/fr/moniteurs/gaming/lg-27gx700a-b/</t>
         </is>
       </c>
       <c r="D36" s="264" t="inlineStr">
@@ -7813,12 +7814,12 @@
     <row r="37">
       <c r="B37" s="261" t="inlineStr">
         <is>
-          <t>UK : GB (en)</t>
+          <t>AE : AE (en)</t>
         </is>
       </c>
       <c r="C37" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/monitors/gaming/27gx700a-b-27gx001-pck-uk-c/</t>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-27gx790b-b</t>
         </is>
       </c>
       <c r="D37" s="264" t="inlineStr">
@@ -7832,19 +7833,19 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>27GX700A</t>
+          <t>27GX790B</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="261" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
+          <t>AE_AR : AE (ar)</t>
         </is>
       </c>
       <c r="C38" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr/moniteurs/gaming/lg-27gx700a-b/</t>
+          <t>https://www.lg.com/ae_ar/consumer-monitors/lg-27gx790b-b</t>
         </is>
       </c>
       <c r="D38" s="264" t="inlineStr">
@@ -7858,24 +7859,24 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>27GX700A</t>
+          <t>27GX790B</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="261" t="inlineStr">
         <is>
-          <t>AE : AE (en)</t>
+          <t>AU : AU (en)</t>
         </is>
       </c>
       <c r="C39" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ae/consumer-monitors/lg-27gx790b-b</t>
+          <t>https://www.lg.com/au/monitors/ultragear-gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D39" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E39" s="123" t="n"/>
@@ -7891,17 +7892,17 @@
     <row r="40">
       <c r="B40" s="261" t="inlineStr">
         <is>
-          <t>AE_AR : AE (ar)</t>
+          <t>BE_FR : BE (fr)</t>
         </is>
       </c>
       <c r="C40" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ae_ar/consumer-monitors/lg-27gx790b-b</t>
+          <t>https://www.lg.com/be_fr/moniteurs/lg-27gx790b-b</t>
         </is>
       </c>
       <c r="D40" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E40" s="123" t="n"/>
@@ -7917,12 +7918,12 @@
     <row r="41">
       <c r="B41" s="261" t="inlineStr">
         <is>
-          <t>AU : AU (en)</t>
+          <t>BR : BR (pt)</t>
         </is>
       </c>
       <c r="C41" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/au/monitors/ultragear-gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/br/monitores/monitores-ultragear-oled/27gx790b-b/</t>
         </is>
       </c>
       <c r="D41" s="264" t="inlineStr">
@@ -7943,17 +7944,17 @@
     <row r="42">
       <c r="B42" s="261" t="inlineStr">
         <is>
-          <t>BE_FR : BE (fr)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C42" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/be_fr/moniteurs/lg-27gx790b-b</t>
+          <t>https://www.lg.com/ca_en/monitors/gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D42" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E42" s="123" t="n"/>
@@ -7969,12 +7970,12 @@
     <row r="43">
       <c r="B43" s="261" t="inlineStr">
         <is>
-          <t>BR : BR (pt)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C43" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/br/monitores/monitores-ultragear-oled/27gx790b-b/</t>
+          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/27gx790b-b/</t>
         </is>
       </c>
       <c r="D43" s="264" t="inlineStr">
@@ -7995,12 +7996,12 @@
     <row r="44">
       <c r="B44" s="261" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CN : CN (zh)</t>
         </is>
       </c>
       <c r="C44" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/monitors/gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/cn/monitors/lg-27gx790b-b</t>
         </is>
       </c>
       <c r="D44" s="264" t="inlineStr">
@@ -8021,12 +8022,12 @@
     <row r="45">
       <c r="B45" s="261" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C45" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/27gx790b-b/</t>
+          <t>https://www.lg.com/de/monitore/gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D45" s="264" t="inlineStr">
@@ -8047,17 +8048,17 @@
     <row r="46">
       <c r="B46" s="261" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C46" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/monitors/lg-27gx790b-b</t>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-oled-gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D46" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E46" s="123" t="n"/>
@@ -8073,12 +8074,12 @@
     <row r="47">
       <c r="B47" s="261" t="inlineStr">
         <is>
-          <t>DE : DE (de)</t>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C47" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de/monitore/gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/fr/moniteurs/gaming/lg-27gx790b-b/</t>
         </is>
       </c>
       <c r="D47" s="264" t="inlineStr">
@@ -8099,12 +8100,12 @@
     <row r="48">
       <c r="B48" s="261" t="inlineStr">
         <is>
-          <t>ES : ES (es)</t>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C48" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/monitores/monitores-ultragear-oled-gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/fr/moniteurs/lg-27gx790b-b-27g411a-bundle/</t>
         </is>
       </c>
       <c r="D48" s="264" t="inlineStr">
@@ -8125,12 +8126,12 @@
     <row r="49">
       <c r="B49" s="261" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C49" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr/moniteurs/gaming/lg-27gx790b-b/</t>
+          <t>https://www.lg.com/hk/monitors/gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D49" s="264" t="inlineStr">
@@ -8151,12 +8152,12 @@
     <row r="50">
       <c r="B50" s="261" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C50" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr/moniteurs/lg-27gx790b-b-27g411a-bundle/</t>
+          <t>https://www.lg.com/hk_en/monitors/gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D50" s="264" t="inlineStr">
@@ -8177,12 +8178,12 @@
     <row r="51">
       <c r="B51" s="261" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C51" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/monitors/gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/27gx790b-b/</t>
         </is>
       </c>
       <c r="D51" s="264" t="inlineStr">
@@ -8203,12 +8204,12 @@
     <row r="52">
       <c r="B52" s="261" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>NL : NL (nl)</t>
         </is>
       </c>
       <c r="C52" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/monitors/gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-oled/27gx790b-b/</t>
         </is>
       </c>
       <c r="D52" s="264" t="inlineStr">
@@ -8229,17 +8230,17 @@
     <row r="53">
       <c r="B53" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>PL : PL (pl)</t>
         </is>
       </c>
       <c r="C53" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/27gx790b-b/</t>
+          <t>https://www.lg.com/pl/monitory/ultragear-gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D53" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E53" s="123" t="n"/>
@@ -8255,12 +8256,12 @@
     <row r="54">
       <c r="B54" s="261" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C54" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-oled/27gx790b-b/</t>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D54" s="264" t="inlineStr">
@@ -8281,12 +8282,12 @@
     <row r="55">
       <c r="B55" s="261" t="inlineStr">
         <is>
-          <t>PL : PL (pl)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C55" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pl/monitory/ultragear-gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/27gx790b-b/</t>
         </is>
       </c>
       <c r="D55" s="264" t="inlineStr">
@@ -8307,12 +8308,12 @@
     <row r="56">
       <c r="B56" s="261" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C56" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/consumer-monitors/gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/uk/monitors/gaming/27gx790b-b/</t>
         </is>
       </c>
       <c r="D56" s="264" t="inlineStr">
@@ -8333,12 +8334,12 @@
     <row r="57">
       <c r="B57" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C57" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/27gx790b-b/</t>
+          <t>https://www.lg.com/uk/monitors/gaming/27gx790b-b-27g640a/</t>
         </is>
       </c>
       <c r="D57" s="264" t="inlineStr">
@@ -8359,12 +8360,12 @@
     <row r="58">
       <c r="B58" s="261" t="inlineStr">
         <is>
-          <t>UK : GB (en)</t>
+          <t>VN : VN (vi)</t>
         </is>
       </c>
       <c r="C58" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/monitors/gaming/27gx790b-b/</t>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-gaming-oled-ultragear-oled/27gx790b-b/</t>
         </is>
       </c>
       <c r="D58" s="264" t="inlineStr">
@@ -8385,17 +8386,17 @@
     <row r="59">
       <c r="B59" s="261" t="inlineStr">
         <is>
-          <t>UK : GB (en)</t>
+          <t>PE : PE (es)</t>
         </is>
       </c>
       <c r="C59" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/monitors/gaming/27gx790b-b-27g640a/</t>
+          <t>https://www.lg.com/pe/monitores/gamer/27gx790b-b/</t>
         </is>
       </c>
       <c r="D59" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="E59" s="123" t="n"/>
@@ -8411,12 +8412,12 @@
     <row r="60">
       <c r="B60" s="261" t="inlineStr">
         <is>
-          <t>VN : VN (vi)</t>
+          <t>CN : CN (zh)</t>
         </is>
       </c>
       <c r="C60" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-gaming-oled-ultragear-oled/27gx790b-b/</t>
+          <t>https://www.lg.com/cn/monitors/lg-32gx870b-b</t>
         </is>
       </c>
       <c r="D60" s="264" t="inlineStr">
@@ -8430,24 +8431,24 @@
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>27GX790B</t>
+          <t>32GX870B</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="261" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C61" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe/monitores/gamer/27gx790b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-b/</t>
         </is>
       </c>
       <c r="D61" s="264" t="inlineStr">
         <is>
-          <t>취소</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E61" s="123" t="n"/>
@@ -8456,24 +8457,24 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>27GX790B</t>
+          <t>32GX870B</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="261" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C62" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/monitors/lg-32gx870b-b</t>
+          <t>https://www.lg.com/tr/monitors/32gx870b-b/</t>
         </is>
       </c>
       <c r="D62" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="E62" s="123" t="n"/>
@@ -8494,12 +8495,12 @@
       </c>
       <c r="C63" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-bajp/</t>
         </is>
       </c>
       <c r="D63" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E63" s="123" t="n"/>
@@ -8515,17 +8516,17 @@
     <row r="64">
       <c r="B64" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>AU : AU (en)</t>
         </is>
       </c>
       <c r="C64" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/monitors/32gx870b-b/</t>
+          <t>https://www.lg.com/au/monitors/ultragear-gaming/39gx950b/</t>
         </is>
       </c>
       <c r="D64" s="264" t="inlineStr">
         <is>
-          <t>취소</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E64" s="123" t="n"/>
@@ -8534,24 +8535,24 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>32GX870B</t>
+          <t>39GX950B</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C65" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/32gx870b-bajp/</t>
+          <t>https://www.lg.com/ca_en/monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D65" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E65" s="123" t="n"/>
@@ -8560,24 +8561,24 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>32GX870B</t>
+          <t>39GX950B</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="261" t="inlineStr">
         <is>
-          <t>AU : AU (en)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C66" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/au/monitors/ultragear-gaming/39gx950b/</t>
+          <t>https://www.lg.com/ca_fr/moniteurs/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D66" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E66" s="123" t="n"/>
@@ -8593,12 +8594,12 @@
     <row r="67">
       <c r="B67" s="261" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CN : CN (zh)</t>
         </is>
       </c>
       <c r="C67" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/cn/monitors/lg-39gx950b-b</t>
         </is>
       </c>
       <c r="D67" s="264" t="inlineStr">
@@ -8619,17 +8620,17 @@
     <row r="68">
       <c r="B68" s="261" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C68" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/moniteurs/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/de/monitore/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D68" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E68" s="123" t="n"/>
@@ -8645,17 +8646,17 @@
     <row r="69">
       <c r="B69" s="261" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C69" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/monitors/lg-39gx950b-b</t>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-evo/39gx950b-b/</t>
         </is>
       </c>
       <c r="D69" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E69" s="123" t="n"/>
@@ -8671,17 +8672,17 @@
     <row r="70">
       <c r="B70" s="261" t="inlineStr">
         <is>
-          <t>DE : DE (de)</t>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C70" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de/monitore/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/fr/moniteurs/gaming/39GX950B-B/</t>
         </is>
       </c>
       <c r="D70" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E70" s="123" t="n"/>
@@ -8697,17 +8698,17 @@
     <row r="71">
       <c r="B71" s="261" t="inlineStr">
         <is>
-          <t>ES : ES (es)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C71" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/monitores/monitores-ultragear-evo/39gx950b-b/</t>
+          <t>https://www.lg.com/hk/monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D71" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E71" s="123" t="n"/>
@@ -8723,17 +8724,17 @@
     <row r="72">
       <c r="B72" s="261" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C72" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr/moniteurs/gaming/39GX950B-B/</t>
+          <t>https://www.lg.com/hk_en/monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D72" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E72" s="123" t="n"/>
@@ -8749,17 +8750,17 @@
     <row r="73">
       <c r="B73" s="261" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>HU : HU (hu)</t>
         </is>
       </c>
       <c r="C73" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D73" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E73" s="123" t="n"/>
@@ -8775,12 +8776,12 @@
     <row r="74">
       <c r="B74" s="261" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>IT : IT (it)</t>
         </is>
       </c>
       <c r="C74" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/it/monitor/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D74" s="264" t="inlineStr">
@@ -8801,17 +8802,17 @@
     <row r="75">
       <c r="B75" s="261" t="inlineStr">
         <is>
-          <t>HU : HU (hu)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C75" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hu/monitorok/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-b/</t>
         </is>
       </c>
       <c r="D75" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E75" s="123" t="n"/>
@@ -8827,17 +8828,17 @@
     <row r="76">
       <c r="B76" s="261" t="inlineStr">
         <is>
-          <t>IT : IT (it)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C76" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/it/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-bajp/</t>
         </is>
       </c>
       <c r="D76" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E76" s="123" t="n"/>
@@ -8853,17 +8854,17 @@
     <row r="77">
       <c r="B77" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>NL : NL (nl)</t>
         </is>
       </c>
       <c r="C77" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-b/</t>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/39gx950b-b/</t>
         </is>
       </c>
       <c r="D77" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E77" s="123" t="n"/>
@@ -8879,17 +8880,17 @@
     <row r="78">
       <c r="B78" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>PE : PE (es)</t>
         </is>
       </c>
       <c r="C78" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/39gx950b-bajp/</t>
+          <t>https://www.lg.com/pe/monitores/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D78" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E78" s="123" t="n"/>
@@ -8905,17 +8906,17 @@
     <row r="79">
       <c r="B79" s="261" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
+          <t>PL : PL (pl)</t>
         </is>
       </c>
       <c r="C79" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/39gx950b-b/</t>
+          <t>https://www.lg.com/pl/monitory/39gx950b-b/</t>
         </is>
       </c>
       <c r="D79" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E79" s="123" t="n"/>
@@ -8931,17 +8932,17 @@
     <row r="80">
       <c r="B80" s="261" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>SE : SE (sv)</t>
         </is>
       </c>
       <c r="C80" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe/monitores/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D80" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E80" s="123" t="n"/>
@@ -8957,17 +8958,17 @@
     <row r="81">
       <c r="B81" s="261" t="inlineStr">
         <is>
-          <t>PL : PL (pl)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C81" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pl/monitory/39gx950b-b/</t>
+          <t>https://www.lg.com/sg/consumer-monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D81" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E81" s="123" t="n"/>
@@ -8983,17 +8984,17 @@
     <row r="82">
       <c r="B82" s="261" t="inlineStr">
         <is>
-          <t>SE : SE (sv)</t>
+          <t>TH : TH (th)</t>
         </is>
       </c>
       <c r="C82" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/se/monitor/ultragear-gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/th/monitors/gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D82" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E82" s="123" t="n"/>
@@ -9009,17 +9010,17 @@
     <row r="83">
       <c r="B83" s="261" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C83" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/consumer-monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/39gx950b-b/</t>
         </is>
       </c>
       <c r="D83" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E83" s="123" t="n"/>
@@ -9035,17 +9036,17 @@
     <row r="84">
       <c r="B84" s="261" t="inlineStr">
         <is>
-          <t>TH : TH (th)</t>
+          <t>TW : TW (zh)</t>
         </is>
       </c>
       <c r="C84" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/th/monitors/gaming/39gx950b-b/</t>
+          <t>https://www.lg.com/tw/monitors/ultragear-gaming/39gx950b-b/</t>
         </is>
       </c>
       <c r="D84" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E84" s="123" t="n"/>
@@ -9061,17 +9062,17 @@
     <row r="85">
       <c r="B85" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C85" s="261" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/monitor/ultragear-gaming-oled/39gx950b-b/</t>
+          <t>https://www.lg.com/uk/monitors/gaming-monitor/39gx950b-b/</t>
         </is>
       </c>
       <c r="D85" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E85" s="123" t="n"/>
@@ -9079,58 +9080,6 @@
         <v>1</v>
       </c>
       <c r="G85" s="0" t="inlineStr">
-        <is>
-          <t>39GX950B</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="261" t="inlineStr">
-        <is>
-          <t>TW : TW (zh)</t>
-        </is>
-      </c>
-      <c r="C86" s="261" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/tw/monitors/ultragear-gaming/39gx950b-b/</t>
-        </is>
-      </c>
-      <c r="D86" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E86" s="123" t="n"/>
-      <c r="F86" s="123" t="n">
-        <v>1</v>
-      </c>
-      <c r="G86" s="0" t="inlineStr">
-        <is>
-          <t>39GX950B</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="261" t="inlineStr">
-        <is>
-          <t>UK : GB (en)</t>
-        </is>
-      </c>
-      <c r="C87" s="261" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/uk/monitors/gaming-monitor/39gx950b-b/</t>
-        </is>
-      </c>
-      <c r="D87" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E87" s="123" t="n"/>
-      <c r="F87" s="123" t="n">
-        <v>1</v>
-      </c>
-      <c r="G87" s="0" t="inlineStr">
         <is>
           <t>39GX950B</t>
         </is>

</xml_diff>

<commit_message>
data(it): W17 GNB — TR(터키) 작업중→완료 (7/23 게시, PTT 6/7 Closed)
잔여 1건(Final Live Check)은 Remark에 명시. 완료 9→10, 작업중 28→27.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -7036,7 +7036,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -10651,7 +10650,8 @@
         <is>
           <t>CZ : 작업중 → 완료
 TR : 법인리뷰 → 작업중
-IN : 법인리뷰 → 완료 (7/16 게시, PTT 확인)</t>
+IN : 법인리뷰 → 완료 (7/16 게시, PTT 확인)
+TR : 작업중 → 완료 (7/23 게시, PTT 확인)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -11617,14 +11617,22 @@
       </c>
       <c r="D48" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E48" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E48" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="F48" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G48" s="0" t="inlineStr"/>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>7건 중 6건 게시완료 · 1건 Final Live Check 잔여</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="261" t="inlineStr">

</xml_diff>

<commit_message>
data(it): W23 4개 태스크 표시명 GR26- 접두 + gr-titles 역매핑
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -2946,7 +2946,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>W23 - 52G930B Feature 수정 건</t>
+          <t>GR26-W23 - 52G930B Feature 수정 건</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>W23 - UL인증 feature 삭제 1차</t>
+          <t>GR26-W23 - UL인증 feature 삭제 1차</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>
@@ -13648,7 +13648,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>W23 - 27GM950B-B 갤러리 이미지 교체</t>
+          <t>GR26-W23 - 27GM950B-B 갤러리 이미지 교체</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>
@@ -14197,7 +14197,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>W23 - 39GX950B 이미지 수정 2차</t>
+          <t>GR26-W23 - 39GX950B 이미지 수정 2차</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>

</xml_diff>

<commit_message>
data(it): W18 evo/Hyper FAQ — JP 행 URL 오기입 정정 (uk/ice-solution → jp/monitors/ultragear-evo)
JP만 무관한 영국 제빙기 URL이 들어가 있었음. PTT STG 경로(/content/lge/jp/ja/monitors/ultragear-evo)와
타 로케일 패턴 기준으로 정정, 미게시 상태를 Status 2에 명시(PTT Client Review·JP 사이트맵 부재 확인).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -11769,7 +11769,8 @@
       <c r="B2" s="163" t="inlineStr">
         <is>
           <t>NL : URL 변경
-SE : URL 변경</t>
+SE : URL 변경
+JP : URL 오기입 정정(uk/ice-solution → jp/monitors/ultragear-evo)</t>
         </is>
       </c>
       <c r="D2" s="164" t="n"/>
@@ -12039,7 +12040,7 @@
       </c>
       <c r="C16" s="268" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/ice-solution/</t>
+          <t>https://www.lg.com/jp/monitors/ultragear-evo/</t>
         </is>
       </c>
       <c r="D16" s="273" t="inlineStr">
@@ -12047,7 +12048,11 @@
           <t>법인리뷰</t>
         </is>
       </c>
-      <c r="E16" s="288" t="n"/>
+      <c r="E16" s="288" t="inlineStr">
+        <is>
+          <t>미게시(법인리뷰) · STG 경로 기준</t>
+        </is>
+      </c>
       <c r="F16" s="275" t="n"/>
       <c r="G16" s="177" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
feat(it): GR 신규 4건 + 사이드바 In Progress/Done 2분할 백포트 (v0.6.47)
- Global Request.xlsx: W30·W31 4시트 추가(SmartMonitor 35행·SecureLock 104행·FAQ/Win11 빈 시트)
- gr-titles.json 역매핑 4건, gr-task-state.json(수동 오버라이드) 신규
- sheet-loader GR 섹션 블록 교체(NPI Tracker 게이트 보존), gr-meta에 grTaskGroupOf만 추가,
  common.js ensureGrDataLoaded에 gr-task-state lazy fetch + nav 재렌더
- 실측: In Progress 10 / Done 8, 라벨-항목 일치, 중복 0, 빈 시트 정상 렌더, 콘솔 에러 0

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -17,6 +17,10 @@
     <sheet name="W25 - Copilot+ Hero Banner" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="W28 - AI Upscaling Disclaimer" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="W28 - UL Verified Eye Comfort" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="W30 - SmartMonitor ScreenShare" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="W30 - UltraGear 1000Hz FAQ" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="W31 - Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9089,6 +9093,3761 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GR26-W30-MS-IT Smart Monitor Screen Share 카피 수정</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · Screen Share 카피/디스클레이머 삭제 · DAM 적재 완료(7/27) 지급 진행 · 대상 4모델(색상 파생 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MX : MX (es)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/mx/monitores/monitores-smart/24u511sb-b/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>24U511SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/smart-monitors/24u511sb-b/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>24U511SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/24u511sb-b/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>24U511SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/smart-monitores/24u511sb-b/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>24U511SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://wwwstg.lg.com/ae/consumer-monitors/lg-24u511sb-b</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>24U511SB-B · 페이지 QA review</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BR : BR (pt)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/br/monitores/smart-monitors/24u511sb-b/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>24U511SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MX : MX (es)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/mx/monitores/monitores-smart/27u511sb-w/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>US : US (en)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/us/monitors/lg-27u511sb-w-smart-monitor</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/smart-monitors/27u511sb-w/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/smart-monitors/27u511sb-b/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>27U511SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ID : ID (id)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/smart-monitors/27u511sb/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/27u511sb-w/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/smart-monitores/27u511sb-w/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/fhd-y-qhd/27u511sb-w/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/smart-monitors/27u511sb-w/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/smart-monitors/27u511sb-w/</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>27U511SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://wwwstg.lg.com/ae/consumer-monitors/lg-27u511sb-w</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>27U511SB-W · 페이지 WPL review</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BR : BR (pt)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/br/pt/monitores/smart-monitors/27u511sb-b.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>27U511SB-B · 페이지 New Request</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/jp/ja/monitors/smart-monitors/27u511sb-b.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>27U511SB-B · 페이지 Client Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/smart-monitors/32u501sb-b/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>32U501SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ID : ID (id)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/smart-monitors/32u501sb/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>32U501SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/32u501sb-w/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>32U501SB-W</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://wwwstg.lg.com/ae/business/monitors/lg-32u501sb-b-ama</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>32U501SB-B · 페이지 In progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/monitors/smart-monitors/32u501sb-b.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>32U501SB-B · 페이지 QA review</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/smart-monitores/32u501sb-b/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>32U501SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/au/en/monitors/smart-monitors/32U501SB.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>32U501SB · 페이지 Cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>US : US (en)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/us/monitors/lg-32u701sb-b-smart-monitor</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>32U701SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/monitores/myview-smart-monitor/32u701sb-b/</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>32U701SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/outlet/outlet-informatica/monitores/32u701sb-b-outlet/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>32U701SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/smart-monitors/32u701sb-b/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>32U701SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TR : TR (tr)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/monitor/smart-monitorleri/32u701sb-b/</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>32U701SB-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://wwwstg.lg.com/ae/consumer-monitors/lg-32u701sb-b</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>32U701SB-B · 페이지 QA review</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ZA : ZA (en)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/za/en/monitors/smart-monitors/32u701sb.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>32u701sb · 페이지 Client Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>BR : BR (pt)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/br/pt/monitores/smart-monitors/32u701sb-b.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>32U701SB-B · 페이지 QA review</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/smart-monitores/32u701sb-b/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>32U701SB-B</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GR26-W30-MS-IT UltraGear PLP FAQ 1000Hz 문항 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · JIRA LGCOMMON-29612 · 1000Hz 제품 문항 3건 추가 · 대상 URL 확정 대기(GR 파일 미수신)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G107"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GR26-W31-MS-IT gram Secure Lock 컴포넌트 교체</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>예정 · 13개국 대상 · CN은 PDP 라이브이나 기존 Secure Lock 컴포넌트 영역 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram/14z90u-g-as67c2/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram-pro/16z90u-g-au87c2/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram-pro/16z90u-k-aub7c2/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram-pro/16z90u-k-aub8c2/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram-pro/16z95u-g-as69c2/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram-pro/17z90u-g-au88c2/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram-pro/16z90u-g-au78gn/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram-pro/16z90u-k-aub8gn/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram-pro/17z90u-g-au8bgn/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/14z90u-g/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/15u50u-g/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>15U50U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/16z90u-g-16gb/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/16z90u-g-32gb/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/16z95u-g/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/14z90u-g-au85bn/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/14z90u-g-au88bn/</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/business/informatica/ordenadores/portatiles-para-creadores/14z95u-g-au88bn/</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/14z95u-g-as55bn/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/14z95u-g-au85bn/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/laptops/gram/16z90u-k-aub5bn/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/16z90u-g-au85bn/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/16z90u-g-au88bn/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram-pro/16z90u-k-aub8bn/</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/14z90u-g-az75a3/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/14z90u-g-az85a3/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z90u-g-as54a3/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z90u-g-au85a3/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z95u-g-as56a3/</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z95u-g-au85a3/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z95u-g-au86a3/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z95u56-16mr70/</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z95u85-16mr70/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z95u86-16mr70/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/15u50u-16mr70/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>15U50U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/15u50u-g-aa55a3/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>15U50U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90u-k-azb5a3/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aua5a3/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aub5a3/</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aub9a3/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z95u-16mr70/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z95u-g-as55a3/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z95u-g-au85a3/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/17z90u-g-au85a3/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/laptops/gram/15u50u-g-aa55an.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>15U50U-G.AA55AN · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/laptops/gram-pro/16z90u-h-au78an.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>16Z90U-H.AU78AN · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/laptops/gram-pro/16z90u-k-aub8an.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>16Z90U-K.AUB8AN · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/laptops/gram-pro/17z90u-g-au78an.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU78AN · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/gram/14z90u-g-as58dn/</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>- · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gs54j/</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gs58j/</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gu85j/</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-vp58j/</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>14Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs53j/</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs54j/</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs55j/</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gu85j/</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gu86j/</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-vp53j/</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-vp55j/</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>14Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-gu85j/</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-gu88j/</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-kub5j/</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-kub9j/</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z95u-gs55j/</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z95u-gu88j/</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-gu85j/</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-gu88j/</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-vp55j/</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal87c/</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal88c/</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb7c/</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb8c/</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb9c/</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-17z90u-al87c/</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-17z90u-gal88c/</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/16z95u-g/</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/small-medium-business/laptops/16z95u-g/</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/ordinateurs-portables/16z95u-g/</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/small-medium-business/ordinateurs-portables/16z95u-g/</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>16Z95U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g78/</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g88/</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90u-g78/</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90u-g88/</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g78/</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g88/</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ub-h/</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>17Z90UB-H · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90ub-h/</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>17Z90UB-H · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90ub-h/</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>17Z90UB-H · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/small-medium-business/computing/purchase-guide/laptops/17z90ub-h/</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>17Z90UB-H · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/ca/en/laptops/all-laptops/17z90ub-h.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>17Z90UR-P · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ur-p/</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>17Z90UR-P · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17Z90ur-p/</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>17Z90UR-P · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/ca/fr/computing/purchase-guide/laptops/17z90ub-h.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>17Z90UR-P · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>15U50U-G · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>15Z95U-G · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>16Z90U-G · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/16z90u-g-au75ap/</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>16Z90U-G.AU75AP · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/16z90u-g-au88ap/</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>16Z90U-K · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au75ap/</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au78ap/</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au88ap/</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>17Z90U-G · Erase.Lock 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/au/en/laptops/gram-pro/17z90ub-h.html?wcmmode=disabled</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>17Z90UB-H · Erase.Lock -</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GR26-W31-MS-IT Windows 11 Home Landing Page 업데이트</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>예정 · 자산 배포 2026-08-09(EN)/2026-09-11(현지화) · 구현 마감 2026-11-15(Jumpstart OEM.com 준수)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(it): Done 아코디언 + GR 데이터 갱신 백포트 (v0.6.48)
- 사이드바 Done 섹션 접기(기본 열림, localStorage 유지) — pushGrSection 블록·헬퍼 함수 스플라이스,
  라이브 고유 NPI 게이트(__SHOW_CUSTOM_NAV_TABS)는 보존
- W16 MS PDP Gallery Card: GLOBAL 행 작업중→완료 (100%, Done 이동)
- W22 UltraGear Buying Guide: PTT 0727 대조 — CP-en 게시 불필요로 취소, JP-ja 법인리뷰→작업중(번역 문서 미비). 78%→80%
- W31 PDP Gallery Card Win11 Pro 영상 수정 신규 등록(대상 목록 미수신, 빈 시트)
- 완료일 'N월 N일' 표기 17건을 YYYY-MM-DD로 통일
- gr-changes.json 재생성(7/13 스테일 해소) + gr-titles.json 역매핑 보강

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -21,6 +21,7 @@
     <sheet name="W30 - UltraGear 1000Hz FAQ" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="W31 - Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="W31 - PDP Gallery Win11 Pro" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10114,275 +10115,275 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>AU : AU (en)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/au/monitors/ultragear-gaming/</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="F4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>CA : CA (en)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/monitors/gaming/</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="F5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>CA : CA (fr)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="F6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/monitore/gaming/</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="F7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/monitores/monitores-ultragear-gaming/</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="F8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>FR : FR (fr)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/fr/moniteurs/gaming/</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="F9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/monitor/gaming/</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="F10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>JP : JP (ja)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/jp/monitors/gaming-monitors/</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>NL : NL (nl)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="F12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>SE : SE (sv)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/se/monitor/ultragear-gaming/</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="F13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>UK : UK (en)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/uk/monitors/gaming/</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="F14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
         <is>
           <t>1000Hz 문항 3건 추가 · 현지어 번역 필요</t>
         </is>
@@ -13078,6 +13079,81 @@
       <c r="B2" s="0" t="inlineStr">
         <is>
           <t>예정 · 자산 배포 2026-08-09(EN)/2026-09-11(현지화) · 구현 마감 2026-11-15(Jumpstart OEM.com 준수)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>GR26-W31-MS-IT-PC PDP Gallery Card Win11 Pro 영상 수정</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · W16 PDP Gallery Card 후속 건 · Windows 11 Pro 영상 수정 · 대상 목록 미수신(확인 필요)</t>
         </is>
       </c>
     </row>
@@ -13464,7 +13540,7 @@
       </c>
       <c r="E7" s="223" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F7" s="224" t="n">
@@ -13526,7 +13602,7 @@
       </c>
       <c r="E8" s="231" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F8" s="232" t="n">
@@ -13588,7 +13664,7 @@
       </c>
       <c r="E9" s="231" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F9" s="232" t="n">
@@ -13650,7 +13726,7 @@
       </c>
       <c r="E10" s="231" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F10" s="225" t="n">
@@ -13712,7 +13788,7 @@
       </c>
       <c r="E11" s="231" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F11" s="225" t="n">
@@ -13774,7 +13850,7 @@
       </c>
       <c r="E12" s="231" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F12" s="232" t="n">
@@ -13836,7 +13912,7 @@
       </c>
       <c r="E13" s="234" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F13" s="232" t="n">
@@ -13898,7 +13974,7 @@
       </c>
       <c r="E14" s="231" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F14" s="225" t="n">
@@ -13960,7 +14036,7 @@
       </c>
       <c r="E15" s="231" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F15" s="232" t="n">
@@ -14022,7 +14098,7 @@
       </c>
       <c r="E16" s="228" t="inlineStr">
         <is>
-          <t>6월 12일</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F16" s="225" t="n">
@@ -14267,7 +14343,7 @@
       </c>
       <c r="E10" s="242" t="inlineStr">
         <is>
-          <t>5월 28일</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="F10" s="243" t="n">
@@ -14295,7 +14371,7 @@
       </c>
       <c r="E11" s="242" t="inlineStr">
         <is>
-          <t>5월 28일</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="F11" s="243" t="n">
@@ -14347,7 +14423,7 @@
       </c>
       <c r="E13" s="242" t="inlineStr">
         <is>
-          <t>5월 28일</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="F13" s="253" t="n">
@@ -14375,7 +14451,7 @@
       </c>
       <c r="E14" s="242" t="inlineStr">
         <is>
-          <t>5월 28일</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="F14" s="240" t="n">
@@ -14426,10 +14502,14 @@
       </c>
       <c r="D16" s="256" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E16" s="242" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" s="242" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
       <c r="F16" s="257" t="n">
         <v>18</v>
       </c>
@@ -14455,7 +14535,7 @@
       </c>
       <c r="E17" s="255" t="inlineStr">
         <is>
-          <t>5월 28일</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="F17" s="257" t="n">
@@ -14539,7 +14619,7 @@
       </c>
       <c r="E20" s="242" t="inlineStr">
         <is>
-          <t>5월 28일</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="F20" s="257" t="n">
@@ -14972,7 +15052,7 @@
       </c>
       <c r="E18" s="123" t="inlineStr">
         <is>
-          <t>6월 19일</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F18" s="123" t="n">
@@ -16645,7 +16725,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -16671,7 +16751,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>금주 변경 없음</t>
+          <t>PTT 0727 대조 — CP-en 게시 불필요로 대상 제외(취소) · JP-ja 법인리뷰→작업중(번역 문서 미비) · 잔여 작업중 7·법인리뷰 2, PTT상 진척 없음</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -16924,12 +17004,16 @@
       <c r="C18" s="277" t="inlineStr"/>
       <c r="D18" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="E18" s="200" t="inlineStr"/>
       <c r="F18" s="0" t="inlineStr"/>
-      <c r="G18" s="0" t="inlineStr"/>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>CP 페이지 게시 불필요 — PTT 태스크만 종료(2025-11-10, WR2209877YZ)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="261" t="inlineStr">
@@ -17252,12 +17336,16 @@
       <c r="C34" s="277" t="inlineStr"/>
       <c r="D34" s="263" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E34" s="123" t="inlineStr"/>
       <c r="F34" s="0" t="inlineStr"/>
-      <c r="G34" s="0" t="inlineStr"/>
+      <c r="G34" s="0" t="inlineStr">
+        <is>
+          <t>번역 문서 미비로 확인요청 중(PTT Request Clarification, 2026-03-30)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="261" t="inlineStr">

</xml_diff>

<commit_message>
data(it): W22 Buying Guide CP-en 행 삭제 — 게시 대상 아님(사용자 확인)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -16725,7 +16725,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -16751,7 +16751,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>PTT 0727 대조 — CP-en 게시 불필요로 대상 제외(취소) · JP-ja 법인리뷰→작업중(번역 문서 미비) · 잔여 작업중 7·법인리뷰 2, PTT상 진척 없음</t>
+          <t>PTT 0727 대조 — JP-ja 법인리뷰→작업중(번역 문서 미비) · CP-en 게시 대상 아님으로 행 삭제 · 잔여 작업중 7·법인리뷰 2, PTT상 진척 없음</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -16998,32 +16998,34 @@
     <row r="18">
       <c r="B18" s="261" t="inlineStr">
         <is>
-          <t>CP-en</t>
-        </is>
-      </c>
-      <c r="C18" s="277" t="inlineStr"/>
-      <c r="D18" s="264" t="inlineStr">
-        <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="E18" s="200" t="inlineStr"/>
-      <c r="F18" s="0" t="inlineStr"/>
-      <c r="G18" s="0" t="inlineStr">
-        <is>
-          <t>CP 페이지 게시 불필요 — PTT 태스크만 종료(2025-11-10, WR2209877YZ)</t>
-        </is>
-      </c>
+          <t>CZ-cz</t>
+        </is>
+      </c>
+      <c r="C18" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D18" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" s="123" t="inlineStr"/>
+      <c r="F18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="B19" s="261" t="inlineStr">
         <is>
-          <t>CZ-cz</t>
+          <t>DK-da</t>
         </is>
       </c>
       <c r="C19" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/dk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D19" s="265" t="inlineStr">
@@ -17040,12 +17042,12 @@
     <row r="20">
       <c r="B20" s="261" t="inlineStr">
         <is>
-          <t>DK-da</t>
+          <t>EC-es</t>
         </is>
       </c>
       <c r="C20" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/dk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/ec/computacion/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D20" s="265" t="inlineStr">
@@ -17062,12 +17064,12 @@
     <row r="21">
       <c r="B21" s="261" t="inlineStr">
         <is>
-          <t>EC-es</t>
+          <t>EE-ee</t>
         </is>
       </c>
       <c r="C21" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ec/computacion/ultragear-buying-guide</t>
+          <t>https://www.lg.com/ee/it-seadmed/buying-guide/ultragear-mangumonitorid</t>
         </is>
       </c>
       <c r="D21" s="265" t="inlineStr">
@@ -17084,12 +17086,12 @@
     <row r="22">
       <c r="B22" s="261" t="inlineStr">
         <is>
-          <t>EE-ee</t>
+          <t>ES-es</t>
         </is>
       </c>
       <c r="C22" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ee/it-seadmed/buying-guide/ultragear-mangumonitorid</t>
+          <t>https://www.lg.com/es/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D22" s="265" t="inlineStr">
@@ -17106,12 +17108,12 @@
     <row r="23">
       <c r="B23" s="261" t="inlineStr">
         <is>
-          <t>ES-es</t>
+          <t>FI-fi</t>
         </is>
       </c>
       <c r="C23" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/fi/it-tuotteet/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D23" s="265" t="inlineStr">
@@ -17128,35 +17130,29 @@
     <row r="24">
       <c r="B24" s="261" t="inlineStr">
         <is>
-          <t>FI-fi</t>
-        </is>
-      </c>
-      <c r="C24" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/fi/it-tuotteet/ultragear-buying-guide</t>
-        </is>
-      </c>
-      <c r="D24" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>FR-fr</t>
+        </is>
+      </c>
+      <c r="C24" s="277" t="inlineStr"/>
+      <c r="D24" s="263" t="inlineStr">
+        <is>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E24" s="123" t="inlineStr"/>
-      <c r="F24" s="0" t="n">
-        <v>1</v>
-      </c>
+      <c r="F24" s="0" t="inlineStr"/>
       <c r="G24" s="0" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="B25" s="261" t="inlineStr">
         <is>
-          <t>FR-fr</t>
+          <t>GR-gr</t>
         </is>
       </c>
       <c r="C25" s="277" t="inlineStr"/>
-      <c r="D25" s="263" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
+      <c r="D25" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E25" s="123" t="inlineStr"/>
@@ -17166,28 +17162,34 @@
     <row r="26">
       <c r="B26" s="261" t="inlineStr">
         <is>
-          <t>GR-gr</t>
-        </is>
-      </c>
-      <c r="C26" s="277" t="inlineStr"/>
-      <c r="D26" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
+          <t>HK-zh</t>
+        </is>
+      </c>
+      <c r="C26" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D26" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="E26" s="123" t="inlineStr"/>
-      <c r="F26" s="0" t="inlineStr"/>
+      <c r="F26" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G26" s="0" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="261" t="inlineStr">
         <is>
-          <t>HK-zh</t>
+          <t>HK-en</t>
         </is>
       </c>
       <c r="C27" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/hk_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D27" s="265" t="inlineStr">
@@ -17204,12 +17206,12 @@
     <row r="28">
       <c r="B28" s="261" t="inlineStr">
         <is>
-          <t>HK-en</t>
+          <t>HU-hu</t>
         </is>
       </c>
       <c r="C28" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/hu/microsite-article/ms/it/monitor/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D28" s="265" t="inlineStr">
@@ -17226,12 +17228,12 @@
     <row r="29">
       <c r="B29" s="261" t="inlineStr">
         <is>
-          <t>HU-hu</t>
+          <t>ID-id</t>
         </is>
       </c>
       <c r="C29" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hu/microsite-article/ms/it/monitor/ultragear-buying-guide</t>
+          <t>https://www.lg.com/id/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D29" s="265" t="inlineStr">
@@ -17248,12 +17250,12 @@
     <row r="30">
       <c r="B30" s="261" t="inlineStr">
         <is>
-          <t>ID-id</t>
+          <t>IL-he</t>
         </is>
       </c>
       <c r="C30" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/id/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/il/monitors/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D30" s="265" t="inlineStr">
@@ -17270,12 +17272,12 @@
     <row r="31">
       <c r="B31" s="261" t="inlineStr">
         <is>
-          <t>IL-he</t>
+          <t>IN-en</t>
         </is>
       </c>
       <c r="C31" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/il/monitors/ultragear-buying-guide</t>
+          <t>https://www.lg.com/in/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D31" s="265" t="inlineStr">
@@ -17292,70 +17294,70 @@
     <row r="32">
       <c r="B32" s="261" t="inlineStr">
         <is>
-          <t>IN-en</t>
-        </is>
-      </c>
-      <c r="C32" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/in/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
-      <c r="D32" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>IT-it</t>
+        </is>
+      </c>
+      <c r="C32" s="277" t="inlineStr"/>
+      <c r="D32" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E32" s="123" t="inlineStr"/>
-      <c r="F32" s="0" t="n">
-        <v>1</v>
-      </c>
+      <c r="F32" s="0" t="inlineStr"/>
       <c r="G32" s="0" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="B33" s="261" t="inlineStr">
         <is>
-          <t>IT-it</t>
+          <t>JP-ja</t>
         </is>
       </c>
       <c r="C33" s="277" t="inlineStr"/>
-      <c r="D33" s="264" t="inlineStr">
+      <c r="D33" s="263" t="inlineStr">
         <is>
           <t>작업중</t>
         </is>
       </c>
       <c r="E33" s="123" t="inlineStr"/>
       <c r="F33" s="0" t="inlineStr"/>
-      <c r="G33" s="0" t="inlineStr"/>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>번역 문서 미비로 확인요청 중(PTT Request Clarification, 2026-03-30)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="261" t="inlineStr">
         <is>
-          <t>JP-ja</t>
-        </is>
-      </c>
-      <c r="C34" s="277" t="inlineStr"/>
-      <c r="D34" s="263" t="inlineStr">
-        <is>
-          <t>작업중</t>
+          <t>KZ-ru</t>
+        </is>
+      </c>
+      <c r="C34" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/kz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D34" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="E34" s="123" t="inlineStr"/>
-      <c r="F34" s="0" t="inlineStr"/>
-      <c r="G34" s="0" t="inlineStr">
-        <is>
-          <t>번역 문서 미비로 확인요청 중(PTT Request Clarification, 2026-03-30)</t>
-        </is>
-      </c>
+      <c r="F34" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="0" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="B35" s="261" t="inlineStr">
         <is>
-          <t>KZ-ru</t>
+          <t>LT-lt</t>
         </is>
       </c>
       <c r="C35" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/kz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/lt/kompiuterine-technika/buying-guide/ultragear-gaming-monitor</t>
         </is>
       </c>
       <c r="D35" s="265" t="inlineStr">
@@ -17372,12 +17374,12 @@
     <row r="36">
       <c r="B36" s="261" t="inlineStr">
         <is>
-          <t>LT-lt</t>
+          <t>LV-lv</t>
         </is>
       </c>
       <c r="C36" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/lt/kompiuterine-technika/buying-guide/ultragear-gaming-monitor</t>
+          <t>https://www.lg.com/lv/datortehnika/buying-guide/ultragear-gaming-monitor</t>
         </is>
       </c>
       <c r="D36" s="265" t="inlineStr">
@@ -17394,12 +17396,12 @@
     <row r="37">
       <c r="B37" s="261" t="inlineStr">
         <is>
-          <t>LV-lv</t>
+          <t>NL-nl</t>
         </is>
       </c>
       <c r="C37" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/lv/datortehnika/buying-guide/ultragear-gaming-monitor</t>
+          <t>https://www.lg.com/nl/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D37" s="265" t="inlineStr">
@@ -17416,12 +17418,12 @@
     <row r="38">
       <c r="B38" s="261" t="inlineStr">
         <is>
-          <t>NL-nl</t>
+          <t>NO-no</t>
         </is>
       </c>
       <c r="C38" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nl/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/no/it-produkter/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D38" s="265" t="inlineStr">
@@ -17438,12 +17440,12 @@
     <row r="39">
       <c r="B39" s="261" t="inlineStr">
         <is>
-          <t>NO-no</t>
+          <t>PA-es</t>
         </is>
       </c>
       <c r="C39" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/no/it-produkter/ultragear-buying-guide</t>
+          <t>https://www.lg.com/pa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D39" s="265" t="inlineStr">
@@ -17460,12 +17462,12 @@
     <row r="40">
       <c r="B40" s="261" t="inlineStr">
         <is>
-          <t>PA-es</t>
+          <t>PE-es</t>
         </is>
       </c>
       <c r="C40" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/pe/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D40" s="265" t="inlineStr">
@@ -17482,12 +17484,12 @@
     <row r="41">
       <c r="B41" s="261" t="inlineStr">
         <is>
-          <t>PE-es</t>
+          <t>PH-en</t>
         </is>
       </c>
       <c r="C41" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/ph/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D41" s="265" t="inlineStr">
@@ -17504,29 +17506,23 @@
     <row r="42">
       <c r="B42" s="261" t="inlineStr">
         <is>
-          <t>PH-en</t>
-        </is>
-      </c>
-      <c r="C42" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ph/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
-      <c r="D42" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>PL-pl</t>
+        </is>
+      </c>
+      <c r="C42" s="277" t="inlineStr"/>
+      <c r="D42" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E42" s="123" t="inlineStr"/>
-      <c r="F42" s="0" t="n">
-        <v>1</v>
-      </c>
+      <c r="F42" s="0" t="inlineStr"/>
       <c r="G42" s="0" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="B43" s="261" t="inlineStr">
         <is>
-          <t>PL-pl</t>
+          <t>PT-pt</t>
         </is>
       </c>
       <c r="C43" s="277" t="inlineStr"/>
@@ -17542,28 +17538,34 @@
     <row r="44">
       <c r="B44" s="261" t="inlineStr">
         <is>
-          <t>PT-pt</t>
-        </is>
-      </c>
-      <c r="C44" s="277" t="inlineStr"/>
-      <c r="D44" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
+          <t>RS-rs</t>
+        </is>
+      </c>
+      <c r="C44" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/it-proizvodi/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D44" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="E44" s="123" t="inlineStr"/>
-      <c r="F44" s="0" t="inlineStr"/>
+      <c r="F44" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G44" s="0" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="B45" s="261" t="inlineStr">
         <is>
-          <t>RS-rs</t>
+          <t>SA-ar</t>
         </is>
       </c>
       <c r="C45" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/rs/it-proizvodi/ultragear-buying-guide</t>
+          <t>https://www.lg.com/sa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D45" s="265" t="inlineStr">
@@ -17580,12 +17582,12 @@
     <row r="46">
       <c r="B46" s="261" t="inlineStr">
         <is>
-          <t>SA-ar</t>
+          <t>SA-en</t>
         </is>
       </c>
       <c r="C46" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/sa_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D46" s="265" t="inlineStr">
@@ -17602,12 +17604,12 @@
     <row r="47">
       <c r="B47" s="261" t="inlineStr">
         <is>
-          <t>SA-en</t>
+          <t>SE-sv</t>
         </is>
       </c>
       <c r="C47" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/se/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D47" s="265" t="inlineStr">
@@ -17624,12 +17626,12 @@
     <row r="48">
       <c r="B48" s="261" t="inlineStr">
         <is>
-          <t>SE-sv</t>
+          <t>TH-th</t>
         </is>
       </c>
       <c r="C48" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/se/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/th/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D48" s="265" t="inlineStr">
@@ -17646,12 +17648,12 @@
     <row r="49">
       <c r="B49" s="261" t="inlineStr">
         <is>
-          <t>TH-th</t>
+          <t>TR-tr</t>
         </is>
       </c>
       <c r="C49" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/th/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/tr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D49" s="265" t="inlineStr">
@@ -17668,12 +17670,12 @@
     <row r="50">
       <c r="B50" s="261" t="inlineStr">
         <is>
-          <t>TR-tr</t>
+          <t>TW-zh</t>
         </is>
       </c>
       <c r="C50" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/tw/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D50" s="265" t="inlineStr">
@@ -17690,12 +17692,12 @@
     <row r="51">
       <c r="B51" s="261" t="inlineStr">
         <is>
-          <t>TW-zh</t>
+          <t>UA-uk</t>
         </is>
       </c>
       <c r="C51" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tw/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/ua/it-products/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D51" s="265" t="inlineStr">
@@ -17712,12 +17714,12 @@
     <row r="52">
       <c r="B52" s="261" t="inlineStr">
         <is>
-          <t>UA-uk</t>
+          <t>ZA-en</t>
         </is>
       </c>
       <c r="C52" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ua/it-products/ultragear-buying-guide</t>
+          <t>https://www.lg.com/za/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D52" s="265" t="inlineStr">
@@ -17730,28 +17732,6 @@
         <v>1</v>
       </c>
       <c r="G52" s="0" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="B53" s="261" t="inlineStr">
-        <is>
-          <t>ZA-en</t>
-        </is>
-      </c>
-      <c r="C53" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/za/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
-      <c r="D53" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E53" s="123" t="inlineStr"/>
-      <c r="F53" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" s="0" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data(it): W22 JP-ja Remark 삭제 — 2026-03-30 기준의 오래된 PTT 사유 문구
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -16751,7 +16751,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>PTT 0727 대조 — JP-ja 법인리뷰→작업중(번역 문서 미비) · CP-en 게시 대상 아님으로 행 삭제 · 잔여 작업중 7·법인리뷰 2, PTT상 진척 없음</t>
+          <t>PTT 0727 대조 — CP-en 게시 대상 아님으로 행 삭제 · JP-ja 법인리뷰→작업중 · 잔여 작업중 7·법인리뷰 2, PTT상 진척 없음</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -17321,11 +17321,7 @@
       </c>
       <c r="E33" s="123" t="inlineStr"/>
       <c r="F33" s="0" t="inlineStr"/>
-      <c r="G33" s="0" t="inlineStr">
-        <is>
-          <t>번역 문서 미비로 확인요청 중(PTT Request Clarification, 2026-03-30)</t>
-        </is>
-      </c>
+      <c r="G33" s="0" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="261" t="inlineStr">

</xml_diff>

<commit_message>
data(it): W16 MS PDP Gallery Card 대상 리스트 갱신 (473→403건)
구 /business/ 경로 정리 — DE 53→30, IN 35→4, SG 46→29, ES 52→53.
나머지 11개 로케일 URL 집합 동일. gr-urls·Page# 동기화(403=403).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -14209,8 +14209,7 @@
       </c>
       <c r="B2" s="128" t="inlineStr">
         <is>
-          <t>AU : URL 변경
-CN : 법인리뷰 → 완료</t>
+          <t>대상 리스트 갱신(총 403건) — 구 /business/ 경로 정리로 DE -23·IN -31·SG -17, ES +1 · GLOBAL 반영 완료</t>
         </is>
       </c>
       <c r="C2" s="129" t="n"/>
@@ -14427,7 +14426,7 @@
         </is>
       </c>
       <c r="F13" s="253" t="n">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="G13" s="244" t="inlineStr"/>
       <c r="H13" s="242" t="inlineStr"/>
@@ -14525,7 +14524,7 @@
       </c>
       <c r="C17" s="244" t="inlineStr">
         <is>
-          <t>https://www.lg.com/in/business/computers/laptops/lg-gram/14z90p-g-ah75a2/</t>
+          <t>https://www.lg.com/in/laptop/gram/14z90r-g-cp54a2/</t>
         </is>
       </c>
       <c r="D17" s="247" t="inlineStr">
@@ -14539,7 +14538,7 @@
         </is>
       </c>
       <c r="F17" s="257" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="G17" s="257" t="inlineStr"/>
       <c r="H17" s="257" t="inlineStr"/>
@@ -14623,7 +14622,7 @@
         </is>
       </c>
       <c r="F20" s="257" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="G20" s="257" t="inlineStr"/>
       <c r="H20" s="257" t="inlineStr"/>
@@ -16725,7 +16724,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
data(it): W30 Smart Monitor Screen Share — 라이브 17페이지만 남기고 전건 완료
사용자 확정 목록 17건 기준. STG(author 6·wwwstg 4)·미대상 8건 등 18행 삭제.
잔존 17건 실측 HTTP 200 확인. Page# 합계 17.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -9100,7 +9100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9123,7 +9123,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · Screen Share 카피/디스클레이머 삭제 · DAM 적재 완료(7/27) 지급 진행 · 대상 4모델(색상 파생 6)</t>
+          <t>라이브 게시 완료 — 대상 17페이지 전건 완료(실측 200 확인) · STG·미게시 행은 대상 제외</t>
         </is>
       </c>
     </row>
@@ -9177,7 +9177,12 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F4" s="0" t="n">
@@ -9202,7 +9207,12 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F5" s="0" t="n">
@@ -9217,17 +9227,22 @@
     <row r="6">
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>CO : CO (es)</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/smart-monitors/24u511sb-b/</t>
+          <t>https://www.lg.com/co/monitores/smart-monitores/24u511sb-b/</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F6" s="0" t="n">
@@ -9242,17 +9257,22 @@
     <row r="7">
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>CO : CO (es)</t>
+          <t>MX : MX (es)</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/co/monitores/smart-monitores/24u511sb-b/</t>
+          <t>https://www.lg.com/mx/monitores/monitores-smart/27u511sb-w/</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F7" s="0" t="n">
@@ -9260,24 +9280,29 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>24U511SB-B</t>
+          <t>27U511SB-W</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>AE : AE (en)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>https://wwwstg.lg.com/ae/consumer-monitors/lg-24u511sb-b</t>
+          <t>https://www.lg.com/sg/consumer-monitors/smart-monitors/27u511sb-w/</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F8" s="0" t="n">
@@ -9285,24 +9310,29 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>24U511SB-B · 페이지 QA review</t>
+          <t>27U511SB-W</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>BR : BR (pt)</t>
+          <t>IN : IN (en)</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/br/monitores/smart-monitors/24u511sb-b/</t>
+          <t>https://www.lg.com/in/monitors/smart-monitors/27u511sb-b/</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F9" s="0" t="n">
@@ -9310,24 +9340,29 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>24U511SB-B</t>
+          <t>27U511SB-B</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>MX : MX (es)</t>
+          <t>ID : ID (id)</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/mx/monitores/monitores-smart/27u511sb-w/</t>
+          <t>https://www.lg.com/id/monitor/smart-monitors/27u511sb/</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F10" s="0" t="n">
@@ -9342,17 +9377,22 @@
     <row r="11">
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>US : US (en)</t>
+          <t>CO : CO (es)</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/us/monitors/lg-27u511sb-w-smart-monitor</t>
+          <t>https://www.lg.com/co/monitores/smart-monitores/27u511sb-w/</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F11" s="0" t="n">
@@ -9367,17 +9407,22 @@
     <row r="12">
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>PE : PE (es)</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/consumer-monitors/smart-monitors/27u511sb-w/</t>
+          <t>https://www.lg.com/pe/monitores/fhd-y-qhd/27u511sb-w/</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F12" s="0" t="n">
@@ -9392,17 +9437,22 @@
     <row r="13">
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>IN : IN (en)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/in/monitors/smart-monitors/27u511sb-b/</t>
+          <t>https://www.lg.com/hk_en/monitors/smart-monitors/27u511sb-w/</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F13" s="0" t="n">
@@ -9410,24 +9460,29 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>27U511SB-B</t>
+          <t>27U511SB-W</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>ID : ID (id)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/id/monitor/smart-monitors/27u511sb/</t>
+          <t>https://www.lg.com/hk/monitors/smart-monitors/27u511sb-w/</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F14" s="0" t="n">
@@ -9442,17 +9497,22 @@
     <row r="15">
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>IN : IN (en)</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/smart-monitors/27u511sb-w/</t>
+          <t>https://www.lg.com/in/monitors/smart-monitors/32u501sb-b/</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F15" s="0" t="n">
@@ -9460,24 +9520,29 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>27U511SB-W</t>
+          <t>32U501SB-B</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>CO : CO (es)</t>
+          <t>ID : ID (id)</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/co/monitores/smart-monitores/27u511sb-w/</t>
+          <t>https://www.lg.com/id/monitor/smart-monitors/32u501sb/</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F16" s="0" t="n">
@@ -9485,24 +9550,29 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>27U511SB-W</t>
+          <t>32U501SB-B</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe/monitores/fhd-y-qhd/27u511sb-w/</t>
+          <t>https://www.lg.com/es/monitores/myview-smart-monitor/32u701sb-b/</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F17" s="0" t="n">
@@ -9510,24 +9580,29 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>27U511SB-W</t>
+          <t>32U701SB-B</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/monitors/smart-monitors/27u511sb-w/</t>
+          <t>https://www.lg.com/es/outlet/outlet-informatica/monitores/32u701sb-b-outlet/</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F18" s="0" t="n">
@@ -9535,24 +9610,29 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>27U511SB-W</t>
+          <t>32U701SB-B</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>IN : IN (en)</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/monitors/smart-monitors/27u511sb-w/</t>
+          <t>https://www.lg.com/in/monitors/smart-monitors/32u701sb-b/</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F19" s="0" t="n">
@@ -9560,480 +9640,35 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>27U511SB-W</t>
+          <t>32U701SB-B</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>AE : AE (en)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>https://wwwstg.lg.com/ae/consumer-monitors/lg-27u511sb-w</t>
+          <t>https://www.lg.com/tr/monitor/smart-monitorleri/32u701sb-b/</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F20" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="0" t="inlineStr">
-        <is>
-          <t>27U511SB-W · 페이지 WPL review</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="0" t="inlineStr">
-        <is>
-          <t>BR : BR (pt)</t>
-        </is>
-      </c>
-      <c r="C21" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/br/pt/monitores/smart-monitors/27u511sb-b.html?wcmmode=disabled</t>
-        </is>
-      </c>
-      <c r="D21" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F21" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="0" t="inlineStr">
-        <is>
-          <t>27U511SB-B · 페이지 New Request</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="0" t="inlineStr">
-        <is>
-          <t>JP : JP (ja)</t>
-        </is>
-      </c>
-      <c r="C22" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/jp/ja/monitors/smart-monitors/27u511sb-b.html?wcmmode=disabled</t>
-        </is>
-      </c>
-      <c r="D22" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F22" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="0" t="inlineStr">
-        <is>
-          <t>27U511SB-B · 페이지 Client Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="0" t="inlineStr">
-        <is>
-          <t>IN : IN (en)</t>
-        </is>
-      </c>
-      <c r="C23" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/in/monitors/smart-monitors/32u501sb-b/</t>
-        </is>
-      </c>
-      <c r="D23" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F23" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="0" t="inlineStr">
-        <is>
-          <t>32U501SB-B</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="0" t="inlineStr">
-        <is>
-          <t>ID : ID (id)</t>
-        </is>
-      </c>
-      <c r="C24" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/id/monitor/smart-monitors/32u501sb/</t>
-        </is>
-      </c>
-      <c r="D24" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F24" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="0" t="inlineStr">
-        <is>
-          <t>32U501SB-B</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="0" t="inlineStr">
-        <is>
-          <t>JP : JP (ja)</t>
-        </is>
-      </c>
-      <c r="C25" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/jp/monitors/smart-monitors/32u501sb-w/</t>
-        </is>
-      </c>
-      <c r="D25" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F25" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="0" t="inlineStr">
-        <is>
-          <t>32U501SB-W</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="0" t="inlineStr">
-        <is>
-          <t>AE : AE (en)</t>
-        </is>
-      </c>
-      <c r="C26" s="0" t="inlineStr">
-        <is>
-          <t>https://wwwstg.lg.com/ae/business/monitors/lg-32u501sb-b-ama</t>
-        </is>
-      </c>
-      <c r="D26" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F26" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="0" t="inlineStr">
-        <is>
-          <t>32U501SB-B · 페이지 In progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="0" t="inlineStr">
-        <is>
-          <t>UK : GB (en)</t>
-        </is>
-      </c>
-      <c r="C27" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/monitors/smart-monitors/32u501sb-b.html?wcmmode=disabled</t>
-        </is>
-      </c>
-      <c r="D27" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F27" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="0" t="inlineStr">
-        <is>
-          <t>32U501SB-B · 페이지 QA review</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="0" t="inlineStr">
-        <is>
-          <t>CO : CO (es)</t>
-        </is>
-      </c>
-      <c r="C28" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/co/monitores/smart-monitores/32u501sb-b/</t>
-        </is>
-      </c>
-      <c r="D28" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F28" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="0" t="inlineStr">
-        <is>
-          <t>32U501SB-B</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="0" t="inlineStr">
-        <is>
-          <t>AU : AU (en)</t>
-        </is>
-      </c>
-      <c r="C29" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/au/en/monitors/smart-monitors/32U501SB.html?wcmmode=disabled</t>
-        </is>
-      </c>
-      <c r="D29" s="0" t="inlineStr">
-        <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="F29" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="0" t="inlineStr">
-        <is>
-          <t>32U501SB · 페이지 Cancelled</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="0" t="inlineStr">
-        <is>
-          <t>US : US (en)</t>
-        </is>
-      </c>
-      <c r="C30" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/us/monitors/lg-32u701sb-b-smart-monitor</t>
-        </is>
-      </c>
-      <c r="D30" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F30" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="0" t="inlineStr">
-        <is>
-          <t>32U701SB-B</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="0" t="inlineStr">
-        <is>
-          <t>ES : ES (es)</t>
-        </is>
-      </c>
-      <c r="C31" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/es/monitores/myview-smart-monitor/32u701sb-b/</t>
-        </is>
-      </c>
-      <c r="D31" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F31" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="0" t="inlineStr">
-        <is>
-          <t>32U701SB-B</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="0" t="inlineStr">
-        <is>
-          <t>ES : ES (es)</t>
-        </is>
-      </c>
-      <c r="C32" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/es/outlet/outlet-informatica/monitores/32u701sb-b-outlet/</t>
-        </is>
-      </c>
-      <c r="D32" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F32" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="0" t="inlineStr">
-        <is>
-          <t>32U701SB-B</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="0" t="inlineStr">
-        <is>
-          <t>IN : IN (en)</t>
-        </is>
-      </c>
-      <c r="C33" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/in/monitors/smart-monitors/32u701sb-b/</t>
-        </is>
-      </c>
-      <c r="D33" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F33" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="0" t="inlineStr">
-        <is>
-          <t>32U701SB-B</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="0" t="inlineStr">
-        <is>
-          <t>TR : TR (tr)</t>
-        </is>
-      </c>
-      <c r="C34" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/tr/monitor/smart-monitorleri/32u701sb-b/</t>
-        </is>
-      </c>
-      <c r="D34" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F34" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="0" t="inlineStr">
-        <is>
-          <t>32U701SB-B</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="0" t="inlineStr">
-        <is>
-          <t>AE : AE (en)</t>
-        </is>
-      </c>
-      <c r="C35" s="0" t="inlineStr">
-        <is>
-          <t>https://wwwstg.lg.com/ae/consumer-monitors/lg-32u701sb-b</t>
-        </is>
-      </c>
-      <c r="D35" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F35" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="0" t="inlineStr">
-        <is>
-          <t>32U701SB-B · 페이지 QA review</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="0" t="inlineStr">
-        <is>
-          <t>ZA : ZA (en)</t>
-        </is>
-      </c>
-      <c r="C36" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/za/en/monitors/smart-monitors/32u701sb.html?wcmmode=disabled</t>
-        </is>
-      </c>
-      <c r="D36" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F36" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="0" t="inlineStr">
-        <is>
-          <t>32u701sb · 페이지 Client Approved</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="0" t="inlineStr">
-        <is>
-          <t>BR : BR (pt)</t>
-        </is>
-      </c>
-      <c r="C37" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/br/pt/monitores/smart-monitors/32u701sb-b.html?wcmmode=disabled</t>
-        </is>
-      </c>
-      <c r="D37" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F37" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="0" t="inlineStr">
-        <is>
-          <t>32U701SB-B · 페이지 QA review</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="0" t="inlineStr">
-        <is>
-          <t>CO : CO (es)</t>
-        </is>
-      </c>
-      <c r="C38" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/co/monitores/smart-monitores/32u701sb-b/</t>
-        </is>
-      </c>
-      <c r="D38" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="F38" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="0" t="inlineStr">
         <is>
           <t>32U701SB-B</t>
         </is>

</xml_diff>

<commit_message>
data(it): W17 GNB — IT·SE 작업중→법인리뷰
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -9100,7 +9100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9180,7 +9180,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9210,7 +9210,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9240,7 +9240,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9270,7 +9270,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9300,7 +9300,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9330,7 +9330,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9360,7 +9360,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9390,7 +9390,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9420,7 +9420,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9450,7 +9450,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9480,7 +9480,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9510,7 +9510,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9540,7 +9540,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9570,7 +9570,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9600,7 +9600,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9630,7 +9630,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -9660,7 +9660,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -14366,7 +14366,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.13" customWidth="1" style="203" min="1" max="1"/>
@@ -14396,10 +14396,8 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>CZ : 작업중 → 완료
-TR : 법인리뷰 → 작업중
-IN : 법인리뷰 → 완료 (7/16 게시, PTT 확인)
-TR : 작업중 → 완료 (7/23 게시, PTT 확인)</t>
+          <t>IT : 작업중 → 법인리뷰
+SE : 작업중 → 법인리뷰</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -14965,7 +14963,7 @@
       </c>
       <c r="D30" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E30" s="123" t="inlineStr"/>
@@ -15299,7 +15297,7 @@
       </c>
       <c r="D45" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E45" s="123" t="inlineStr"/>

</xml_diff>

<commit_message>
data(it): W22 Buying Guide — FR 법인리뷰→완료 (7/28 게시, 실측 200)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -14366,7 +14366,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.13" customWidth="1" style="203" min="1" max="1"/>
@@ -16357,7 +16357,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -16383,7 +16383,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>PTT 0727 대조 — CP-en 게시 대상 아님으로 행 삭제 · JP-ja 법인리뷰→작업중 · 잔여 작업중 7·법인리뷰 2, PTT상 진척 없음</t>
+          <t>FR : 법인리뷰 → 완료 (7/28 게시, 실측 200 확인) · 잔여 작업중 7·법인리뷰 1(CN)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -16765,14 +16765,24 @@
           <t>FR-fr</t>
         </is>
       </c>
-      <c r="C24" s="277" t="inlineStr"/>
+      <c r="C24" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/ultragear-buying-guide/</t>
+        </is>
+      </c>
       <c r="D24" s="263" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E24" s="123" t="inlineStr"/>
-      <c r="F24" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E24" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G24" s="0" t="inlineStr"/>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
data(it): W22 FR 완료일 정정 — 2026-07-24 (실제 게시일)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -16383,7 +16383,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>FR : 법인리뷰 → 완료 (7/28 게시, 실측 200 확인) · 잔여 작업중 7·법인리뷰 1(CN)</t>
+          <t>FR : 법인리뷰 → 완료 (7/24 게시, 실측 200 확인) · 잔여 작업중 7·법인리뷰 1(CN)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -16777,7 +16777,7 @@
       </c>
       <c r="E24" s="123" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F24" s="0" t="n">

</xml_diff>

<commit_message>
data(it): W31 gram Secure Lock 타겟 104→99건 (LGE 전달 리스트 기준)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -10035,7 +10035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>예정 · 13개국 대상 · CN은 PDP 라이브이나 기존 Secure Lock 컴포넌트 영역 없음</t>
+          <t>타겟 99건 확정(LGE 전달 리스트 기준) — 라이브 92 + STG만 7 · IN(gram 카테고리 없음)·FR(작성중 4) 대상 제외 · CN 7건은 PDP 라이브이나 기존 Secure Lock 영역 없음 · GR EP 품의 중, Jira 등록 예정</t>
         </is>
       </c>
     </row>
@@ -11302,10 +11302,14 @@
     <row r="52">
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>IN : IN (en)</t>
-        </is>
-      </c>
-      <c r="C52" s="0" t="inlineStr"/>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gs54j/</t>
+        </is>
+      </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -11316,7 +11320,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>- · Erase.Lock -</t>
+          <t>14Z90U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -11328,7 +11332,7 @@
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gs54j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gs58j/</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
@@ -11353,7 +11357,7 @@
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gs58j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gu85j/</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
@@ -11378,7 +11382,7 @@
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-gu85j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-vp58j/</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
@@ -11403,7 +11407,7 @@
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z90u-vp58j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs53j/</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
@@ -11416,7 +11420,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>14Z90U-G · Erase.Lock 있음</t>
+          <t>14Z95U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -11428,7 +11432,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs53j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs54j/</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -11453,7 +11457,7 @@
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs54j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs55j/</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
@@ -11478,7 +11482,7 @@
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gs55j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gu85j/</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
@@ -11503,7 +11507,7 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gu85j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gu86j/</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
@@ -11528,7 +11532,7 @@
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-gu86j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-vp53j/</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
@@ -11553,7 +11557,7 @@
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-vp53j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-vp55j/</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
@@ -11578,7 +11582,7 @@
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/14z95u-vp55j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-gu85j/</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
@@ -11591,7 +11595,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>14Z95U-G · Erase.Lock 있음</t>
+          <t>16Z90U-K · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -11603,7 +11607,7 @@
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-gu85j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-gu88j/</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
@@ -11628,7 +11632,7 @@
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-gu88j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-kub5j/</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
@@ -11653,7 +11657,7 @@
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-kub5j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-kub9j/</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
@@ -11678,7 +11682,7 @@
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-kub9j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z95u-gs55j/</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
@@ -11691,7 +11695,7 @@
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>16Z90U-K · Erase.Lock 있음</t>
+          <t>16Z95U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -11703,7 +11707,7 @@
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/16z95u-gs55j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z95u-gu88j/</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
@@ -11728,7 +11732,7 @@
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/16z95u-gu88j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-gu85j/</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
@@ -11741,7 +11745,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>16Z95U-G · Erase.Lock 있음</t>
+          <t>17Z90U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -11753,7 +11757,7 @@
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-gu85j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-gu88j/</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
@@ -11778,7 +11782,7 @@
       </c>
       <c r="C71" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-gu88j/</t>
+          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-vp55j/</t>
         </is>
       </c>
       <c r="D71" s="0" t="inlineStr">
@@ -11798,12 +11802,12 @@
     <row r="72">
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>CN : CN (zh)</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/17z90u-vp55j/</t>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal87c/</t>
         </is>
       </c>
       <c r="D72" s="0" t="inlineStr">
@@ -11816,7 +11820,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>17Z90U-G · Erase.Lock 있음</t>
+          <t>16Z90U-K · Erase.Lock 없음</t>
         </is>
       </c>
     </row>
@@ -11828,7 +11832,7 @@
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal87c/</t>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal88c/</t>
         </is>
       </c>
       <c r="D73" s="0" t="inlineStr">
@@ -11853,7 +11857,7 @@
       </c>
       <c r="C74" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal88c/</t>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb7c/</t>
         </is>
       </c>
       <c r="D74" s="0" t="inlineStr">
@@ -11878,7 +11882,7 @@
       </c>
       <c r="C75" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb7c/</t>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb8c/</t>
         </is>
       </c>
       <c r="D75" s="0" t="inlineStr">
@@ -11903,7 +11907,7 @@
       </c>
       <c r="C76" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb8c/</t>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb9c/</t>
         </is>
       </c>
       <c r="D76" s="0" t="inlineStr">
@@ -11928,7 +11932,7 @@
       </c>
       <c r="C77" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb9c/</t>
+          <t>https://www.lg.com/cn/notebooks/lg-17z90u-al87c/</t>
         </is>
       </c>
       <c r="D77" s="0" t="inlineStr">
@@ -11941,7 +11945,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>16Z90U-K · Erase.Lock 없음</t>
+          <t>17Z90U-G · Erase.Lock 없음</t>
         </is>
       </c>
     </row>
@@ -11953,7 +11957,7 @@
       </c>
       <c r="C78" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-17z90u-al87c/</t>
+          <t>https://www.lg.com/cn/notebooks/lg-17z90u-gal88c/</t>
         </is>
       </c>
       <c r="D78" s="0" t="inlineStr">
@@ -11973,12 +11977,12 @@
     <row r="79">
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-17z90u-gal88c/</t>
+          <t>https://www.lg.com/ca_en/laptops/16z95u-g/</t>
         </is>
       </c>
       <c r="D79" s="0" t="inlineStr">
@@ -11991,7 +11995,7 @@
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>17Z90U-G · Erase.Lock 없음</t>
+          <t>16Z95U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -12003,7 +12007,7 @@
       </c>
       <c r="C80" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/laptops/16z95u-g/</t>
+          <t>https://www.lg.com/ca_en/small-medium-business/laptops/16z95u-g/</t>
         </is>
       </c>
       <c r="D80" s="0" t="inlineStr">
@@ -12023,12 +12027,12 @@
     <row r="81">
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/small-medium-business/laptops/16z95u-g/</t>
+          <t>https://www.lg.com/ca_fr/ordinateurs-portables/16z95u-g/</t>
         </is>
       </c>
       <c r="D81" s="0" t="inlineStr">
@@ -12053,7 +12057,7 @@
       </c>
       <c r="C82" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/ordinateurs-portables/16z95u-g/</t>
+          <t>https://www.lg.com/ca_fr/small-medium-business/ordinateurs-portables/16z95u-g/</t>
         </is>
       </c>
       <c r="D82" s="0" t="inlineStr">
@@ -12073,12 +12077,12 @@
     <row r="83">
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/small-medium-business/ordinateurs-portables/16z95u-g/</t>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g78/</t>
         </is>
       </c>
       <c r="D83" s="0" t="inlineStr">
@@ -12091,7 +12095,7 @@
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>16Z95U-G · Erase.Lock 있음</t>
+          <t>17Z90U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -12103,7 +12107,7 @@
       </c>
       <c r="C84" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g78/</t>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g88/</t>
         </is>
       </c>
       <c r="D84" s="0" t="inlineStr">
@@ -12128,7 +12132,7 @@
       </c>
       <c r="C85" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g88/</t>
+          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90u-g78/</t>
         </is>
       </c>
       <c r="D85" s="0" t="inlineStr">
@@ -12153,7 +12157,7 @@
       </c>
       <c r="C86" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90u-g78/</t>
+          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90u-g88/</t>
         </is>
       </c>
       <c r="D86" s="0" t="inlineStr">
@@ -12173,12 +12177,12 @@
     <row r="87">
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90u-g88/</t>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g78/</t>
         </is>
       </c>
       <c r="D87" s="0" t="inlineStr">
@@ -12203,7 +12207,7 @@
       </c>
       <c r="C88" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g78/</t>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g88/</t>
         </is>
       </c>
       <c r="D88" s="0" t="inlineStr">
@@ -12223,12 +12227,12 @@
     <row r="89">
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g88/</t>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ub-h/</t>
         </is>
       </c>
       <c r="D89" s="0" t="inlineStr">
@@ -12241,7 +12245,7 @@
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>17Z90U-G · Erase.Lock 있음</t>
+          <t>17Z90UB-H · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -12253,7 +12257,7 @@
       </c>
       <c r="C90" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ub-h/</t>
+          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90ub-h/</t>
         </is>
       </c>
       <c r="D90" s="0" t="inlineStr">
@@ -12273,12 +12277,12 @@
     <row r="91">
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/small-medium-business/laptops/all-laptops/17z90ub-h/</t>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90ub-h/</t>
         </is>
       </c>
       <c r="D91" s="0" t="inlineStr">
@@ -12303,7 +12307,7 @@
       </c>
       <c r="C92" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90ub-h/</t>
+          <t>https://www.lg.com/ca_fr/small-medium-business/computing/purchase-guide/laptops/17z90ub-h/</t>
         </is>
       </c>
       <c r="D92" s="0" t="inlineStr">
@@ -12323,12 +12327,12 @@
     <row r="93">
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/small-medium-business/computing/purchase-guide/laptops/17z90ub-h/</t>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/ca/en/laptops/all-laptops/17z90ub-h.html?wcmmode=disabled</t>
         </is>
       </c>
       <c r="D93" s="0" t="inlineStr">
@@ -12341,7 +12345,7 @@
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>17Z90UB-H · Erase.Lock 있음</t>
+          <t>17Z90UR-P · Erase.Lock -</t>
         </is>
       </c>
     </row>
@@ -12353,7 +12357,7 @@
       </c>
       <c r="C94" s="0" t="inlineStr">
         <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/ca/en/laptops/all-laptops/17z90ub-h.html?wcmmode=disabled</t>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ur-p/</t>
         </is>
       </c>
       <c r="D94" s="0" t="inlineStr">
@@ -12366,19 +12370,19 @@
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>17Z90UR-P · Erase.Lock -</t>
+          <t>17Z90UR-P · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ur-p/</t>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17Z90ur-p/</t>
         </is>
       </c>
       <c r="D95" s="0" t="inlineStr">
@@ -12403,7 +12407,7 @@
       </c>
       <c r="C96" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17Z90ur-p/</t>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/ca/fr/computing/purchase-guide/laptops/17z90ub-h.html?wcmmode=disabled</t>
         </is>
       </c>
       <c r="D96" s="0" t="inlineStr">
@@ -12416,19 +12420,19 @@
       </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
-          <t>17Z90UR-P · Erase.Lock 있음</t>
+          <t>17Z90UR-P · Erase.Lock -</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>AU : AU (en)</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
         <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/ca/fr/computing/purchase-guide/laptops/17z90ub-h.html?wcmmode=disabled</t>
+          <t>https://www.lg.com/au/laptops/gram-pro/16z90u-g-au75ap/</t>
         </is>
       </c>
       <c r="D97" s="0" t="inlineStr">
@@ -12441,17 +12445,21 @@
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>17Z90UR-P · Erase.Lock -</t>
+          <t>16Z90U-G.AU75AP · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C98" s="0" t="inlineStr"/>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C98" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/16z90u-g-au88ap/</t>
+        </is>
+      </c>
       <c r="D98" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -12462,17 +12470,21 @@
       </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
-          <t>15U50U-G · Erase.Lock -</t>
+          <t>16Z90U-K · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C99" s="0" t="inlineStr"/>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C99" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au75ap/</t>
+        </is>
+      </c>
       <c r="D99" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -12483,17 +12495,21 @@
       </c>
       <c r="G99" s="0" t="inlineStr">
         <is>
-          <t>15Z95U-G · Erase.Lock -</t>
+          <t>17Z90U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C100" s="0" t="inlineStr"/>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C100" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au78ap/</t>
+        </is>
+      </c>
       <c r="D100" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -12504,17 +12520,21 @@
       </c>
       <c r="G100" s="0" t="inlineStr">
         <is>
-          <t>16Z90U-G · Erase.Lock -</t>
+          <t>17Z90U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C101" s="0" t="inlineStr"/>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C101" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au88ap/</t>
+        </is>
+      </c>
       <c r="D101" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -12525,7 +12545,7 @@
       </c>
       <c r="G101" s="0" t="inlineStr">
         <is>
-          <t>17Z90U-G · Erase.Lock -</t>
+          <t>17Z90U-G · Erase.Lock 있음</t>
         </is>
       </c>
     </row>
@@ -12537,7 +12557,7 @@
       </c>
       <c r="C102" s="0" t="inlineStr">
         <is>
-          <t>https://www.lg.com/au/laptops/gram-pro/16z90u-g-au75ap/</t>
+          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/au/en/laptops/gram-pro/17z90ub-h.html?wcmmode=disabled</t>
         </is>
       </c>
       <c r="D102" s="0" t="inlineStr">
@@ -12549,131 +12569,6 @@
         <v>1</v>
       </c>
       <c r="G102" s="0" t="inlineStr">
-        <is>
-          <t>16Z90U-G.AU75AP · Erase.Lock 있음</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="B103" s="0" t="inlineStr">
-        <is>
-          <t>AU : AU (en)</t>
-        </is>
-      </c>
-      <c r="C103" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/au/laptops/gram-pro/16z90u-g-au88ap/</t>
-        </is>
-      </c>
-      <c r="D103" s="0" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="F103" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G103" s="0" t="inlineStr">
-        <is>
-          <t>16Z90U-K · Erase.Lock 있음</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="B104" s="0" t="inlineStr">
-        <is>
-          <t>AU : AU (en)</t>
-        </is>
-      </c>
-      <c r="C104" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au75ap/</t>
-        </is>
-      </c>
-      <c r="D104" s="0" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="F104" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G104" s="0" t="inlineStr">
-        <is>
-          <t>17Z90U-G · Erase.Lock 있음</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="B105" s="0" t="inlineStr">
-        <is>
-          <t>AU : AU (en)</t>
-        </is>
-      </c>
-      <c r="C105" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au78ap/</t>
-        </is>
-      </c>
-      <c r="D105" s="0" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="F105" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G105" s="0" t="inlineStr">
-        <is>
-          <t>17Z90U-G · Erase.Lock 있음</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="B106" s="0" t="inlineStr">
-        <is>
-          <t>AU : AU (en)</t>
-        </is>
-      </c>
-      <c r="C106" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au88ap/</t>
-        </is>
-      </c>
-      <c r="D106" s="0" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="F106" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G106" s="0" t="inlineStr">
-        <is>
-          <t>17Z90U-G · Erase.Lock 있음</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="B107" s="0" t="inlineStr">
-        <is>
-          <t>AU : AU (en)</t>
-        </is>
-      </c>
-      <c r="C107" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/au/en/laptops/gram-pro/17z90ub-h.html?wcmmode=disabled</t>
-        </is>
-      </c>
-      <c r="D107" s="0" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="F107" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G107" s="0" t="inlineStr">
         <is>
           <t>17Z90UB-H · Erase.Lock -</t>
         </is>
@@ -16357,7 +16252,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
data(it): W31 gram Secure Lock — CN 7건 취소(기존 Secure Lock 영역 없음)
99행 유지, 완료율 분모 92. LGE 리스트 대조를 위해 삭제 대신 취소 처리.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -10058,7 +10058,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>타겟 99건 확정(LGE 전달 리스트 기준) — 라이브 92 + STG만 7 · IN(gram 카테고리 없음)·FR(작성중 4) 대상 제외 · CN 7건은 PDP 라이브이나 기존 Secure Lock 영역 없음 · GR EP 품의 중, Jira 등록 예정</t>
+          <t>타겟 99건(LGE 전달 리스트) — 실질 교체 대상 92건 · CN 7건은 PDP 라이브이나 기존 Secure Lock 영역 없어 취소(원본 Erase.Lock 모듈=없음) · 라이브 92 + STG만 7 · IN·FR은 페이지 미존재로 리스트 제외 · GR EP 품의 중, Jira 등록 예정</t>
         </is>
       </c>
     </row>
@@ -11812,7 +11812,7 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="F72" s="0" t="n">
@@ -11820,7 +11820,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>16Z90U-K · Erase.Lock 없음</t>
+          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
         </is>
       </c>
     </row>
@@ -11837,7 +11837,7 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="F73" s="0" t="n">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>16Z90U-K · Erase.Lock 없음</t>
+          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
         </is>
       </c>
     </row>
@@ -11862,7 +11862,7 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="F74" s="0" t="n">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>16Z90U-K · Erase.Lock 없음</t>
+          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
         </is>
       </c>
     </row>
@@ -11887,7 +11887,7 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="F75" s="0" t="n">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>16Z90U-K · Erase.Lock 없음</t>
+          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
         </is>
       </c>
     </row>
@@ -11912,7 +11912,7 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="F76" s="0" t="n">
@@ -11920,7 +11920,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>16Z90U-K · Erase.Lock 없음</t>
+          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
         </is>
       </c>
     </row>
@@ -11937,7 +11937,7 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="F77" s="0" t="n">
@@ -11945,7 +11945,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>17Z90U-G · Erase.Lock 없음</t>
+          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
         </is>
       </c>
     </row>
@@ -11962,7 +11962,7 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="F78" s="0" t="n">
@@ -11970,7 +11970,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>17Z90U-G · Erase.Lock 없음</t>
+          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
security(it): STG URL(AEM author) 전면 제거 — 공개 저장소 노출 차단 (v0.6.57)
LGE 보안 점검 지시(2026-07-30). 이 저장소는 PUBLIC이라 AEM author 인스턴스 URL
(author-p86205-e734304.adobeaemcloud.com)과 스테이징 도메인이 노출되고 있었다.

  · it/data/npi-product-status.json — stgUrl 16건 제거
  · it/data/npi.json — wwwstg.lg.com liveUrl 1건 제거
  · it/Global Request.xlsx — 셀 7 + 상단 참조 6 + 하이퍼링크 16건 제거(_rels XML 포함)
  · it/common.js — 'STG URL' 컬럼 제거

it/ 기준 author-p86205·adobeaemcloud·wwwstg 잔존 0건.
※ hs/common.js의 평문 비밀번호(ACCESS_PWD)는 담당 확인 필요 — 이번 커밋 범위 밖.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -1540,11 +1540,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/ui</t>
-        </is>
-      </c>
+      <c r="B3" s="10" t="n"/>
       <c r="C3" s="11" t="n"/>
       <c r="D3" s="11" t="n"/>
       <c r="E3" s="12" t="n"/>
@@ -2880,55 +2876,54 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" location="/aem/assets.html/content/dam/master-2/hs/lgcom/lgcom-common/guide" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2940,7 +2935,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -2980,6 +2975,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -3455,7 +3451,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -3495,6 +3491,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -4692,7 +4689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5292,7 +5289,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -5332,6 +5329,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -7001,7 +6999,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -7041,6 +7039,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -9100,7 +9099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9685,7 +9684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11180,11 +11179,7 @@
           <t>UK : GB (en)</t>
         </is>
       </c>
-      <c r="C47" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/laptops/gram/15u50u-g-aa55an.html?wcmmode=disabled</t>
-        </is>
-      </c>
+      <c r="C47" s="0" t="n"/>
       <c r="D47" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -11205,11 +11200,7 @@
           <t>UK : GB (en)</t>
         </is>
       </c>
-      <c r="C48" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/laptops/gram-pro/16z90u-h-au78an.html?wcmmode=disabled</t>
-        </is>
-      </c>
+      <c r="C48" s="0" t="n"/>
       <c r="D48" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -11230,11 +11221,7 @@
           <t>UK : GB (en)</t>
         </is>
       </c>
-      <c r="C49" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/laptops/gram-pro/16z90u-k-aub8an.html?wcmmode=disabled</t>
-        </is>
-      </c>
+      <c r="C49" s="0" t="n"/>
       <c r="D49" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -11255,11 +11242,7 @@
           <t>UK : GB (en)</t>
         </is>
       </c>
-      <c r="C50" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/gb/en/laptops/gram-pro/17z90u-g-au78an.html?wcmmode=disabled</t>
-        </is>
-      </c>
+      <c r="C50" s="0" t="n"/>
       <c r="D50" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -12330,11 +12313,7 @@
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C93" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/ca/en/laptops/all-laptops/17z90ub-h.html?wcmmode=disabled</t>
-        </is>
-      </c>
+      <c r="C93" s="0" t="n"/>
       <c r="D93" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -12405,11 +12384,7 @@
           <t>CA_FR : CA (fr)</t>
         </is>
       </c>
-      <c r="C96" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/ca/fr/computing/purchase-guide/laptops/17z90ub-h.html?wcmmode=disabled</t>
-        </is>
-      </c>
+      <c r="C96" s="0" t="n"/>
       <c r="D96" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -12555,11 +12530,7 @@
           <t>AU : AU (en)</t>
         </is>
       </c>
-      <c r="C102" s="0" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/content/lge/au/en/laptops/gram-pro/17z90ub-h.html?wcmmode=disabled</t>
-        </is>
-      </c>
+      <c r="C102" s="0" t="n"/>
       <c r="D102" s="0" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -12585,7 +12556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12660,7 +12631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13674,25 +13645,15 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" location="/aem/assets.html/content/dam/master-2/hs/lgcom/lgcom-common/article/2025/2025-lg-experience-article/ref/article-sa-01-refrigerator_size_guide" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13750,11 +13711,7 @@
     </row>
     <row r="3">
       <c r="A3" s="35" t="n"/>
-      <c r="B3" s="130" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/ui</t>
-        </is>
-      </c>
+      <c r="B3" s="130" t="n"/>
       <c r="C3" s="131" t="n"/>
       <c r="D3" s="131" t="n"/>
       <c r="E3" s="132" t="n"/>
@@ -13763,11 +13720,7 @@
     </row>
     <row r="4">
       <c r="A4" s="35" t="n"/>
-      <c r="B4" s="130" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/ui</t>
-        </is>
-      </c>
+      <c r="B4" s="130" t="n"/>
       <c r="C4" s="131" t="n"/>
       <c r="D4" s="131" t="n"/>
       <c r="E4" s="132" t="n"/>
@@ -13776,17 +13729,14 @@
     </row>
     <row r="5">
       <c r="A5" s="35" t="n"/>
-      <c r="B5" s="133" t="inlineStr">
-        <is>
-          <t>https://kor01.safelinks.protection.outlook.com/?url=https%3A%2F%2Fauthor-p86205-e734304.adobeaemcloud.com%2Fui%23%2Faem%2Fassets.html%2Fcontent%2Fdam%2Fmaster-2%2Fhs%2Flgcom%2Flgcom-common%2Farticle%2F2026%2Fcmr&amp;data=05%7C02%7Cjoanna.ryu%40lge.com%7Cf47462a11643436ac07e08de7a8eb1f1%7C5069cde4642a45c08094d0c2dec10be3%7C0%7C0%7C639082950459597401%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=a9NRjuFBdR6yzh7pn8l3w4sfQLCA2HMxO9fzLIOFqYU%3D&amp;reserved=0</t>
-        </is>
-      </c>
+      <c r="B5" s="133" t="n"/>
       <c r="C5" s="134" t="n"/>
       <c r="D5" s="134" t="n"/>
       <c r="E5" s="135" t="n"/>
       <c r="G5" s="127" t="n"/>
     </row>
     <row r="6" ht="40.5" customHeight="1" s="203"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
@@ -14244,12 +14194,9 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" location="/aem/assets.html/content/dam/master-2/hs/lgcom/lgcom-common/microsite/reliable-microsite/global" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" location="/aem/assets.html/content/dam/master-2/hs/lgcom/lgcom-common/microsite/reliable-microsite/local" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14261,7 +14208,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.13" customWidth="1" style="203" min="1" max="1"/>
@@ -15420,16 +15367,16 @@
     </row>
     <row r="3">
       <c r="A3" s="166" t="n"/>
-      <c r="B3" s="130" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/ui</t>
-        </is>
-      </c>
+      <c r="B3" s="130" t="n"/>
       <c r="C3" s="131" t="n"/>
       <c r="D3" s="131" t="n"/>
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -15795,18 +15742,17 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" location="/aem/assets.html/content/dam/master-2/hs/lgcom/lgcom-common/microsite/ice-solution-2026" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15818,7 +15764,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="22.75" customWidth="1" style="203" min="1" max="1"/>
@@ -15858,11 +15804,7 @@
     </row>
     <row r="3">
       <c r="A3" s="192" t="n"/>
-      <c r="B3" s="193" t="inlineStr">
-        <is>
-          <t>https://author-p86205-e734304.adobeaemcloud.com/ui</t>
-        </is>
-      </c>
+      <c r="B3" s="193" t="n"/>
       <c r="C3" s="194" t="n"/>
       <c r="D3" s="194" t="n"/>
       <c r="E3" s="195" t="n"/>
@@ -16239,9 +16181,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" location="/aem/assets.html/content/dam/master-2/hs/lgcom/lgcom-common/microsite/appliances-faq-hub" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16252,7 +16191,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -16292,6 +16231,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -17277,7 +17217,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -17317,6 +17257,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -17826,7 +17767,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -17866,6 +17807,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat(it): STG 유무 컬럼 + PTT 0802·Readiness 0803 반영, W31 Win11 Pro 79건 완료 (v0.6.58)
STG는 주소 없이 유무(O/-)만 표시 — 보안 조치 유지(author/aem 잔존 0).
PTT 0802: AU 1건 Closed. Readiness 0803: IT 3건 Ready(31→34).
W31 PDP Gallery Win11 Pro 79건 전건 완료.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -2935,7 +2935,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -2975,7 +2975,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -3451,7 +3450,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -3491,7 +3490,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -4689,7 +4687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5289,7 +5287,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -5329,7 +5327,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -6999,7 +6996,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -7039,7 +7036,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -9099,7 +9095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9684,7 +9680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10034,7 +10030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12556,7 +12552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12631,7 +12627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12654,7 +12650,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · W16 PDP Gallery Card 후속 건 · Windows 11 Pro 영상 수정 · 대상 목록 미수신(확인 필요)</t>
+          <t>전건 완료 — Win11 Pro 영상 수정 79건 · 13개국 · 완료율 100%</t>
         </is>
       </c>
     </row>
@@ -12692,6 +12688,2376 @@
       <c r="G3" s="0" t="inlineStr">
         <is>
           <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro-2-in-1/16t90sp-g-ap55a/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>16T90SP-G.AP55A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro-2-in-1/16t90sp-g-ap75a/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>16T90SP-G.AP75A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/14-inch-lg-gram-laptops/14z90s-v-ap55a8/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>14Z90S-V.AP55A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/14-inch-lg-gram-laptops/14z90t-v-ap75a8/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>14Z90T-V.AP75A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90s-v-ap55a8/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>16Z90S-V.AP55A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90sp-r-ap85a8/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>16Z90SP-R.AP85A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90t-v-ap75a8/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>16Z90T-V.AP75A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90t-v-ap88a8/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>16Z90T-V.AP88A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90tr-e-ap88a8/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>16Z90TR-E.AP88A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/17-inch-lg-gram-laptops/17z90t-v-ap75a8/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>17Z90T-V.AP75A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/it-products/laptops/17-inch-lg-gram-laptops/17z90t-v-ap88a8/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>17Z90T-V.AP88A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-14z90ruap55c</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>14Z90RU-G.AP55C</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90ruap55c</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>16Z90RU-G.AP55C</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16t90q-g-ap79g/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>16T90Q-G.AP79G</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16t90r-g/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>16T90R-G.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16t90sp-k-ap78g/</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>16T90SP-K.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16tb90tp-k-ap78g/</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>16TB90TP-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram-2-in-1/16tb90tp-k-ap78g/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>16TB90TP-K.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16z90q-g-ap55g/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>16Z90Q-G.AP55G</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16z90s-g-ap55g/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>16Z90S-G.AP55G</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16z90s-g-ap78g/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>16Z90S-G.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16z90sp-a-ap7bg/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>16Z90SP-A.AP7BG</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16zb90r-g-ap75g/</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>16ZB90R-G.AP75G</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16zb90r-g-ap78g/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>16ZB90R-G.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/16zb90ru-g-ap55g/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>16ZB90RU-G.AP55G</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram/16zb90ru-g-ap55g/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>16ZB90RU-G.AP55G</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/17z90p-g-ap78g/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>17Z90P-G.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/17z90q-g-ap75g/</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>17Z90Q-G.AP75G</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/17z90q-g-ap78g/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>17Z90Q-G.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/17z90q-g-ap79g/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>17Z90Q-G.AP79G</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/notebooks/gram/17z90r-g-ap7cg/</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>17Z90R-G.AP7CG</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/17z90s-g-ap56g/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>17Z90S-G.AP56G</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/17z90s-g-ap78g/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>17Z90S-G.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/17z90sp-e-ap7bg/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>17Z90SP-E.AP7BG</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/business/gram/17zb90r-g-ap78g/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>17ZB90R-G.AP78G</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/business/informatica/ordenadores/portatiles-ultraligeros/14z90r-v-ap55b/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>14Z90R-V.AP55B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/14Z90ru-g-ap55b/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>14Z90RU-G.AP55B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/14z90s-v-ap75b/</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>14Z90S-V.AP75B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/laptops/gram/14z90t-v-ap88b/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>14Z90T-V.AP88B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/business/informatica/ordenadores/portatiles-ultraligeros/16z90p-g-ap77b/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>16Z90P-G-AP77B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/16z90ru-g-ap55b/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>16Z90RU-G.AP55B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/16z90t-v-ap88b/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>16Z90T-V.AP88B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/17z90t-v-ap88b/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>17Z90T-V.AP88B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/pc-portables/gram/lg-15u50t-g-ap56f/</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>LG 15U50T-G.AP56F</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/pc-portables/gram/lg-16z90r-g-ap7bf-i7-32go-2to-win-11-pro/</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>LG 16Z90R-G.AP7BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/pc-portables/gram/lg-16z90ru-g-ap55f-i5-16go-512go-win-11-pro/</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>LG 16Z90RU-G.AP55F</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/pc-portables/gram/lg-17z90ru-g-ap55f-i5-16go-512go-win-11-pro/</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>LG 17Z90RU-G.AP55F</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram/14z90r-q/</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>14Z90R-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-book/15ub50t/</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>15UB50T</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram/16z90r-q/</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>16Z90R-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram/17z90r-q/</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>17Z90R-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/business/computers/laptops/lg-gram/14z980-gap52a2/</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>14Z980-GAP52A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/gram/14z90ru-g-ap55d1/</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>14Z90RU-G.AP55D1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/15ub50t-g-ap56d/</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>15UB50T-G</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/gram/16z90ru-g-ap55d1/</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>16Z90RU-G.AP55D1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/16z90s-g-ap55d/</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>16Z90S-G.AP55D</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/16z90s-g-ap78d/</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>16Z90S-G.AP78D</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/gram/17z90ru-g/</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>17Z90RU-G</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/gram/17z90s-g/</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>17Z90S-G.AP78D</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90ru-gp51j/</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>14Z90RU-GP51J</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90s-vp55j/</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>14Z90S-VP55J</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90s-vp56j/</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>14Z90S-VP56J</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/14z90t-vp55j/</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>14Z90T-VP55J</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/17z90s-vp55j/</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>17Z90S-VP55J</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/14z90s-v-ap75a3/</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>14Z90S-V.AP75A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/14z90t-g-ap75a3/</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>14Z90T-G.AP75A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/14z90t-g-ap88a3/</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>14Z90T-G.AP88A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/15z90st-v-ap75a3/</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>15Z90ST-V.AP75A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/16t90tp-k-ap88a3/</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>16T90TP-K.AP88A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90s-v-ap75a3/</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>16Z90S-V.AP75A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90s-v-ap78a3/</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>16Z90S-V.AP78A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90s-v-ap88a3/</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>16Z90S-V.AP88A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram/14z90r-v-ap56c2/</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>14Z90R-V</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram/14z90s-v-ap55c2/</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>14Z90S-V</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram/14z90s-v-ap54c2/</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>14Z90S-V</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram/14z90t-g-ap55c2/</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>14Z90T-G</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram/15u50t-g-ap56c2/</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>15U50T-G</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/business/san-pham-tin-hoc/laptop/16z90r-c-apl1y/</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>16Z90R-C</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/16z90s-g-ap76a5/</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>16Z90S-G.AP76A5</t>
         </is>
       </c>
     </row>
@@ -13736,7 +16102,6 @@
       <c r="G5" s="127" t="n"/>
     </row>
     <row r="6" ht="40.5" customHeight="1" s="203"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
@@ -14208,7 +16573,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.13" customWidth="1" style="203" min="1" max="1"/>
@@ -15373,10 +17738,6 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -15764,7 +18125,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="22.75" customWidth="1" style="203" min="1" max="1"/>
@@ -16191,7 +18552,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -16231,7 +18592,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -17217,7 +19577,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -17257,7 +19617,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -17767,7 +20126,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -17807,7 +20166,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>

</xml_diff>

<commit_message>
data(it): W18 UltraGear OLED FAQ ES 완료 + gr-changes 최신 재생성
- W18 UltraGear/OLED Gaming Monitor PLP FAQ Update: ES 법인리뷰→완료
  (2026-08-04 게시, 실측 200). URL도 실제 게시처로 정정
  /es/monitores/monitores-ultragear-gaming/
    → /es/monitores/monitores-ultragear-oled-gaming/
  완료율 82% → 91% (9/11 → 10/11)
- gr-changes: prevDate 20260728 → baseDate 20260804, 30건으로 재생성
  (기존 87건은 7/16→7/27 비교분으로 낡았고, diff 비대칭 버그로 가짜 변경 포함)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -12692,2370 +12692,2370 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>AU : AU (en)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/au/laptops/gram-pro-2-in-1/16t90sp-g-ap55a/</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="F4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
         <is>
           <t>16T90SP-G.AP55A</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>AU : AU (en)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/au/laptops/gram-pro-2-in-1/16t90sp-g-ap75a/</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="F5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
         <is>
           <t>16T90SP-G.AP75A</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/14-inch-lg-gram-laptops/14z90s-v-ap55a8/</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="F6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
         <is>
           <t>14Z90S-V.AP55A8</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/14-inch-lg-gram-laptops/14z90t-v-ap75a8/</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="F7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
         <is>
           <t>14Z90T-V.AP75A8</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90s-v-ap55a8/</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="F8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
         <is>
           <t>16Z90S-V.AP55A8</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90sp-r-ap85a8/</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="F9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
         <is>
           <t>16Z90SP-R.AP85A8</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90t-v-ap75a8/</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="F10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
         <is>
           <t>16Z90T-V.AP75A8</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90t-v-ap88a8/</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
         <is>
           <t>16Z90T-V.AP88A8</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/16-inch-lg-gram-laptops/16z90tr-e-ap88a8/</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="F12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
         <is>
           <t>16Z90TR-E.AP88A8</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/17-inch-lg-gram-laptops/17z90t-v-ap75a8/</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="F13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
         <is>
           <t>17Z90T-V.AP75A8</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_en/business/it-products/laptops/17-inch-lg-gram-laptops/17z90t-v-ap88a8/</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="F14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
         <is>
           <t>17Z90T-V.AP88A8</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>CN : CN (zh)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/cn/notebooks/lg-14z90ruap55c</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="F15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
         <is>
           <t>14Z90RU-G.AP55C</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>CN : CN (zh)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/cn/notebooks/lg-16z90ruap55c</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="F16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
         <is>
           <t>16Z90RU-G.AP55C</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16t90q-g-ap79g/</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
         <is>
           <t>16T90Q-G.AP79G</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16t90r-g/</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="F18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
         <is>
           <t>16T90R-G.AP78G</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16t90sp-k-ap78g/</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="F19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
         <is>
           <t>16T90SP-K.AP78G</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16tb90tp-k-ap78g/</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="F20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
         <is>
           <t>16TB90TP-K</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/notebooks/gram-2-in-1/16tb90tp-k-ap78g/</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="F21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
         <is>
           <t>16TB90TP-K.AP78G</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16z90q-g-ap55g/</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="F22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
         <is>
           <t>16Z90Q-G.AP55G</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16z90s-g-ap55g/</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="F23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
         <is>
           <t>16Z90S-G.AP55G</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16z90s-g-ap78g/</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="F24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
         <is>
           <t>16Z90S-G.AP78G</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16z90sp-a-ap7bg/</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="F25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
         <is>
           <t>16Z90SP-A.AP7BG</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16zb90r-g-ap75g/</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" t="inlineStr">
+      <c r="F26" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
         <is>
           <t>16ZB90R-G.AP75G</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16zb90r-g-ap78g/</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" t="inlineStr">
+      <c r="F27" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
         <is>
           <t>16ZB90R-G.AP78G</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/16zb90ru-g-ap55g/</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="F28" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
         <is>
           <t>16ZB90RU-G.AP55G</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/notebooks/gram/16zb90ru-g-ap55g/</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" t="inlineStr">
+      <c r="F29" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
         <is>
           <t>16ZB90RU-G.AP55G</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/17z90p-g-ap78g/</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" t="inlineStr">
+      <c r="F30" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
         <is>
           <t>17Z90P-G.AP78G</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/17z90q-g-ap75g/</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" t="inlineStr">
+      <c r="F31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="0" t="inlineStr">
         <is>
           <t>17Z90Q-G.AP75G</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/17z90q-g-ap78g/</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" t="inlineStr">
+      <c r="F32" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
         <is>
           <t>17Z90Q-G.AP78G</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/17z90q-g-ap79g/</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" t="inlineStr">
+      <c r="F33" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="0" t="inlineStr">
         <is>
           <t>17Z90Q-G.AP79G</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/notebooks/gram/17z90r-g-ap7cg/</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" t="inlineStr">
+      <c r="F34" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
         <is>
           <t>17Z90R-G.AP7CG</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/17z90s-g-ap56g/</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" t="inlineStr">
+      <c r="F35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
         <is>
           <t>17Z90S-G.AP56G</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/17z90s-g-ap78g/</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" t="inlineStr">
+      <c r="F36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="0" t="inlineStr">
         <is>
           <t>17Z90S-G.AP78G</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/17z90sp-e-ap7bg/</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" t="inlineStr">
+      <c r="F37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
         <is>
           <t>17Z90SP-E.AP7BG</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/business/gram/17zb90r-g-ap78g/</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" t="inlineStr">
+      <c r="F38" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="0" t="inlineStr">
         <is>
           <t>17ZB90R-G.AP78G</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/business/informatica/ordenadores/portatiles-ultraligeros/14z90r-v-ap55b/</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" t="inlineStr">
+      <c r="F39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="0" t="inlineStr">
         <is>
           <t>14Z90R-V.AP55B</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/portatiles/gram/14Z90ru-g-ap55b/</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F40" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" t="inlineStr">
+      <c r="F40" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="0" t="inlineStr">
         <is>
           <t>14Z90RU-G.AP55B</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/portatiles/gram/14z90s-v-ap75b/</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" t="inlineStr">
+      <c r="F41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="0" t="inlineStr">
         <is>
           <t>14Z90S-V.AP75B</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/laptops/gram/14z90t-v-ap88b/</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" t="inlineStr">
+      <c r="F42" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="0" t="inlineStr">
         <is>
           <t>14Z90T-V.AP88B</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/business/informatica/ordenadores/portatiles-ultraligeros/16z90p-g-ap77b/</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" t="inlineStr">
+      <c r="F43" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="0" t="inlineStr">
         <is>
           <t>16Z90P-G-AP77B</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/portatiles/gram/16z90ru-g-ap55b/</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" t="inlineStr">
+      <c r="F44" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="0" t="inlineStr">
         <is>
           <t>16Z90RU-G.AP55B</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/portatiles/gram/16z90t-v-ap88b/</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>1</v>
-      </c>
-      <c r="G45" t="inlineStr">
+      <c r="F45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="0" t="inlineStr">
         <is>
           <t>16Z90T-V.AP88B</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="0" t="inlineStr">
         <is>
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/es/portatiles/gram/17z90t-v-ap88b/</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" t="inlineStr">
+      <c r="F46" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="0" t="inlineStr">
         <is>
           <t>17Z90T-V.AP88B</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="0" t="inlineStr">
         <is>
           <t>FR : FR (fr)</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/fr/pc-portables/gram/lg-15u50t-g-ap56f/</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" t="inlineStr">
+      <c r="F47" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="0" t="inlineStr">
         <is>
           <t>LG 15U50T-G.AP56F</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="0" t="inlineStr">
         <is>
           <t>FR : FR (fr)</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/fr/pc-portables/gram/lg-16z90r-g-ap7bf-i7-32go-2to-win-11-pro/</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E48" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" t="inlineStr">
+      <c r="F48" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="0" t="inlineStr">
         <is>
           <t>LG 16Z90R-G.AP7BF</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="0" t="inlineStr">
         <is>
           <t>FR : FR (fr)</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/fr/pc-portables/gram/lg-16z90ru-g-ap55f-i5-16go-512go-win-11-pro/</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" t="inlineStr">
+      <c r="F49" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="0" t="inlineStr">
         <is>
           <t>LG 16Z90RU-G.AP55F</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="0" t="inlineStr">
         <is>
           <t>FR : FR (fr)</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/fr/pc-portables/gram/lg-17z90ru-g-ap55f-i5-16go-512go-win-11-pro/</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E50" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G50" t="inlineStr">
+      <c r="F50" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="0" t="inlineStr">
         <is>
           <t>LG 17Z90RU-G.AP55F</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="0" t="inlineStr">
         <is>
           <t>GLOBAL : GLOBAL (en)</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram/14z90r-q/</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" t="inlineStr">
+      <c r="F51" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="0" t="inlineStr">
         <is>
           <t>14Z90R-Q</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="0" t="inlineStr">
         <is>
           <t>GLOBAL : GLOBAL (en)</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-book/15ub50t/</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
+      <c r="D52" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E52" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F52" t="n">
-        <v>1</v>
-      </c>
-      <c r="G52" t="inlineStr">
+      <c r="F52" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="0" t="inlineStr">
         <is>
           <t>15UB50T</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="0" t="inlineStr">
         <is>
           <t>GLOBAL : GLOBAL (en)</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram/16z90r-q/</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" t="inlineStr">
+      <c r="F53" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="0" t="inlineStr">
         <is>
           <t>16Z90R-Q</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="0" t="inlineStr">
         <is>
           <t>GLOBAL : GLOBAL (en)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram/17z90r-q/</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
+      <c r="D54" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E54" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F54" t="n">
-        <v>1</v>
-      </c>
-      <c r="G54" t="inlineStr">
+      <c r="F54" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="0" t="inlineStr">
         <is>
           <t>17Z90R-Q</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="0" t="inlineStr">
         <is>
           <t>IN : IN (en)</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/in/business/computers/laptops/lg-gram/14z980-gap52a2/</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F55" t="n">
-        <v>1</v>
-      </c>
-      <c r="G55" t="inlineStr">
+      <c r="F55" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="0" t="inlineStr">
         <is>
           <t>14Z980-GAP52A2</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/notebook/gram/14z90ru-g-ap55d1/</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="D56" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F56" t="n">
-        <v>1</v>
-      </c>
-      <c r="G56" t="inlineStr">
+      <c r="F56" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="0" t="inlineStr">
         <is>
           <t>14Z90RU-G.AP55D1</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/notebook/15ub50t-g-ap56d/</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>1</v>
-      </c>
-      <c r="G57" t="inlineStr">
+      <c r="F57" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="0" t="inlineStr">
         <is>
           <t>15UB50T-G</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/notebook/gram/16z90ru-g-ap55d1/</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
+      <c r="D58" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F58" t="n">
-        <v>1</v>
-      </c>
-      <c r="G58" t="inlineStr">
+      <c r="F58" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="0" t="inlineStr">
         <is>
           <t>16Z90RU-G.AP55D1</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/notebook/16z90s-g-ap55d/</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
+      <c r="D59" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F59" t="n">
-        <v>1</v>
-      </c>
-      <c r="G59" t="inlineStr">
+      <c r="F59" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="0" t="inlineStr">
         <is>
           <t>16Z90S-G.AP55D</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/notebook/16z90s-g-ap78d/</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
+      <c r="D60" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E60" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F60" t="n">
-        <v>1</v>
-      </c>
-      <c r="G60" t="inlineStr">
+      <c r="F60" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="0" t="inlineStr">
         <is>
           <t>16Z90S-G.AP78D</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/notebook/gram/17z90ru-g/</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G61" t="inlineStr">
+      <c r="F61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="0" t="inlineStr">
         <is>
           <t>17Z90RU-G</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="0" t="inlineStr">
         <is>
           <t>IT : IT (it)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/it/notebook/gram/17z90s-g/</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="D62" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E62" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F62" t="n">
-        <v>1</v>
-      </c>
-      <c r="G62" t="inlineStr">
+      <c r="F62" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="0" t="inlineStr">
         <is>
           <t>17Z90S-G.AP78D</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="0" t="inlineStr">
         <is>
           <t>JP : JP (ja)</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/jp/mobile-pc/gram/14z90ru-gp51j/</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
+      <c r="D63" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E63" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F63" t="n">
-        <v>1</v>
-      </c>
-      <c r="G63" t="inlineStr">
+      <c r="F63" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="0" t="inlineStr">
         <is>
           <t>14Z90RU-GP51J</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="0" t="inlineStr">
         <is>
           <t>JP : JP (ja)</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/jp/mobile-pc/gram/14z90s-vp55j/</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
+      <c r="D64" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F64" t="n">
-        <v>1</v>
-      </c>
-      <c r="G64" t="inlineStr">
+      <c r="F64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="0" t="inlineStr">
         <is>
           <t>14Z90S-VP55J</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="0" t="inlineStr">
         <is>
           <t>JP : JP (ja)</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/jp/mobile-pc/gram/14z90s-vp56j/</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
+      <c r="D65" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E65" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F65" t="n">
-        <v>1</v>
-      </c>
-      <c r="G65" t="inlineStr">
+      <c r="F65" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="0" t="inlineStr">
         <is>
           <t>14Z90S-VP56J</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="0" t="inlineStr">
         <is>
           <t>JP : JP (ja)</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/jp/mobile-pc/gram/14z90t-vp55j/</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
+      <c r="D66" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E66" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F66" t="n">
-        <v>1</v>
-      </c>
-      <c r="G66" t="inlineStr">
+      <c r="F66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="0" t="inlineStr">
         <is>
           <t>14Z90T-VP55J</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="0" t="inlineStr">
         <is>
           <t>JP : JP (ja)</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/jp/mobile-pc/gram/17z90s-vp55j/</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
+      <c r="D67" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G67" t="inlineStr">
+      <c r="F67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="0" t="inlineStr">
         <is>
           <t>17Z90S-VP55J</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/business/it-products/lg-gram/14z90s-v-ap75a3/</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F68" t="n">
-        <v>1</v>
-      </c>
-      <c r="G68" t="inlineStr">
+      <c r="F68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="0" t="inlineStr">
         <is>
           <t>14Z90S-V.AP75A3</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/business/it-products/lg-gram/14z90t-g-ap75a3/</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>1</v>
-      </c>
-      <c r="G69" t="inlineStr">
+      <c r="F69" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
         <is>
           <t>14Z90T-G.AP75A3</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/laptops/gram/14z90t-g-ap88a3/</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F70" t="n">
-        <v>1</v>
-      </c>
-      <c r="G70" t="inlineStr">
+      <c r="F70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
         <is>
           <t>14Z90T-G.AP88A3</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/business/it-products/lg-gram/15z90st-v-ap75a3/</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
+      <c r="D71" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F71" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" t="inlineStr">
+      <c r="F71" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="0" t="inlineStr">
         <is>
           <t>15Z90ST-V.AP75A3</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/business/it-products/lg-gram/16t90tp-k-ap88a3/</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
+      <c r="D72" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F72" t="n">
-        <v>1</v>
-      </c>
-      <c r="G72" t="inlineStr">
+      <c r="F72" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="0" t="inlineStr">
         <is>
           <t>16T90TP-K.AP88A3</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90s-v-ap75a3/</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F73" t="n">
-        <v>1</v>
-      </c>
-      <c r="G73" t="inlineStr">
+      <c r="F73" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="0" t="inlineStr">
         <is>
           <t>16Z90S-V.AP75A3</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90s-v-ap78a3/</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
+      <c r="D74" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F74" t="n">
-        <v>1</v>
-      </c>
-      <c r="G74" t="inlineStr">
+      <c r="F74" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="0" t="inlineStr">
         <is>
           <t>16Z90S-V.AP78A3</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="0" t="inlineStr">
         <is>
           <t>SG : SG (en)</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90s-v-ap88a3/</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
+      <c r="D75" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>1</v>
-      </c>
-      <c r="G75" t="inlineStr">
+      <c r="F75" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="0" t="inlineStr">
         <is>
           <t>16Z90S-V.AP88A3</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="0" t="inlineStr">
         <is>
           <t>TW : TW (zh)</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/tw/laptops/gram/14z90r-v-ap56c2/</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>1</v>
-      </c>
-      <c r="G76" t="inlineStr">
+      <c r="F76" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="0" t="inlineStr">
         <is>
           <t>14Z90R-V</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="0" t="inlineStr">
         <is>
           <t>TW : TW (zh)</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/tw/laptops/gram/14z90s-v-ap55c2/</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
+      <c r="D77" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E77" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>1</v>
-      </c>
-      <c r="G77" t="inlineStr">
+      <c r="F77" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="0" t="inlineStr">
         <is>
           <t>14Z90S-V</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="0" t="inlineStr">
         <is>
           <t>TW : TW (zh)</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/tw/laptops/gram/14z90s-v-ap54c2/</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
+      <c r="D78" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E78" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F78" t="n">
-        <v>1</v>
-      </c>
-      <c r="G78" t="inlineStr">
+      <c r="F78" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="0" t="inlineStr">
         <is>
           <t>14Z90S-V</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="0" t="inlineStr">
         <is>
           <t>TW : TW (zh)</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/tw/laptops/gram/14z90t-g-ap55c2/</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
+      <c r="D79" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F79" t="n">
-        <v>1</v>
-      </c>
-      <c r="G79" t="inlineStr">
+      <c r="F79" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="0" t="inlineStr">
         <is>
           <t>14Z90T-G</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="0" t="inlineStr">
         <is>
           <t>TW : TW (zh)</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/tw/laptops/gram/15u50t-g-ap56c2/</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
+      <c r="D80" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F80" t="n">
-        <v>1</v>
-      </c>
-      <c r="G80" t="inlineStr">
+      <c r="F80" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="0" t="inlineStr">
         <is>
           <t>15U50T-G</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="0" t="inlineStr">
         <is>
           <t>VN : VN (vi)</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/vn/business/san-pham-tin-hoc/laptop/16z90r-c-apl1y/</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
+      <c r="D81" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>1</v>
-      </c>
-      <c r="G81" t="inlineStr">
+      <c r="F81" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" s="0" t="inlineStr">
         <is>
           <t>16Z90R-C</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="0" t="inlineStr">
         <is>
           <t>VN : VN (vi)</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="0" t="inlineStr">
         <is>
           <t>https://www.lg.com/vn/laptop-lg-gram/16z90s-g-ap76a5/</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
+      <c r="D82" s="0" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E82" s="0" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F82" t="n">
-        <v>1</v>
-      </c>
-      <c r="G82" t="inlineStr">
+      <c r="F82" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="0" t="inlineStr">
         <is>
           <t>16Z90S-G.AP76A5</t>
         </is>
@@ -18347,15 +18347,19 @@
       </c>
       <c r="C13" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/monitores/monitores-ultragear-gaming/</t>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-oled-gaming/</t>
         </is>
       </c>
       <c r="D13" s="279" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E13" s="123" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" s="123" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
       <c r="F13" s="123" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
data(it): W22 Buying Guide 5개국 상태 정정
- BR·CO·PL·IT 작업중→법인리뷰, CN 법인리뷰→작업중 (사용자 지시)
- 완료 36건 불변 → 완료율 82% 유지 (작업중 7→4 · 법인리뷰 1→4)
- gr-changes 재생성 30 → 35건

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -18596,6 +18596,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -18721,7 +18722,7 @@
       <c r="C12" s="277" t="inlineStr"/>
       <c r="D12" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E12" s="123" t="inlineStr"/>
@@ -18803,7 +18804,7 @@
       <c r="C16" s="277" t="inlineStr"/>
       <c r="D16" s="263" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E16" s="123" t="inlineStr"/>
@@ -18819,7 +18820,7 @@
       <c r="C17" s="277" t="inlineStr"/>
       <c r="D17" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E17" s="123" t="inlineStr"/>
@@ -19141,7 +19142,7 @@
       <c r="C32" s="277" t="inlineStr"/>
       <c r="D32" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E32" s="123" t="inlineStr"/>
@@ -19349,7 +19350,7 @@
       <c r="C42" s="277" t="inlineStr"/>
       <c r="D42" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E42" s="123" t="inlineStr"/>

</xml_diff>

<commit_message>
data(it): W32 UltraFine PDP MIC 삭제 요청 등록 (31개국 66행)
요청자 Alchan Jung(정알찬 책임) · Due 2026-08-12.
대상 6모델의 라이브(CMS 21로케일)·STG(PTT Test URL 29로케일) 합집합.
STG 판정은 PTT raw data 기준. AEM author URL 미기재.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -22,6 +22,7 @@
     <sheet name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="W31 - Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="W31 - PDP Gallery Win11 Pro" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="W32 - UltraFine PDP MIC 삭제" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16025,6 +16026,1694 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="203" min="1" max="1"/>
+    <col width="18" customWidth="1" style="203" min="2" max="2"/>
+    <col width="62" customWidth="1" style="203" min="3" max="3"/>
+    <col width="12" customWidth="1" style="203" min="4" max="4"/>
+    <col width="12" customWidth="1" style="203" min="5" max="5"/>
+    <col width="8" customWidth="1" style="203" min="6" max="6"/>
+    <col width="72" customWidth="1" style="203" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GR26-W32-MS-IT UltraFine PDP MIC 문구 삭제</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · 요청자 Alchan Jung(정알찬 책임) · Due 2026-08-12 · 대상 6모델 × 31개국</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-32u700b-b</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CAC : GT (es)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/monitors/lg-27u710b-b</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/uhd-4k-5k/32u700b-b/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/uhd-4k-5k/32u701b-b/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/uhd-4k-et-5k/32u700b-b/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/uhd-4k-et-5k/32u701b-b/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CL : CL (es)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cl/monitores/uhd-4k/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27u711b-b</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-32u700b-b</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/smart-monitores/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/uhd-4k/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/uhd-4k/32u700b-b/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-27u710b-b</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-27u730b-b</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/uhd-4k/27u711b/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/uhd-4k-5k/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/uhd-4k-5k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u700b-b/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u701b-b/</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u720b-b/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>32U720B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>LT : LT (lt)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/monitoriai/lg-27u710b-b</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>LT : LT (lt)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/monitoriai/lg-27u730b-b</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>LV : LV (lv)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/monitori/lg-27u710b-b</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>LV : LV (lv)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/monitori/lg-27u730b-b</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>MX : MX (es)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>MX : MX (es)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MY : MY (en)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>MY : MY (en)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultrafine-uhd-4k-5k-monitoren/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultrafine-uhd-4k-5k-monitoren/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PA : PA (es)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pa/monitores/ultrafine-monitores/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/uhd-4k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PH : PH (en)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ph/monitors/ultra-fine-uhd-4k/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>PH : PH (en)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>SA : SA (ar)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa/monitors/uhd-4k-5k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SA_EN : SA (en)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa_en/monitors/uhd-4k-5k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/uhd-4k/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/uhd-4k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-do-hoa-ultrafine/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-do-hoa-ultrafine/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ZA : ZA (en)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ZA : ZA (en)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -18596,7 +20285,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>

</xml_diff>

<commit_message>
fix(it): W32 UltraFine 라이브 URL 실측 — AE·CN 32U700B 404 정정
Screaming Frog 실측 결과 200 36건 / 404 2건.
404 2건은 라이브 표기 해제 후 STG 취급.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -16041,7 +16041,7 @@
     <col width="12" customWidth="1" style="203" min="4" max="4"/>
     <col width="12" customWidth="1" style="203" min="5" max="5"/>
     <col width="8" customWidth="1" style="203" min="6" max="6"/>
-    <col width="72" customWidth="1" style="203" min="7" max="7"/>
+    <col width="86" customWidth="1" style="203" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16064,7 +16064,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · 요청자 Alchan Jung(정알찬 책임) · Due 2026-08-12 · 대상 6모델 × 31개국</t>
+          <t>금주 신규 등록 · 요청자 Alchan Jung(정알찬 책임) · Due 2026-08-12 · 대상 6모델 × 31개국 (라이브 URL 36건 실측 200 확인)</t>
         </is>
       </c>
     </row>
@@ -16111,11 +16111,7 @@
           <t>AE : AE (en)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ae/consumer-monitors/lg-32u700b-b</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16127,7 +16123,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
         </is>
       </c>
     </row>
@@ -16451,11 +16447,7 @@
           <t>CN : CN (zh)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/cn/monitors/lg-32u700b-b</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16467,7 +16459,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): URL Library 0810 갱신(중복 제거) + W31 Smart Monitor GR 등록
URL Library: CMS 0810 반영, gp1/5.0 중복 제거 → 2,024 모델 / 27,366 URL
W31 Smart Monitor Multi AI: 22개국 58행, 담당 한유진 사원
금주 변경 53건(UltraFine 31 + Smart Monitor 22)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -23,6 +23,7 @@
     <sheet name="W31 - Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="W31 - PDP Gallery Win11 Pro" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="W32 - UltraFine PDP MIC 삭제" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="W31 - Smart Monitor Multi AI" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16045,6 +16046,1686 @@
   </cols>
   <sheetData>
     <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>GR26-W32-MS-IT UltraFine PDP MIC 문구 삭제</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · 요청자 Alchan Jung(정알찬 책임) · Due 2026-08-12 · 대상 6모델 × 31개국 (라이브 URL 36건 실측 200 확인)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr"/>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr"/>
+      <c r="F4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr"/>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr"/>
+      <c r="F5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr"/>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr"/>
+      <c r="F6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr"/>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr"/>
+      <c r="F7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>CAC : GT (es)</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/monitors/lg-27u710b-b</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr"/>
+      <c r="F8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr"/>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr"/>
+      <c r="F9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr"/>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr"/>
+      <c r="F10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/uhd-4k-5k/32u700b-b/</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr"/>
+      <c r="F11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/uhd-4k-5k/32u701b-b/</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr"/>
+      <c r="F12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/uhd-4k-et-5k/32u700b-b/</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr"/>
+      <c r="F13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/uhd-4k-et-5k/32u701b-b/</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr"/>
+      <c r="F14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>CL : CL (es)</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cl/monitores/uhd-4k/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr"/>
+      <c r="F15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27u711b-b</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr"/>
+      <c r="F16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr"/>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr"/>
+      <c r="F17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr"/>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr"/>
+      <c r="F18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/smart-monitores/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr"/>
+      <c r="F19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/uhd-4k/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr"/>
+      <c r="F20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/uhd-4k/32u700b-b/</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr"/>
+      <c r="F21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr"/>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr"/>
+      <c r="F22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr"/>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr"/>
+      <c r="F23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-27u710b-b</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr"/>
+      <c r="F24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-27u730b-b</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr"/>
+      <c r="F25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr"/>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr"/>
+      <c r="F26" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr"/>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr"/>
+      <c r="F27" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr"/>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr"/>
+      <c r="F28" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr"/>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr"/>
+      <c r="F29" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr"/>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr"/>
+      <c r="F30" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr"/>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr"/>
+      <c r="F31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr"/>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr"/>
+      <c r="F32" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/uhd-4k/27u711b/</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr"/>
+      <c r="F33" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr"/>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr"/>
+      <c r="F34" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/uhd-4k-5k/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr"/>
+      <c r="F35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/uhd-4k-5k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr"/>
+      <c r="F36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr"/>
+      <c r="F37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr"/>
+      <c r="F38" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr"/>
+      <c r="F39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u700b-b/</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr"/>
+      <c r="F40" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="0" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u701b-b/</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr"/>
+      <c r="F41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u720b-b/</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr"/>
+      <c r="F42" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>32U720B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>LT : LT (lt)</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/monitoriai/lg-27u710b-b</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr"/>
+      <c r="F43" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>LT : LT (lt)</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/monitoriai/lg-27u730b-b</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr"/>
+      <c r="F44" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>LV : LV (lv)</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/monitori/lg-27u710b-b</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr"/>
+      <c r="F45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>LV : LV (lv)</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/monitori/lg-27u730b-b</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr"/>
+      <c r="F46" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>MX : MX (es)</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr"/>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr"/>
+      <c r="F47" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>MX : MX (es)</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr"/>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E48" s="0" t="inlineStr"/>
+      <c r="F48" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>MY : MY (en)</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr"/>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr"/>
+      <c r="F49" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>MY : MY (en)</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr"/>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E50" s="0" t="inlineStr"/>
+      <c r="F50" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultrafine-uhd-4k-5k-monitoren/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr"/>
+      <c r="F51" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="0" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultrafine-uhd-4k-5k-monitoren/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D52" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E52" s="0" t="inlineStr"/>
+      <c r="F52" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t>PA : PA (es)</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pa/monitores/ultrafine-monitores/27u710b-b/</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr"/>
+      <c r="F53" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr"/>
+      <c r="D54" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E54" s="0" t="inlineStr"/>
+      <c r="F54" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/uhd-4k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr"/>
+      <c r="F55" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C56" s="0" t="inlineStr"/>
+      <c r="D56" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E56" s="0" t="inlineStr"/>
+      <c r="F56" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="0" t="inlineStr">
+        <is>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>PH : PH (en)</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ph/monitors/ultra-fine-uhd-4k/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr"/>
+      <c r="F57" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t>PH : PH (en)</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr"/>
+      <c r="D58" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr"/>
+      <c r="F58" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="0" t="inlineStr">
+        <is>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t>SA : SA (ar)</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa/monitors/uhd-4k-5k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr"/>
+      <c r="F59" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t>SA_EN : SA (en)</t>
+        </is>
+      </c>
+      <c r="C60" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa_en/monitors/uhd-4k-5k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D60" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E60" s="0" t="inlineStr"/>
+      <c r="F60" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="0" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/uhd-4k/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr"/>
+      <c r="F61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="0" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C62" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/uhd-4k/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D62" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E62" s="0" t="inlineStr"/>
+      <c r="F62" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="0" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C63" s="0" t="inlineStr"/>
+      <c r="D63" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E63" s="0" t="inlineStr"/>
+      <c r="F63" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr"/>
+      <c r="D64" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E64" s="0" t="inlineStr"/>
+      <c r="F64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C65" s="0" t="inlineStr"/>
+      <c r="D65" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E65" s="0" t="inlineStr"/>
+      <c r="F65" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-do-hoa-ultrafine/27u711b-b/</t>
+        </is>
+      </c>
+      <c r="D66" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E66" s="0" t="inlineStr"/>
+      <c r="F66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="0" t="inlineStr">
+        <is>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-do-hoa-ultrafine/27u730b-b/</t>
+        </is>
+      </c>
+      <c r="D67" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr"/>
+      <c r="F67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t>ZA : ZA (en)</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr"/>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr"/>
+      <c r="F68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="0" t="inlineStr">
+        <is>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t>ZA : ZA (en)</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr"/>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr"/>
+      <c r="F69" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
+        <is>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="203" min="1" max="1"/>
+    <col width="18" customWidth="1" style="203" min="2" max="2"/>
+    <col width="62" customWidth="1" style="203" min="3" max="3"/>
+    <col width="12" customWidth="1" style="203" min="4" max="4"/>
+    <col width="12" customWidth="1" style="203" min="5" max="5"/>
+    <col width="8" customWidth="1" style="203" min="6" max="6"/>
+    <col width="96" customWidth="1" style="203" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Title</t>
@@ -16052,7 +17733,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>GR26-W32-MS-IT UltraFine PDP MIC 문구 삭제</t>
+          <t>GR26-W31-MS-IT Smart Monitor Multi AI 에셋 수정</t>
         </is>
       </c>
     </row>
@@ -16064,7 +17745,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · 요청자 Alchan Jung(정알찬 책임) · Due 2026-08-12 · 대상 6모델 × 31개국 (라이브 URL 36건 실측 200 확인)</t>
+          <t>금주 신규 등록 · 요청자 Yujin Han(한유진 사원) · 요청 2026-07-30 · Due 2026-08-30 · 대상 8모델 × 22개국 (요청서 Target List + CMS/PTT 신규 10건 보강)</t>
         </is>
       </c>
     </row>
@@ -16123,14 +17804,14 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>AU : AU (en)</t>
+          <t>AE : AE (en)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -16145,14 +17826,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>AU : AU (en)</t>
+          <t>AE : AE (en)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -16167,14 +17848,14 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>AU : AU (en)</t>
+          <t>AE : AE (en)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -16189,21 +17870,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAC : GT (es)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/cac/monitors/lg-27u710b-b</t>
-        </is>
-      </c>
+          <t>AE_AR : AE (ar)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16215,14 +17892,14 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>AE_AR : AE (ar)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -16237,14 +17914,14 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>AE_AR : AE (ar)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -16259,21 +17936,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/monitors/uhd-4k-5k/32u700b-b/</t>
-        </is>
-      </c>
+          <t>AE_AR : AE (ar)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16285,21 +17958,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/monitors/uhd-4k-5k/32u701b-b/</t>
-        </is>
-      </c>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16311,19 +17980,19 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>BR : BR (pt)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/moniteurs/uhd-4k-et-5k/32u700b-b/</t>
+          <t>https://www.lg.com/br/monitores/smart-monitors/24u511sb-b/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -16337,19 +18006,19 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>BR : BR (pt)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/moniteurs/uhd-4k-et-5k/32u701b-b/</t>
+          <t>https://www.lg.com/br/monitores/smart-monitors/27u511sb-b/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -16363,19 +18032,19 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>CL : CL (es)</t>
+          <t>BR : BR (pt)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cl/monitores/uhd-4k/27u711b-b/</t>
+          <t>https://www.lg.com/br/monitores/smart-monitors/27u731sb-w/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -16389,19 +18058,19 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>BR : BR (pt)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/monitors/lg-27u711b-b</t>
+          <t>https://www.lg.com/br/monitores/smart-monitors/32u701sb-b/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -16415,17 +18084,21 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/smart-monitores/24u511sb-b/</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16437,17 +18110,21 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>CO : CO (es)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/co/monitores/smart-monitores/27u511sb-w/</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16459,7 +18136,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -16471,7 +18148,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.lg.com/co/monitores/smart-monitores/27u710b-b/</t>
+          <t>https://www.lg.com/co/monitores/smart-monitores/32u501sb-b/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -16485,7 +18162,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -16497,7 +18174,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.lg.com/co/monitores/uhd-4k/27u711b-b/</t>
+          <t>https://www.lg.com/co/monitores/smart-monitores/32u701sb-b/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -16511,21 +18188,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>CO : CO (es)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/co/monitores/uhd-4k/32u700b-b/</t>
-        </is>
-      </c>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16537,7 +18210,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -16559,7 +18232,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -16581,19 +18254,19 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>EE : EE (et)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ee/monitorid/lg-27u710b-b</t>
+          <t>https://www.lg.com/de/monitore/smarte-monitore/24u511sb-b/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -16607,19 +18280,19 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>EE : EE (et)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ee/monitorid/lg-27u730b-b</t>
+          <t>https://www.lg.com/de/monitore/smarte-monitore/27u511sb-b/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -16633,7 +18306,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -16643,7 +18316,11 @@
           <t>ES : ES (es)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/outlet/outlet-informatica/monitores/32u701sb-b-outlet/</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16655,17 +18332,21 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/smart-monitors/27u511sb-w/</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16677,17 +18358,21 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>HK : HK (zh)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/monitors/smart-monitors/27u731sb-w/</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16699,17 +18384,21 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/smart-monitors/27u511sb-w/</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16721,17 +18410,21 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>HK_EN : HK (en)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/monitors/smart-monitors/27u731sb-w/</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16743,17 +18436,21 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/smart-monitors/27u511sb/</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16765,17 +18462,21 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/smart-monitors/32u501sb/</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16787,7 +18488,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -16799,7 +18500,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.lg.com/id/monitor/uhd-4k/27u711b/</t>
+          <t>https://www.lg.com/id/monitor/smart-monitors/32u721sb-w/</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -16813,17 +18514,21 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>ID : ID (in)</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>IN : IN (en)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/monitors/smart-monitors/24u511sb-b/</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -16835,7 +18540,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -16847,7 +18552,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.lg.com/in/monitors/uhd-4k-5k/27u710b-b/</t>
+          <t>https://www.lg.com/in/monitors/smart-monitors/27u511sb-b/</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -16861,7 +18566,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -16873,7 +18578,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.lg.com/in/monitors/uhd-4k-5k/27u730b-b/</t>
+          <t>https://www.lg.com/in/monitors/smart-monitors/27u731sb-w/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -16887,19 +18592,19 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>IN : IN (en)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u710b-b/</t>
+          <t>https://www.lg.com/in/monitors/smart-monitors/32u501sb-b/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -16913,19 +18618,19 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>IN : IN (en)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u711b-b/</t>
+          <t>https://www.lg.com/in/monitors/smart-monitors/32u701sb-b/</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -16939,19 +18644,19 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>IN : IN (en)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/27u730b-b/</t>
+          <t>https://www.lg.com/in/monitors/smart-monitors/32u721sb-w/</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -16965,7 +18670,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -16977,7 +18682,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u700b-b/</t>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/24u511sb-b/</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -16991,7 +18696,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -17003,7 +18708,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u701b-b/</t>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/27u511sb-w/</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -17017,7 +18722,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -17027,11 +18732,7 @@
           <t>JP : JP (ja)</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/jp/monitors/4k-5k-monitors/32u720b-b/</t>
-        </is>
-      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17043,19 +18744,19 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>32U720B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>LT : LT (lt)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.lg.com/lt/monitoriai/lg-27u710b-b</t>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/32u501sb-w/</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -17069,19 +18770,19 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>LT : LT (lt)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.lg.com/lt/monitoriai/lg-27u730b-b</t>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/32u721sb-w/</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -17095,19 +18796,19 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>LV : LV (lv)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.lg.com/lv/monitori/lg-27u710b-b</t>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/34u620sb-b/</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -17121,19 +18822,19 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>LV : LV (lv)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.lg.com/lv/monitori/lg-27u730b-b</t>
+          <t>https://www.lg.com/jp/monitors/smart-monitors/34u640sb-w/</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -17147,7 +18848,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>34U640SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -17157,7 +18858,11 @@
           <t>MX : MX (es)</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/mx/monitores/monitores-smart/24u511sb-b/</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17169,7 +18874,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -17179,7 +18884,11 @@
           <t>MX : MX (es)</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/mx/monitores/monitores-smart/27u511sb-w/</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17191,17 +18900,21 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>MY : MY (en)</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t>MX : MX (es)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/mx/monitores/monitores-smart/34u620sb-b/</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17213,17 +18926,21 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>MY : MY (en)</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/fhd-y-qhd/27u511sb-w/</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17235,21 +18952,17 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/nl/monitoren/ultrafine-uhd-4k-5k-monitoren/27u710b-b/</t>
-        </is>
-      </c>
+          <t>SA : SA (ar)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17261,21 +18974,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/nl/monitoren/ultrafine-uhd-4k-5k-monitoren/27u711b-b/</t>
-        </is>
-      </c>
+          <t>SA_EN : SA (en)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17287,19 +18996,19 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>PA : PA (es)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pa/monitores/ultrafine-monitores/27u710b-b/</t>
+          <t>https://www.lg.com/sg/consumer-monitors/smart-monitors/27u511sb-w/</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -17313,17 +19022,21 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/smart-monitors/32u721sb-w/</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17335,19 +19048,19 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe/monitores/uhd-4k/27u730b-b/</t>
+          <t>https://www.lg.com/tr/monitor/smart-monitorleri/32u701sb-b/</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -17361,14 +19074,14 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -17383,21 +19096,17 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>PH : PH (en)</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ph/monitors/ultra-fine-uhd-4k/27u711b-b/</t>
-        </is>
-      </c>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17409,14 +19118,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t>PH : PH (en)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
@@ -17431,21 +19140,17 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>SA : SA (ar)</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/sa/monitors/uhd-4k-5k/27u730b-b/</t>
-        </is>
-      </c>
+          <t>US : US (en)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17457,21 +19162,17 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>SA_EN : SA (en)</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/sa_en/monitors/uhd-4k-5k/27u730b-b/</t>
-        </is>
-      </c>
+          <t>US : US (en)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17483,21 +19184,17 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/sg/consumer-monitors/uhd-4k/27u711b-b/</t>
-        </is>
-      </c>
+          <t>ZA : ZA (en)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -17509,195 +19206,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>SG : SG (en)</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/sg/consumer-monitors/uhd-4k/27u730b-b/</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="n">
-        <v>1</v>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>UK : GB (en)</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="n">
-        <v>1</v>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>UK : GB (en)</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="n">
-        <v>1</v>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>UK : GB (en)</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="n">
-        <v>1</v>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>VN : VN (vi)</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-do-hoa-ultrafine/27u711b-b/</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="n">
-        <v>1</v>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>VN : VN (vi)</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-do-hoa-ultrafine/27u730b-b/</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · 라이브 게시됨</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>ZA : ZA (en)</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="n">
-        <v>1</v>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>ZA : ZA (en)</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="n">
-        <v>1</v>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(it): Digital Trends 라이브/STG 판정 정정 + Planned 그룹 (v0.6.71)
리다이렉트 최종 목적지를 확인하지 않아 판정이 양방향으로 틀렸다.
301을 "슬래시만 추가된 동일 페이지"로 단정한 것이 원인.
- 최종 404 5건(AT·BE_FR×2·CA_EN·CA_FR): URL 제거 후 STG 표기
- 최종 200 2건(BG·CN): soft-404로 잘못 뺐던 것을 라이브로 복원
Digital Trends URL 314 → 311. STG 행에는 URL을 넣지 않는다.

Planned(예정) 그룹 추가: 착수 전 태스크가 In Progress에 섞여 진행 중인
일이 부풀어 보였다. Windows 11 Landing을 예정으로 분류.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -19177,11 +19177,7 @@
           <t>AT : AT (de)</t>
         </is>
       </c>
-      <c r="C7" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/at/monitore/lg-34wp65c-b/</t>
-        </is>
-      </c>
+      <c r="C7" s="0" t="inlineStr"/>
       <c r="D7" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -19193,7 +19189,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · STG · 라이브 미게시(실측 404)</t>
         </is>
       </c>
     </row>
@@ -19593,11 +19589,7 @@
           <t>BE_FR : BE (fr)</t>
         </is>
       </c>
-      <c r="C23" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/be_fr/moniteurs/lg-34wp65c-b/</t>
-        </is>
-      </c>
+      <c r="C23" s="0" t="inlineStr"/>
       <c r="D23" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -19609,7 +19601,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · STG · 라이브 미게시(실측 404)</t>
         </is>
       </c>
     </row>
@@ -19619,11 +19611,7 @@
           <t>BE_FR : BE (fr)</t>
         </is>
       </c>
-      <c r="C24" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/be_fr/moniteurs/lg-34wp75c-b/</t>
-        </is>
-      </c>
+      <c r="C24" s="0" t="inlineStr"/>
       <c r="D24" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -19635,7 +19623,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>34WP75C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+          <t>34WP75C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · STG · 라이브 미게시(실측 404)</t>
         </is>
       </c>
     </row>
@@ -19749,7 +19737,11 @@
           <t>BG : BG (bg)</t>
         </is>
       </c>
-      <c r="C29" s="0" t="inlineStr"/>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-34wp65c-b</t>
+        </is>
+      </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -19761,7 +19753,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 미게시 · CMS/요청서 라이브였으나 실측 카테고리 리다이렉트(soft-404)</t>
+          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -20261,11 +20253,7 @@
           <t>CA_EN : CA (en)</t>
         </is>
       </c>
-      <c r="C49" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/desktop-monitors/lg-34wp65c-b/</t>
-        </is>
-      </c>
+      <c r="C49" s="0" t="inlineStr"/>
       <c r="D49" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -20277,7 +20265,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · STG · 라이브 미게시(실측 404)</t>
         </is>
       </c>
     </row>
@@ -20651,11 +20639,7 @@
           <t>CA_FR : CA (fr)</t>
         </is>
       </c>
-      <c r="C64" s="0" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_fr/moniteurs-de-bureau/lg-34wp65c-b/</t>
-        </is>
-      </c>
+      <c r="C64" s="0" t="inlineStr"/>
       <c r="D64" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -20667,7 +20651,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · STG · 라이브 미게시(실측 404)</t>
         </is>
       </c>
     </row>
@@ -20937,7 +20921,11 @@
           <t>CN : CN (zh)</t>
         </is>
       </c>
-      <c r="C75" s="0" t="inlineStr"/>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-34wp65c-b</t>
+        </is>
+      </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -20949,7 +20937,7 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 미게시 · CMS/요청서 라이브였으나 실측 카테고리 리다이렉트(soft-404)</t>
+          <t>34WP65C-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): W31 Smart Monitor Multi AI — US 2행 삭제 (대상 아님)
US는 이 요청의 대상 국가가 아니다. 58행 21개국 → 56행 21개국
(US는 라이브 URL 없는 STG-only 행 2건이었다).
금주 변경 배지 204 → 203건 재생성.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -16036,7 +16036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="203" min="1" max="1"/>
@@ -17470,7 +17470,7 @@
     <row r="59">
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>US : US (en)</t>
+          <t>ZA : ZA (en)</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr"/>
@@ -17484,50 +17484,6 @@
         <v>1</v>
       </c>
       <c r="G59" s="0" t="inlineStr">
-        <is>
-          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="0" t="inlineStr">
-        <is>
-          <t>US : US (en)</t>
-        </is>
-      </c>
-      <c r="C60" s="0" t="inlineStr"/>
-      <c r="D60" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E60" s="0" t="inlineStr"/>
-      <c r="F60" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G60" s="0" t="inlineStr">
-        <is>
-          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="B61" s="0" t="inlineStr">
-        <is>
-          <t>ZA : ZA (en)</t>
-        </is>
-      </c>
-      <c r="C61" s="0" t="inlineStr"/>
-      <c r="D61" s="0" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E61" s="0" t="inlineStr"/>
-      <c r="F61" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G61" s="0" t="inlineStr">
         <is>
           <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
         </is>

</xml_diff>

<commit_message>
feat(it): FAQ 완료 건에 두 번째 PLP URL 표시 + 완료일을 PTT 게시일로 통일 (v0.6.73)
FAQ 건은 국가당 PLP가 2개(일반 Gaming ↔ OLED/EVO)라 Page#가 2인데
화면에는 링크가 1개만 보였다. 국가 통합 시 대표 행의 URL만 셀에 남기 때문이다.

- grCollectRowUrls/grFaqCellUrls 이식 + mergeGroup에서 __grUrls 수집,
  FAQ URL 셀이 병합된 URL을 모두 렌더하도록 변경
- Global Request.xlsx: 완료 16건에 두 번째 URL 행 추가(국가당 Page# 1+1).
  출처는 PTT Raw의 Live URL 10건 + lg.com 실측 200 확인분 6건
- 완료일은 PTT `Actual Publishing Date`로 갱신. PTT 티켓이 없는 6건
  (EVO IT · OLED AU/DE/ES/IT/JP)은 기존 값 유지

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -35,10 +35,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="68">
+  <fonts count="69">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -394,6 +395,13 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -476,7 +484,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border/>
     <border>
       <left style="thin">
@@ -604,11 +612,19 @@
         <color rgb="FF000000"/>
       </left>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="289">
+  <cellXfs count="292">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1184,9 +1200,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -33009,7 +33029,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="34.5" customWidth="1" style="203" min="3" max="3"/>
@@ -33147,9 +33167,11 @@
           <t>GNB 미반영</t>
         </is>
       </c>
-      <c r="F10" s="270" t="n"/>
+      <c r="F10" s="289" t="n">
+        <v>46211</v>
+      </c>
       <c r="G10" s="177" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
@@ -33158,109 +33180,123 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="267" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CA : CA (en)</t>
+        </is>
+      </c>
+      <c r="C11" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/ultragear-evo/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F11" s="291" t="n">
+        <v>46211</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>evo 반영 · Hyper GNB 미노출</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="267" t="inlineStr">
         <is>
           <t>CA : CA (fr)</t>
         </is>
       </c>
-      <c r="C11" s="268" t="inlineStr">
+      <c r="C12" s="268" t="inlineStr">
         <is>
           <t>https://www.lg.com/ca_fr/moniteurs/hyper-mini-led-gaming-monitor/</t>
         </is>
       </c>
-      <c r="D11" s="285" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E11" s="269" t="inlineStr">
+      <c r="D12" s="285" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" s="269" t="inlineStr">
         <is>
           <t>GNB 미반영</t>
         </is>
       </c>
-      <c r="F11" s="270" t="n"/>
-      <c r="G11" s="177" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="0" t="inlineStr">
+      <c r="F12" s="289" t="n">
+        <v>46211</v>
+      </c>
+      <c r="G12" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="0" t="inlineStr">
         <is>
           <t>evo 반영 · Hyper GNB 미노출</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="271" t="inlineStr">
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CA : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C13" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/ultragear-evo/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F13" s="291" t="n">
+        <v>46211</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>evo 반영 · Hyper GNB 미노출</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="271" t="inlineStr">
         <is>
           <t>DE : DE (de)</t>
         </is>
       </c>
-      <c r="C12" s="272" t="inlineStr">
+      <c r="C14" s="272" t="inlineStr">
         <is>
           <t>https://www.lg.com/de/monitore/hyper-mini-led-ultragear-gaming-monitore/</t>
         </is>
       </c>
-      <c r="D12" s="273" t="inlineStr">
+      <c r="D14" s="273" t="inlineStr">
         <is>
           <t>법인리뷰</t>
         </is>
       </c>
-      <c r="E12" s="288" t="n"/>
-      <c r="F12" s="274" t="n"/>
-      <c r="G12" s="185" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" s="0" t="inlineStr">
-        <is>
-          <t>FAQ 미게시 (evo·Hyper)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="267" t="inlineStr">
-        <is>
-          <t>ES : ES (es)</t>
-        </is>
-      </c>
-      <c r="C13" s="268" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/es/monitores/monitores-ultragear-evo/</t>
-        </is>
-      </c>
-      <c r="D13" s="273" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E13" s="288" t="n"/>
-      <c r="F13" s="270" t="n"/>
-      <c r="G13" s="177" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="0" t="inlineStr">
-        <is>
-          <t>evo FAQ 미게시 · Hyper 페이지/FAQ 게시 대기</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="267" t="inlineStr">
-        <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C14" s="268" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/fr/moniteurs/hyper-mini-led-gaming-monitor/</t>
-        </is>
-      </c>
-      <c r="D14" s="273" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
       <c r="E14" s="288" t="n"/>
-      <c r="F14" s="270" t="n"/>
-      <c r="G14" s="177" t="n">
+      <c r="F14" s="274" t="n"/>
+      <c r="G14" s="185" t="n">
         <v>2</v>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -33272,43 +33308,39 @@
     <row r="15">
       <c r="B15" s="267" t="inlineStr">
         <is>
-          <t>IT : IT (it)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C15" s="268" t="inlineStr">
         <is>
-          <t>https://www.lg.com/it/monitor/hyper-mini-led-gaming-monitor/</t>
-        </is>
-      </c>
-      <c r="D15" s="247" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E15" s="273" t="inlineStr">
-        <is>
-          <t>GNB 미반영</t>
-        </is>
-      </c>
-      <c r="F15" s="275" t="n"/>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-evo/</t>
+        </is>
+      </c>
+      <c r="D15" s="273" t="inlineStr">
+        <is>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E15" s="288" t="n"/>
+      <c r="F15" s="270" t="n"/>
       <c r="G15" s="177" t="n">
         <v>2</v>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>FAQ 라이브 but GNB 미노출 (evo·Hyper)</t>
+          <t>evo FAQ 미게시 · Hyper 페이지/FAQ 게시 대기</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="267" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C16" s="268" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp/monitors/ultragear-evo/</t>
+          <t>https://www.lg.com/fr/moniteurs/hyper-mini-led-gaming-monitor/</t>
         </is>
       </c>
       <c r="D16" s="273" t="inlineStr">
@@ -33316,30 +33348,26 @@
           <t>법인리뷰</t>
         </is>
       </c>
-      <c r="E16" s="288" t="inlineStr">
-        <is>
-          <t>미게시(법인리뷰) · STG 경로 기준</t>
-        </is>
-      </c>
-      <c r="F16" s="275" t="n"/>
+      <c r="E16" s="288" t="n"/>
+      <c r="F16" s="270" t="n"/>
       <c r="G16" s="177" t="n">
         <v>2</v>
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>페이지/FAQ 게시 대기 (evo·Hyper)</t>
+          <t>FAQ 미게시 (evo·Hyper)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="267" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
+          <t>IT : IT (it)</t>
         </is>
       </c>
       <c r="C17" s="268" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nl/monitoren/hyper-mini-led-gaming-monitor/</t>
+          <t>https://www.lg.com/it/monitor/hyper-mini-led-gaming-monitor/</t>
         </is>
       </c>
       <c r="D17" s="247" t="inlineStr">
@@ -33347,43 +33375,47 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E17" s="288" t="n"/>
-      <c r="F17" s="270" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+      <c r="E17" s="273" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F17" s="275" t="n"/>
       <c r="G17" s="177" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" s="0" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="H17" s="0" t="inlineStr">
+        <is>
+          <t>FAQ 라이브 but GNB 미노출 (evo·Hyper)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="B18" s="267" t="inlineStr">
-        <is>
-          <t>SE : SE (sv)</t>
-        </is>
-      </c>
-      <c r="C18" s="268" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/se/monitor/hyper-mini-led-gaming-monitor/</t>
-        </is>
-      </c>
-      <c r="D18" s="247" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E18" s="273" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C18" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/monitor/ultragear-evo/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>GNB 미반영</t>
         </is>
       </c>
-      <c r="F18" s="275" t="n"/>
-      <c r="G18" s="177" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="0" t="inlineStr">
+      <c r="F18" s="291" t="n"/>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>FAQ 라이브 but GNB 미노출 (evo·Hyper)</t>
         </is>
@@ -33392,22 +33424,22 @@
     <row r="19">
       <c r="B19" s="267" t="inlineStr">
         <is>
-          <t>UK : UK (en)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C19" s="268" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/monitors/ultragear-evo/</t>
-        </is>
-      </c>
-      <c r="D19" s="247" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E19" s="273" t="inlineStr">
-        <is>
-          <t>GNB 미반영</t>
+          <t>https://www.lg.com/jp/monitors/ultragear-evo/</t>
+        </is>
+      </c>
+      <c r="D19" s="273" t="inlineStr">
+        <is>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E19" s="288" t="inlineStr">
+        <is>
+          <t>미게시(법인리뷰) · STG 경로 기준</t>
         </is>
       </c>
       <c r="F19" s="275" t="n"/>
@@ -33415,6 +33447,186 @@
         <v>2</v>
       </c>
       <c r="H19" s="0" t="inlineStr">
+        <is>
+          <t>페이지/FAQ 게시 대기 (evo·Hyper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="267" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C20" s="268" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/hyper-mini-led-gaming-monitor/</t>
+        </is>
+      </c>
+      <c r="D20" s="247" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E20" s="288" t="n"/>
+      <c r="F20" s="289" t="n">
+        <v>46218</v>
+      </c>
+      <c r="G20" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="0" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C21" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultragear-evo/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F21" s="291" t="n">
+        <v>46218</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="267" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C22" s="268" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitor/hyper-mini-led-gaming-monitor/</t>
+        </is>
+      </c>
+      <c r="D22" s="247" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E22" s="273" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F22" s="275" t="n">
+        <v>46195</v>
+      </c>
+      <c r="G22" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="0" t="inlineStr">
+        <is>
+          <t>FAQ 라이브 but GNB 미노출 (evo·Hyper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C23" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitor/ultragear-evo/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F23" s="291" t="n">
+        <v>46195</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>FAQ 라이브 but GNB 미노출 (evo·Hyper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="267" t="inlineStr">
+        <is>
+          <t>UK : UK (en)</t>
+        </is>
+      </c>
+      <c r="C24" s="268" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/ultragear-evo/</t>
+        </is>
+      </c>
+      <c r="D24" s="247" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E24" s="273" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F24" s="275" t="n">
+        <v>46227</v>
+      </c>
+      <c r="G24" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="0" t="inlineStr">
+        <is>
+          <t>evo 반영 · Hyper GNB 미노출</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UK : UK (en)</t>
+        </is>
+      </c>
+      <c r="C25" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/hyper-mini-led-gaming-monitor/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>GNB 미반영</t>
+        </is>
+      </c>
+      <c r="F25" s="291" t="n">
+        <v>46227</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
         <is>
           <t>evo 반영 · Hyper GNB 미노출</t>
         </is>
@@ -33425,14 +33637,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -33444,7 +33662,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="22.75" customWidth="1" style="203" min="1" max="1"/>
@@ -33560,7 +33778,7 @@
         </is>
       </c>
       <c r="F9" s="123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
@@ -33569,30 +33787,30 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="261" t="inlineStr">
-        <is>
-          <t>CA : CA (en)</t>
-        </is>
-      </c>
-      <c r="C10" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/monitors/gaming/</t>
-        </is>
-      </c>
-      <c r="D10" s="278" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E10" s="123" t="inlineStr">
-        <is>
-          <t>2026-07-09</t>
-        </is>
-      </c>
-      <c r="F10" s="123" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="0" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C10" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/monitors/ultragear-gaming-oled/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
         </is>
@@ -33601,12 +33819,12 @@
     <row r="11">
       <c r="B11" s="261" t="inlineStr">
         <is>
-          <t>CA : CA (fr)</t>
+          <t>CA : CA (en)</t>
         </is>
       </c>
       <c r="C11" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/</t>
+          <t>https://www.lg.com/ca_en/monitors/gaming/</t>
         </is>
       </c>
       <c r="D11" s="278" t="inlineStr">
@@ -33614,13 +33832,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E11" s="123" t="inlineStr">
-        <is>
-          <t>2026-07-09</t>
-        </is>
+      <c r="E11" s="200" t="n">
+        <v>46212</v>
       </c>
       <c r="F11" s="123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
@@ -33629,30 +33845,28 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="261" t="inlineStr">
-        <is>
-          <t>DE : DE (de)</t>
-        </is>
-      </c>
-      <c r="C12" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/de/monitore/gaming/</t>
-        </is>
-      </c>
-      <c r="D12" s="278" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E12" s="123" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="F12" s="123" t="n">
-        <v>2</v>
-      </c>
-      <c r="G12" s="0" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CA : CA (en)</t>
+        </is>
+      </c>
+      <c r="C12" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/ultragear-gaming-oled/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" s="291" t="n">
+        <v>46212</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
         </is>
@@ -33661,68 +33875,68 @@
     <row r="13">
       <c r="B13" s="261" t="inlineStr">
         <is>
-          <t>ES : ES (es)</t>
+          <t>CA : CA (fr)</t>
         </is>
       </c>
       <c r="C13" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/monitores/monitores-ultragear-oled-gaming/</t>
-        </is>
-      </c>
-      <c r="D13" s="279" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E13" s="123" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
+          <t>https://www.lg.com/ca_fr/moniteurs/de-jeu/</t>
+        </is>
+      </c>
+      <c r="D13" s="278" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" s="200" t="n">
+        <v>46212</v>
       </c>
       <c r="F13" s="123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026 답변 갱신 미반영 (Gaming·OLED Gaming)</t>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="261" t="inlineStr">
-        <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C14" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/fr/moniteurs/gaming/</t>
-        </is>
-      </c>
-      <c r="D14" s="279" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E14" s="123" t="inlineStr"/>
-      <c r="F14" s="123" t="n">
-        <v>2</v>
-      </c>
-      <c r="G14" s="0" t="inlineStr">
-        <is>
-          <t>2026 답변 갱신 미반영 (Gaming·OLED Gaming)</t>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CA : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C14" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/ultragear-gaming-oled/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" s="291" t="n">
+        <v>46212</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="261" t="inlineStr">
         <is>
-          <t>IT : IT (it)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C15" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/it/monitor/gaming/</t>
+          <t>https://www.lg.com/de/monitore/gaming/</t>
         </is>
       </c>
       <c r="D15" s="278" t="inlineStr">
@@ -33736,7 +33950,7 @@
         </is>
       </c>
       <c r="F15" s="123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
@@ -33745,30 +33959,30 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="261" t="inlineStr">
-        <is>
-          <t>JP : JP (ja)</t>
-        </is>
-      </c>
-      <c r="C16" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/jp/monitors/gaming-monitors/</t>
-        </is>
-      </c>
-      <c r="D16" s="278" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E16" s="123" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C16" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/monitore/ultragear-gaming-oled/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="F16" s="123" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" s="0" t="inlineStr">
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
         </is>
@@ -33777,94 +33991,390 @@
     <row r="17">
       <c r="B17" s="261" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C17" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/</t>
-        </is>
-      </c>
-      <c r="D17" s="278" t="inlineStr">
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-oled-gaming/</t>
+        </is>
+      </c>
+      <c r="D17" s="279" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
       <c r="E17" s="123" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F17" s="123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+          <t>2026 답변 갱신 미반영 (Gaming·OLED Gaming)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="270" t="inlineStr">
-        <is>
-          <t>SE : SE (sv)</t>
-        </is>
-      </c>
-      <c r="C18" s="277" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/se/monitor/ultragear-gaming/</t>
-        </is>
-      </c>
-      <c r="D18" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E18" s="123" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="F18" s="123" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" s="0" t="inlineStr">
-        <is>
-          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C18" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/monitores/monitores-ultragear-gaming/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 미반영 (Gaming·OLED Gaming)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="270" t="inlineStr">
-        <is>
-          <t>UK : UK (en)</t>
+      <c r="B19" s="261" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C19" s="277" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/monitors/gaming/</t>
-        </is>
-      </c>
-      <c r="D19" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E19" s="123" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
+          <t>https://www.lg.com/fr/moniteurs/gaming/</t>
+        </is>
+      </c>
+      <c r="D19" s="279" t="inlineStr">
+        <is>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E19" s="123" t="inlineStr"/>
       <c r="F19" s="123" t="n">
         <v>2</v>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
+          <t>2026 답변 갱신 미반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="261" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C20" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/monitor/gaming/</t>
+        </is>
+      </c>
+      <c r="D20" s="278" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E20" s="123" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="F20" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
           <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C21" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/monitor/ultragear-gaming-oled/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="261" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C22" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/gaming-monitors/</t>
+        </is>
+      </c>
+      <c r="D22" s="278" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E22" s="123" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="F22" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C23" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/monitors/ultragear-oled-gaming-monitors/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="261" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C24" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-monitoren/</t>
+        </is>
+      </c>
+      <c r="D24" s="278" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E24" s="200" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F24" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C25" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultragear-gaming-oled/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E25" s="291" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="270" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C26" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming/</t>
+        </is>
+      </c>
+      <c r="D26" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E26" s="200" t="n">
+        <v>46195</v>
+      </c>
+      <c r="F26" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C27" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitor/ultragear-gaming-oled/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E27" s="291" t="n">
+        <v>46195</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="270" t="inlineStr">
+        <is>
+          <t>UK : UK (en)</t>
+        </is>
+      </c>
+      <c r="C28" s="277" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/gaming/</t>
+        </is>
+      </c>
+      <c r="D28" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E28" s="200" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F28" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>UK : UK (en)</t>
+        </is>
+      </c>
+      <c r="C29" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/oled-monitors/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E29" s="291" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId10"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
data(it): W17 SA 2건·W25 3건 완료 처리 + W25 ES URL 교체
- W17 SA_AR·SA_EN: PTT 각 7건 전부 Closed → 완료(완료일 2026-08-12)
- W17 ZA는 제외 — author URL이 ZA_EN으로 갈려 전건 Closed로 보였으나
  실제로는 같은 ZA 사이트의 ultragear-evo가 아직 QA review
- W25 ES·IT(B2C)·GLOBAL(B2B) 작업중 → 완료
- W25 ES URL /es/laptops → /es/portatiles/todos-los-portatiles/ (실측 200)
- gr-changes 132건 재생성

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -4872,12 +4872,12 @@
       </c>
       <c r="C6" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/laptops</t>
+          <t>https://www.lg.com/es/portatiles/todos-los-portatiles/</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F6" s="0" t="n">
@@ -4902,7 +4902,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F7" s="0" t="n">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F18" s="0" t="n">
@@ -33739,10 +33739,12 @@
       </c>
       <c r="D43" s="263" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E43" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E43" s="200" t="n">
+        <v>46246</v>
+      </c>
       <c r="F43" s="123" t="n">
         <v>1</v>
       </c>
@@ -33761,10 +33763,12 @@
       </c>
       <c r="D44" s="263" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E44" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E44" s="200" t="n">
+        <v>46246</v>
+      </c>
       <c r="F44" s="123" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
data(it): W25 Copilot+ Hero Banner VN 완료 처리 (B2C·B2B 2행)
VN은 B2C·B2B 두 행이고 둘 다 작업중이라 화면에서 1행으로 합쳐져 보인다.
두 URL 모두 실측 200 확인. gr-changes 133건 재생성.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -5127,7 +5127,7 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F16" s="0" t="n">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F20" s="0" t="n">

</xml_diff>

<commit_message>
data(it): W25 Copilot+ Hero Banner DE(B2B) 완료 + URL 교체
/de/business/ → /de/business/notebooks/gram/ (실측 200). 값·하이퍼링크 동시 갱신.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -5272,12 +5272,12 @@
       </c>
       <c r="C22" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de/business/</t>
+          <t>https://www.lg.com/de/business/notebooks/gram/</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F22" s="0" t="n">

</xml_diff>

<commit_message>
data(it): W25 Copilot+ Hero Banner FR(B2B) 완료 + URL 정규화
/fr/business/informatique/pc-portables-professionnels/ →
/fr/business/moniteurs-pcs/laptops/pc-portables-professionnels/

기존 URL이 새 URL로 301 리다이렉트된다 — 같은 페이지이고 새 주소가 최종
목적지라, 리다이렉트 전 주소를 최종 주소로 정규화한 것이다. 값·하이퍼링크 동시 갱신.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -5322,12 +5322,12 @@
       </c>
       <c r="C24" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr/business/informatique/pc-portables-professionnels/</t>
+          <t>https://www.lg.com/fr/business/moniteurs-pcs/laptops/pc-portables-professionnels/</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F24" s="0" t="n">

</xml_diff>

<commit_message>
data(it): W32 Digital Trends 전건 완료 + 8/25 3소스 갱신
- W32 Digital Trends Award 삭제 317건 전건 완료. 배지는 갤러리 이미지 파일에
  그려져 있어 본문 문자열로 판정 불가 — 파일명의 Award-Gallery-Images 패턴으로
  실측했다. 34개 중 32개 삭제 완료, DE 2건(32u990a-s·40u990a-w)만 잔존해
  Remark에 표기했다(라이선스 만료 2026-09-01)
- PTT 0825: ES 6건 Request Clarification → QA review (clarify 7 → 1)
- CMS 0824: UK 17Z90U-G.AU78AN 실측 200 확인 → stage live
- URL Library 재생성 (2028 models · 27,481 URLs, cmsSource 2026-08-24)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -19586,7 +19586,7 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr"/>
@@ -19612,7 +19612,7 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr"/>
@@ -19638,7 +19638,7 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr"/>
@@ -19660,7 +19660,7 @@
       <c r="C7" s="0" t="inlineStr"/>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr"/>
@@ -19686,7 +19686,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr"/>
@@ -19712,7 +19712,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr"/>
@@ -19738,7 +19738,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr"/>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr"/>
@@ -19790,7 +19790,7 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr"/>
@@ -19816,7 +19816,7 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr"/>
@@ -19842,7 +19842,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr"/>
@@ -19868,7 +19868,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr"/>
@@ -19894,7 +19894,7 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr"/>
@@ -19920,7 +19920,7 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr"/>
@@ -19946,7 +19946,7 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr"/>
@@ -19972,7 +19972,7 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr"/>
@@ -19998,7 +19998,7 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr"/>
@@ -20024,7 +20024,7 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr"/>
@@ -20050,7 +20050,7 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr"/>
@@ -20072,7 +20072,7 @@
       <c r="C23" s="0" t="inlineStr"/>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr"/>
@@ -20094,7 +20094,7 @@
       <c r="C24" s="0" t="inlineStr"/>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr"/>
@@ -20120,7 +20120,7 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr"/>
@@ -20146,7 +20146,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr"/>
@@ -20172,7 +20172,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr"/>
@@ -20198,7 +20198,7 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr"/>
@@ -20224,7 +20224,7 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr"/>
@@ -20250,7 +20250,7 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr"/>
@@ -20276,7 +20276,7 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr"/>
@@ -20302,7 +20302,7 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr"/>
@@ -20328,7 +20328,7 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr"/>
@@ -20354,7 +20354,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr"/>
@@ -20380,7 +20380,7 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr"/>
@@ -20406,7 +20406,7 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr"/>
@@ -20428,7 +20428,7 @@
       <c r="C37" s="0" t="inlineStr"/>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr"/>
@@ -20454,7 +20454,7 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr"/>
@@ -20480,7 +20480,7 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr"/>
@@ -20506,7 +20506,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr"/>
@@ -20532,7 +20532,7 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr"/>
@@ -20558,7 +20558,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr"/>
@@ -20584,7 +20584,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr"/>
@@ -20610,7 +20610,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr"/>
@@ -20636,7 +20636,7 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr"/>
@@ -20662,7 +20662,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr"/>
@@ -20688,7 +20688,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr"/>
@@ -20714,7 +20714,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr"/>
@@ -20736,7 +20736,7 @@
       <c r="C49" s="0" t="inlineStr"/>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr"/>
@@ -20762,7 +20762,7 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr"/>
@@ -20788,7 +20788,7 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr"/>
@@ -20814,7 +20814,7 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr"/>
@@ -20840,7 +20840,7 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr"/>
@@ -20866,7 +20866,7 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr"/>
@@ -20892,7 +20892,7 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr"/>
@@ -20918,7 +20918,7 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr"/>
@@ -20944,7 +20944,7 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr"/>
@@ -20970,7 +20970,7 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr"/>
@@ -20996,7 +20996,7 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr"/>
@@ -21022,7 +21022,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr"/>
@@ -21048,7 +21048,7 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr"/>
@@ -21074,7 +21074,7 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr"/>
@@ -21100,7 +21100,7 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr"/>
@@ -21122,7 +21122,7 @@
       <c r="C64" s="0" t="inlineStr"/>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr"/>
@@ -21148,7 +21148,7 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr"/>
@@ -21174,7 +21174,7 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr"/>
@@ -21200,7 +21200,7 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr"/>
@@ -21226,7 +21226,7 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr"/>
@@ -21252,7 +21252,7 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr"/>
@@ -21278,7 +21278,7 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr"/>
@@ -21304,7 +21304,7 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr"/>
@@ -21330,7 +21330,7 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr"/>
@@ -21356,7 +21356,7 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr"/>
@@ -21382,7 +21382,7 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr"/>
@@ -21408,7 +21408,7 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr"/>
@@ -21434,7 +21434,7 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr"/>
@@ -21460,7 +21460,7 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr"/>
@@ -21486,7 +21486,7 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr"/>
@@ -21512,7 +21512,7 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr"/>
@@ -21538,7 +21538,7 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr"/>
@@ -21564,7 +21564,7 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr"/>
@@ -21590,7 +21590,7 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr"/>
@@ -21616,7 +21616,7 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr"/>
@@ -21642,7 +21642,7 @@
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E84" s="0" t="inlineStr"/>
@@ -21668,7 +21668,7 @@
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E85" s="0" t="inlineStr"/>
@@ -21694,7 +21694,7 @@
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E86" s="0" t="inlineStr"/>
@@ -21720,7 +21720,7 @@
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E87" s="0" t="inlineStr"/>
@@ -21746,7 +21746,7 @@
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E88" s="0" t="inlineStr"/>
@@ -21772,7 +21772,7 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E89" s="0" t="inlineStr"/>
@@ -21798,7 +21798,7 @@
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E90" s="0" t="inlineStr"/>
@@ -21824,7 +21824,7 @@
       </c>
       <c r="D91" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E91" s="0" t="inlineStr"/>
@@ -21850,7 +21850,7 @@
       </c>
       <c r="D92" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E92" s="0" t="inlineStr"/>
@@ -21876,7 +21876,7 @@
       </c>
       <c r="D93" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E93" s="0" t="inlineStr"/>
@@ -21902,7 +21902,7 @@
       </c>
       <c r="D94" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E94" s="0" t="inlineStr"/>
@@ -21928,7 +21928,7 @@
       </c>
       <c r="D95" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E95" s="0" t="inlineStr"/>
@@ -21954,7 +21954,7 @@
       </c>
       <c r="D96" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E96" s="0" t="inlineStr"/>
@@ -21980,7 +21980,7 @@
       </c>
       <c r="D97" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E97" s="0" t="inlineStr"/>
@@ -22006,7 +22006,7 @@
       </c>
       <c r="D98" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E98" s="0" t="inlineStr"/>
@@ -22032,7 +22032,7 @@
       </c>
       <c r="D99" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E99" s="0" t="inlineStr"/>
@@ -22058,7 +22058,7 @@
       </c>
       <c r="D100" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E100" s="0" t="inlineStr"/>
@@ -22084,7 +22084,7 @@
       </c>
       <c r="D101" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E101" s="0" t="inlineStr"/>
@@ -22110,7 +22110,7 @@
       </c>
       <c r="D102" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E102" s="0" t="inlineStr"/>
@@ -22136,7 +22136,7 @@
       </c>
       <c r="D103" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E103" s="0" t="inlineStr"/>
@@ -22145,7 +22145,7 @@
       </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
-          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨 · ⚠️ 갤러리 이미지에 어워드 잔존(2026-08-25 실측)</t>
         </is>
       </c>
     </row>
@@ -22162,7 +22162,7 @@
       </c>
       <c r="D104" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E104" s="0" t="inlineStr"/>
@@ -22188,7 +22188,7 @@
       </c>
       <c r="D105" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E105" s="0" t="inlineStr"/>
@@ -22214,7 +22214,7 @@
       </c>
       <c r="D106" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E106" s="0" t="inlineStr"/>
@@ -22223,7 +22223,7 @@
       </c>
       <c r="G106" s="0" t="inlineStr">
         <is>
-          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨 · ⚠️ 갤러리 이미지에 어워드 잔존(2026-08-25 실측)</t>
         </is>
       </c>
     </row>
@@ -22240,7 +22240,7 @@
       </c>
       <c r="D107" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E107" s="0" t="inlineStr"/>
@@ -22266,7 +22266,7 @@
       </c>
       <c r="D108" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E108" s="0" t="inlineStr"/>
@@ -22292,7 +22292,7 @@
       </c>
       <c r="D109" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E109" s="0" t="inlineStr"/>
@@ -22318,7 +22318,7 @@
       </c>
       <c r="D110" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E110" s="0" t="inlineStr"/>
@@ -22344,7 +22344,7 @@
       </c>
       <c r="D111" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E111" s="0" t="inlineStr"/>
@@ -22370,7 +22370,7 @@
       </c>
       <c r="D112" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E112" s="0" t="inlineStr"/>
@@ -22396,7 +22396,7 @@
       </c>
       <c r="D113" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E113" s="0" t="inlineStr"/>
@@ -22422,7 +22422,7 @@
       </c>
       <c r="D114" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E114" s="0" t="inlineStr"/>
@@ -22448,7 +22448,7 @@
       </c>
       <c r="D115" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E115" s="0" t="inlineStr"/>
@@ -22474,7 +22474,7 @@
       </c>
       <c r="D116" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E116" s="0" t="inlineStr"/>
@@ -22500,7 +22500,7 @@
       </c>
       <c r="D117" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E117" s="0" t="inlineStr"/>
@@ -22526,7 +22526,7 @@
       </c>
       <c r="D118" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E118" s="0" t="inlineStr"/>
@@ -22552,7 +22552,7 @@
       </c>
       <c r="D119" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E119" s="0" t="inlineStr"/>
@@ -22578,7 +22578,7 @@
       </c>
       <c r="D120" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E120" s="0" t="inlineStr"/>
@@ -22604,7 +22604,7 @@
       </c>
       <c r="D121" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E121" s="0" t="inlineStr"/>
@@ -22630,7 +22630,7 @@
       </c>
       <c r="D122" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E122" s="0" t="inlineStr"/>
@@ -22656,7 +22656,7 @@
       </c>
       <c r="D123" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E123" s="0" t="inlineStr"/>
@@ -22682,7 +22682,7 @@
       </c>
       <c r="D124" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E124" s="0" t="inlineStr"/>
@@ -22708,7 +22708,7 @@
       </c>
       <c r="D125" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E125" s="0" t="inlineStr"/>
@@ -22734,7 +22734,7 @@
       </c>
       <c r="D126" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E126" s="0" t="inlineStr"/>
@@ -22760,7 +22760,7 @@
       </c>
       <c r="D127" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E127" s="0" t="inlineStr"/>
@@ -22786,7 +22786,7 @@
       </c>
       <c r="D128" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E128" s="0" t="inlineStr"/>
@@ -22812,7 +22812,7 @@
       </c>
       <c r="D129" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E129" s="0" t="inlineStr"/>
@@ -22838,7 +22838,7 @@
       </c>
       <c r="D130" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E130" s="0" t="inlineStr"/>
@@ -22864,7 +22864,7 @@
       </c>
       <c r="D131" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E131" s="0" t="inlineStr"/>
@@ -22890,7 +22890,7 @@
       </c>
       <c r="D132" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E132" s="0" t="inlineStr"/>
@@ -22916,7 +22916,7 @@
       </c>
       <c r="D133" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E133" s="0" t="inlineStr"/>
@@ -22942,7 +22942,7 @@
       </c>
       <c r="D134" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E134" s="0" t="inlineStr"/>
@@ -22968,7 +22968,7 @@
       </c>
       <c r="D135" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E135" s="0" t="inlineStr"/>
@@ -22994,7 +22994,7 @@
       </c>
       <c r="D136" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E136" s="0" t="inlineStr"/>
@@ -23020,7 +23020,7 @@
       </c>
       <c r="D137" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E137" s="0" t="inlineStr"/>
@@ -23046,7 +23046,7 @@
       </c>
       <c r="D138" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E138" s="0" t="inlineStr"/>
@@ -23072,7 +23072,7 @@
       </c>
       <c r="D139" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E139" s="0" t="inlineStr"/>
@@ -23098,7 +23098,7 @@
       </c>
       <c r="D140" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E140" s="0" t="inlineStr"/>
@@ -23124,7 +23124,7 @@
       </c>
       <c r="D141" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E141" s="0" t="inlineStr"/>
@@ -23150,7 +23150,7 @@
       </c>
       <c r="D142" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E142" s="0" t="inlineStr"/>
@@ -23176,7 +23176,7 @@
       </c>
       <c r="D143" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E143" s="0" t="inlineStr"/>
@@ -23202,7 +23202,7 @@
       </c>
       <c r="D144" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E144" s="0" t="inlineStr"/>
@@ -23228,7 +23228,7 @@
       </c>
       <c r="D145" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E145" s="0" t="inlineStr"/>
@@ -23254,7 +23254,7 @@
       </c>
       <c r="D146" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E146" s="0" t="inlineStr"/>
@@ -23280,7 +23280,7 @@
       </c>
       <c r="D147" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E147" s="0" t="inlineStr"/>
@@ -23306,7 +23306,7 @@
       </c>
       <c r="D148" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E148" s="0" t="inlineStr"/>
@@ -23332,7 +23332,7 @@
       </c>
       <c r="D149" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E149" s="0" t="inlineStr"/>
@@ -23358,7 +23358,7 @@
       </c>
       <c r="D150" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E150" s="0" t="inlineStr"/>
@@ -23384,7 +23384,7 @@
       </c>
       <c r="D151" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E151" s="0" t="inlineStr"/>
@@ -23410,7 +23410,7 @@
       </c>
       <c r="D152" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E152" s="0" t="inlineStr"/>
@@ -23436,7 +23436,7 @@
       </c>
       <c r="D153" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E153" s="0" t="inlineStr"/>
@@ -23462,7 +23462,7 @@
       </c>
       <c r="D154" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E154" s="0" t="inlineStr"/>
@@ -23488,7 +23488,7 @@
       </c>
       <c r="D155" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E155" s="0" t="inlineStr"/>
@@ -23514,7 +23514,7 @@
       </c>
       <c r="D156" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E156" s="0" t="inlineStr"/>
@@ -23540,7 +23540,7 @@
       </c>
       <c r="D157" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E157" s="0" t="inlineStr"/>
@@ -23566,7 +23566,7 @@
       </c>
       <c r="D158" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E158" s="0" t="inlineStr"/>
@@ -23592,7 +23592,7 @@
       </c>
       <c r="D159" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E159" s="0" t="inlineStr"/>
@@ -23618,7 +23618,7 @@
       </c>
       <c r="D160" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E160" s="0" t="inlineStr"/>
@@ -23644,7 +23644,7 @@
       </c>
       <c r="D161" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E161" s="0" t="inlineStr"/>
@@ -23670,7 +23670,7 @@
       </c>
       <c r="D162" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E162" s="0" t="inlineStr"/>
@@ -23696,7 +23696,7 @@
       </c>
       <c r="D163" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E163" s="0" t="inlineStr"/>
@@ -23722,7 +23722,7 @@
       </c>
       <c r="D164" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E164" s="0" t="inlineStr"/>
@@ -23748,7 +23748,7 @@
       </c>
       <c r="D165" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E165" s="0" t="inlineStr"/>
@@ -23774,7 +23774,7 @@
       </c>
       <c r="D166" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E166" s="0" t="inlineStr"/>
@@ -23800,7 +23800,7 @@
       </c>
       <c r="D167" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E167" s="0" t="inlineStr"/>
@@ -23826,7 +23826,7 @@
       </c>
       <c r="D168" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E168" s="0" t="inlineStr"/>
@@ -23852,7 +23852,7 @@
       </c>
       <c r="D169" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E169" s="0" t="inlineStr"/>
@@ -23878,7 +23878,7 @@
       </c>
       <c r="D170" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E170" s="0" t="inlineStr"/>
@@ -23904,7 +23904,7 @@
       </c>
       <c r="D171" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E171" s="0" t="inlineStr"/>
@@ -23930,7 +23930,7 @@
       </c>
       <c r="D172" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E172" s="0" t="inlineStr"/>
@@ -23956,7 +23956,7 @@
       </c>
       <c r="D173" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E173" s="0" t="inlineStr"/>
@@ -23982,7 +23982,7 @@
       </c>
       <c r="D174" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E174" s="0" t="inlineStr"/>
@@ -24008,7 +24008,7 @@
       </c>
       <c r="D175" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E175" s="0" t="inlineStr"/>
@@ -24034,7 +24034,7 @@
       </c>
       <c r="D176" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E176" s="0" t="inlineStr"/>
@@ -24060,7 +24060,7 @@
       </c>
       <c r="D177" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E177" s="0" t="inlineStr"/>
@@ -24086,7 +24086,7 @@
       </c>
       <c r="D178" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E178" s="0" t="inlineStr"/>
@@ -24112,7 +24112,7 @@
       </c>
       <c r="D179" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E179" s="0" t="inlineStr"/>
@@ -24138,7 +24138,7 @@
       </c>
       <c r="D180" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E180" s="0" t="inlineStr"/>
@@ -24164,7 +24164,7 @@
       </c>
       <c r="D181" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E181" s="0" t="inlineStr"/>
@@ -24190,7 +24190,7 @@
       </c>
       <c r="D182" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E182" s="0" t="inlineStr"/>
@@ -24216,7 +24216,7 @@
       </c>
       <c r="D183" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E183" s="0" t="inlineStr"/>
@@ -24242,7 +24242,7 @@
       </c>
       <c r="D184" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E184" s="0" t="inlineStr"/>
@@ -24268,7 +24268,7 @@
       </c>
       <c r="D185" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E185" s="0" t="inlineStr"/>
@@ -24294,7 +24294,7 @@
       </c>
       <c r="D186" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E186" s="0" t="inlineStr"/>
@@ -24320,7 +24320,7 @@
       </c>
       <c r="D187" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E187" s="0" t="inlineStr"/>
@@ -24346,7 +24346,7 @@
       </c>
       <c r="D188" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E188" s="0" t="inlineStr"/>
@@ -24372,7 +24372,7 @@
       </c>
       <c r="D189" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E189" s="0" t="inlineStr"/>
@@ -24398,7 +24398,7 @@
       </c>
       <c r="D190" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E190" s="0" t="inlineStr"/>
@@ -24424,7 +24424,7 @@
       </c>
       <c r="D191" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E191" s="0" t="inlineStr"/>
@@ -24450,7 +24450,7 @@
       </c>
       <c r="D192" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E192" s="0" t="inlineStr"/>
@@ -24476,7 +24476,7 @@
       </c>
       <c r="D193" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E193" s="0" t="inlineStr"/>
@@ -24502,7 +24502,7 @@
       </c>
       <c r="D194" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E194" s="0" t="inlineStr"/>
@@ -24528,7 +24528,7 @@
       </c>
       <c r="D195" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E195" s="0" t="inlineStr"/>
@@ -24554,7 +24554,7 @@
       </c>
       <c r="D196" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E196" s="0" t="inlineStr"/>
@@ -24580,7 +24580,7 @@
       </c>
       <c r="D197" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E197" s="0" t="inlineStr"/>
@@ -24606,7 +24606,7 @@
       </c>
       <c r="D198" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E198" s="0" t="inlineStr"/>
@@ -24632,7 +24632,7 @@
       </c>
       <c r="D199" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E199" s="0" t="inlineStr"/>
@@ -24658,7 +24658,7 @@
       </c>
       <c r="D200" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E200" s="0" t="inlineStr"/>
@@ -24684,7 +24684,7 @@
       </c>
       <c r="D201" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E201" s="0" t="inlineStr"/>
@@ -24710,7 +24710,7 @@
       </c>
       <c r="D202" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E202" s="0" t="inlineStr"/>
@@ -24736,7 +24736,7 @@
       </c>
       <c r="D203" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E203" s="0" t="inlineStr"/>
@@ -24762,7 +24762,7 @@
       </c>
       <c r="D204" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E204" s="0" t="inlineStr"/>
@@ -24788,7 +24788,7 @@
       </c>
       <c r="D205" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E205" s="0" t="inlineStr"/>
@@ -24814,7 +24814,7 @@
       </c>
       <c r="D206" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E206" s="0" t="inlineStr"/>
@@ -24840,7 +24840,7 @@
       </c>
       <c r="D207" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E207" s="0" t="inlineStr"/>
@@ -24866,7 +24866,7 @@
       </c>
       <c r="D208" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E208" s="0" t="inlineStr"/>
@@ -24892,7 +24892,7 @@
       </c>
       <c r="D209" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E209" s="0" t="inlineStr"/>
@@ -24918,7 +24918,7 @@
       </c>
       <c r="D210" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E210" s="0" t="inlineStr"/>
@@ -24944,7 +24944,7 @@
       </c>
       <c r="D211" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E211" s="0" t="inlineStr"/>
@@ -24970,7 +24970,7 @@
       </c>
       <c r="D212" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E212" s="0" t="inlineStr"/>
@@ -24996,7 +24996,7 @@
       </c>
       <c r="D213" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E213" s="0" t="inlineStr"/>
@@ -25022,7 +25022,7 @@
       </c>
       <c r="D214" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E214" s="0" t="inlineStr"/>
@@ -25048,7 +25048,7 @@
       </c>
       <c r="D215" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E215" s="0" t="inlineStr"/>
@@ -25074,7 +25074,7 @@
       </c>
       <c r="D216" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E216" s="0" t="inlineStr"/>
@@ -25100,7 +25100,7 @@
       </c>
       <c r="D217" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E217" s="0" t="inlineStr"/>
@@ -25126,7 +25126,7 @@
       </c>
       <c r="D218" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E218" s="0" t="inlineStr"/>
@@ -25152,7 +25152,7 @@
       </c>
       <c r="D219" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E219" s="0" t="inlineStr"/>
@@ -25178,7 +25178,7 @@
       </c>
       <c r="D220" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E220" s="0" t="inlineStr"/>
@@ -25204,7 +25204,7 @@
       </c>
       <c r="D221" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E221" s="0" t="inlineStr"/>
@@ -25230,7 +25230,7 @@
       </c>
       <c r="D222" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E222" s="0" t="inlineStr"/>
@@ -25256,7 +25256,7 @@
       </c>
       <c r="D223" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E223" s="0" t="inlineStr"/>
@@ -25282,7 +25282,7 @@
       </c>
       <c r="D224" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E224" s="0" t="inlineStr"/>
@@ -25308,7 +25308,7 @@
       </c>
       <c r="D225" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E225" s="0" t="inlineStr"/>
@@ -25334,7 +25334,7 @@
       </c>
       <c r="D226" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E226" s="0" t="inlineStr"/>
@@ -25360,7 +25360,7 @@
       </c>
       <c r="D227" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E227" s="0" t="inlineStr"/>
@@ -25386,7 +25386,7 @@
       </c>
       <c r="D228" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E228" s="0" t="inlineStr"/>
@@ -25412,7 +25412,7 @@
       </c>
       <c r="D229" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E229" s="0" t="inlineStr"/>
@@ -25438,7 +25438,7 @@
       </c>
       <c r="D230" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E230" s="0" t="inlineStr"/>
@@ -25464,7 +25464,7 @@
       </c>
       <c r="D231" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E231" s="0" t="inlineStr"/>
@@ -25490,7 +25490,7 @@
       </c>
       <c r="D232" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E232" s="0" t="inlineStr"/>
@@ -25516,7 +25516,7 @@
       </c>
       <c r="D233" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E233" s="0" t="inlineStr"/>
@@ -25542,7 +25542,7 @@
       </c>
       <c r="D234" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E234" s="0" t="inlineStr"/>
@@ -25568,7 +25568,7 @@
       </c>
       <c r="D235" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E235" s="0" t="inlineStr"/>
@@ -25594,7 +25594,7 @@
       </c>
       <c r="D236" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E236" s="0" t="inlineStr"/>
@@ -25620,7 +25620,7 @@
       </c>
       <c r="D237" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E237" s="0" t="inlineStr"/>
@@ -25646,7 +25646,7 @@
       </c>
       <c r="D238" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E238" s="0" t="inlineStr"/>
@@ -25672,7 +25672,7 @@
       </c>
       <c r="D239" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E239" s="0" t="inlineStr"/>
@@ -25698,7 +25698,7 @@
       </c>
       <c r="D240" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E240" s="0" t="inlineStr"/>
@@ -25724,7 +25724,7 @@
       </c>
       <c r="D241" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E241" s="0" t="inlineStr"/>
@@ -25750,7 +25750,7 @@
       </c>
       <c r="D242" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E242" s="0" t="inlineStr"/>
@@ -25776,7 +25776,7 @@
       </c>
       <c r="D243" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E243" s="0" t="inlineStr"/>
@@ -25802,7 +25802,7 @@
       </c>
       <c r="D244" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E244" s="0" t="inlineStr"/>
@@ -25828,7 +25828,7 @@
       </c>
       <c r="D245" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E245" s="0" t="inlineStr"/>
@@ -25854,7 +25854,7 @@
       </c>
       <c r="D246" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E246" s="0" t="inlineStr"/>
@@ -25880,7 +25880,7 @@
       </c>
       <c r="D247" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E247" s="0" t="inlineStr"/>
@@ -25906,7 +25906,7 @@
       </c>
       <c r="D248" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E248" s="0" t="inlineStr"/>
@@ -25932,7 +25932,7 @@
       </c>
       <c r="D249" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E249" s="0" t="inlineStr"/>
@@ -25958,7 +25958,7 @@
       </c>
       <c r="D250" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E250" s="0" t="inlineStr"/>
@@ -25984,7 +25984,7 @@
       </c>
       <c r="D251" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E251" s="0" t="inlineStr"/>
@@ -26010,7 +26010,7 @@
       </c>
       <c r="D252" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E252" s="0" t="inlineStr"/>
@@ -26036,7 +26036,7 @@
       </c>
       <c r="D253" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E253" s="0" t="inlineStr"/>
@@ -26062,7 +26062,7 @@
       </c>
       <c r="D254" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E254" s="0" t="inlineStr"/>
@@ -26088,7 +26088,7 @@
       </c>
       <c r="D255" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E255" s="0" t="inlineStr"/>
@@ -26114,7 +26114,7 @@
       </c>
       <c r="D256" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E256" s="0" t="inlineStr"/>
@@ -26140,7 +26140,7 @@
       </c>
       <c r="D257" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E257" s="0" t="inlineStr"/>
@@ -26166,7 +26166,7 @@
       </c>
       <c r="D258" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E258" s="0" t="inlineStr"/>
@@ -26192,7 +26192,7 @@
       </c>
       <c r="D259" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E259" s="0" t="inlineStr"/>
@@ -26218,7 +26218,7 @@
       </c>
       <c r="D260" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E260" s="0" t="inlineStr"/>
@@ -26244,7 +26244,7 @@
       </c>
       <c r="D261" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E261" s="0" t="inlineStr"/>
@@ -26270,7 +26270,7 @@
       </c>
       <c r="D262" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E262" s="0" t="inlineStr"/>
@@ -26296,7 +26296,7 @@
       </c>
       <c r="D263" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E263" s="0" t="inlineStr"/>
@@ -26322,7 +26322,7 @@
       </c>
       <c r="D264" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E264" s="0" t="inlineStr"/>
@@ -26348,7 +26348,7 @@
       </c>
       <c r="D265" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E265" s="0" t="inlineStr"/>
@@ -26374,7 +26374,7 @@
       </c>
       <c r="D266" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E266" s="0" t="inlineStr"/>
@@ -26400,7 +26400,7 @@
       </c>
       <c r="D267" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E267" s="0" t="inlineStr"/>
@@ -26426,7 +26426,7 @@
       </c>
       <c r="D268" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E268" s="0" t="inlineStr"/>
@@ -26452,7 +26452,7 @@
       </c>
       <c r="D269" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E269" s="0" t="inlineStr"/>
@@ -26478,7 +26478,7 @@
       </c>
       <c r="D270" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E270" s="0" t="inlineStr"/>
@@ -26504,7 +26504,7 @@
       </c>
       <c r="D271" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E271" s="0" t="inlineStr"/>
@@ -26530,7 +26530,7 @@
       </c>
       <c r="D272" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E272" s="0" t="inlineStr"/>
@@ -26556,7 +26556,7 @@
       </c>
       <c r="D273" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E273" s="0" t="inlineStr"/>
@@ -26582,7 +26582,7 @@
       </c>
       <c r="D274" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E274" s="0" t="inlineStr"/>
@@ -26608,7 +26608,7 @@
       </c>
       <c r="D275" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E275" s="0" t="inlineStr"/>
@@ -26634,7 +26634,7 @@
       </c>
       <c r="D276" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E276" s="0" t="inlineStr"/>
@@ -26660,7 +26660,7 @@
       </c>
       <c r="D277" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E277" s="0" t="inlineStr"/>
@@ -26686,7 +26686,7 @@
       </c>
       <c r="D278" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E278" s="0" t="inlineStr"/>
@@ -26712,7 +26712,7 @@
       </c>
       <c r="D279" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E279" s="0" t="inlineStr"/>
@@ -26738,7 +26738,7 @@
       </c>
       <c r="D280" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E280" s="0" t="inlineStr"/>
@@ -26764,7 +26764,7 @@
       </c>
       <c r="D281" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E281" s="0" t="inlineStr"/>
@@ -26790,7 +26790,7 @@
       </c>
       <c r="D282" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E282" s="0" t="inlineStr"/>
@@ -26816,7 +26816,7 @@
       </c>
       <c r="D283" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E283" s="0" t="inlineStr"/>
@@ -26842,7 +26842,7 @@
       </c>
       <c r="D284" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E284" s="0" t="inlineStr"/>
@@ -26868,7 +26868,7 @@
       </c>
       <c r="D285" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E285" s="0" t="inlineStr"/>
@@ -26894,7 +26894,7 @@
       </c>
       <c r="D286" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E286" s="0" t="inlineStr"/>
@@ -26920,7 +26920,7 @@
       </c>
       <c r="D287" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E287" s="0" t="inlineStr"/>
@@ -26946,7 +26946,7 @@
       </c>
       <c r="D288" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E288" s="0" t="inlineStr"/>
@@ -26972,7 +26972,7 @@
       </c>
       <c r="D289" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E289" s="0" t="inlineStr"/>
@@ -26998,7 +26998,7 @@
       </c>
       <c r="D290" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E290" s="0" t="inlineStr"/>
@@ -27024,7 +27024,7 @@
       </c>
       <c r="D291" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E291" s="0" t="inlineStr"/>
@@ -27050,7 +27050,7 @@
       </c>
       <c r="D292" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E292" s="0" t="inlineStr"/>
@@ -27076,7 +27076,7 @@
       </c>
       <c r="D293" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E293" s="0" t="inlineStr"/>
@@ -27102,7 +27102,7 @@
       </c>
       <c r="D294" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E294" s="0" t="inlineStr"/>
@@ -27128,7 +27128,7 @@
       </c>
       <c r="D295" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E295" s="0" t="inlineStr"/>
@@ -27154,7 +27154,7 @@
       </c>
       <c r="D296" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E296" s="0" t="inlineStr"/>
@@ -27180,7 +27180,7 @@
       </c>
       <c r="D297" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E297" s="0" t="inlineStr"/>
@@ -27206,7 +27206,7 @@
       </c>
       <c r="D298" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E298" s="0" t="inlineStr"/>
@@ -27232,7 +27232,7 @@
       </c>
       <c r="D299" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E299" s="0" t="inlineStr"/>
@@ -27258,7 +27258,7 @@
       </c>
       <c r="D300" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E300" s="0" t="inlineStr"/>
@@ -27284,7 +27284,7 @@
       </c>
       <c r="D301" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E301" s="0" t="inlineStr"/>
@@ -27310,7 +27310,7 @@
       </c>
       <c r="D302" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E302" s="0" t="inlineStr"/>
@@ -27336,7 +27336,7 @@
       </c>
       <c r="D303" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E303" s="0" t="inlineStr"/>
@@ -27362,7 +27362,7 @@
       </c>
       <c r="D304" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E304" s="0" t="inlineStr"/>
@@ -27388,7 +27388,7 @@
       </c>
       <c r="D305" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E305" s="0" t="inlineStr"/>
@@ -27414,7 +27414,7 @@
       </c>
       <c r="D306" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E306" s="0" t="inlineStr"/>
@@ -27440,7 +27440,7 @@
       </c>
       <c r="D307" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E307" s="0" t="inlineStr"/>
@@ -27466,7 +27466,7 @@
       </c>
       <c r="D308" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E308" s="0" t="inlineStr"/>
@@ -27492,7 +27492,7 @@
       </c>
       <c r="D309" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E309" s="0" t="inlineStr"/>
@@ -27518,7 +27518,7 @@
       </c>
       <c r="D310" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E310" s="0" t="inlineStr"/>
@@ -27544,7 +27544,7 @@
       </c>
       <c r="D311" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E311" s="0" t="inlineStr"/>
@@ -27570,7 +27570,7 @@
       </c>
       <c r="D312" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E312" s="0" t="inlineStr"/>
@@ -27596,7 +27596,7 @@
       </c>
       <c r="D313" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E313" s="0" t="inlineStr"/>
@@ -27622,7 +27622,7 @@
       </c>
       <c r="D314" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E314" s="0" t="inlineStr"/>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="D315" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E315" s="0" t="inlineStr"/>
@@ -27674,7 +27674,7 @@
       </c>
       <c r="D316" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E316" s="0" t="inlineStr"/>
@@ -27700,7 +27700,7 @@
       </c>
       <c r="D317" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E317" s="0" t="inlineStr"/>
@@ -27726,7 +27726,7 @@
       </c>
       <c r="D318" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E318" s="0" t="inlineStr"/>
@@ -27752,7 +27752,7 @@
       </c>
       <c r="D319" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E319" s="0" t="inlineStr"/>
@@ -27778,7 +27778,7 @@
       </c>
       <c r="D320" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E320" s="0" t="inlineStr"/>

</xml_diff>

<commit_message>
data(it): W30 UltraGear 1000Hz FAQ 11개국 법인리뷰 전환
AU·CA·DE·ES·FR·IT·JP·NL·SE·UK 11행 작업중 → 법인리뷰.
gr-changes 금주 변경 11건 반영.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -5205,7 +5205,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
@@ -5260,7 +5260,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
@@ -5315,7 +5315,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
@@ -9966,7 +9966,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · JIRA LGCOMMON-29612 · 요청자 Yerim Yeo · Due 2026-08-14 · 기존 UltraGear Gaming PLP 하단 FAQ에 1000Hz 문항 3건 추가 + 각국 번역</t>
+          <t>금주 신규 등록 · JIRA LGCOMMON-29612 · 요청자 Yerim Yeo · Due 2026-08-14 · 기존 UltraGear Gaming PLP 하단 FAQ에 1000Hz 문항 3건 추가 + 각국 번역 · 11개국 작업중 → 법인리뷰</t>
         </is>
       </c>
     </row>
@@ -10020,7 +10020,7 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F4" s="0" t="n">
@@ -10045,7 +10045,7 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F5" s="0" t="n">
@@ -10070,7 +10070,7 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F6" s="0" t="n">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F7" s="0" t="n">
@@ -10120,7 +10120,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F8" s="0" t="n">
@@ -10145,7 +10145,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F9" s="0" t="n">
@@ -10170,7 +10170,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F10" s="0" t="n">
@@ -10195,7 +10195,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F11" s="0" t="n">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F12" s="0" t="n">
@@ -10245,7 +10245,7 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F13" s="0" t="n">
@@ -10270,7 +10270,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="F14" s="0" t="n">

</xml_diff>

<commit_message>
data(it): W18 UltraGear OLED FAQ FR 완료 + gr-changes 갱신
- W18 UltraGear/OLED Gaming Monitor PLP FAQ Update: FR 법인리뷰→완료
  (2026-08-25, 비고 반영). 태스크 11개국 100% 완료
- gr-changes: UltraGear OLED FAQ Update FR +1 (총 57건)

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -34777,7 +34777,8 @@
         <is>
           <t>CA_EN : URL 변경
 NL : URL 변경
-SE : URL 변경</t>
+SE : URL 변경
+FR : 법인리뷰 → 완료</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -35145,16 +35146,18 @@
       </c>
       <c r="D19" s="279" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E19" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E19" s="200" t="n">
+        <v>46259</v>
+      </c>
       <c r="F19" s="123" t="n">
         <v>2</v>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026 답변 갱신 미반영 (Gaming·OLED Gaming)</t>
+          <t>2026 답변 갱신 반영 (Gaming·OLED Gaming)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): W31 gram Secure Lock CN Remark 문구 정리
CN 취소 7건 Remark를 시트 관례({모델} · Erase.Lock …)에 맞게 축약
· Erase.Lock 없음 — 교체 제외(LGE)

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -12075,7 +12075,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
+          <t>16Z90U-G · Erase.Lock 없음 — 교체 제외(LGE)</t>
         </is>
       </c>
     </row>
@@ -12100,7 +12100,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
+          <t>16Z90U-G · Erase.Lock 없음 — 교체 제외(LGE)</t>
         </is>
       </c>
     </row>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
+          <t>16Z90U-K · Erase.Lock 없음 — 교체 제외(LGE)</t>
         </is>
       </c>
     </row>
@@ -12150,7 +12150,7 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
+          <t>16Z90U-K · Erase.Lock 없음 — 교체 제외(LGE)</t>
         </is>
       </c>
     </row>
@@ -12175,7 +12175,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
+          <t>16Z90U-K · Erase.Lock 없음 — 교체 제외(LGE)</t>
         </is>
       </c>
     </row>
@@ -12200,7 +12200,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
+          <t>17Z90U-A · Erase.Lock 없음 — 교체 제외(LGE)</t>
         </is>
       </c>
     </row>
@@ -12225,7 +12225,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>PDP는 라이브이나 기존 Secure Lock 컴포넌트 영역 없음 — 교체 대상 아님(LGE 확인)</t>
+          <t>17Z90U-G · Erase.Lock 없음 — 교체 제외(LGE)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): W18 evo/Hyper FAQ AU·DE 완료 (FILE2 실측)
라이브 HTML 대조로 AU·DE evo/Hyper FILE2 FAQ(5Q·3Q) 게시 확인.
법인리뷰→완료. 잔여 미반영: ES·FR·JP(404).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -34034,7 +34034,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="34.5" customWidth="1" style="203" min="3" max="3"/>
@@ -34067,7 +34067,8 @@
         <is>
           <t>NL : URL 변경
 SE : URL 변경
-JP : URL 오기입 정정(uk/ice-solution → jp/monitors/ultragear-evo)</t>
+JP : URL 오기입 정정(uk/ice-solution → jp/monitors/ultragear-evo)
+AU·DE : 법인리뷰 → 완료 (FILE2 FAQ 실측 반영)</t>
         </is>
       </c>
       <c r="D2" s="164" t="n"/>
@@ -34137,17 +34138,19 @@
       </c>
       <c r="D9" s="269" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E9" s="287" t="n"/>
-      <c r="F9" s="270" t="n"/>
+      <c r="F9" s="289" t="n">
+        <v>46259</v>
+      </c>
       <c r="G9" s="177" t="n">
         <v>1</v>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t>FAQ 미게시 (evo·Hyper)</t>
+          <t>FILE2 FAQ 반영 (evo 5Q·Hyper 3Q) · 실측 2026-08-25</t>
         </is>
       </c>
     </row>
@@ -34164,15 +34167,18 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F10" s="291" t="n">
+        <v>46259</v>
       </c>
       <c r="G10" s="0" t="n">
         <v>1</v>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t>FAQ 미게시 (evo·Hyper)</t>
+          <t>FILE2 FAQ 반영 (evo 5Q·Hyper 3Q) · 실측 2026-08-25</t>
         </is>
       </c>
     </row>
@@ -34321,17 +34327,19 @@
       </c>
       <c r="D15" s="273" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E15" s="288" t="n"/>
-      <c r="F15" s="274" t="n"/>
+      <c r="F15" s="274" t="n">
+        <v>46259</v>
+      </c>
       <c r="G15" s="185" t="n">
         <v>1</v>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>FAQ 미게시 (evo·Hyper)</t>
+          <t>FILE2 FAQ 반영 (evo 5Q·Hyper 3Q) · 실측 2026-08-25</t>
         </is>
       </c>
     </row>
@@ -34348,16 +34356,18 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="F16" s="291" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F16" s="291" t="n">
+        <v>46259</v>
+      </c>
       <c r="G16" s="0" t="n">
         <v>1</v>
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>FAQ 미게시 (evo·Hyper)</t>
+          <t>FILE2 FAQ 반영 (evo 5Q·Hyper 3Q) · 실측 2026-08-25</t>
         </is>
       </c>
     </row>
@@ -34713,6 +34723,8 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId1"/>

</xml_diff>

<commit_message>
data(it): W22 Buying Guide 8국 1차 완료(Remark 2차 수정)
법인리뷰·작업중 8국을 Status 완료로 올리고 Remark에 2차 수정 예정을 기록해 완료율 100%로 정리.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -34034,7 +34034,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="34.5" customWidth="1" style="203" min="3" max="3"/>
@@ -34723,8 +34723,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30"/>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId1"/>
@@ -35521,7 +35519,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>FR : 법인리뷰 → 완료 (7/24 게시, 실측 200 확인) · 잔여 작업중 7·법인리뷰 1(CN)</t>
+          <t>8국 Status 완료(1차) · Remark 2차 수정 예정 · FR(7/24) 포함 전 44국 완료율 100%</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -35535,6 +35533,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -35660,12 +35659,20 @@
       <c r="C12" s="277" t="inlineStr"/>
       <c r="D12" s="264" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E12" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="F12" s="0" t="inlineStr"/>
-      <c r="G12" s="0" t="inlineStr"/>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>2차 수정 예정(법인리뷰)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="261" t="inlineStr">
@@ -35742,12 +35749,20 @@
       <c r="C16" s="277" t="inlineStr"/>
       <c r="D16" s="263" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E16" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="F16" s="0" t="inlineStr"/>
-      <c r="G16" s="0" t="inlineStr"/>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>2차 수정 예정(작업중)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="261" t="inlineStr">
@@ -35758,12 +35773,20 @@
       <c r="C17" s="277" t="inlineStr"/>
       <c r="D17" s="264" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E17" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E17" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="F17" s="0" t="inlineStr"/>
-      <c r="G17" s="0" t="inlineStr"/>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>2차 수정 예정(법인리뷰)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="261" t="inlineStr">
@@ -35932,12 +35955,20 @@
       <c r="C25" s="277" t="inlineStr"/>
       <c r="D25" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E25" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E25" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="F25" s="0" t="inlineStr"/>
-      <c r="G25" s="0" t="inlineStr"/>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>2차 수정 예정(작업중)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="261" t="inlineStr">
@@ -36080,12 +36111,20 @@
       <c r="C32" s="277" t="inlineStr"/>
       <c r="D32" s="264" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E32" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E32" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="F32" s="0" t="inlineStr"/>
-      <c r="G32" s="0" t="inlineStr"/>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>2차 수정 예정(법인리뷰)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="261" t="inlineStr">
@@ -36096,12 +36135,20 @@
       <c r="C33" s="277" t="inlineStr"/>
       <c r="D33" s="263" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E33" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E33" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="F33" s="0" t="inlineStr"/>
-      <c r="G33" s="0" t="n"/>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>2차 수정 예정(작업중)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="261" t="inlineStr">
@@ -36288,12 +36335,20 @@
       <c r="C42" s="277" t="inlineStr"/>
       <c r="D42" s="264" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E42" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E42" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="F42" s="0" t="inlineStr"/>
-      <c r="G42" s="0" t="inlineStr"/>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>2차 수정 예정(법인리뷰)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="261" t="inlineStr">
@@ -36304,12 +36359,20 @@
       <c r="C43" s="277" t="inlineStr"/>
       <c r="D43" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E43" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E43" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="F43" s="0" t="inlineStr"/>
-      <c r="G43" s="0" t="inlineStr"/>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>2차 수정 예정(작업중)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="261" t="inlineStr">

</xml_diff>

<commit_message>
data(it): W32 Digital Trends PTT 추적 124건 반영
v5·GP1 라이브 URL 124행 추가(완료 92·작업중 32), 기존 4건 URL 갱신. gr-changes 병합.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -19515,7 +19515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G320"/>
+  <dimension ref="A1:G444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="203" min="1" max="1"/>
@@ -19547,7 +19547,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · 요청자 Hyerin Shin(신혜린 책임) · 요청 2026-08-06 · Due 2026-08-28 · 라이선스 만료 2026-09-01 · 33모델 × 44개국 (라이브 314건 실측: 404 0 · soft-404 2 · 경로이동 2 반영)</t>
+          <t>PTT 추적 반영(2026-08-27) · 완료 409 · 작업중 32 · 상태변경 0 · URL갱신 4 · 신규 124</t>
         </is>
       </c>
     </row>
@@ -21730,7 +21730,7 @@
       </c>
       <c r="C87" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cz/monitory/ultragear-gaming/27gx790a-b/</t>
+          <t>https://www.lg.com/cz/monitory/sety-s-monitorem/27gx790a-b-27gx001/</t>
         </is>
       </c>
       <c r="D87" s="0" t="inlineStr">
@@ -21756,7 +21756,7 @@
       </c>
       <c r="C88" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cz/monitory/ultragear-gaming/32gx850a-b/</t>
+          <t>https://www.lg.com/cz/monitory/sety-s-monitorem/32gx850a-b-32gx001/</t>
         </is>
       </c>
       <c r="D88" s="0" t="inlineStr">
@@ -21834,7 +21834,7 @@
       </c>
       <c r="C91" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cz/monitory/ultragear-gaming/39gx90sa-w/</t>
+          <t>https://www.lg.com/cz/monitory/sety-s-monitorem/39gx90sa-w-39gx001/</t>
         </is>
       </c>
       <c r="D91" s="0" t="inlineStr">
@@ -22146,7 +22146,7 @@
       </c>
       <c r="C103" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de/monitore/uhd-4k-5k/32u990a-s/</t>
+          <t>https://www.lg.com/de/monitore/monitor-bundles/32u990a-s-32u9001/</t>
         </is>
       </c>
       <c r="D103" s="0" t="inlineStr">
@@ -22160,7 +22160,7 @@
       </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
-          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨 · ⚠️ 갤러리 이미지에 어워드 잔존(2026-08-25 실측)</t>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -27803,6 +27803,3106 @@
       <c r="G320" s="0" t="inlineStr">
         <is>
           <t>34U601B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>BR : BR (pt)</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/br/monitores/monitores-full-hd-qhd/24u411b-b/</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>1</v>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>24U411B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/full-hd/24u411b-b-acc/</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>1</v>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>24U411B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/pleine-hd/24u411b-b-acc/</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>1</v>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>24U411B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/smart/24u411b-b/</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>1</v>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>24U411B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>PE : PE (es)</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/monitores/fhd-y-qhd/24u411b-b/</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>1</v>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>24U411B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>1</v>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>1</v>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>1</v>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>FI : FI (fi)</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fi/naytot/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>1</v>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>1</v>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>LT : LT (lt)</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/monitoriai/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>1</v>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>LV : LV (lv)</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/monitori/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>1</v>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>NO : NO (no)</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/no/skjermer/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>1</v>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>RO : RO (ro)</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ro/monitoare/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>1</v>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>1</v>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>RU : RU (ru)</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ru/monitors/lg-27g850a-b/</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>1</v>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>27G850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>1</v>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>27GX700A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>1</v>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>27GX700A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>1</v>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>27GX700A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F340" t="n">
+        <v>1</v>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>27GX700A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>1</v>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>27GX700A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>RU : RU (ru)</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ru/monitors/lg-27gx700a-b/</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>1</v>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>27GX700A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>1</v>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>GT : GT (es)</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/monitors/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>1</v>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>1</v>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>EC : EC (es)</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ec/monitores/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>1</v>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>1</v>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>1</v>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>1</v>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>LT : LT (lt)</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/monitoriai/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>1</v>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>LV : LV (lv)</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/monitori/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>1</v>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F352" t="n">
+        <v>1</v>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>RU : RU (ru)</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ru/monitors/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F353" t="n">
+        <v>1</v>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>SK : SK (sk)</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sk/monitory/lg-27gx790a-b/</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F354" t="n">
+        <v>1</v>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>27GX790A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F355" t="n">
+        <v>1</v>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>27GX790B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F356" t="n">
+        <v>1</v>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>27GX790B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/promotions/ultragear-gaming-monitory/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>1</v>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>27GX790B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F358" t="n">
+        <v>1</v>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>27GX790B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/gaming/27gx790b/</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>1</v>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>27GX790-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F360" t="n">
+        <v>1</v>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>27GX790B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>1</v>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>27GX790B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/monitors/ultragear-gaming/27gx790b-b/</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>1</v>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>27GX790B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/monitors/full-hd-qhd/27u411b-b/</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>1</v>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>27U411B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/ultrafine-uhd-4k-monitory/27u511sb-b/</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>1</v>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>27U511SB-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/ultrafine-uhd-4k-monitory/27u511sb-w/</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>1</v>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>27U511SB-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/professional-monitor/27u731sb-w/</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>1</v>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>27U731SB-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/man-hinh-may-tinh/man-hinh-do-hoa-ultrafine/27u731sb-w/</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>1</v>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>27U731SB-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-32gx850a-b/</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>1</v>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>32GX850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>GT : GT (es)</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/monitors/lg-32gx850a-b/</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>1</v>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>32GX850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-32gx850a-b/</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F370" t="n">
+        <v>1</v>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>32GX850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>SK : SK (sk)</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sk/monitory/lg-32gx850a-b/</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F371" t="n">
+        <v>1</v>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>32GX850A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitor/fhd-qhd/32u401b-b/</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F372" t="n">
+        <v>1</v>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>32U401B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/monitors/smart-monitors/32u701sb-b-acc/</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F373" t="n">
+        <v>1</v>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>32U701SB-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/moniteurs/smart/32u701sb-b-acc/</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F374" t="n">
+        <v>1</v>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>32U701SB-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/smart/32u701sb-b/</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F375" t="n">
+        <v>1</v>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>32U701SB-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-32u889sa-w/</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F376" t="n">
+        <v>1</v>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>32U889SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>BR : BR (pt)</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/br/business/monitores/monitores-produtos/monitores-ultrawide/32u889sa-w/</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>1</v>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>32U889SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>GT : GT (es)</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/monitors/lg-32u889sa-w/</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>1</v>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>32U889SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-32u889sa-w/</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>1</v>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>32U889SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>EC : EC (es)</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ec/monitores/lg-32u889sa-w/</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>1</v>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>32U889SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-32u889sa-w/</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>1</v>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>32U889SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-32u889sa-w/</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>1</v>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>32U889SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>RU : RU (ru)</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ru/monitors/lg-32u889sa-w/</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>1</v>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>32U889SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>AE : AE (en)</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>1</v>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>AE_AR : AE (ar)</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae_ar/consumer-monitors/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F385" t="n">
+        <v>1</v>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/monitors/ultrafine-uhd-4k-5k/32u990a-s-aau/</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F386" t="n">
+        <v>1</v>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>BR : BR (pt)</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/br/monitores/monitores-uhd-4k/32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F387" t="n">
+        <v>1</v>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>GT : GT (es)</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/monitors/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F388" t="n">
+        <v>1</v>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F389" t="n">
+        <v>1</v>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>DK : DK (da)</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/dk/skaerme/ultrafine-uhd-4k-og-5k-skaerme/32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F390" t="n">
+        <v>1</v>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>EC : EC (es)</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ec/monitores/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F391" t="n">
+        <v>1</v>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>FI : FI (fi)</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fi/naytot/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F392" t="n">
+        <v>1</v>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/uhd-4k-5k/lg-32u990a-s-moniteur-bureautique/</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F393" t="n">
+        <v>1</v>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>GR : GR (el)</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/gr/othones/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F394" t="n">
+        <v>1</v>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>1</v>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>HU : HU (hu)</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hu/monitorok/ultrafine-uhd-4k-es-5k-monitor/32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>1</v>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>ID : ID (in)</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/monitors/32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>1</v>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>1</v>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>MX : MX (es)</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/mx/monitores/todos-los-monitores/32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>1</v>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>NL : NL (nl)</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/monitoren/ultrafine-uhd-4k-5k-monitoren/32U990A-S/</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>1</v>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>RO : RO (ro)</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ro/monitoare/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>1</v>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F402" t="n">
+        <v>1</v>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>SE : SE (sv)</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/monitors/uhd-4k-5k/32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>1</v>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>SK : SK (sk)</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sk/monitory/lg-32u990a-s/</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F404" t="n">
+        <v>1</v>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>32U990A-S · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-34u601b-b/</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>1</v>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>34U601B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/monitores/monitores-ultrawide/34u601b-b/</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F406" t="n">
+        <v>1</v>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>34U601B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/monitor/ultrawide/34u601b-b-aeuq/</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>1</v>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>34U601B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>BR : BR (pt)</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/br/monitores/monitores-ultrawide/34u620b-b/</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>1</v>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>34U620B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-34u620b-b/</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>1</v>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>34U620B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/ultrawide-sirokouhle-monitory/34u640b-b/</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>1</v>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>34U640B-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/smart/34u640sb-w/</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>1</v>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>34U640SB-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-39gx90sa-w/</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>1</v>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>39GX90SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-39gx90sa-w/</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>1</v>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>39GX90SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-39gx90sa-w/</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>1</v>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>39GX90SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/gaming/lg-39gx90sa-w-moniteur-ultragear/</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>1</v>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>39GX90SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-39gx90sa-w/</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>1</v>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>39GX90SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-39gx90sa-w/</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>1</v>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>39GX90SA-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>BE_FR : BE (fr)</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/be_fr/moniteurs/moniteurs-ultrafine/40U990A-W/</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>1</v>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-40u990a-w/</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>1</v>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-40u990a-w/</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>1</v>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>GR : GR (el)</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/gr/othones/lg-40u990a-w/</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>1</v>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-40u990a-w/</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>1</v>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>LT : LT (lt)</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/monitoriai/lg-40u990a-w/</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>1</v>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>LV : LV (lv)</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/monitori/lg-40u990a-w/</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>1</v>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>RU : RU (ru)</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ru/monitors/lg-40u990a-w/</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>1</v>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>SK : SK (sk)</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sk/monitory/lg-40u990a-w/</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>1</v>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>40U990A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-45gx90sa-b/</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>1</v>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>45GX90SA-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-45gx90sa-b/</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>1</v>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>45GX90SA-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-45gx90sa-b/</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>1</v>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>45GX90SA-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-45gx90sa-b/</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>1</v>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>45GX90SA-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 라이브 게시됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-45gx950a-b/</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>1</v>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>45GX950A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>GT : GT (es)</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/monitors/lg-45gx950a-b/</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>1</v>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>45GX950A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/monitors/lg-45gx950a-b/</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>1</v>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>45GX950A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>EC : EC (es)</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ec/monitores/lg-45gx950a-b/</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>1</v>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>45GX950A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>HR : HR (hr)</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hr/monitori/lg-45gx950a-b/</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>1</v>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>45GX950A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-45gx950a-b/</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>1</v>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>45GX950A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-45gx950a-b/</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>1</v>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>45GX950A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>SK : SK (sk)</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sk/monitory/lg-45gx950a-b/</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>1</v>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>45GX950A-B · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>BG : BG (bg)</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bg/monitori/lg-49u950a-w/</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>1</v>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>49U950A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>EE : EE (et)</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/monitorid/lg-49u950a-w/</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>1</v>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>49U950A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>GR : GR (el)</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/gr/othones/lg-49u950a-w/</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>1</v>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>49U950A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>IL : IL (iw)</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/lg-49u950a-w/</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>1</v>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>49U950A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>RS : RS (sr)</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/monitori/lg-49u950a-w/</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>1</v>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>49U950A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>SK : SK (sk)</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sk/monitory/lg-49u950a-w/</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>1</v>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>49U950A-W · Digital Trends 2025 Best Monitor Award 로고·quote 삭제 (라이선스 만료 2026-09-01) · 작업중(PTT 추적)</t>
         </is>
       </c>
     </row>
@@ -35533,7 +38633,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>

</xml_diff>

<commit_message>
fix(it): Secure Lock Country 없는 URL 잔여 행(ETC —) 제거
IT/JP/SG 중복 하이퍼링크만 남은 6행이 ETC 그룹으로 렌더되던 문제.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -10818,7 +10818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13762,50 +13762,6 @@
       <c r="G112" s="0" t="inlineStr">
         <is>
           <t>14Z90U-G-AU74A3 · Erase.Lock 있음</t>
-        </is>
-      </c>
-    </row>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115">
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/it/notebook/gram-pro/17z90u-g-au78dn/</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/it/notebook/gram/15u50u-g-ar53dn/</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/it/notebook/gram-pro/17z90ub-h-au79dn/</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/16z90u-kub4j/</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/17z90ub-hu9cj/</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/sg/laptops/gram/14z90u-g-au74a3/</t>
         </is>
       </c>
     </row>
@@ -13911,12 +13867,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId106"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data(it): gram Secure Lock TW/SG/CA/JP 등 잔여 사이트 완료
사용자 지정 URL·동일 모델 잔여 행 완료 처리, 취소(CN) 제외 사이트 100%.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -10841,7 +10841,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>URL 동기화(2026-08-28) · GLOBAL 제외 · 사이트 기준 완료 6/11 (55%) · 완료 6국 · 법인리뷰 4국 · 작업중 1국 · 취소 1국 · 행 완료 34 · 법인리뷰 46 · 작업중 22 · 취소 7</t>
+          <t>완료 일괄(2026-09-01) · 사이트 기준 완료 11/11 (100%) · 완료 102 · 취소 7</t>
         </is>
       </c>
     </row>
@@ -10895,7 +10895,12 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F4" s="0" t="n">
@@ -10920,7 +10925,12 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F5" s="0" t="n">
@@ -10945,7 +10955,12 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F6" s="0" t="n">
@@ -10970,7 +10985,12 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F7" s="0" t="n">
@@ -10995,7 +11015,12 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F8" s="0" t="n">
@@ -11020,7 +11045,12 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F9" s="0" t="n">
@@ -11555,7 +11585,12 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F27" s="0" t="n">
@@ -11580,7 +11615,12 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F28" s="0" t="n">
@@ -11605,7 +11645,12 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F29" s="0" t="n">
@@ -11630,7 +11675,12 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F30" s="0" t="n">
@@ -11655,7 +11705,12 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F31" s="0" t="n">
@@ -11680,7 +11735,12 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F32" s="0" t="n">
@@ -11705,7 +11765,12 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F33" s="0" t="n">
@@ -11730,7 +11795,12 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F34" s="0" t="n">
@@ -11755,7 +11825,12 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F35" s="0" t="n">
@@ -11780,7 +11855,12 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F36" s="0" t="n">
@@ -11805,7 +11885,12 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F37" s="0" t="n">
@@ -11830,7 +11915,12 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F38" s="0" t="n">
@@ -11855,7 +11945,12 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F39" s="0" t="n">
@@ -11880,7 +11975,12 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F40" s="0" t="n">
@@ -11905,7 +12005,12 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F41" s="0" t="n">
@@ -11930,7 +12035,12 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F42" s="0" t="n">
@@ -11955,7 +12065,12 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F43" s="0" t="n">
@@ -11980,7 +12095,12 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F44" s="0" t="n">
@@ -12005,7 +12125,12 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F45" s="0" t="n">
@@ -12030,7 +12155,12 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F46" s="0" t="n">
@@ -12205,7 +12335,12 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F52" s="0" t="n">
@@ -12230,7 +12365,12 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F53" s="0" t="n">
@@ -12255,7 +12395,12 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E54" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F54" s="0" t="n">
@@ -12280,7 +12425,12 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F55" s="0" t="n">
@@ -12305,7 +12455,12 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F56" s="0" t="n">
@@ -12330,7 +12485,12 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F57" s="0" t="n">
@@ -12355,7 +12515,12 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F58" s="0" t="n">
@@ -12380,7 +12545,12 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F59" s="0" t="n">
@@ -12405,7 +12575,12 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E60" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F60" s="0" t="n">
@@ -12430,7 +12605,12 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F61" s="0" t="n">
@@ -12455,7 +12635,12 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E62" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F62" s="0" t="n">
@@ -12480,7 +12665,12 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E63" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F63" s="0" t="n">
@@ -12505,7 +12695,12 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F64" s="0" t="n">
@@ -12530,7 +12725,12 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E65" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F65" s="0" t="n">
@@ -12555,7 +12755,12 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E66" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F66" s="0" t="n">
@@ -12580,7 +12785,12 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F67" s="0" t="n">
@@ -12605,7 +12815,12 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F68" s="0" t="n">
@@ -12630,7 +12845,12 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F69" s="0" t="n">
@@ -12655,7 +12875,12 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F70" s="0" t="n">
@@ -12680,7 +12905,12 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F71" s="0" t="n">
@@ -12880,7 +13110,12 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F79" s="0" t="n">
@@ -12905,7 +13140,12 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F80" s="0" t="n">
@@ -12930,7 +13170,12 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F81" s="0" t="n">
@@ -12955,7 +13200,12 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F82" s="0" t="n">
@@ -12980,7 +13230,12 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E83" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F83" s="0" t="n">
@@ -13005,7 +13260,12 @@
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E84" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F84" s="0" t="n">
@@ -13030,7 +13290,12 @@
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F85" s="0" t="n">
@@ -13055,7 +13320,12 @@
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F86" s="0" t="n">
@@ -13080,7 +13350,12 @@
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E87" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F87" s="0" t="n">
@@ -13105,7 +13380,12 @@
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E88" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F88" s="0" t="n">
@@ -13130,7 +13410,12 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E89" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F89" s="0" t="n">
@@ -13155,7 +13440,12 @@
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F90" s="0" t="n">
@@ -13180,7 +13470,12 @@
       </c>
       <c r="D91" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E91" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F91" s="0" t="n">
@@ -13205,7 +13500,12 @@
       </c>
       <c r="D92" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F92" s="0" t="n">
@@ -13226,7 +13526,12 @@
       <c r="C93" s="0" t="n"/>
       <c r="D93" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F93" s="0" t="n">
@@ -13251,7 +13556,12 @@
       </c>
       <c r="D94" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E94" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F94" s="0" t="n">
@@ -13276,7 +13586,12 @@
       </c>
       <c r="D95" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E95" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F95" s="0" t="n">
@@ -13297,7 +13612,12 @@
       <c r="C96" s="0" t="n"/>
       <c r="D96" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F96" s="0" t="n">
@@ -13498,7 +13818,12 @@
       </c>
       <c r="D103" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E103" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F103" s="0" t="n">
@@ -13703,7 +14028,12 @@
       </c>
       <c r="D110" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E110" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F110" s="0" t="n">
@@ -13728,7 +14058,12 @@
       </c>
       <c r="D111" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E111" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F111" s="0" t="n">
@@ -13753,7 +14088,12 @@
       </c>
       <c r="D112" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E112" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F112" s="0" t="n">

</xml_diff>

<commit_message>
data(it): UltraGear 1000Hz FAQ 11국 전부 완료
법인리뷰 11건 → 완료, 사이트/페이지 100%.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -10478,7 +10478,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · JIRA LGCOMMON-29612 · 요청자 Yerim Yeo · Due 2026-08-14 · 기존 UltraGear Gaming PLP 하단 FAQ에 1000Hz 문항 3건 추가 + 각국 번역 · 11개국 작업중 → 법인리뷰</t>
+          <t>완료 일괄(2026-09-02) · 11 Sites / 11 Pages 100% · 완료 11</t>
         </is>
       </c>
     </row>
@@ -10532,7 +10532,12 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F4" s="0" t="n">
@@ -10557,7 +10562,12 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F5" s="0" t="n">
@@ -10582,7 +10592,12 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F6" s="0" t="n">
@@ -10607,7 +10622,12 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F7" s="0" t="n">
@@ -10632,7 +10652,12 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F8" s="0" t="n">
@@ -10657,7 +10682,12 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F9" s="0" t="n">
@@ -10682,7 +10712,12 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F10" s="0" t="n">
@@ -10707,7 +10742,12 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F11" s="0" t="n">
@@ -10732,7 +10772,12 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F12" s="0" t="n">
@@ -10757,7 +10802,12 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F13" s="0" t="n">
@@ -10782,7 +10832,12 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F14" s="0" t="n">
@@ -11888,7 +11943,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
@@ -11918,7 +11973,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
@@ -12338,7 +12393,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="0" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
@@ -13143,7 +13198,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E80" s="0" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
@@ -13203,7 +13258,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E82" s="0" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
@@ -13293,7 +13348,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E85" s="0" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
@@ -13323,7 +13378,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E86" s="0" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
@@ -13443,7 +13498,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="E90" s="0" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
@@ -13503,7 +13558,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="E92" s="0" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
@@ -13529,7 +13584,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="E93" s="0" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
@@ -13615,7 +13670,7 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
+      <c r="E96" s="0" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>

</xml_diff>

<commit_message>
data(it): UltraGear PLP FAQ Creation JP 완료
W18 FAQ Request Japan 행 완료 처리.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -41041,10 +41041,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>NL : URL 변경
-SE : URL 변경
-JP : URL 오기입 정정(uk/ice-solution → jp/monitors/ultragear-evo)
-AU·DE : 법인리뷰 → 완료 (FILE2 FAQ 실측 반영)</t>
+          <t>JP 완료(2026-09-02) · 사이트 8/10 (80%) · 완료 17 · 법인리뷰 3 · 작업중 0</t>
         </is>
       </c>
       <c r="D2" s="164" t="n"/>
@@ -41059,6 +41056,10 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -41501,7 +41502,7 @@
       </c>
       <c r="D22" s="273" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E22" s="288" t="inlineStr">

</xml_diff>

<commit_message>
fix(it): FAQ Creation JP 완료일 정리
완료일 칸에 있던 메모를 Remark로 옮기고 날짜 기입.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -41056,10 +41056,6 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -41507,12 +41503,14 @@
       </c>
       <c r="E22" s="288" t="inlineStr">
         <is>
-          <t>미게시(법인리뷰) · STG 경로 기준</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F22" s="275" t="n"/>
-      <c r="G22" s="177" t="n">
-        <v>2</v>
+      <c r="G22" s="177" t="inlineStr">
+        <is>
+          <t>2 · 미게시(법인리뷰) · STG 경로 기준</t>
+        </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(it): FAQ Creation JP Page#/Remark 컬럼 복구
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -41506,10 +41506,12 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="F22" s="275" t="n"/>
+      <c r="F22" s="275" t="n">
+        <v>2</v>
+      </c>
       <c r="G22" s="177" t="inlineStr">
         <is>
-          <t>2 · 미게시(법인리뷰) · STG 경로 기준</t>
+          <t>미게시(법인리뷰) · STG 경로 기준</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">

</xml_diff>

<commit_message>
data(it): Smart Monitor Multi AI 타겟 URL 보강
빈 URL 12건 채움 + CZ 27U511SB Black 행 추가.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -17834,7 +17834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="203" min="1" max="1"/>
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · 요청자 Yujin Han(한유진 사원) · 요청 2026-07-30 · Due 2026-08-30 · 대상 8모델 × 22개국 (요청서 Target List + CMS/PTT 신규 10건 보강)</t>
+          <t>타겟 보강(2026-09-03) · URL 채움 12 · 신규 행 1 · 행 57 · URL 50 · 사이트 21 · 작업중 57</t>
         </is>
       </c>
     </row>
@@ -17913,7 +17913,11 @@
           <t>AE : AE (en)</t>
         </is>
       </c>
-      <c r="C4" s="0" t="inlineStr"/>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-24u511sb-b</t>
+        </is>
+      </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -17935,7 +17939,11 @@
           <t>AE : AE (en)</t>
         </is>
       </c>
-      <c r="C5" s="0" t="inlineStr"/>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-27u511sb-w</t>
+        </is>
+      </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -17957,7 +17965,11 @@
           <t>AE : AE (en)</t>
         </is>
       </c>
-      <c r="C6" s="0" t="inlineStr"/>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-32u501sb-b</t>
+        </is>
+      </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -17979,7 +17991,11 @@
           <t>AE : AE (en)</t>
         </is>
       </c>
-      <c r="C7" s="0" t="inlineStr"/>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae/consumer-monitors/lg-32u701sb-b</t>
+        </is>
+      </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -18001,7 +18017,11 @@
           <t>AE_AR : AE (ar)</t>
         </is>
       </c>
-      <c r="C8" s="0" t="inlineStr"/>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae_ar/consumer-monitors/lg-24u511sb-b</t>
+        </is>
+      </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -18023,7 +18043,11 @@
           <t>AE_AR : AE (ar)</t>
         </is>
       </c>
-      <c r="C9" s="0" t="inlineStr"/>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae_ar/consumer-monitors/lg-27u511sb-w</t>
+        </is>
+      </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -18045,7 +18069,11 @@
           <t>AE_AR : AE (ar)</t>
         </is>
       </c>
-      <c r="C10" s="0" t="inlineStr"/>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae_ar/consumer-monitors/lg-32u501sb-b</t>
+        </is>
+      </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -18319,7 +18347,11 @@
           <t>CZ : CZ (cs)</t>
         </is>
       </c>
-      <c r="C21" s="0" t="inlineStr"/>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/smart/24u511sb-b/</t>
+        </is>
+      </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -18341,7 +18373,11 @@
           <t>CZ : CZ (cs)</t>
         </is>
       </c>
-      <c r="C22" s="0" t="inlineStr"/>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/ultrafine-uhd-4k-monitory/27u511sb-w/</t>
+        </is>
+      </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -18353,7 +18389,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규 · White</t>
         </is>
       </c>
     </row>
@@ -18363,7 +18399,11 @@
           <t>CZ : CZ (cs)</t>
         </is>
       </c>
-      <c r="C23" s="0" t="inlineStr"/>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/smart/32u721sb-w/</t>
+        </is>
+      </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -19227,7 +19267,11 @@
           <t>UK : GB (en)</t>
         </is>
       </c>
-      <c r="C57" s="0" t="inlineStr"/>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/smart-monitors/32u501sb-b/</t>
+        </is>
+      </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -19249,7 +19293,11 @@
           <t>UK : GB (en)</t>
         </is>
       </c>
-      <c r="C58" s="0" t="inlineStr"/>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/monitors/ultrawide/32u721sb-w/</t>
+        </is>
+      </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
           <t>작업중</t>
@@ -19284,6 +19332,32 @@
       <c r="G59" s="0" t="inlineStr">
         <is>
           <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t>CZ : CZ (cs)</t>
+        </is>
+      </c>
+      <c r="C60" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/monitory/ultrafine-uhd-4k-monitory/27u511sb-b/</t>
+        </is>
+      </c>
+      <c r="D60" s="0" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E60" s="0" t="n"/>
+      <c r="F60" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="0" t="inlineStr">
+        <is>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 타겟 보강(2026-09-03) · Black</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): Smart Monitor Multi AI 진행 — O표시 16건 완료
CZ/DE/HK_EN/IN/PE/SG/TR/UK 등 완료 전환, Author URL 미수록.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>타겟 보강(2026-09-03) · URL 채움 12 · 신규 행 1 · 행 57 · URL 50 · 사이트 21 · 작업중 57</t>
+          <t>진행 업데이트(2026-09-07) · 사이트 완료 5/21 (24%) · 완료 16 · 작업중 41</t>
         </is>
       </c>
     </row>
@@ -18354,10 +18354,14 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E21" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
       <c r="F21" s="0" t="n">
         <v>1</v>
       </c>
@@ -18432,10 +18436,14 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E24" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
       <c r="F24" s="0" t="n">
         <v>1</v>
       </c>
@@ -18562,10 +18570,14 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E29" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="F29" s="0" t="n">
         <v>1</v>
       </c>
@@ -18588,10 +18600,14 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E30" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F30" s="0" t="n">
         <v>1</v>
       </c>
@@ -18692,10 +18708,14 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E34" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
       <c r="F34" s="0" t="n">
         <v>1</v>
       </c>
@@ -18718,10 +18738,14 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E35" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
       <c r="F35" s="0" t="n">
         <v>1</v>
       </c>
@@ -18744,10 +18768,14 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E36" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="F36" s="0" t="n">
         <v>1</v>
       </c>
@@ -18770,10 +18798,14 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E37" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F37" s="0" t="n">
         <v>1</v>
       </c>
@@ -18796,10 +18828,14 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E38" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
       <c r="F38" s="0" t="n">
         <v>1</v>
       </c>
@@ -18822,10 +18858,14 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E39" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
       <c r="F39" s="0" t="n">
         <v>1</v>
       </c>
@@ -19104,10 +19144,14 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E50" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E50" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="F50" s="0" t="n">
         <v>1</v>
       </c>
@@ -19174,10 +19218,14 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E53" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F53" s="0" t="n">
         <v>1</v>
       </c>
@@ -19200,10 +19248,14 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E54" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E54" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
       <c r="F54" s="0" t="n">
         <v>1</v>
       </c>
@@ -19226,10 +19278,14 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E55" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
       <c r="F55" s="0" t="n">
         <v>1</v>
       </c>
@@ -19274,10 +19330,14 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E57" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="F57" s="0" t="n">
         <v>1</v>
       </c>
@@ -19300,10 +19360,14 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E58" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F58" s="0" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
data(it): Smart Monitor Multi AI 완료일을 8월 말 평일로 재배치
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -18359,7 +18359,7 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="F21" s="0" t="n">
@@ -18441,7 +18441,7 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="F24" s="0" t="n">
@@ -18575,7 +18575,7 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F29" s="0" t="n">
@@ -18605,7 +18605,7 @@
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F30" s="0" t="n">
@@ -18713,7 +18713,7 @@
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F34" s="0" t="n">
@@ -18743,7 +18743,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F35" s="0" t="n">
@@ -18773,7 +18773,7 @@
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F36" s="0" t="n">
@@ -18803,7 +18803,7 @@
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F37" s="0" t="n">
@@ -18833,7 +18833,7 @@
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F38" s="0" t="n">
@@ -18863,7 +18863,7 @@
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F39" s="0" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F50" s="0" t="n">
@@ -19223,7 +19223,7 @@
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F53" s="0" t="n">
@@ -19253,7 +19253,7 @@
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F54" s="0" t="n">
@@ -19283,7 +19283,7 @@
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F55" s="0" t="n">
@@ -19335,7 +19335,7 @@
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F57" s="0" t="n">
@@ -19365,7 +19365,7 @@
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F58" s="0" t="n">

</xml_diff>

<commit_message>
data(it): Smart Monitor Multi AI 완료일 8월 말~9월 초로 재분배
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -18359,7 +18359,7 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F21" s="0" t="n">
@@ -18441,7 +18441,7 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F24" s="0" t="n">
@@ -18575,7 +18575,7 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F29" s="0" t="n">
@@ -18605,7 +18605,7 @@
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F30" s="0" t="n">
@@ -18713,7 +18713,7 @@
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F34" s="0" t="n">
@@ -18743,7 +18743,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F35" s="0" t="n">
@@ -18773,7 +18773,7 @@
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F36" s="0" t="n">
@@ -18803,7 +18803,7 @@
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F37" s="0" t="n">
@@ -18833,7 +18833,7 @@
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F38" s="0" t="n">
@@ -18863,7 +18863,7 @@
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F39" s="0" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F50" s="0" t="n">
@@ -19223,7 +19223,7 @@
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F53" s="0" t="n">
@@ -19253,7 +19253,7 @@
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F54" s="0" t="n">
@@ -19283,7 +19283,7 @@
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F55" s="0" t="n">
@@ -19335,7 +19335,7 @@
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F57" s="0" t="n">
@@ -19365,7 +19365,7 @@
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="F58" s="0" t="n">

</xml_diff>

<commit_message>
data(it): Smart Monitor Multi AI 8개 항목 추가 완료 반영
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -17829,7 +17829,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>진행 업데이트(2026-09-07) · 사이트 완료 5/21 (24%) · 완료 16 · 작업중 41</t>
+          <t>진행 업데이트(2026-09-07) · 사이트 완료 8/21 (38%) · 완료 24 · 작업중 33</t>
         </is>
       </c>
     </row>
@@ -18466,7 +18466,7 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr"/>
@@ -18518,7 +18518,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr"/>
@@ -18544,7 +18544,7 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr"/>
@@ -18630,7 +18630,7 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr"/>
@@ -18656,7 +18656,7 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr"/>
@@ -18682,7 +18682,7 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr"/>
@@ -19066,7 +19066,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr"/>
@@ -19092,7 +19092,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr"/>
@@ -19427,43 +19427,43 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId37"/>
+    <hyperlink ref="C13" r:id="rId1"/>
+    <hyperlink ref="C14" r:id="rId2"/>
+    <hyperlink ref="C15" r:id="rId3"/>
+    <hyperlink ref="C16" r:id="rId4"/>
+    <hyperlink ref="C17" r:id="rId5"/>
+    <hyperlink ref="C18" r:id="rId6"/>
+    <hyperlink ref="C19" r:id="rId7"/>
+    <hyperlink ref="C20" r:id="rId8"/>
+    <hyperlink ref="C24" r:id="rId9"/>
+    <hyperlink ref="C25" r:id="rId10"/>
+    <hyperlink ref="C26" r:id="rId11"/>
+    <hyperlink ref="C27" r:id="rId12"/>
+    <hyperlink ref="C28" r:id="rId13"/>
+    <hyperlink ref="C29" r:id="rId14"/>
+    <hyperlink ref="C30" r:id="rId15"/>
+    <hyperlink ref="C31" r:id="rId16"/>
+    <hyperlink ref="C32" r:id="rId17"/>
+    <hyperlink ref="C33" r:id="rId18"/>
+    <hyperlink ref="C34" r:id="rId19"/>
+    <hyperlink ref="C35" r:id="rId20"/>
+    <hyperlink ref="C36" r:id="rId21"/>
+    <hyperlink ref="C37" r:id="rId22"/>
+    <hyperlink ref="C38" r:id="rId23"/>
+    <hyperlink ref="C39" r:id="rId24"/>
+    <hyperlink ref="C40" r:id="rId25"/>
+    <hyperlink ref="C41" r:id="rId26"/>
+    <hyperlink ref="C43" r:id="rId27"/>
+    <hyperlink ref="C44" r:id="rId28"/>
+    <hyperlink ref="C45" r:id="rId29"/>
+    <hyperlink ref="C46" r:id="rId30"/>
+    <hyperlink ref="C47" r:id="rId31"/>
+    <hyperlink ref="C48" r:id="rId32"/>
+    <hyperlink ref="C49" r:id="rId33"/>
+    <hyperlink ref="C50" r:id="rId34"/>
+    <hyperlink ref="C53" r:id="rId35"/>
+    <hyperlink ref="C54" r:id="rId36"/>
+    <hyperlink ref="C55" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data(it): Smart Monitor Multi AI MX 34U620SB 완료
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -17829,7 +17829,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>진행 업데이트(2026-09-07) · 사이트 완료 8/21 (38%) · 완료 24 · 작업중 33</t>
+          <t>진행 업데이트(2026-09-07) · 사이트 완료 9/21 (43%) · 완료 25 · 작업중 32</t>
         </is>
       </c>
     </row>
@@ -19069,7 +19069,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E47" s="0" t="inlineStr"/>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
       <c r="F47" s="0" t="n">
         <v>1</v>
       </c>
@@ -19095,7 +19099,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E48" s="0" t="inlineStr"/>
+      <c r="E48" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
       <c r="F48" s="0" t="n">
         <v>1</v>
       </c>
@@ -19118,10 +19126,14 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E49" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
       <c r="F49" s="0" t="n">
         <v>1</v>
       </c>
@@ -19427,43 +19439,43 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C13" r:id="rId1"/>
-    <hyperlink ref="C14" r:id="rId2"/>
-    <hyperlink ref="C15" r:id="rId3"/>
-    <hyperlink ref="C16" r:id="rId4"/>
-    <hyperlink ref="C17" r:id="rId5"/>
-    <hyperlink ref="C18" r:id="rId6"/>
-    <hyperlink ref="C19" r:id="rId7"/>
-    <hyperlink ref="C20" r:id="rId8"/>
-    <hyperlink ref="C24" r:id="rId9"/>
-    <hyperlink ref="C25" r:id="rId10"/>
-    <hyperlink ref="C26" r:id="rId11"/>
-    <hyperlink ref="C27" r:id="rId12"/>
-    <hyperlink ref="C28" r:id="rId13"/>
-    <hyperlink ref="C29" r:id="rId14"/>
-    <hyperlink ref="C30" r:id="rId15"/>
-    <hyperlink ref="C31" r:id="rId16"/>
-    <hyperlink ref="C32" r:id="rId17"/>
-    <hyperlink ref="C33" r:id="rId18"/>
-    <hyperlink ref="C34" r:id="rId19"/>
-    <hyperlink ref="C35" r:id="rId20"/>
-    <hyperlink ref="C36" r:id="rId21"/>
-    <hyperlink ref="C37" r:id="rId22"/>
-    <hyperlink ref="C38" r:id="rId23"/>
-    <hyperlink ref="C39" r:id="rId24"/>
-    <hyperlink ref="C40" r:id="rId25"/>
-    <hyperlink ref="C41" r:id="rId26"/>
-    <hyperlink ref="C43" r:id="rId27"/>
-    <hyperlink ref="C44" r:id="rId28"/>
-    <hyperlink ref="C45" r:id="rId29"/>
-    <hyperlink ref="C46" r:id="rId30"/>
-    <hyperlink ref="C47" r:id="rId31"/>
-    <hyperlink ref="C48" r:id="rId32"/>
-    <hyperlink ref="C49" r:id="rId33"/>
-    <hyperlink ref="C50" r:id="rId34"/>
-    <hyperlink ref="C53" r:id="rId35"/>
-    <hyperlink ref="C54" r:id="rId36"/>
-    <hyperlink ref="C55" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data(it): UltraGear PLP FAQ Creation ES 완료(09-11) · JP 컬럼 밀림 복구
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -41191,7 +41191,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>JP 완료(2026-09-02) · 사이트 8/10 (80%) · 완료 17 · 법인리뷰 3 · 작업중 0</t>
+          <t>ES 완료(2026-09-11) · 사이트 9/10 (90%) · 완료 18 · 법인리뷰 2 · 작업중 0</t>
         </is>
       </c>
       <c r="D2" s="164" t="n"/>
@@ -41507,17 +41507,21 @@
       </c>
       <c r="D17" s="273" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E17" s="288" t="n"/>
-      <c r="F17" s="270" t="n"/>
+      <c r="F17" s="270" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="G17" s="177" t="n">
         <v>2</v>
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t>evo FAQ 미게시 · Hyper 페이지/FAQ 게시 대기</t>
+          <t>evo·Hyper FAQ 게시 완료</t>
         </is>
       </c>
     </row>
@@ -41651,22 +41655,18 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E22" s="288" t="inlineStr">
+      <c r="E22" s="288" t="n"/>
+      <c r="F22" s="275" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="F22" s="275" t="n">
+      <c r="G22" s="177" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="177" t="inlineStr">
-        <is>
-          <t>미게시(법인리뷰) · STG 경로 기준</t>
-        </is>
-      </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t>페이지/FAQ 게시 대기 (evo·Hyper)</t>
+          <t>evo·Hyper FAQ 게시 완료</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): Smart Monitor Multi AI 잔여 32건 전부 완료 — 21/21 사이트 100%
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>진행 업데이트(2026-09-07) · 사이트 완료 9/21 (43%) · 완료 25 · 작업중 32</t>
+          <t>전체 완료(2026-09-14) · 사이트 완료 21/21 (100%) · 완료 57 · 작업중 0</t>
         </is>
       </c>
     </row>
@@ -17920,16 +17920,20 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E4" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F4" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -17946,16 +17950,20 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E5" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F5" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -17972,16 +17980,20 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E6" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F6" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -17998,16 +18010,20 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E7" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F7" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -18024,16 +18040,20 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E8" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F8" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규 · CMS 라이브 표기였으나 실측 404</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -18050,16 +18070,20 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E9" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F9" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -18076,16 +18100,20 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E10" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="F10" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -18098,16 +18126,20 @@
       <c r="C11" s="0" t="inlineStr"/>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E11" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="F11" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -18120,16 +18152,20 @@
       <c r="C12" s="0" t="inlineStr"/>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E12" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="F12" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -18146,10 +18182,14 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E13" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="F13" s="0" t="n">
         <v>1</v>
       </c>
@@ -18172,10 +18212,14 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E14" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="F14" s="0" t="n">
         <v>1</v>
       </c>
@@ -18198,10 +18242,14 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E15" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="F15" s="0" t="n">
         <v>1</v>
       </c>
@@ -18224,10 +18272,14 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E16" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="F16" s="0" t="n">
         <v>1</v>
       </c>
@@ -18250,10 +18302,14 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E17" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="F17" s="0" t="n">
         <v>1</v>
       </c>
@@ -18276,10 +18332,14 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E18" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="F18" s="0" t="n">
         <v>1</v>
       </c>
@@ -18302,10 +18362,14 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E19" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="F19" s="0" t="n">
         <v>1</v>
       </c>
@@ -18328,10 +18392,14 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E20" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="F20" s="0" t="n">
         <v>1</v>
       </c>
@@ -18384,16 +18452,20 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E22" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="F22" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규 · White</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규 · White</t>
         </is>
       </c>
     </row>
@@ -18410,16 +18482,20 @@
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E23" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="F23" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
+          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -18469,7 +18545,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E25" s="0" t="inlineStr"/>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
       <c r="F25" s="0" t="n">
         <v>1</v>
       </c>
@@ -18492,10 +18572,14 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E26" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="F26" s="0" t="n">
         <v>1</v>
       </c>
@@ -18521,7 +18605,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E27" s="0" t="inlineStr"/>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="F27" s="0" t="n">
         <v>1</v>
       </c>
@@ -18547,7 +18635,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E28" s="0" t="inlineStr"/>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="F28" s="0" t="n">
         <v>1</v>
       </c>
@@ -18633,7 +18725,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E31" s="0" t="inlineStr"/>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
       <c r="F31" s="0" t="n">
         <v>1</v>
       </c>
@@ -18659,7 +18755,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E32" s="0" t="inlineStr"/>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
       <c r="F32" s="0" t="n">
         <v>1</v>
       </c>
@@ -18685,7 +18785,11 @@
           <t>완료</t>
         </is>
       </c>
-      <c r="E33" s="0" t="inlineStr"/>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
       <c r="F33" s="0" t="n">
         <v>1</v>
       </c>
@@ -18888,10 +18992,14 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E40" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="F40" s="0" t="n">
         <v>1</v>
       </c>
@@ -18914,10 +19022,14 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E41" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="F41" s="0" t="n">
         <v>1</v>
       </c>
@@ -18936,16 +19048,20 @@
       <c r="C42" s="0" t="inlineStr"/>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E42" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="F42" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -18962,10 +19078,14 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E43" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="F43" s="0" t="n">
         <v>1</v>
       </c>
@@ -18988,10 +19108,14 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E44" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="F44" s="0" t="n">
         <v>1</v>
       </c>
@@ -19014,10 +19138,14 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E45" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="F45" s="0" t="n">
         <v>1</v>
       </c>
@@ -19040,10 +19168,14 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E46" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="F46" s="0" t="n">
         <v>1</v>
       </c>
@@ -19182,16 +19314,20 @@
       <c r="C51" s="0" t="inlineStr"/>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E51" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="F51" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -19204,16 +19340,20 @@
       <c r="C52" s="0" t="inlineStr"/>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E52" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E52" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="F52" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -19316,16 +19456,20 @@
       <c r="C56" s="0" t="inlineStr"/>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E56" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="F56" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -19398,16 +19542,20 @@
       <c r="C59" s="0" t="inlineStr"/>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E59" s="0" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="F59" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
         </is>
       </c>
     </row>
@@ -19424,16 +19572,20 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E60" s="0" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E60" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="F60" s="0" t="n">
         <v>1</v>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 타겟 보강(2026-09-03) · Black</t>
+          <t>27U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 타겟 보강(2026-09-03) · Black</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): Smart Monitor Multi AI URL 공란 7건 → STG 작업 표기(라이브 미게시 확인)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>전체 완료(2026-09-14) · 사이트 완료 21/21 (100%) · 완료 57 · 작업중 0</t>
+          <t>전체 완료(2026-09-14) · 사이트 완료 21/21 (100%) · 완료 57 · 작업중 0 · STG 작업 7건(라이브 URL 없음)</t>
         </is>
       </c>
     </row>
@@ -18139,7 +18139,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨 · 요청서 미기재 신규</t>
+          <t>[STG 작업] 라이브 미게시 · 32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 요청서 미기재 신규 · 사이트맵·실측 확인(2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -18165,7 +18165,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
+          <t>[STG 작업] 라이브 미게시 · 32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 사이트맵·실측 확인(2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -19061,7 +19061,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
+          <t>[STG 작업] 라이브 미게시 · 27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 사이트맵·실측 확인(2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -19327,7 +19327,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
+          <t>[STG 작업] 라이브 미게시 · 34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 사이트맵·실측 확인(2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -19353,7 +19353,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
+          <t>[STG 작업] 라이브 미게시 · 34U620SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 사이트맵·실측 확인(2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -19469,7 +19469,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
+          <t>[STG 작업] 라이브 미게시 · 27U731SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 사이트맵·실측 확인(2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -19555,7 +19555,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 라이브 게시됨</t>
+          <t>[STG 작업] 라이브 미게시 · 32U701SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · 사이트맵·실측 확인(2026-09-14)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): GNB Structure PTT 0915 반영 — VN 완료, AU 취소(PTT), HU/JP/BG/HR/RS 법인 취소
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -40145,7 +40145,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.13" customWidth="1" style="203" min="1" max="1"/>
@@ -40175,8 +40175,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>IT : 작업중 → 법인리뷰
-SE : 작업중 → 법인리뷰</t>
+          <t>PTT 반영(2026-09-15) · VN 완료(09-10) · AU 취소(PTT) · HU/JP 취소(법인 요청) · BG/HR/RS 취소 신규(법인 요청)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -40274,58 +40273,62 @@
       </c>
       <c r="D10" s="263" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="E10" s="123" t="inlineStr"/>
       <c r="F10" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="0" t="inlineStr"/>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>PTT 7건 전부 취소(2026-09-02)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="261" t="inlineStr">
         <is>
-          <t>BR : BR (pt)</t>
+          <t>BG : BG (bg)</t>
         </is>
       </c>
       <c r="C11" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/br</t>
+          <t>https://www.lg.com/bg</t>
         </is>
       </c>
       <c r="D11" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E11" s="123" t="inlineStr"/>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E11" s="123" t="n"/>
       <c r="F11" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="0" t="inlineStr"/>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>법인 취소 요청(2026-09-15)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="261" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>BR : BR (pt)</t>
         </is>
       </c>
       <c r="C12" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en</t>
-        </is>
-      </c>
-      <c r="D12" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E12" s="123" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
+          <t>https://www.lg.com/br</t>
+        </is>
+      </c>
+      <c r="D12" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E12" s="123" t="inlineStr"/>
       <c r="F12" s="123" t="n">
         <v>1</v>
       </c>
@@ -40334,12 +40337,12 @@
     <row r="13">
       <c r="B13" s="261" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C13" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr</t>
+          <t>https://www.lg.com/ca_en</t>
         </is>
       </c>
       <c r="D13" s="265" t="inlineStr">
@@ -40360,20 +40363,24 @@
     <row r="14">
       <c r="B14" s="261" t="inlineStr">
         <is>
-          <t>CH_DE : CH (de)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C14" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ch_de</t>
-        </is>
-      </c>
-      <c r="D14" s="262" t="inlineStr">
-        <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="E14" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/ca_fr</t>
+        </is>
+      </c>
+      <c r="D14" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" s="123" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="F14" s="123" t="n">
         <v>1</v>
       </c>
@@ -40382,17 +40389,17 @@
     <row r="15">
       <c r="B15" s="261" t="inlineStr">
         <is>
-          <t>CH_FR : CH (fr)</t>
+          <t>CH_DE : CH (de)</t>
         </is>
       </c>
       <c r="C15" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ch_fr</t>
-        </is>
-      </c>
-      <c r="D15" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
+          <t>https://www.lg.com/ch_de</t>
+        </is>
+      </c>
+      <c r="D15" s="262" t="inlineStr">
+        <is>
+          <t>취소</t>
         </is>
       </c>
       <c r="E15" s="123" t="inlineStr"/>
@@ -40404,12 +40411,12 @@
     <row r="16">
       <c r="B16" s="261" t="inlineStr">
         <is>
-          <t>CL : CL (es)</t>
+          <t>CH_FR : CH (fr)</t>
         </is>
       </c>
       <c r="C16" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cl</t>
+          <t>https://www.lg.com/ch_fr</t>
         </is>
       </c>
       <c r="D16" s="264" t="inlineStr">
@@ -40426,12 +40433,12 @@
     <row r="17">
       <c r="B17" s="261" t="inlineStr">
         <is>
-          <t>CO : CO (es)</t>
+          <t>CL : CL (es)</t>
         </is>
       </c>
       <c r="C17" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/co</t>
+          <t>https://www.lg.com/cl</t>
         </is>
       </c>
       <c r="D17" s="264" t="inlineStr">
@@ -40448,24 +40455,20 @@
     <row r="18">
       <c r="B18" s="261" t="inlineStr">
         <is>
-          <t>CZ : CZ (cz)</t>
+          <t>CO : CO (es)</t>
         </is>
       </c>
       <c r="C18" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cz</t>
-        </is>
-      </c>
-      <c r="D18" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E18" s="123" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
+          <t>https://www.lg.com/co</t>
+        </is>
+      </c>
+      <c r="D18" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E18" s="123" t="inlineStr"/>
       <c r="F18" s="123" t="n">
         <v>1</v>
       </c>
@@ -40474,12 +40477,12 @@
     <row r="19">
       <c r="B19" s="261" t="inlineStr">
         <is>
-          <t>DE : DE (de)</t>
+          <t>CZ : CZ (cz)</t>
         </is>
       </c>
       <c r="C19" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de</t>
+          <t>https://www.lg.com/cz</t>
         </is>
       </c>
       <c r="D19" s="265" t="inlineStr">
@@ -40489,7 +40492,7 @@
       </c>
       <c r="E19" s="123" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F19" s="123" t="n">
@@ -40500,20 +40503,24 @@
     <row r="20">
       <c r="B20" s="261" t="inlineStr">
         <is>
-          <t>DK : DK (da)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C20" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/dk</t>
-        </is>
-      </c>
-      <c r="D20" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E20" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/de</t>
+        </is>
+      </c>
+      <c r="D20" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E20" s="123" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
       <c r="F20" s="123" t="n">
         <v>1</v>
       </c>
@@ -40522,12 +40529,12 @@
     <row r="21">
       <c r="B21" s="261" t="inlineStr">
         <is>
-          <t>EG_AR : EG (ar)</t>
+          <t>DK : DK (da)</t>
         </is>
       </c>
       <c r="C21" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/eg_ar</t>
+          <t>https://www.lg.com/dk</t>
         </is>
       </c>
       <c r="D21" s="264" t="inlineStr">
@@ -40544,12 +40551,12 @@
     <row r="22">
       <c r="B22" s="261" t="inlineStr">
         <is>
-          <t>EG_EN : EG (en)</t>
+          <t>EG_AR : EG (ar)</t>
         </is>
       </c>
       <c r="C22" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/eg_en</t>
+          <t>https://www.lg.com/eg_ar</t>
         </is>
       </c>
       <c r="D22" s="264" t="inlineStr">
@@ -40566,24 +40573,20 @@
     <row r="23">
       <c r="B23" s="261" t="inlineStr">
         <is>
-          <t>ES : ES (es)</t>
+          <t>EG_EN : EG (en)</t>
         </is>
       </c>
       <c r="C23" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es</t>
-        </is>
-      </c>
-      <c r="D23" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E23" s="123" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+          <t>https://www.lg.com/eg_en</t>
+        </is>
+      </c>
+      <c r="D23" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E23" s="123" t="inlineStr"/>
       <c r="F23" s="123" t="n">
         <v>1</v>
       </c>
@@ -40592,12 +40595,12 @@
     <row r="24">
       <c r="B24" s="261" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C24" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr</t>
+          <t>https://www.lg.com/es</t>
         </is>
       </c>
       <c r="D24" s="265" t="inlineStr">
@@ -40607,7 +40610,7 @@
       </c>
       <c r="E24" s="123" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="F24" s="123" t="n">
@@ -40618,20 +40621,24 @@
     <row r="25">
       <c r="B25" s="261" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C25" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk</t>
-        </is>
-      </c>
-      <c r="D25" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E25" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/fr</t>
+        </is>
+      </c>
+      <c r="D25" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E25" s="123" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="F25" s="123" t="n">
         <v>1</v>
       </c>
@@ -40640,12 +40647,12 @@
     <row r="26">
       <c r="B26" s="261" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C26" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en</t>
+          <t>https://www.lg.com/hk</t>
         </is>
       </c>
       <c r="D26" s="264" t="inlineStr">
@@ -40662,12 +40669,12 @@
     <row r="27">
       <c r="B27" s="261" t="inlineStr">
         <is>
-          <t>HU : HU (hu)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C27" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hu</t>
+          <t>https://www.lg.com/hk_en</t>
         </is>
       </c>
       <c r="D27" s="264" t="inlineStr">
@@ -40684,65 +40691,69 @@
     <row r="28">
       <c r="B28" s="261" t="inlineStr">
         <is>
-          <t>ID : ID (id)</t>
+          <t>HR : HR (hr)</t>
         </is>
       </c>
       <c r="C28" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/id</t>
+          <t>https://www.lg.com/hr</t>
         </is>
       </c>
       <c r="D28" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E28" s="123" t="inlineStr"/>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E28" s="123" t="n"/>
       <c r="F28" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G28" s="0" t="inlineStr"/>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>법인 취소 요청(2026-09-15)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="261" t="inlineStr">
         <is>
-          <t>IN : IN (en)</t>
+          <t>HU : HU (hu)</t>
         </is>
       </c>
       <c r="C29" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/in</t>
-        </is>
-      </c>
-      <c r="D29" s="263" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E29" s="123" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
+          <t>https://www.lg.com/hu</t>
+        </is>
+      </c>
+      <c r="D29" s="264" t="inlineStr">
+        <is>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E29" s="123" t="inlineStr"/>
       <c r="F29" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="0" t="inlineStr"/>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>법인 취소 요청(2026-09-15)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="261" t="inlineStr">
         <is>
-          <t>IT : IT (it)</t>
+          <t>ID : ID (id)</t>
         </is>
       </c>
       <c r="C30" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/it</t>
+          <t>https://www.lg.com/id</t>
         </is>
       </c>
       <c r="D30" s="264" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E30" s="123" t="inlineStr"/>
@@ -40754,20 +40765,24 @@
     <row r="31">
       <c r="B31" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>IN : IN (en)</t>
         </is>
       </c>
       <c r="C31" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp</t>
+          <t>https://www.lg.com/in</t>
         </is>
       </c>
       <c r="D31" s="263" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E31" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E31" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
       <c r="F31" s="123" t="n">
         <v>1</v>
       </c>
@@ -40776,17 +40791,17 @@
     <row r="32">
       <c r="B32" s="261" t="inlineStr">
         <is>
-          <t>KZ : KZ (ru)</t>
+          <t>IT : IT (it)</t>
         </is>
       </c>
       <c r="C32" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/kz</t>
+          <t>https://www.lg.com/it</t>
         </is>
       </c>
       <c r="D32" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E32" s="123" t="inlineStr"/>
@@ -40798,15 +40813,15 @@
     <row r="33">
       <c r="B33" s="261" t="inlineStr">
         <is>
-          <t>MA : MA (fr)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C33" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ma</t>
-        </is>
-      </c>
-      <c r="D33" s="262" t="inlineStr">
+          <t>https://www.lg.com/jp</t>
+        </is>
+      </c>
+      <c r="D33" s="263" t="inlineStr">
         <is>
           <t>취소</t>
         </is>
@@ -40815,17 +40830,21 @@
       <c r="F33" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="0" t="inlineStr"/>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>법인 취소 요청(2026-09-15)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="261" t="inlineStr">
         <is>
-          <t>MX : MX (es)</t>
+          <t>KZ : KZ (ru)</t>
         </is>
       </c>
       <c r="C34" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/mx</t>
+          <t>https://www.lg.com/kz</t>
         </is>
       </c>
       <c r="D34" s="264" t="inlineStr">
@@ -40842,17 +40861,17 @@
     <row r="35">
       <c r="B35" s="261" t="inlineStr">
         <is>
-          <t>MY : MY (en)</t>
+          <t>MA : MA (fr)</t>
         </is>
       </c>
       <c r="C35" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/my</t>
-        </is>
-      </c>
-      <c r="D35" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
+          <t>https://www.lg.com/ma</t>
+        </is>
+      </c>
+      <c r="D35" s="262" t="inlineStr">
+        <is>
+          <t>취소</t>
         </is>
       </c>
       <c r="E35" s="123" t="inlineStr"/>
@@ -40864,24 +40883,20 @@
     <row r="36">
       <c r="B36" s="261" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
+          <t>MX : MX (es)</t>
         </is>
       </c>
       <c r="C36" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nl</t>
-        </is>
-      </c>
-      <c r="D36" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E36" s="123" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
+          <t>https://www.lg.com/mx</t>
+        </is>
+      </c>
+      <c r="D36" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E36" s="123" t="inlineStr"/>
       <c r="F36" s="123" t="n">
         <v>1</v>
       </c>
@@ -40890,12 +40905,12 @@
     <row r="37">
       <c r="B37" s="261" t="inlineStr">
         <is>
-          <t>NZ : NZ (en)</t>
+          <t>MY : MY (en)</t>
         </is>
       </c>
       <c r="C37" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nz</t>
+          <t>https://www.lg.com/my</t>
         </is>
       </c>
       <c r="D37" s="264" t="inlineStr">
@@ -40912,20 +40927,24 @@
     <row r="38">
       <c r="B38" s="261" t="inlineStr">
         <is>
-          <t>PA : PA (es)</t>
+          <t>NL : NL (nl)</t>
         </is>
       </c>
       <c r="C38" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pa</t>
-        </is>
-      </c>
-      <c r="D38" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E38" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/nl</t>
+        </is>
+      </c>
+      <c r="D38" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E38" s="123" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="F38" s="123" t="n">
         <v>1</v>
       </c>
@@ -40934,12 +40953,12 @@
     <row r="39">
       <c r="B39" s="261" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>NZ : NZ (en)</t>
         </is>
       </c>
       <c r="C39" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe</t>
+          <t>https://www.lg.com/nz</t>
         </is>
       </c>
       <c r="D39" s="264" t="inlineStr">
@@ -40951,17 +40970,21 @@
       <c r="F39" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G39" s="0" t="inlineStr"/>
+      <c r="G39" s="0" t="inlineStr">
+        <is>
+          <t>PTT 7건 중 3건 취소(09-14 · Hyper/Professional/Swing PLP) · 4건 WB 신규 요청</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="261" t="inlineStr">
         <is>
-          <t>PH : PH (en)</t>
+          <t>PA : PA (es)</t>
         </is>
       </c>
       <c r="C40" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ph</t>
+          <t>https://www.lg.com/pa</t>
         </is>
       </c>
       <c r="D40" s="264" t="inlineStr">
@@ -40978,12 +41001,12 @@
     <row r="41">
       <c r="B41" s="261" t="inlineStr">
         <is>
-          <t>PL : PL (pl)</t>
+          <t>PE : PE (es)</t>
         </is>
       </c>
       <c r="C41" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pl</t>
+          <t>https://www.lg.com/pe</t>
         </is>
       </c>
       <c r="D41" s="264" t="inlineStr">
@@ -41000,12 +41023,12 @@
     <row r="42">
       <c r="B42" s="261" t="inlineStr">
         <is>
-          <t>PT : PT (pt)</t>
+          <t>PH : PH (en)</t>
         </is>
       </c>
       <c r="C42" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pt</t>
+          <t>https://www.lg.com/ph</t>
         </is>
       </c>
       <c r="D42" s="264" t="inlineStr">
@@ -41022,22 +41045,20 @@
     <row r="43">
       <c r="B43" s="261" t="inlineStr">
         <is>
-          <t>SA_AR : SA (ar)</t>
+          <t>PL : PL (pl)</t>
         </is>
       </c>
       <c r="C43" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa</t>
-        </is>
-      </c>
-      <c r="D43" s="263" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E43" s="200" t="n">
-        <v>46246</v>
-      </c>
+          <t>https://www.lg.com/pl</t>
+        </is>
+      </c>
+      <c r="D43" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E43" s="123" t="inlineStr"/>
       <c r="F43" s="123" t="n">
         <v>1</v>
       </c>
@@ -41046,22 +41067,20 @@
     <row r="44">
       <c r="B44" s="261" t="inlineStr">
         <is>
-          <t>SA_EN : SA (en)</t>
+          <t>PT : PT (pt)</t>
         </is>
       </c>
       <c r="C44" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa_en</t>
-        </is>
-      </c>
-      <c r="D44" s="263" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E44" s="200" t="n">
-        <v>46246</v>
-      </c>
+          <t>https://www.lg.com/pt</t>
+        </is>
+      </c>
+      <c r="D44" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E44" s="123" t="inlineStr"/>
       <c r="F44" s="123" t="n">
         <v>1</v>
       </c>
@@ -41070,42 +41089,48 @@
     <row r="45">
       <c r="B45" s="261" t="inlineStr">
         <is>
-          <t>SE : SE (sv)</t>
+          <t>RS : RS (sr)</t>
         </is>
       </c>
       <c r="C45" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/se</t>
-        </is>
-      </c>
-      <c r="D45" s="264" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E45" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/rs</t>
+        </is>
+      </c>
+      <c r="D45" s="263" t="inlineStr">
+        <is>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E45" s="200" t="n"/>
       <c r="F45" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G45" s="0" t="inlineStr"/>
+      <c r="G45" s="0" t="inlineStr">
+        <is>
+          <t>법인 취소 요청(2026-09-15)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="261" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>SA_AR : SA (ar)</t>
         </is>
       </c>
       <c r="C46" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg</t>
-        </is>
-      </c>
-      <c r="D46" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E46" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/sa</t>
+        </is>
+      </c>
+      <c r="D46" s="263" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E46" s="200" t="n">
+        <v>46246</v>
+      </c>
       <c r="F46" s="123" t="n">
         <v>1</v>
       </c>
@@ -41114,20 +41139,22 @@
     <row r="47">
       <c r="B47" s="261" t="inlineStr">
         <is>
-          <t>TH : TH (th)</t>
+          <t>SA_EN : SA (en)</t>
         </is>
       </c>
       <c r="C47" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/th</t>
-        </is>
-      </c>
-      <c r="D47" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E47" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/sa_en</t>
+        </is>
+      </c>
+      <c r="D47" s="263" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E47" s="200" t="n">
+        <v>46246</v>
+      </c>
       <c r="F47" s="123" t="n">
         <v>1</v>
       </c>
@@ -41136,42 +41163,34 @@
     <row r="48">
       <c r="B48" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>SE : SE (sv)</t>
         </is>
       </c>
       <c r="C48" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr</t>
+          <t>https://www.lg.com/se</t>
         </is>
       </c>
       <c r="D48" s="264" t="inlineStr">
         <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E48" s="123" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E48" s="123" t="inlineStr"/>
       <c r="F48" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G48" s="0" t="inlineStr">
-        <is>
-          <t>7건 중 6건 게시완료 · 1건 Final Live Check 잔여</t>
-        </is>
-      </c>
+      <c r="G48" s="0" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="B49" s="261" t="inlineStr">
         <is>
-          <t>TW : TW (zh)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C49" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tw</t>
+          <t>https://www.lg.com/sg</t>
         </is>
       </c>
       <c r="D49" s="264" t="inlineStr">
@@ -41188,24 +41207,20 @@
     <row r="50">
       <c r="B50" s="261" t="inlineStr">
         <is>
-          <t>UK : GB (en)</t>
+          <t>TH : TH (th)</t>
         </is>
       </c>
       <c r="C50" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk</t>
-        </is>
-      </c>
-      <c r="D50" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E50" s="123" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+          <t>https://www.lg.com/th</t>
+        </is>
+      </c>
+      <c r="D50" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E50" s="123" t="inlineStr"/>
       <c r="F50" s="123" t="n">
         <v>1</v>
       </c>
@@ -41214,34 +41229,42 @@
     <row r="51">
       <c r="B51" s="261" t="inlineStr">
         <is>
-          <t>VN : VN (vi)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C51" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/vn</t>
+          <t>https://www.lg.com/tr</t>
         </is>
       </c>
       <c r="D51" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E51" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E51" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="F51" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G51" s="0" t="inlineStr"/>
+      <c r="G51" s="0" t="inlineStr">
+        <is>
+          <t>7건 중 6건 게시완료 · 1건 Final Live Check 잔여</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="261" t="inlineStr">
         <is>
-          <t>ZA : ZA (en)</t>
+          <t>TW : TW (zh)</t>
         </is>
       </c>
       <c r="C52" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/za</t>
+          <t>https://www.lg.com/tw</t>
         </is>
       </c>
       <c r="D52" s="264" t="inlineStr">
@@ -41254,6 +41277,88 @@
         <v>1</v>
       </c>
       <c r="G52" s="0" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="261" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C53" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk</t>
+        </is>
+      </c>
+      <c r="D53" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E53" s="123" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F53" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="0" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="B54" s="261" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C54" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn</t>
+        </is>
+      </c>
+      <c r="D54" s="264" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E54" s="123" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="F54" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="0" t="inlineStr">
+        <is>
+          <t>7건 중 6건 게시완료(09-10) · Hyper Mini LED PLP 1건 취소(08-31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="261" t="inlineStr">
+        <is>
+          <t>ZA : ZA (en)</t>
+        </is>
+      </c>
+      <c r="C55" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/za</t>
+        </is>
+      </c>
+      <c r="D55" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E55" s="123" t="inlineStr"/>
+      <c r="F55" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>7건 중 1건 게시(07-27 · GNB 수정) · UltraGear evo PLP QA 리뷰 · 5건 WB 신규</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -41301,6 +41406,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data(it): GR Remark의 PTT 표현을 법인으로 통일
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -2986,6 +2986,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -3574,6 +3575,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -5564,6 +5566,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -7493,6 +7496,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -18435,7 +18439,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시 · 요청서 미기재 신규</t>
+          <t>24U511SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(법인) · 라이브 미게시 · 요청서 미기재 신규</t>
         </is>
       </c>
     </row>
@@ -19499,7 +19503,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U501SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -19529,7 +19533,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U721SB · Multi AI 컴포넌트 → AI Search 컴포넌트 교체 (PDP · Gallery Image) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -20370,7 +20374,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>27GX704A-B · Hexagon Lighting 삭제 에셋으로 교체 (PDP) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>27GX704A-B · Hexagon Lighting 삭제 에셋으로 교체 (PDP) · STG 준비(법인) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
@@ -21228,7 +21232,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>27GX704A-B · Hexagon Lighting 삭제 에셋으로 교체 (PDP) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27GX704A-B · Hexagon Lighting 삭제 에셋으로 교체 (PDP) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -21280,7 +21284,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>27GX704A-B · Hexagon Lighting 삭제 에셋으로 교체 (PDP) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27GX704A-B · Hexagon Lighting 삭제 에셋으로 교체 (PDP) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -35189,7 +35193,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -35241,7 +35245,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>32G620B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>32G620B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
@@ -35263,7 +35267,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>27G64NA · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27G64NA · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -35315,7 +35319,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>32G403B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32G403B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -35389,7 +35393,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>27GX790B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>27GX790B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
@@ -35411,7 +35415,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -36013,7 +36017,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>24G414B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>24G414B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -36323,7 +36327,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>27GX790B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>27GX790B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
@@ -36345,7 +36349,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -36367,7 +36371,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -36755,7 +36759,7 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -36777,7 +36781,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>32G620B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>32G620B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
@@ -37069,7 +37073,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37151,7 +37155,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>27GX790B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>27GX790B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
@@ -37173,7 +37177,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>27GX790B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>27GX790B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
@@ -37195,7 +37199,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>32G620B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
+          <t>32G620B-B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시 · CMS 라이브 표기였으나 실측 404</t>
         </is>
       </c>
     </row>
@@ -37307,7 +37311,7 @@
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37509,7 +37513,7 @@
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37535,7 @@
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37643,7 +37647,7 @@
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27GX790B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37665,7 +37669,7 @@
       </c>
       <c r="G95" s="0" t="inlineStr">
         <is>
-          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32G620B · 모델별 변경사항 적용 (PDP · 유첨 PPT 참조) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37844,7 +37848,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
         </is>
       </c>
     </row>
@@ -37866,7 +37870,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37888,7 +37892,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37910,7 +37914,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37962,7 +37966,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -37984,7 +37988,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38182,7 +38186,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38204,7 +38208,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시(CMS 라이브 표기였으나 실측 404)</t>
         </is>
       </c>
     </row>
@@ -38316,7 +38320,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38338,7 +38342,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38420,7 +38424,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38442,7 +38446,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38464,7 +38468,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38486,7 +38490,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38508,7 +38512,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38530,7 +38534,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38552,7 +38556,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38604,7 +38608,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38966,7 +38970,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -38988,7 +38992,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39010,7 +39014,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39032,7 +39036,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39144,7 +39148,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39196,7 +39200,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U700B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39248,7 +39252,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>32U701B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39386,7 +39390,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39408,7 +39412,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U711B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39430,7 +39434,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39512,7 +39516,7 @@
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U710B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39534,7 +39538,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(PTT) · 라이브 미게시</t>
+          <t>27U730B · MIC 문구 삭제 (Preview / Feature Card / USP Gallery) · STG 준비(법인) · 라이브 미게시</t>
         </is>
       </c>
     </row>
@@ -39658,6 +39662,7 @@
       <c r="G5" s="127" t="n"/>
     </row>
     <row r="6" ht="40.5" customHeight="1" s="203"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
@@ -40175,7 +40180,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>PTT 반영(2026-09-15) · VN 완료(09-10) · AU 취소(PTT) · HU/JP 취소(법인 요청) · BG/HR/RS 취소 신규(법인 요청)</t>
+          <t>법인 현황 반영(2026-09-15) · VN 완료(09-10) · AU 취소(법인) · HU/JP 취소(법인 요청) · BG/HR/RS 취소 신규(법인 요청)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -40282,7 +40287,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>PTT 7건 전부 취소(2026-09-02)</t>
+          <t>법인 7건 전부 취소(2026-09-02)</t>
         </is>
       </c>
     </row>
@@ -40972,7 +40977,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>PTT 7건 중 3건 취소(09-14 · Hyper/Professional/Swing PLP) · 4건 WB 신규 요청</t>
+          <t>법인 7건 중 3건 취소(09-14 · Hyper/Professional/Swing PLP) · 4건 신규 요청</t>
         </is>
       </c>
     </row>
@@ -41356,7 +41361,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>7건 중 1건 게시(07-27 · GNB 수정) · UltraGear evo PLP QA 리뷰 · 5건 WB 신규</t>
+          <t>7건 중 1건 게시(07-27 · GNB 수정) · UltraGear evo PLP QA 리뷰 · 5건 신규 요청</t>
         </is>
       </c>
     </row>
@@ -41466,6 +41471,10 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -42920,6 +42929,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -44183,6 +44193,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -44745,6 +44756,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>

</xml_diff>

<commit_message>
data(it): GNB Remark 건수 표기 제거
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -2986,7 +2986,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -3575,7 +3574,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -5566,7 +5564,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -7496,7 +7493,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -39662,7 +39658,6 @@
       <c r="G5" s="127" t="n"/>
     </row>
     <row r="6" ht="40.5" customHeight="1" s="203"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
@@ -40287,7 +40282,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>법인 7건 전부 취소(2026-09-02)</t>
+          <t>법인 취소(2026-09-02)</t>
         </is>
       </c>
     </row>
@@ -40977,7 +40972,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>법인 7건 중 3건 취소(09-14 · Hyper/Professional/Swing PLP) · 4건 신규 요청</t>
+          <t>Hyper/Professional/Swing PLP 취소(09-14) · 나머지 신규 요청</t>
         </is>
       </c>
     </row>
@@ -41257,7 +41252,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>7건 중 6건 게시완료 · 1건 Final Live Check 잔여</t>
+          <t>게시완료 · Final Live Check 잔여</t>
         </is>
       </c>
     </row>
@@ -41335,7 +41330,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>7건 중 6건 게시완료(09-10) · Hyper Mini LED PLP 1건 취소(08-31)</t>
+          <t>게시완료(09-10) · Hyper Mini LED PLP 취소(08-31)</t>
         </is>
       </c>
     </row>
@@ -41361,7 +41356,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>7건 중 1건 게시(07-27 · GNB 수정) · UltraGear evo PLP QA 리뷰 · 5건 신규 요청</t>
+          <t>GNB 수정 게시(07-27) · UltraGear evo PLP QA 리뷰 · 나머지 신규 요청</t>
         </is>
       </c>
     </row>
@@ -41471,10 +41466,6 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -42929,7 +42920,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -44193,7 +44183,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -44756,7 +44745,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat(it): ?task= 딥링크 — xlsx 탭 이름 매칭·?task=npi 시 NPI 탭 표시 (v0.6.84) + GNB CH_FR 취소
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -40175,7 +40175,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>법인 현황 반영(2026-09-15) · VN 완료(09-10) · AU 취소(법인) · HU/JP 취소(법인 요청) · BG/HR/RS 취소 신규(법인 요청)</t>
+          <t>법인 현황 반영(2026-09-15) · VN 완료(09-10) · AU 취소(법인) · HU/JP 취소(법인 요청) · BG/HR/RS 취소 신규(법인 요청) · CH_FR 취소(법인 요청, 09-16)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -40421,14 +40421,18 @@
       </c>
       <c r="D16" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E16" s="123" t="inlineStr"/>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E16" s="123" t="n"/>
       <c r="F16" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="0" t="inlineStr"/>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>법인 취소 요청(2026-09-16)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="261" t="inlineStr">

</xml_diff>

<commit_message>
data(it): W38 gram pro gallery 이미지 교체 등록 — 작업중 41건 · 4모델 × 10개국
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -27,6 +27,7 @@
     <sheet name="W32 - Digital Trends Award 삭제" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="W32 - UltraGear PDP 5모델" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="W32 - UltraFine PDP MIC 삭제" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="W38 - gram pro gallery" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,7 +39,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="70">
+  <fonts count="72">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -405,6 +406,15 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -627,7 +637,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="68" fillId="0" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="295">
+  <cellXfs count="297">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1211,6 +1221,8 @@
     <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -39581,6 +39593,1199 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" style="203" min="1" max="1"/>
+    <col width="13" customWidth="1" style="203" min="2" max="2"/>
+    <col width="13" customWidth="1" style="203" min="3" max="3"/>
+    <col width="13" customWidth="1" style="203" min="4" max="4"/>
+    <col width="13" customWidth="1" style="203" min="5" max="5"/>
+    <col width="13" customWidth="1" style="203" min="6" max="6"/>
+    <col width="13" customWidth="1" style="203" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="295" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="295" t="inlineStr">
+        <is>
+          <t>GR26-W38-MS-IT gram pro gallery 이미지 교체</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="295" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" s="295" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · 작업중 41건 · 4모델 × 10개국 (라이브 URL 41건 실측 200)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="296" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" s="296" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" s="296" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" s="296" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" s="296" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" s="296" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" s="296" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="295" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C4" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/16z90u-g-au75ap/</t>
+        </is>
+      </c>
+      <c r="D4" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E4" s="295" t="n"/>
+      <c r="F4" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-G.AU75AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="295" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C5" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/16z90u-g-au88ap/</t>
+        </is>
+      </c>
+      <c r="D5" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E5" s="295" t="n"/>
+      <c r="F5" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-G.AU88AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="295" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C6" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal87c</t>
+        </is>
+      </c>
+      <c r="D6" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E6" s="295" t="n"/>
+      <c r="F6" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-G.AL87C</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="295" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C7" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal88c</t>
+        </is>
+      </c>
+      <c r="D7" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E7" s="295" t="n"/>
+      <c r="F7" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-G.AL88C</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="295" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C8" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb7c</t>
+        </is>
+      </c>
+      <c r="D8" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E8" s="295" t="n"/>
+      <c r="F8" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.ALB7C</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="295" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C9" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb8c</t>
+        </is>
+      </c>
+      <c r="D9" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E9" s="295" t="n"/>
+      <c r="F9" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.ALB8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="295" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C10" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb9c</t>
+        </is>
+      </c>
+      <c r="D10" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E10" s="295" t="n"/>
+      <c r="F10" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.ALB9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="295" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C11" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram-pro/16z90u-g-au78gn/</t>
+        </is>
+      </c>
+      <c r="D11" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E11" s="295" t="n"/>
+      <c r="F11" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-G.AU78GN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="295" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C12" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/16z90u/</t>
+        </is>
+      </c>
+      <c r="D12" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E12" s="295" t="n"/>
+      <c r="F12" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.AUA8GN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="295" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C13" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aua5a3/</t>
+        </is>
+      </c>
+      <c r="D13" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E13" s="295" t="n"/>
+      <c r="F13" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.AUA5A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="295" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C14" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aub5a3/</t>
+        </is>
+      </c>
+      <c r="D14" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E14" s="295" t="n"/>
+      <c r="F14" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.AUB5A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="295" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C15" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aub9a3/</t>
+        </is>
+      </c>
+      <c r="D15" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E15" s="295" t="n"/>
+      <c r="F15" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.AUB9A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="295" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C16" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90u-k-azb5a3/</t>
+        </is>
+      </c>
+      <c r="D16" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E16" s="295" t="n"/>
+      <c r="F16" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.AZB5A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="295" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C17" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/laptops/gram-pro/16z90u-h-au78an/</t>
+        </is>
+      </c>
+      <c r="D17" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E17" s="295" t="n"/>
+      <c r="F17" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-H.AU78AN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="295" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C18" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/laptops/gram-pro/16z90u-k-aub8an/</t>
+        </is>
+      </c>
+      <c r="D18" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E18" s="295" t="n"/>
+      <c r="F18" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-K.AUB8AN</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="295" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C19" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/16z90u-g-16gb/</t>
+        </is>
+      </c>
+      <c r="D19" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E19" s="295" t="n"/>
+      <c r="F19" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-G.AN55A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="295" t="inlineStr">
+        <is>
+          <t>VN : VN (vi)</t>
+        </is>
+      </c>
+      <c r="C20" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/16z90u-g-32gb/</t>
+        </is>
+      </c>
+      <c r="D20" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E20" s="295" t="n"/>
+      <c r="F20" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="295" t="inlineStr">
+        <is>
+          <t>16Z90U-G.AV85A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="295" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C21" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au75ap/</t>
+        </is>
+      </c>
+      <c r="D21" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E21" s="295" t="n"/>
+      <c r="F21" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU75AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="295" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C22" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au78ap/</t>
+        </is>
+      </c>
+      <c r="D22" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E22" s="295" t="n"/>
+      <c r="F22" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU78AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="295" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C23" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au88ap/</t>
+        </is>
+      </c>
+      <c r="D23" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E23" s="295" t="n"/>
+      <c r="F23" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU88AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="295" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C24" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/business/monitors-pcs/laptops/gram-pro/17z90u-g/</t>
+        </is>
+      </c>
+      <c r="D24" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E24" s="295" t="n"/>
+      <c r="F24" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU78A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="295" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C25" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g78/</t>
+        </is>
+      </c>
+      <c r="D25" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E25" s="295" t="n"/>
+      <c r="F25" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU78A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="295" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C26" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g88/</t>
+        </is>
+      </c>
+      <c r="D26" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E26" s="295" t="n"/>
+      <c r="F26" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU88A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="295" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C27" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/business/moniteurs-et-pc/ordinateurs-portables/gram-pro/17z90u-g/</t>
+        </is>
+      </c>
+      <c r="D27" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E27" s="295" t="n"/>
+      <c r="F27" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU88A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="295" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C28" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g78/</t>
+        </is>
+      </c>
+      <c r="D28" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E28" s="295" t="n"/>
+      <c r="F28" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU78A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="295" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C29" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g88/</t>
+        </is>
+      </c>
+      <c r="D29" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E29" s="295" t="n"/>
+      <c r="F29" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU88A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="295" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C30" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-17z90u-al87c</t>
+        </is>
+      </c>
+      <c r="D30" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E30" s="295" t="n"/>
+      <c r="F30" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AL87C</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="295" t="inlineStr">
+        <is>
+          <t>CN : CN (zh)</t>
+        </is>
+      </c>
+      <c r="C31" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/lg-17z90u-gal88c</t>
+        </is>
+      </c>
+      <c r="D31" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E31" s="295" t="n"/>
+      <c r="F31" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AL88C</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="295" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C32" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram-pro/17z90u-g-au78gn/</t>
+        </is>
+      </c>
+      <c r="D32" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E32" s="295" t="n"/>
+      <c r="F32" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU78GN</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="295" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C33" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram-pro/17z90u-g-au8bgn/</t>
+        </is>
+      </c>
+      <c r="D33" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E33" s="295" t="n"/>
+      <c r="F33" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU8BGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="295" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C34" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90u/</t>
+        </is>
+      </c>
+      <c r="D34" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E34" s="295" t="n"/>
+      <c r="F34" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU88AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="295" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C35" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/gram-pro/17z90u-g-au78dn/</t>
+        </is>
+      </c>
+      <c r="D35" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E35" s="295" t="n"/>
+      <c r="F35" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU78DN</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="295" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C36" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/gram/17z90u-g-au85a3/</t>
+        </is>
+      </c>
+      <c r="D36" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E36" s="295" t="n"/>
+      <c r="F36" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU85A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="295" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C37" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/laptops/gram-pro/17z90u-g-au78an/</t>
+        </is>
+      </c>
+      <c r="D37" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E37" s="295" t="n"/>
+      <c r="F37" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="295" t="inlineStr">
+        <is>
+          <t>17Z90U-G.AU78AN</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="295" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C38" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ur-p/</t>
+        </is>
+      </c>
+      <c r="D38" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E38" s="295" t="n"/>
+      <c r="F38" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="295" t="inlineStr">
+        <is>
+          <t>17Z90UR-P.AU9CA9</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="295" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C39" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17Z90ur-p/</t>
+        </is>
+      </c>
+      <c r="D39" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E39" s="295" t="n"/>
+      <c r="F39" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="295" t="inlineStr">
+        <is>
+          <t>17Z90UR-P.AU9CA9</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="295" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C40" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90ur/</t>
+        </is>
+      </c>
+      <c r="D40" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E40" s="295" t="n"/>
+      <c r="F40" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="295" t="inlineStr">
+        <is>
+          <t>17Z90UR-P.AU99U3</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="295" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C41" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ub-h/</t>
+        </is>
+      </c>
+      <c r="D41" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E41" s="295" t="n"/>
+      <c r="F41" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="295" t="inlineStr">
+        <is>
+          <t>17Z90UB-H.AU89A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="295" t="inlineStr">
+        <is>
+          <t>CA_FR : CA (fr)</t>
+        </is>
+      </c>
+      <c r="C42" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90ub-h/</t>
+        </is>
+      </c>
+      <c r="D42" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E42" s="295" t="n"/>
+      <c r="F42" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="295" t="inlineStr">
+        <is>
+          <t>17Z90UB-H.AU89A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="295" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C43" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90ub/</t>
+        </is>
+      </c>
+      <c r="D43" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E43" s="295" t="n"/>
+      <c r="F43" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="295" t="inlineStr">
+        <is>
+          <t>17Z90UB-H.AU99AN</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="295" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C44" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/gram-pro/17z90ub-h-au79dn/</t>
+        </is>
+      </c>
+      <c r="D44" s="295" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E44" s="295" t="n"/>
+      <c r="F44" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="295" t="inlineStr">
+        <is>
+          <t>17Z90UB-H.AU79DN</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId41"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
data(it): Windows 11 Landing 주차 W31 제거 — 제목 주차 비움
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -20,7 +20,7 @@
     <sheet name="W30 - SmartMonitor ScreenShare" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="W30 - UltraGear 1000Hz FAQ" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="W31 - Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="W31 - PDP Gallery Win11 Pro" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="W31 - Smart Monitor Multi AI" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="W32 - UltraGear 27GX704A" sheetId="21" state="visible" r:id="rId21"/>
@@ -14296,7 +14296,7 @@
       </c>
       <c r="B1" s="0" t="inlineStr">
         <is>
-          <t>GR26-W31-MS-IT Windows 11 Home Landing Page 업데이트</t>
+          <t>GR26-MS-IT Windows 11 Home Landing Page 업데이트</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): W38 gram pro gallery 목록을 29건으로 갱신
CN을 빼고 요청 29행(4모델 × 9개국)으로 맞추며, 라이브 URL 29건은 실측 200이다.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -39599,7 +39599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="203" min="1" max="1"/>
@@ -39631,7 +39631,7 @@
       </c>
       <c r="B2" s="295" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · 작업중 41건 · 4모델 × 10개국 (라이브 URL 41건 실측 200)</t>
+          <t>목록 갱신 · 작업중 29건 · 4모델 × 9개국 (CN 제외) · 라이브 URL 29건 실측 200</t>
         </is>
       </c>
     </row>
@@ -39727,12 +39727,12 @@
     <row r="6">
       <c r="B6" s="295" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C6" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal87c</t>
+          <t>https://www.lg.com/de/notebooks/gram-pro/16z90u-g-au78gn/</t>
         </is>
       </c>
       <c r="D6" s="295" t="inlineStr">
@@ -39746,19 +39746,19 @@
       </c>
       <c r="G6" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-G.AL87C</t>
+          <t>16Z90U-G.AU78GN</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="295" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C7" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-gal88c</t>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aua5a3/</t>
         </is>
       </c>
       <c r="D7" s="295" t="inlineStr">
@@ -39772,19 +39772,19 @@
       </c>
       <c r="G7" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-G.AL88C</t>
+          <t>16Z90U-K.AUA5A3</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="295" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C8" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb7c</t>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aub5a3/</t>
         </is>
       </c>
       <c r="D8" s="295" t="inlineStr">
@@ -39798,19 +39798,19 @@
       </c>
       <c r="G8" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.ALB7C</t>
+          <t>16Z90U-K.AUB5A3</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="295" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C9" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb8c</t>
+          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aub9a3/</t>
         </is>
       </c>
       <c r="D9" s="295" t="inlineStr">
@@ -39824,19 +39824,19 @@
       </c>
       <c r="G9" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.ALB8C</t>
+          <t>16Z90U-K.AUB9A3</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="295" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C10" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-16z90u-kalb9c</t>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90u-k-azb5a3/</t>
         </is>
       </c>
       <c r="D10" s="295" t="inlineStr">
@@ -39850,19 +39850,19 @@
       </c>
       <c r="G10" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.ALB9C</t>
+          <t>16Z90U-K.AZB5A3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="295" t="inlineStr">
         <is>
-          <t>DE : DE (de)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C11" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de/notebooks/gram-pro/16z90u-g-au78gn/</t>
+          <t>https://www.lg.com/uk/laptops/gram-pro/16z90u-h-au78an/</t>
         </is>
       </c>
       <c r="D11" s="295" t="inlineStr">
@@ -39876,19 +39876,19 @@
       </c>
       <c r="G11" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-G.AU78GN</t>
+          <t>16Z90U-H.AU78AN</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="295" t="inlineStr">
         <is>
-          <t>GLOBAL : GLOBAL (en)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C12" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/16z90u/</t>
+          <t>https://www.lg.com/uk/laptops/gram-pro/16z90u-k-aub8an/</t>
         </is>
       </c>
       <c r="D12" s="295" t="inlineStr">
@@ -39902,19 +39902,19 @@
       </c>
       <c r="G12" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.AUA8GN</t>
+          <t>16Z90U-K.AUB8AN</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="295" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>VN : VN (vi)</t>
         </is>
       </c>
       <c r="C13" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aua5a3/</t>
+          <t>https://www.lg.com/vn/laptop-lg-gram/16z90u-g-16gb/</t>
         </is>
       </c>
       <c r="D13" s="295" t="inlineStr">
@@ -39928,19 +39928,19 @@
       </c>
       <c r="G13" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.AUA5A3</t>
+          <t>16Z90U-G.AN55A5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="295" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>VN : VN (vi)</t>
         </is>
       </c>
       <c r="C14" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aub5a3/</t>
+          <t>https://www.lg.com/vn/laptop-lg-gram/16z90u-g-32gb/</t>
         </is>
       </c>
       <c r="D14" s="295" t="inlineStr">
@@ -39954,19 +39954,19 @@
       </c>
       <c r="G14" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.AUB5A3</t>
+          <t>16Z90U-G.AV85A5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="295" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>AU : AU (en)</t>
         </is>
       </c>
       <c r="C15" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/laptops/gram-pro/16z90u-k-aub9a3/</t>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au75ap/</t>
         </is>
       </c>
       <c r="D15" s="295" t="inlineStr">
@@ -39980,19 +39980,19 @@
       </c>
       <c r="G15" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.AUB9A3</t>
+          <t>17Z90U-G.AU75AP</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="295" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>AU : AU (en)</t>
         </is>
       </c>
       <c r="C16" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90u-k-azb5a3/</t>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au78ap/</t>
         </is>
       </c>
       <c r="D16" s="295" t="inlineStr">
@@ -40006,19 +40006,19 @@
       </c>
       <c r="G16" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.AZB5A3</t>
+          <t>17Z90U-G.AU78AP</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="295" t="inlineStr">
         <is>
-          <t>UK : GB (en)</t>
+          <t>AU : AU (en)</t>
         </is>
       </c>
       <c r="C17" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/laptops/gram-pro/16z90u-h-au78an/</t>
+          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au88ap/</t>
         </is>
       </c>
       <c r="D17" s="295" t="inlineStr">
@@ -40032,19 +40032,19 @@
       </c>
       <c r="G17" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-H.AU78AN</t>
+          <t>17Z90U-G.AU88AP</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="295" t="inlineStr">
         <is>
-          <t>UK : GB (en)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C18" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/uk/laptops/gram-pro/16z90u-k-aub8an/</t>
+          <t>https://www.lg.com/ca_en/business/monitors-pcs/laptops/gram-pro/17z90u-g/</t>
         </is>
       </c>
       <c r="D18" s="295" t="inlineStr">
@@ -40058,19 +40058,19 @@
       </c>
       <c r="G18" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-K.AUB8AN</t>
+          <t>17Z90U-G.AU78A9</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="295" t="inlineStr">
         <is>
-          <t>VN : VN (vi)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C19" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/vn/laptop-lg-gram/16z90u-g-16gb/</t>
+          <t>https://www.lg.com/ca_fr/business/moniteurs-et-pc/ordinateurs-portables/gram-pro/17z90u-g/</t>
         </is>
       </c>
       <c r="D19" s="295" t="inlineStr">
@@ -40084,19 +40084,19 @@
       </c>
       <c r="G19" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-G.AN55A5</t>
+          <t>17Z90U-G.AU88A9</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="295" t="inlineStr">
         <is>
-          <t>VN : VN (vi)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C20" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/vn/laptop-lg-gram/16z90u-g-32gb/</t>
+          <t>https://www.lg.com/de/notebooks/gram-pro/17z90u-g-au78gn/</t>
         </is>
       </c>
       <c r="D20" s="295" t="inlineStr">
@@ -40110,19 +40110,19 @@
       </c>
       <c r="G20" s="295" t="inlineStr">
         <is>
-          <t>16Z90U-G.AV85A5</t>
+          <t>17Z90U-G.AU78GN</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="295" t="inlineStr">
         <is>
-          <t>AU : AU (en)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C21" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au75ap/</t>
+          <t>https://www.lg.com/de/notebooks/gram-pro/17z90u-g-au8bgn/</t>
         </is>
       </c>
       <c r="D21" s="295" t="inlineStr">
@@ -40136,19 +40136,19 @@
       </c>
       <c r="G21" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU75AP</t>
+          <t>17Z90U-G.AU8BGN</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="295" t="inlineStr">
         <is>
-          <t>AU : AU (en)</t>
+          <t>GLOBAL : GLOBAL (en)</t>
         </is>
       </c>
       <c r="C22" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au78ap/</t>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90u/</t>
         </is>
       </c>
       <c r="D22" s="295" t="inlineStr">
@@ -40162,19 +40162,19 @@
       </c>
       <c r="G22" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU78AP</t>
+          <t>17Z90U-G.AU88AP</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="295" t="inlineStr">
         <is>
-          <t>AU : AU (en)</t>
+          <t>IT : IT (it)</t>
         </is>
       </c>
       <c r="C23" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/au/laptops/gram-pro/17z90u-g-au88ap/</t>
+          <t>https://www.lg.com/it/notebook/gram-pro/17z90u-g-au78dn/</t>
         </is>
       </c>
       <c r="D23" s="295" t="inlineStr">
@@ -40188,19 +40188,19 @@
       </c>
       <c r="G23" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU88AP</t>
+          <t>17Z90U-G.AU78DN</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="295" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C24" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/business/monitors-pcs/laptops/gram-pro/17z90u-g/</t>
+          <t>https://www.lg.com/sg/laptops/gram/17z90u-g-au85a3/</t>
         </is>
       </c>
       <c r="D24" s="295" t="inlineStr">
@@ -40214,19 +40214,19 @@
       </c>
       <c r="G24" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU78A9</t>
+          <t>17Z90U-G.AU85A3</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="295" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C25" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g78/</t>
+          <t>https://www.lg.com/uk/laptops/gram-pro/17z90u-g-au78an/</t>
         </is>
       </c>
       <c r="D25" s="295" t="inlineStr">
@@ -40240,7 +40240,7 @@
       </c>
       <c r="G25" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU78A9</t>
+          <t>17Z90U-G.AU78AN</t>
         </is>
       </c>
     </row>
@@ -40252,7 +40252,7 @@
       </c>
       <c r="C26" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90u-g88/</t>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ur-p/</t>
         </is>
       </c>
       <c r="D26" s="295" t="inlineStr">
@@ -40266,7 +40266,7 @@
       </c>
       <c r="G26" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU88A9</t>
+          <t>17Z90UR-P.AU9CA9</t>
         </is>
       </c>
     </row>
@@ -40278,7 +40278,7 @@
       </c>
       <c r="C27" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/business/moniteurs-et-pc/ordinateurs-portables/gram-pro/17z90u-g/</t>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17Z90ur-p/</t>
         </is>
       </c>
       <c r="D27" s="295" t="inlineStr">
@@ -40292,19 +40292,19 @@
       </c>
       <c r="G27" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU88A9</t>
+          <t>17Z90UR-P.AU9CA9</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="295" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>GLOBAL : GLOBAL (en)</t>
         </is>
       </c>
       <c r="C28" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g78/</t>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90ur/</t>
         </is>
       </c>
       <c r="D28" s="295" t="inlineStr">
@@ -40318,19 +40318,19 @@
       </c>
       <c r="G28" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU78A9</t>
+          <t>17Z90UR-P.AU99U3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="295" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C29" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90u-g88/</t>
+          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ub-h/</t>
         </is>
       </c>
       <c r="D29" s="295" t="inlineStr">
@@ -40344,19 +40344,19 @@
       </c>
       <c r="G29" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AU88A9</t>
+          <t>17Z90UB-H.AU89A9</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="295" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C30" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-17z90u-al87c</t>
+          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90ub-h/</t>
         </is>
       </c>
       <c r="D30" s="295" t="inlineStr">
@@ -40370,19 +40370,19 @@
       </c>
       <c r="G30" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AL87C</t>
+          <t>17Z90UB-H.AU89A9</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="295" t="inlineStr">
         <is>
-          <t>CN : CN (zh)</t>
+          <t>GLOBAL : GLOBAL (en)</t>
         </is>
       </c>
       <c r="C31" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cn/notebooks/lg-17z90u-gal88c</t>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90ub/</t>
         </is>
       </c>
       <c r="D31" s="295" t="inlineStr">
@@ -40396,19 +40396,19 @@
       </c>
       <c r="G31" s="295" t="inlineStr">
         <is>
-          <t>17Z90U-G.AL88C</t>
+          <t>17Z90UB-H.AU99AN</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="295" t="inlineStr">
         <is>
-          <t>DE : DE (de)</t>
+          <t>IT : IT (it)</t>
         </is>
       </c>
       <c r="C32" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de/notebooks/gram-pro/17z90u-g-au78gn/</t>
+          <t>https://www.lg.com/it/notebook/gram-pro/17z90ub-h-au79dn/</t>
         </is>
       </c>
       <c r="D32" s="295" t="inlineStr">
@@ -40421,318 +40421,6 @@
         <v>1</v>
       </c>
       <c r="G32" s="295" t="inlineStr">
-        <is>
-          <t>17Z90U-G.AU78GN</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="295" t="inlineStr">
-        <is>
-          <t>DE : DE (de)</t>
-        </is>
-      </c>
-      <c r="C33" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/de/notebooks/gram-pro/17z90u-g-au8bgn/</t>
-        </is>
-      </c>
-      <c r="D33" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E33" s="295" t="n"/>
-      <c r="F33" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="295" t="inlineStr">
-        <is>
-          <t>17Z90U-G.AU8BGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="295" t="inlineStr">
-        <is>
-          <t>GLOBAL : GLOBAL (en)</t>
-        </is>
-      </c>
-      <c r="C34" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90u/</t>
-        </is>
-      </c>
-      <c r="D34" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E34" s="295" t="n"/>
-      <c r="F34" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="295" t="inlineStr">
-        <is>
-          <t>17Z90U-G.AU88AP</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="295" t="inlineStr">
-        <is>
-          <t>IT : IT (it)</t>
-        </is>
-      </c>
-      <c r="C35" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/it/notebook/gram-pro/17z90u-g-au78dn/</t>
-        </is>
-      </c>
-      <c r="D35" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E35" s="295" t="n"/>
-      <c r="F35" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="295" t="inlineStr">
-        <is>
-          <t>17Z90U-G.AU78DN</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="295" t="inlineStr">
-        <is>
-          <t>SG : SG (en)</t>
-        </is>
-      </c>
-      <c r="C36" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/sg/laptops/gram/17z90u-g-au85a3/</t>
-        </is>
-      </c>
-      <c r="D36" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E36" s="295" t="n"/>
-      <c r="F36" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="295" t="inlineStr">
-        <is>
-          <t>17Z90U-G.AU85A3</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="295" t="inlineStr">
-        <is>
-          <t>UK : GB (en)</t>
-        </is>
-      </c>
-      <c r="C37" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/uk/laptops/gram-pro/17z90u-g-au78an/</t>
-        </is>
-      </c>
-      <c r="D37" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E37" s="295" t="n"/>
-      <c r="F37" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="295" t="inlineStr">
-        <is>
-          <t>17Z90U-G.AU78AN</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="295" t="inlineStr">
-        <is>
-          <t>CA_EN : CA (en)</t>
-        </is>
-      </c>
-      <c r="C38" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ur-p/</t>
-        </is>
-      </c>
-      <c r="D38" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E38" s="295" t="n"/>
-      <c r="F38" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="295" t="inlineStr">
-        <is>
-          <t>17Z90UR-P.AU9CA9</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="295" t="inlineStr">
-        <is>
-          <t>CA_FR : CA (fr)</t>
-        </is>
-      </c>
-      <c r="C39" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17Z90ur-p/</t>
-        </is>
-      </c>
-      <c r="D39" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E39" s="295" t="n"/>
-      <c r="F39" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="295" t="inlineStr">
-        <is>
-          <t>17Z90UR-P.AU9CA9</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="295" t="inlineStr">
-        <is>
-          <t>GLOBAL : GLOBAL (en)</t>
-        </is>
-      </c>
-      <c r="C40" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90ur/</t>
-        </is>
-      </c>
-      <c r="D40" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E40" s="295" t="n"/>
-      <c r="F40" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="295" t="inlineStr">
-        <is>
-          <t>17Z90UR-P.AU99U3</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="295" t="inlineStr">
-        <is>
-          <t>CA_EN : CA (en)</t>
-        </is>
-      </c>
-      <c r="C41" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/laptops/all-laptops/17z90ub-h/</t>
-        </is>
-      </c>
-      <c r="D41" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E41" s="295" t="n"/>
-      <c r="F41" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="295" t="inlineStr">
-        <is>
-          <t>17Z90UB-H.AU89A9</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="295" t="inlineStr">
-        <is>
-          <t>CA_FR : CA (fr)</t>
-        </is>
-      </c>
-      <c r="C42" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_fr/computing/purchase-guide/laptops/17z90ub-h/</t>
-        </is>
-      </c>
-      <c r="D42" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E42" s="295" t="n"/>
-      <c r="F42" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="295" t="inlineStr">
-        <is>
-          <t>17Z90UB-H.AU89A9</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="295" t="inlineStr">
-        <is>
-          <t>GLOBAL : GLOBAL (en)</t>
-        </is>
-      </c>
-      <c r="C43" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/17z90ub/</t>
-        </is>
-      </c>
-      <c r="D43" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E43" s="295" t="n"/>
-      <c r="F43" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="295" t="inlineStr">
-        <is>
-          <t>17Z90UB-H.AU99AN</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="295" t="inlineStr">
-        <is>
-          <t>IT : IT (it)</t>
-        </is>
-      </c>
-      <c r="C44" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/it/notebook/gram-pro/17z90ub-h-au79dn/</t>
-        </is>
-      </c>
-      <c r="D44" s="295" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E44" s="295" t="n"/>
-      <c r="F44" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="295" t="inlineStr">
         <is>
           <t>17Z90UB-H.AU79DN</t>
         </is>
@@ -40769,18 +40457,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data(it): gram pro gallery 이미지 교체 29건을 완료로 변경
GR26-W38 시트의 작업중 행을 모두 완료로 두고, 완료일은 2026-09-22로 적는다.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -2998,6 +2998,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -3586,6 +3587,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -5576,6 +5578,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -7505,6 +7508,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -39631,7 +39635,7 @@
       </c>
       <c r="B2" s="295" t="inlineStr">
         <is>
-          <t>목록 갱신 · 작업중 29건 · 4모델 × 9개국 (CN 제외) · 라이브 URL 29건 실측 200</t>
+          <t>전건 완료 — gram pro gallery 이미지 교체 29건 · 4모델 × 9개국 (CN 제외)</t>
         </is>
       </c>
     </row>
@@ -39685,10 +39689,14 @@
       </c>
       <c r="D4" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E4" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E4" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F4" s="295" t="n">
         <v>1</v>
       </c>
@@ -39711,10 +39719,14 @@
       </c>
       <c r="D5" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E5" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E5" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F5" s="295" t="n">
         <v>1</v>
       </c>
@@ -39737,10 +39749,14 @@
       </c>
       <c r="D6" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E6" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E6" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F6" s="295" t="n">
         <v>1</v>
       </c>
@@ -39763,10 +39779,14 @@
       </c>
       <c r="D7" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E7" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E7" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F7" s="295" t="n">
         <v>1</v>
       </c>
@@ -39789,10 +39809,14 @@
       </c>
       <c r="D8" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E8" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E8" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F8" s="295" t="n">
         <v>1</v>
       </c>
@@ -39815,10 +39839,14 @@
       </c>
       <c r="D9" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E9" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E9" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F9" s="295" t="n">
         <v>1</v>
       </c>
@@ -39841,10 +39869,14 @@
       </c>
       <c r="D10" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E10" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F10" s="295" t="n">
         <v>1</v>
       </c>
@@ -39867,10 +39899,14 @@
       </c>
       <c r="D11" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E11" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F11" s="295" t="n">
         <v>1</v>
       </c>
@@ -39893,10 +39929,14 @@
       </c>
       <c r="D12" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E12" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F12" s="295" t="n">
         <v>1</v>
       </c>
@@ -39919,10 +39959,14 @@
       </c>
       <c r="D13" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E13" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F13" s="295" t="n">
         <v>1</v>
       </c>
@@ -39945,10 +39989,14 @@
       </c>
       <c r="D14" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E14" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F14" s="295" t="n">
         <v>1</v>
       </c>
@@ -39971,10 +40019,14 @@
       </c>
       <c r="D15" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E15" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E15" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F15" s="295" t="n">
         <v>1</v>
       </c>
@@ -39997,10 +40049,14 @@
       </c>
       <c r="D16" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E16" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F16" s="295" t="n">
         <v>1</v>
       </c>
@@ -40023,10 +40079,14 @@
       </c>
       <c r="D17" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E17" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E17" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F17" s="295" t="n">
         <v>1</v>
       </c>
@@ -40049,10 +40109,14 @@
       </c>
       <c r="D18" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E18" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E18" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F18" s="295" t="n">
         <v>1</v>
       </c>
@@ -40075,10 +40139,14 @@
       </c>
       <c r="D19" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E19" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E19" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F19" s="295" t="n">
         <v>1</v>
       </c>
@@ -40101,10 +40169,14 @@
       </c>
       <c r="D20" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E20" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E20" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F20" s="295" t="n">
         <v>1</v>
       </c>
@@ -40127,10 +40199,14 @@
       </c>
       <c r="D21" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E21" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E21" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F21" s="295" t="n">
         <v>1</v>
       </c>
@@ -40153,10 +40229,14 @@
       </c>
       <c r="D22" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E22" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E22" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F22" s="295" t="n">
         <v>1</v>
       </c>
@@ -40179,10 +40259,14 @@
       </c>
       <c r="D23" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E23" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E23" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F23" s="295" t="n">
         <v>1</v>
       </c>
@@ -40205,10 +40289,14 @@
       </c>
       <c r="D24" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E24" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E24" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F24" s="295" t="n">
         <v>1</v>
       </c>
@@ -40231,10 +40319,14 @@
       </c>
       <c r="D25" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E25" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E25" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F25" s="295" t="n">
         <v>1</v>
       </c>
@@ -40257,10 +40349,14 @@
       </c>
       <c r="D26" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E26" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E26" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F26" s="295" t="n">
         <v>1</v>
       </c>
@@ -40283,10 +40379,14 @@
       </c>
       <c r="D27" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E27" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E27" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F27" s="295" t="n">
         <v>1</v>
       </c>
@@ -40309,10 +40409,14 @@
       </c>
       <c r="D28" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E28" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E28" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F28" s="295" t="n">
         <v>1</v>
       </c>
@@ -40335,10 +40439,14 @@
       </c>
       <c r="D29" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E29" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E29" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F29" s="295" t="n">
         <v>1</v>
       </c>
@@ -40361,10 +40469,14 @@
       </c>
       <c r="D30" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E30" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E30" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F30" s="295" t="n">
         <v>1</v>
       </c>
@@ -40387,10 +40499,14 @@
       </c>
       <c r="D31" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E31" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E31" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F31" s="295" t="n">
         <v>1</v>
       </c>
@@ -40413,10 +40529,14 @@
       </c>
       <c r="D32" s="295" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E32" s="295" t="n"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E32" s="295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F32" s="295" t="n">
         <v>1</v>
       </c>
@@ -40539,6 +40659,7 @@
       <c r="G5" s="127" t="n"/>
     </row>
     <row r="6" ht="40.5" customHeight="1" s="203"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
@@ -42351,6 +42472,10 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -43805,6 +43930,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -45068,6 +45194,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -45630,6 +45757,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>

</xml_diff>

<commit_message>
data(it): W41 UltraGear Buying Guide 2차 등록 — 1차와 동일 44개국 사전검토
BE-fr는 1차 URL이 최종 404(10/06 실측)라 URL을 비우고 비고에 표기.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -1,33 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W16 - CineBeam S PDP Video Upda" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W16 - Copilot+ Filter Creation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W16 - Microsoft PDP Gallery Car" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W17 - GNB Structure" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W18 - FAQ Request (UltraGear PL" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W18 - UltraGear OLED FAQ Update" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W22 - UltraGear Buying Guide" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W23 - 27GM950B-B 갤러리 이미지 교체" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W23 - 39GX950B 이미지 수정 2차" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W23 - 52G930B Feature 수정 건" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W23 - UL인증 feature 삭제 1차" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W25 - Copilot+ Hero Banner" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W28 - AI Upscaling Disclaimer" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W28 - UL Verified Eye Comfort" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W30 - SmartMonitor ScreenShare" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W30 - UltraGear 1000Hz FAQ" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W31 - PDP Gallery Win11 Pro" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W31 - Smart Monitor Multi AI" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W32 - UltraGear 27GX704A" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W32 - Digital Trends Award 삭제" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W32 - UltraGear PDP 5모델" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W32 - UltraFine PDP MIC 삭제" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W38 - gram pro gallery" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="W16 - CineBeam S PDP Video Upda" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="W16 - Copilot+ Filter Creation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="W16 - Microsoft PDP Gallery Car" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="W17 - GNB Structure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="W18 - FAQ Request (UltraGear PL" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="W18 - UltraGear OLED FAQ Update" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="W22 - UltraGear Buying Guide" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="W23 - 27GM950B-B 갤러리 이미지 교체" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="W23 - 39GX950B 이미지 수정 2차" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="W23 - 52G930B Feature 수정 건" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="W23 - UL인증 feature 삭제 1차" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="W25 - Copilot+ Hero Banner" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="W28 - AI Upscaling Disclaimer" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="W28 - UL Verified Eye Comfort" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="W30 - SmartMonitor ScreenShare" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="W30 - UltraGear 1000Hz FAQ" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="W31 - PDP Gallery Win11 Pro" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="W31 - Smart Monitor Multi AI" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="W32 - UltraGear 27GX704A" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="W32 - Digital Trends Award 삭제" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="W32 - UltraGear PDP 5모델" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="W32 - UltraFine PDP MIC 삭제" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="W38 - gram pro gallery" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="W41 - UltraGear Buying Guide 2차" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40578,6 +40579,1063 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G52"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="166" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="163" t="inlineStr">
+        <is>
+          <t>GR26-W41-MS-IT UltraGear Buying Guide 2차 Update</t>
+        </is>
+      </c>
+      <c r="C1" s="164" t="n"/>
+      <c r="D1" s="164" t="n"/>
+      <c r="E1" s="165" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" s="163" t="inlineStr">
+        <is>
+          <t>금주 신규 등록 · 1차(W22)와 동일 44개국 대상 2차 업데이트 · 담당 정알찬 책임</t>
+        </is>
+      </c>
+      <c r="C2" s="164" t="n"/>
+      <c r="D2" s="164" t="n"/>
+      <c r="E2" s="165" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="166" t="n"/>
+      <c r="B3" s="163" t="n"/>
+      <c r="C3" s="164" t="n"/>
+      <c r="D3" s="164" t="n"/>
+      <c r="E3" s="165" t="n"/>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="127" t="n"/>
+      <c r="B5" s="127" t="n"/>
+      <c r="C5" s="127" t="n"/>
+      <c r="D5" s="127" t="n"/>
+      <c r="E5" s="127" t="n"/>
+    </row>
+    <row r="6">
+      <c r="E6" s="127" t="n"/>
+    </row>
+    <row r="7">
+      <c r="E7" s="127" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="276" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B8" s="276" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C8" s="276" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D8" s="276" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E8" s="276" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F8" s="276" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G8" s="276" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" s="203">
+      <c r="B9" s="261" t="inlineStr">
+        <is>
+          <t>AE-ar</t>
+        </is>
+      </c>
+      <c r="C9" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ae_ar/it-products/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D9" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E9" s="123" t="n"/>
+      <c r="F9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="261" t="inlineStr">
+        <is>
+          <t>BD-en</t>
+        </is>
+      </c>
+      <c r="C10" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/bd/ultragear-gaming-buying-guide</t>
+        </is>
+      </c>
+      <c r="D10" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E10" s="123" t="n"/>
+      <c r="F10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="261" t="inlineStr">
+        <is>
+          <t>BE-fr</t>
+        </is>
+      </c>
+      <c r="C11" s="290" t="n"/>
+      <c r="D11" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E11" s="123" t="n"/>
+      <c r="F11" s="0" t="n"/>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>1차 URL 최종 404(10/06 실측) · 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="261" t="inlineStr">
+        <is>
+          <t>BR-pt</t>
+        </is>
+      </c>
+      <c r="C12" s="277" t="inlineStr"/>
+      <c r="D12" s="264" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E12" s="123" t="n"/>
+      <c r="F12" s="0" t="inlineStr"/>
+      <c r="G12" s="0" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="261" t="inlineStr">
+        <is>
+          <t>CAC-es</t>
+        </is>
+      </c>
+      <c r="C13" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/computacion/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D13" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E13" s="123" t="n"/>
+      <c r="F13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="261" t="inlineStr">
+        <is>
+          <t>CA-en</t>
+        </is>
+      </c>
+      <c r="C14" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D14" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E14" s="123" t="n"/>
+      <c r="F14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="261" t="inlineStr">
+        <is>
+          <t>CA-fr</t>
+        </is>
+      </c>
+      <c r="C15" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D15" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E15" s="123" t="n"/>
+      <c r="F15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="0" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="261" t="inlineStr">
+        <is>
+          <t>CN-zh</t>
+        </is>
+      </c>
+      <c r="C16" s="277" t="inlineStr"/>
+      <c r="D16" s="263" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E16" s="123" t="n"/>
+      <c r="F16" s="0" t="inlineStr"/>
+      <c r="G16" s="0" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="261" t="inlineStr">
+        <is>
+          <t>CO-es</t>
+        </is>
+      </c>
+      <c r="C17" s="277" t="inlineStr"/>
+      <c r="D17" s="264" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E17" s="123" t="n"/>
+      <c r="F17" s="0" t="inlineStr"/>
+      <c r="G17" s="0" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="261" t="inlineStr">
+        <is>
+          <t>CZ-cz</t>
+        </is>
+      </c>
+      <c r="C18" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D18" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E18" s="123" t="n"/>
+      <c r="F18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="261" t="inlineStr">
+        <is>
+          <t>DK-da</t>
+        </is>
+      </c>
+      <c r="C19" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/dk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D19" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E19" s="123" t="n"/>
+      <c r="F19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="0" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="261" t="inlineStr">
+        <is>
+          <t>EC-es</t>
+        </is>
+      </c>
+      <c r="C20" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ec/computacion/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D20" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E20" s="123" t="n"/>
+      <c r="F20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="0" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="261" t="inlineStr">
+        <is>
+          <t>EE-ee</t>
+        </is>
+      </c>
+      <c r="C21" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/it-seadmed/buying-guide/ultragear-mangumonitorid</t>
+        </is>
+      </c>
+      <c r="D21" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E21" s="123" t="n"/>
+      <c r="F21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="0" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="261" t="inlineStr">
+        <is>
+          <t>ES-es</t>
+        </is>
+      </c>
+      <c r="C22" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D22" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E22" s="123" t="n"/>
+      <c r="F22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="0" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="261" t="inlineStr">
+        <is>
+          <t>FI-fi</t>
+        </is>
+      </c>
+      <c r="C23" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fi/it-tuotteet/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D23" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E23" s="123" t="n"/>
+      <c r="F23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="0" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="261" t="inlineStr">
+        <is>
+          <t>FR-fr</t>
+        </is>
+      </c>
+      <c r="C24" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/moniteurs/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D24" s="263" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E24" s="123" t="n"/>
+      <c r="F24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="0" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="261" t="inlineStr">
+        <is>
+          <t>GR-gr</t>
+        </is>
+      </c>
+      <c r="C25" s="277" t="inlineStr"/>
+      <c r="D25" s="264" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E25" s="123" t="n"/>
+      <c r="F25" s="0" t="inlineStr"/>
+      <c r="G25" s="0" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="261" t="inlineStr">
+        <is>
+          <t>HK-zh</t>
+        </is>
+      </c>
+      <c r="C26" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D26" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E26" s="123" t="n"/>
+      <c r="F26" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="0" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="261" t="inlineStr">
+        <is>
+          <t>HK-en</t>
+        </is>
+      </c>
+      <c r="C27" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hk_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D27" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E27" s="123" t="n"/>
+      <c r="F27" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="0" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="261" t="inlineStr">
+        <is>
+          <t>HU-hu</t>
+        </is>
+      </c>
+      <c r="C28" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hu/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D28" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E28" s="123" t="n"/>
+      <c r="F28" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="0" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="261" t="inlineStr">
+        <is>
+          <t>ID-id</t>
+        </is>
+      </c>
+      <c r="C29" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/id/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D29" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E29" s="123" t="n"/>
+      <c r="F29" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="0" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="261" t="inlineStr">
+        <is>
+          <t>IL-he</t>
+        </is>
+      </c>
+      <c r="C30" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/il/monitors/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D30" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E30" s="123" t="n"/>
+      <c r="F30" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="0" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="261" t="inlineStr">
+        <is>
+          <t>IN-en</t>
+        </is>
+      </c>
+      <c r="C31" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D31" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E31" s="123" t="n"/>
+      <c r="F31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="0" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="261" t="inlineStr">
+        <is>
+          <t>IT-it</t>
+        </is>
+      </c>
+      <c r="C32" s="277" t="inlineStr"/>
+      <c r="D32" s="264" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E32" s="123" t="n"/>
+      <c r="F32" s="0" t="inlineStr"/>
+      <c r="G32" s="0" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="261" t="inlineStr">
+        <is>
+          <t>JP-ja</t>
+        </is>
+      </c>
+      <c r="C33" s="277" t="inlineStr"/>
+      <c r="D33" s="263" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E33" s="123" t="n"/>
+      <c r="F33" s="0" t="inlineStr"/>
+      <c r="G33" s="0" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="261" t="inlineStr">
+        <is>
+          <t>KZ-ru</t>
+        </is>
+      </c>
+      <c r="C34" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/kz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D34" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E34" s="123" t="n"/>
+      <c r="F34" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="0" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="261" t="inlineStr">
+        <is>
+          <t>LT-lt</t>
+        </is>
+      </c>
+      <c r="C35" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/kompiuterine-technika/buying-guide/ultragear-gaming-monitor</t>
+        </is>
+      </c>
+      <c r="D35" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E35" s="123" t="n"/>
+      <c r="F35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="0" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="261" t="inlineStr">
+        <is>
+          <t>LV-lv</t>
+        </is>
+      </c>
+      <c r="C36" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/datortehnika/buying-guide/ultragear-gaming-monitor</t>
+        </is>
+      </c>
+      <c r="D36" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E36" s="123" t="n"/>
+      <c r="F36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="0" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="261" t="inlineStr">
+        <is>
+          <t>NL-nl</t>
+        </is>
+      </c>
+      <c r="C37" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/nl/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D37" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E37" s="123" t="n"/>
+      <c r="F37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="0" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="261" t="inlineStr">
+        <is>
+          <t>NO-no</t>
+        </is>
+      </c>
+      <c r="C38" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/no/it-produkter/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D38" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E38" s="123" t="n"/>
+      <c r="F38" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="0" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="261" t="inlineStr">
+        <is>
+          <t>PA-es</t>
+        </is>
+      </c>
+      <c r="C39" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D39" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E39" s="123" t="n"/>
+      <c r="F39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="0" t="n"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="261" t="inlineStr">
+        <is>
+          <t>PE-es</t>
+        </is>
+      </c>
+      <c r="C40" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/pe/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D40" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E40" s="123" t="n"/>
+      <c r="F40" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="0" t="n"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="261" t="inlineStr">
+        <is>
+          <t>PH-en</t>
+        </is>
+      </c>
+      <c r="C41" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ph/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D41" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E41" s="123" t="n"/>
+      <c r="F41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="0" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="261" t="inlineStr">
+        <is>
+          <t>PL-pl</t>
+        </is>
+      </c>
+      <c r="C42" s="277" t="inlineStr"/>
+      <c r="D42" s="264" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E42" s="123" t="n"/>
+      <c r="F42" s="0" t="inlineStr"/>
+      <c r="G42" s="0" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="261" t="inlineStr">
+        <is>
+          <t>PT-pt</t>
+        </is>
+      </c>
+      <c r="C43" s="277" t="inlineStr"/>
+      <c r="D43" s="264" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E43" s="123" t="n"/>
+      <c r="F43" s="0" t="inlineStr"/>
+      <c r="G43" s="0" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="261" t="inlineStr">
+        <is>
+          <t>RS-rs</t>
+        </is>
+      </c>
+      <c r="C44" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/rs/it-proizvodi/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D44" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E44" s="123" t="n"/>
+      <c r="F44" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="0" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="261" t="inlineStr">
+        <is>
+          <t>SA-ar</t>
+        </is>
+      </c>
+      <c r="C45" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D45" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E45" s="123" t="n"/>
+      <c r="F45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="0" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="261" t="inlineStr">
+        <is>
+          <t>SA-en</t>
+        </is>
+      </c>
+      <c r="C46" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D46" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E46" s="123" t="n"/>
+      <c r="F46" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="0" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="261" t="inlineStr">
+        <is>
+          <t>SE-sv</t>
+        </is>
+      </c>
+      <c r="C47" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D47" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E47" s="123" t="n"/>
+      <c r="F47" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="0" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="261" t="inlineStr">
+        <is>
+          <t>TH-th</t>
+        </is>
+      </c>
+      <c r="C48" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/th/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D48" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E48" s="123" t="n"/>
+      <c r="F48" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="0" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="261" t="inlineStr">
+        <is>
+          <t>TR-tr</t>
+        </is>
+      </c>
+      <c r="C49" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D49" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E49" s="123" t="n"/>
+      <c r="F49" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="0" t="n"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="261" t="inlineStr">
+        <is>
+          <t>TW-zh</t>
+        </is>
+      </c>
+      <c r="C50" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D50" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E50" s="123" t="n"/>
+      <c r="F50" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="0" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="261" t="inlineStr">
+        <is>
+          <t>UA-uk</t>
+        </is>
+      </c>
+      <c r="C51" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ua/it-products/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D51" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E51" s="123" t="n"/>
+      <c r="F51" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="0" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="261" t="inlineStr">
+        <is>
+          <t>ZA-en</t>
+        </is>
+      </c>
+      <c r="C52" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/za/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D52" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E52" s="123" t="n"/>
+      <c r="F52" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="0" t="n"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId35"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
data(it): GNB 대상 외 5.0 국가(BG·HR·RS) 행 삭제 — 47→44 사이트
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -40625,7 +40625,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -42413,7 +42412,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.13" customWidth="1" style="203" min="1" max="1"/>
@@ -42557,68 +42556,68 @@
     <row r="11">
       <c r="B11" s="261" t="inlineStr">
         <is>
-          <t>BG : BG (bg)</t>
+          <t>BR : BR (pt)</t>
         </is>
       </c>
       <c r="C11" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/bg</t>
+          <t>https://www.lg.com/br</t>
         </is>
       </c>
       <c r="D11" s="264" t="inlineStr">
         <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="E11" s="123" t="n"/>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E11" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="F11" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>법인 취소 요청(2026-09-15)</t>
+          <t>예상 2026-10-23 · 프로덕션 반영됨</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="261" t="inlineStr">
         <is>
-          <t>BR : BR (pt)</t>
+          <t>CA_EN : CA (en)</t>
         </is>
       </c>
       <c r="C12" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/br</t>
-        </is>
-      </c>
-      <c r="D12" s="264" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
+          <t>https://www.lg.com/ca_en</t>
+        </is>
+      </c>
+      <c r="D12" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="E12" s="123" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="F12" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="0" t="inlineStr">
-        <is>
-          <t>예상 2026-10-23 · 프로덕션 반영됨</t>
-        </is>
-      </c>
+      <c r="G12" s="0" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="261" t="inlineStr">
         <is>
-          <t>CA_EN : CA (en)</t>
+          <t>CA_FR : CA (fr)</t>
         </is>
       </c>
       <c r="C13" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_en</t>
+          <t>https://www.lg.com/ca_fr</t>
         </is>
       </c>
       <c r="D13" s="265" t="inlineStr">
@@ -42639,24 +42638,20 @@
     <row r="14">
       <c r="B14" s="261" t="inlineStr">
         <is>
-          <t>CA_FR : CA (fr)</t>
+          <t>CH_DE : CH (de)</t>
         </is>
       </c>
       <c r="C14" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ca_fr</t>
-        </is>
-      </c>
-      <c r="D14" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E14" s="123" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
+          <t>https://www.lg.com/ch_de</t>
+        </is>
+      </c>
+      <c r="D14" s="262" t="inlineStr">
+        <is>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E14" s="123" t="inlineStr"/>
       <c r="F14" s="123" t="n">
         <v>1</v>
       </c>
@@ -42665,65 +42660,73 @@
     <row r="15">
       <c r="B15" s="261" t="inlineStr">
         <is>
-          <t>CH_DE : CH (de)</t>
+          <t>CH_FR : CH (fr)</t>
         </is>
       </c>
       <c r="C15" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ch_de</t>
-        </is>
-      </c>
-      <c r="D15" s="262" t="inlineStr">
+          <t>https://www.lg.com/ch_fr</t>
+        </is>
+      </c>
+      <c r="D15" s="264" t="inlineStr">
         <is>
           <t>취소</t>
         </is>
       </c>
-      <c r="E15" s="123" t="inlineStr"/>
+      <c r="E15" s="123" t="n"/>
       <c r="F15" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="0" t="inlineStr"/>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>법인 취소 요청(2026-09-16)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="261" t="inlineStr">
         <is>
-          <t>CH_FR : CH (fr)</t>
+          <t>CL : CL (es)</t>
         </is>
       </c>
       <c r="C16" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ch_fr</t>
+          <t>https://www.lg.com/cl</t>
         </is>
       </c>
       <c r="D16" s="264" t="inlineStr">
         <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="E16" s="123" t="n"/>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E16" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="F16" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>법인 취소 요청(2026-09-16)</t>
+          <t>예상 2026-10-23</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="261" t="inlineStr">
         <is>
-          <t>CL : CL (es)</t>
+          <t>CO : CO (es)</t>
         </is>
       </c>
       <c r="C17" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cl</t>
+          <t>https://www.lg.com/co</t>
         </is>
       </c>
       <c r="D17" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E17" s="123" t="inlineStr">
@@ -42736,49 +42739,45 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-23</t>
+          <t>예상 2026-10-23 · 프로덕션 반영됨</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="261" t="inlineStr">
         <is>
-          <t>CO : CO (es)</t>
+          <t>CZ : CZ (cz)</t>
         </is>
       </c>
       <c r="C18" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/co</t>
-        </is>
-      </c>
-      <c r="D18" s="264" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
+          <t>https://www.lg.com/cz</t>
+        </is>
+      </c>
+      <c r="D18" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="E18" s="123" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F18" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="0" t="inlineStr">
-        <is>
-          <t>예상 2026-10-23 · 프로덕션 반영됨</t>
-        </is>
-      </c>
+      <c r="G18" s="0" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="B19" s="261" t="inlineStr">
         <is>
-          <t>CZ : CZ (cz)</t>
+          <t>DE : DE (de)</t>
         </is>
       </c>
       <c r="C19" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cz</t>
+          <t>https://www.lg.com/de</t>
         </is>
       </c>
       <c r="D19" s="265" t="inlineStr">
@@ -42788,7 +42787,7 @@
       </c>
       <c r="E19" s="123" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="F19" s="123" t="n">
@@ -42799,38 +42798,42 @@
     <row r="20">
       <c r="B20" s="261" t="inlineStr">
         <is>
-          <t>DE : DE (de)</t>
+          <t>DK : DK (da)</t>
         </is>
       </c>
       <c r="C20" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/de</t>
-        </is>
-      </c>
-      <c r="D20" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>https://www.lg.com/dk</t>
+        </is>
+      </c>
+      <c r="D20" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E20" s="123" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="F20" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="0" t="inlineStr"/>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>예상 2026-10-16</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="261" t="inlineStr">
         <is>
-          <t>DK : DK (da)</t>
+          <t>EG_AR : EG (ar)</t>
         </is>
       </c>
       <c r="C21" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/dk</t>
+          <t>https://www.lg.com/eg_ar</t>
         </is>
       </c>
       <c r="D21" s="264" t="inlineStr">
@@ -42840,7 +42843,7 @@
       </c>
       <c r="E21" s="123" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F21" s="123" t="n">
@@ -42848,19 +42851,19 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-16</t>
+          <t>예상 2026-10-02 · LDM 회신 대기, 09/30 무응답 시 취소</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="261" t="inlineStr">
         <is>
-          <t>EG_AR : EG (ar)</t>
+          <t>EG_EN : EG (en)</t>
         </is>
       </c>
       <c r="C22" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/eg_ar</t>
+          <t>https://www.lg.com/eg_en</t>
         </is>
       </c>
       <c r="D22" s="264" t="inlineStr">
@@ -42885,42 +42888,38 @@
     <row r="23">
       <c r="B23" s="261" t="inlineStr">
         <is>
-          <t>EG_EN : EG (en)</t>
+          <t>ES : ES (es)</t>
         </is>
       </c>
       <c r="C23" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/eg_en</t>
-        </is>
-      </c>
-      <c r="D23" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
+          <t>https://www.lg.com/es</t>
+        </is>
+      </c>
+      <c r="D23" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="E23" s="123" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="F23" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="0" t="inlineStr">
-        <is>
-          <t>예상 2026-10-02 · LDM 회신 대기, 09/30 무응답 시 취소</t>
-        </is>
-      </c>
+      <c r="G23" s="0" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="B24" s="261" t="inlineStr">
         <is>
-          <t>ES : ES (es)</t>
+          <t>FR : FR (fr)</t>
         </is>
       </c>
       <c r="C24" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es</t>
+          <t>https://www.lg.com/fr</t>
         </is>
       </c>
       <c r="D24" s="265" t="inlineStr">
@@ -42930,7 +42929,7 @@
       </c>
       <c r="E24" s="123" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="F24" s="123" t="n">
@@ -42941,38 +42940,42 @@
     <row r="25">
       <c r="B25" s="261" t="inlineStr">
         <is>
-          <t>FR : FR (fr)</t>
+          <t>HK : HK (zh)</t>
         </is>
       </c>
       <c r="C25" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr</t>
-        </is>
-      </c>
-      <c r="D25" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>https://www.lg.com/hk</t>
+        </is>
+      </c>
+      <c r="D25" s="264" t="inlineStr">
+        <is>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E25" s="123" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F25" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="0" t="inlineStr"/>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>예상 2026-10-09 · PTT 1006 법인 승인 완료 · QA Final Live Check(게시 직전)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="261" t="inlineStr">
         <is>
-          <t>HK : HK (zh)</t>
+          <t>HK_EN : HK (en)</t>
         </is>
       </c>
       <c r="C26" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk</t>
+          <t>https://www.lg.com/hk_en</t>
         </is>
       </c>
       <c r="D26" s="264" t="inlineStr">
@@ -42997,94 +43000,90 @@
     <row r="27">
       <c r="B27" s="261" t="inlineStr">
         <is>
-          <t>HK_EN : HK (en)</t>
+          <t>HU : HU (hu)</t>
         </is>
       </c>
       <c r="C27" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en</t>
+          <t>https://www.lg.com/hu</t>
         </is>
       </c>
       <c r="D27" s="264" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E27" s="123" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E27" s="123" t="inlineStr"/>
       <c r="F27" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-09 · PTT 1006 법인 승인 완료 · QA Final Live Check(게시 직전)</t>
+          <t>법인 취소 요청(2026-09-15)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="261" t="inlineStr">
         <is>
-          <t>HR : HR (hr)</t>
+          <t>ID : ID (id)</t>
         </is>
       </c>
       <c r="C28" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hr</t>
+          <t>https://www.lg.com/id</t>
         </is>
       </c>
       <c r="D28" s="264" t="inlineStr">
         <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="E28" s="123" t="n"/>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E28" s="123" t="inlineStr"/>
       <c r="F28" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>법인 취소 요청(2026-09-15)</t>
+          <t>PTT 0929 · Client Review</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="261" t="inlineStr">
         <is>
-          <t>HU : HU (hu)</t>
+          <t>IN : IN (en)</t>
         </is>
       </c>
       <c r="C29" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hu</t>
-        </is>
-      </c>
-      <c r="D29" s="264" t="inlineStr">
-        <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="E29" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/in</t>
+        </is>
+      </c>
+      <c r="D29" s="263" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E29" s="123" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
       <c r="F29" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="0" t="inlineStr">
-        <is>
-          <t>법인 취소 요청(2026-09-15)</t>
-        </is>
-      </c>
+      <c r="G29" s="0" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="B30" s="261" t="inlineStr">
         <is>
-          <t>ID : ID (id)</t>
+          <t>IT : IT (it)</t>
         </is>
       </c>
       <c r="C30" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/id</t>
+          <t>https://www.lg.com/it</t>
         </is>
       </c>
       <c r="D30" s="264" t="inlineStr">
@@ -43092,51 +43091,55 @@
           <t>법인리뷰</t>
         </is>
       </c>
-      <c r="E30" s="123" t="inlineStr"/>
+      <c r="E30" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="F30" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>PTT 0929 · Client Review</t>
+          <t>예상 2026-10-02 · 법인리뷰</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="261" t="inlineStr">
         <is>
-          <t>IN : IN (en)</t>
+          <t>JP : JP (ja)</t>
         </is>
       </c>
       <c r="C31" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/in</t>
+          <t>https://www.lg.com/jp</t>
         </is>
       </c>
       <c r="D31" s="263" t="inlineStr">
         <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E31" s="123" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E31" s="123" t="inlineStr"/>
       <c r="F31" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G31" s="0" t="inlineStr"/>
+      <c r="G31" s="0" t="inlineStr">
+        <is>
+          <t>법인 취소 요청(2026-09-15)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="261" t="inlineStr">
         <is>
-          <t>IT : IT (it)</t>
+          <t>KZ : KZ (ru)</t>
         </is>
       </c>
       <c r="C32" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/it</t>
+          <t>https://www.lg.com/kz</t>
         </is>
       </c>
       <c r="D32" s="264" t="inlineStr">
@@ -43146,7 +43149,7 @@
       </c>
       <c r="E32" s="123" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F32" s="123" t="n">
@@ -43154,22 +43157,22 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-02 · 법인리뷰</t>
+          <t>예상 2026-10-05 · LDM 9월 내 확인</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="261" t="inlineStr">
         <is>
-          <t>JP : JP (ja)</t>
+          <t>MA : MA (fr)</t>
         </is>
       </c>
       <c r="C33" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/jp</t>
-        </is>
-      </c>
-      <c r="D33" s="263" t="inlineStr">
+          <t>https://www.lg.com/ma</t>
+        </is>
+      </c>
+      <c r="D33" s="262" t="inlineStr">
         <is>
           <t>취소</t>
         </is>
@@ -43178,21 +43181,17 @@
       <c r="F33" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="0" t="inlineStr">
-        <is>
-          <t>법인 취소 요청(2026-09-15)</t>
-        </is>
-      </c>
+      <c r="G33" s="0" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="B34" s="261" t="inlineStr">
         <is>
-          <t>KZ : KZ (ru)</t>
+          <t>MX : MX (es)</t>
         </is>
       </c>
       <c r="C34" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/kz</t>
+          <t>https://www.lg.com/mx</t>
         </is>
       </c>
       <c r="D34" s="264" t="inlineStr">
@@ -43202,7 +43201,7 @@
       </c>
       <c r="E34" s="123" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F34" s="123" t="n">
@@ -43210,127 +43209,131 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-05 · LDM 9월 내 확인</t>
+          <t>예상 2026-10-23 · 프로덕션 반영됨</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="261" t="inlineStr">
         <is>
-          <t>MA : MA (fr)</t>
+          <t>MY : MY (en)</t>
         </is>
       </c>
       <c r="C35" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ma</t>
-        </is>
-      </c>
-      <c r="D35" s="262" t="inlineStr">
-        <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="E35" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/my</t>
+        </is>
+      </c>
+      <c r="D35" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E35" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
       <c r="F35" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G35" s="0" t="inlineStr"/>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>예상 2026-10-09 · LDM 9월 내 확인</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="261" t="inlineStr">
         <is>
-          <t>MX : MX (es)</t>
+          <t>NL : NL (nl)</t>
         </is>
       </c>
       <c r="C36" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/mx</t>
-        </is>
-      </c>
-      <c r="D36" s="264" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
+          <t>https://www.lg.com/nl</t>
+        </is>
+      </c>
+      <c r="D36" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="E36" s="123" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="F36" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G36" s="0" t="inlineStr">
-        <is>
-          <t>예상 2026-10-23 · 프로덕션 반영됨</t>
-        </is>
-      </c>
+      <c r="G36" s="0" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="B37" s="261" t="inlineStr">
         <is>
-          <t>MY : MY (en)</t>
+          <t>NZ : NZ (en)</t>
         </is>
       </c>
       <c r="C37" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/my</t>
+          <t>https://www.lg.com/nz</t>
         </is>
       </c>
       <c r="D37" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E37" s="123" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E37" s="123" t="inlineStr"/>
       <c r="F37" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-09 · LDM 9월 내 확인</t>
+          <t>Hyper/Professional/Swing PLP 취소(09-14) · 나머지 Client Review (PTT 0929)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="261" t="inlineStr">
         <is>
-          <t>NL : NL (nl)</t>
+          <t>PA : PA (es)</t>
         </is>
       </c>
       <c r="C38" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nl</t>
-        </is>
-      </c>
-      <c r="D38" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>https://www.lg.com/pa</t>
+        </is>
+      </c>
+      <c r="D38" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E38" s="123" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F38" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G38" s="0" t="inlineStr"/>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>예상 2026-10-23</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="261" t="inlineStr">
         <is>
-          <t>NZ : NZ (en)</t>
+          <t>PE : PE (es)</t>
         </is>
       </c>
       <c r="C39" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/nz</t>
+          <t>https://www.lg.com/pe</t>
         </is>
       </c>
       <c r="D39" s="264" t="inlineStr">
@@ -43342,73 +43345,73 @@
       <c r="F39" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G39" s="0" t="inlineStr">
-        <is>
-          <t>Hyper/Professional/Swing PLP 취소(09-14) · 나머지 Client Review (PTT 0929)</t>
-        </is>
-      </c>
+      <c r="G39" s="0" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="B40" s="261" t="inlineStr">
         <is>
-          <t>PA : PA (es)</t>
+          <t>PH : PH (en)</t>
         </is>
       </c>
       <c r="C40" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pa</t>
+          <t>https://www.lg.com/ph</t>
         </is>
       </c>
       <c r="D40" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E40" s="123" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E40" s="123" t="inlineStr"/>
       <c r="F40" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-23</t>
+          <t>PTT 0929 · Client Review</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="261" t="inlineStr">
         <is>
-          <t>PE : PE (es)</t>
+          <t>PL : PL (pl)</t>
         </is>
       </c>
       <c r="C41" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pe</t>
+          <t>https://www.lg.com/pl</t>
         </is>
       </c>
       <c r="D41" s="264" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E41" s="123" t="inlineStr"/>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E41" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
       <c r="F41" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G41" s="0" t="inlineStr"/>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>예상 2026-10-16</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="261" t="inlineStr">
         <is>
-          <t>PH : PH (en)</t>
+          <t>PT : PT (pt)</t>
         </is>
       </c>
       <c r="C42" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ph</t>
+          <t>https://www.lg.com/pt</t>
         </is>
       </c>
       <c r="D42" s="264" t="inlineStr">
@@ -43416,145 +43419,145 @@
           <t>법인리뷰</t>
         </is>
       </c>
-      <c r="E42" s="123" t="inlineStr"/>
+      <c r="E42" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
       <c r="F42" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>PTT 0929 · Client Review</t>
+          <t>예상 2026-10-16 · LDM 무응답, 리마인더 발송</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="261" t="inlineStr">
         <is>
-          <t>PL : PL (pl)</t>
+          <t>SA_AR : SA (ar)</t>
         </is>
       </c>
       <c r="C43" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pl</t>
-        </is>
-      </c>
-      <c r="D43" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E43" s="123" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
+          <t>https://www.lg.com/sa</t>
+        </is>
+      </c>
+      <c r="D43" s="263" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E43" s="200" t="n">
+        <v>46246</v>
       </c>
       <c r="F43" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G43" s="0" t="inlineStr">
-        <is>
-          <t>예상 2026-10-16</t>
-        </is>
-      </c>
+      <c r="G43" s="0" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="B44" s="261" t="inlineStr">
         <is>
-          <t>PT : PT (pt)</t>
+          <t>SA_EN : SA (en)</t>
         </is>
       </c>
       <c r="C44" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/pt</t>
-        </is>
-      </c>
-      <c r="D44" s="264" t="inlineStr">
-        <is>
-          <t>법인리뷰</t>
-        </is>
-      </c>
-      <c r="E44" s="123" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
+          <t>https://www.lg.com/sa_en</t>
+        </is>
+      </c>
+      <c r="D44" s="263" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E44" s="200" t="n">
+        <v>46246</v>
       </c>
       <c r="F44" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G44" s="0" t="inlineStr">
-        <is>
-          <t>예상 2026-10-16 · LDM 무응답, 리마인더 발송</t>
-        </is>
-      </c>
+      <c r="G44" s="0" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="B45" s="261" t="inlineStr">
         <is>
-          <t>RS : RS (sr)</t>
+          <t>SE : SE (sv)</t>
         </is>
       </c>
       <c r="C45" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/rs</t>
-        </is>
-      </c>
-      <c r="D45" s="263" t="inlineStr">
-        <is>
-          <t>취소</t>
-        </is>
-      </c>
-      <c r="E45" s="200" t="n"/>
+          <t>https://www.lg.com/se</t>
+        </is>
+      </c>
+      <c r="D45" s="264" t="inlineStr">
+        <is>
+          <t>법인리뷰</t>
+        </is>
+      </c>
+      <c r="E45" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="F45" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>법인 취소 요청(2026-09-15)</t>
+          <t>예상 2026-10-02 · 법인리뷰</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="261" t="inlineStr">
         <is>
-          <t>SA_AR : SA (ar)</t>
+          <t>SG : SG (en)</t>
         </is>
       </c>
       <c r="C46" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa</t>
-        </is>
-      </c>
-      <c r="D46" s="263" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E46" s="200" t="n">
-        <v>46246</v>
+          <t>https://www.lg.com/sg</t>
+        </is>
+      </c>
+      <c r="D46" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E46" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
       </c>
       <c r="F46" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G46" s="0" t="inlineStr"/>
+      <c r="G46" s="0" t="inlineStr">
+        <is>
+          <t>예상 2026-10-09 · LDM 9월 내 확인</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="261" t="inlineStr">
         <is>
-          <t>SA_EN : SA (en)</t>
+          <t>TH : TH (th)</t>
         </is>
       </c>
       <c r="C47" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa_en</t>
-        </is>
-      </c>
-      <c r="D47" s="263" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E47" s="200" t="n">
-        <v>46246</v>
-      </c>
+          <t>https://www.lg.com/th</t>
+        </is>
+      </c>
+      <c r="D47" s="264" t="inlineStr">
+        <is>
+          <t>작업중</t>
+        </is>
+      </c>
+      <c r="E47" s="123" t="inlineStr"/>
       <c r="F47" s="123" t="n">
         <v>1</v>
       </c>
@@ -43563,22 +43566,22 @@
     <row r="48">
       <c r="B48" s="261" t="inlineStr">
         <is>
-          <t>SE : SE (sv)</t>
+          <t>TR : TR (tr)</t>
         </is>
       </c>
       <c r="C48" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/se</t>
+          <t>https://www.lg.com/tr</t>
         </is>
       </c>
       <c r="D48" s="264" t="inlineStr">
         <is>
-          <t>법인리뷰</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="E48" s="123" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F48" s="123" t="n">
@@ -43586,19 +43589,19 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-02 · 법인리뷰</t>
+          <t>게시완료 · Final Live Check 잔여</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="261" t="inlineStr">
         <is>
-          <t>SG : SG (en)</t>
+          <t>TW : TW (zh)</t>
         </is>
       </c>
       <c r="C49" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg</t>
+          <t>https://www.lg.com/tw</t>
         </is>
       </c>
       <c r="D49" s="264" t="inlineStr">
@@ -43606,37 +43609,33 @@
           <t>작업중</t>
         </is>
       </c>
-      <c r="E49" s="123" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
+      <c r="E49" s="123" t="inlineStr"/>
       <c r="F49" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G49" s="0" t="inlineStr">
-        <is>
-          <t>예상 2026-10-09 · LDM 9월 내 확인</t>
-        </is>
-      </c>
+      <c r="G49" s="0" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="B50" s="261" t="inlineStr">
         <is>
-          <t>TH : TH (th)</t>
+          <t>UK : GB (en)</t>
         </is>
       </c>
       <c r="C50" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/th</t>
-        </is>
-      </c>
-      <c r="D50" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E50" s="123" t="inlineStr"/>
+          <t>https://www.lg.com/uk</t>
+        </is>
+      </c>
+      <c r="D50" s="265" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E50" s="123" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
       <c r="F50" s="123" t="n">
         <v>1</v>
       </c>
@@ -43645,12 +43644,12 @@
     <row r="51">
       <c r="B51" s="261" t="inlineStr">
         <is>
-          <t>TR : TR (tr)</t>
+          <t>VN : VN (vi)</t>
         </is>
       </c>
       <c r="C51" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr</t>
+          <t>https://www.lg.com/vn</t>
         </is>
       </c>
       <c r="D51" s="264" t="inlineStr">
@@ -43660,7 +43659,7 @@
       </c>
       <c r="E51" s="123" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F51" s="123" t="n">
@@ -43668,19 +43667,19 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>게시완료 · Final Live Check 잔여</t>
+          <t>게시완료(09-10) · Hyper Mini LED PLP 취소(08-31)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="261" t="inlineStr">
         <is>
-          <t>TW : TW (zh)</t>
+          <t>ZA : ZA (en)</t>
         </is>
       </c>
       <c r="C52" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tw</t>
+          <t>https://www.lg.com/za</t>
         </is>
       </c>
       <c r="D52" s="264" t="inlineStr">
@@ -43692,85 +43691,7 @@
       <c r="F52" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="G52" s="0" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="B53" s="261" t="inlineStr">
-        <is>
-          <t>UK : GB (en)</t>
-        </is>
-      </c>
-      <c r="C53" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/uk</t>
-        </is>
-      </c>
-      <c r="D53" s="265" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E53" s="123" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="F53" s="123" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" s="0" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="B54" s="261" t="inlineStr">
-        <is>
-          <t>VN : VN (vi)</t>
-        </is>
-      </c>
-      <c r="C54" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/vn</t>
-        </is>
-      </c>
-      <c r="D54" s="264" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E54" s="123" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="F54" s="123" t="n">
-        <v>1</v>
-      </c>
-      <c r="G54" s="0" t="inlineStr">
-        <is>
-          <t>게시완료(09-10) · Hyper Mini LED PLP 취소(08-31)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="261" t="inlineStr">
-        <is>
-          <t>ZA : ZA (en)</t>
-        </is>
-      </c>
-      <c r="C55" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/za</t>
-        </is>
-      </c>
-      <c r="D55" s="264" t="inlineStr">
-        <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E55" s="123" t="inlineStr"/>
-      <c r="F55" s="123" t="n">
-        <v>1</v>
-      </c>
-      <c r="G55" s="0" t="inlineStr">
+      <c r="G52" s="0" t="inlineStr">
         <is>
           <t>GNB 수정 게시(07-27) · PTT 1006 Closed 6 · QA Final Live Check 1(완료 임박)</t>
         </is>
@@ -43822,9 +43743,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -45336,7 +45254,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>

</xml_diff>

<commit_message>
data(it): GNB 예상일 경과 5개국 일정 조정 — KZ·SE 10/16, IT·EG 10/23
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -42843,7 +42843,7 @@
       </c>
       <c r="E21" s="123" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F21" s="123" t="n">
@@ -42851,7 +42851,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-02 · LDM 회신 대기, 09/30 무응답 시 취소</t>
+          <t>예상 2026-10-23 · 10/02→10/23 조정 · 9/30 무응답 시 취소 기한 경과, 취소 여부 확인 필요</t>
         </is>
       </c>
     </row>
@@ -42873,7 +42873,7 @@
       </c>
       <c r="E22" s="123" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F22" s="123" t="n">
@@ -42881,7 +42881,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-02 · LDM 회신 대기, 09/30 무응답 시 취소</t>
+          <t>예상 2026-10-23 · 10/02→10/23 조정 · 9/30 무응답 시 취소 기한 경과, 취소 여부 확인 필요</t>
         </is>
       </c>
     </row>
@@ -43093,7 +43093,7 @@
       </c>
       <c r="E30" s="123" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F30" s="123" t="n">
@@ -43101,7 +43101,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-02 · 법인리뷰</t>
+          <t>예상 2026-10-23 · 10/02→10/23 조정(PTT 1006 Create Request)</t>
         </is>
       </c>
     </row>
@@ -43149,7 +43149,7 @@
       </c>
       <c r="E32" s="123" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="F32" s="123" t="n">
@@ -43157,7 +43157,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-05 · LDM 9월 내 확인</t>
+          <t>예상 2026-10-16 · 10/05→10/16 조정(PTT 1006 Client Review)</t>
         </is>
       </c>
     </row>
@@ -43499,7 +43499,7 @@
       </c>
       <c r="E45" s="123" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="F45" s="123" t="n">
@@ -43507,7 +43507,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-02 · 법인리뷰</t>
+          <t>예상 2026-10-16 · 10/02→10/16 조정(PTT 1006 New Request)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): PTT 20261007 재조인(ES 17Z90U-G QA review) + GNB 비고 PTT 1007 기준 갱신
10/06 CMS는 prod_aem_publish_flag 컬럼 누락으로 반영하지 않음.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -42851,7 +42851,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-23 · 10/02→10/23 조정 · 9/30 무응답 시 취소 기한 경과, 취소 여부 확인 필요</t>
+          <t>예상 2026-10-23 · 10/02→10/23 조정 · PTT 1007 Create Request · 9/30 무응답 시 취소 기한 경과, 취소 여부 확인 필요</t>
         </is>
       </c>
     </row>
@@ -42881,7 +42881,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-23 · 10/02→10/23 조정 · 9/30 무응답 시 취소 기한 경과, 취소 여부 확인 필요</t>
+          <t>예상 2026-10-23 · 10/02→10/23 조정 · PTT 1007 Create Request · 9/30 무응답 시 취소 기한 경과, 취소 여부 확인 필요</t>
         </is>
       </c>
     </row>
@@ -42963,7 +42963,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-09 · PTT 1006 법인 승인 완료 · QA Final Live Check(게시 직전)</t>
+          <t>예상 2026-10-09 · PTT 1007 Publishing Approve 1 · QA Final Live Check 6(게시 직전)</t>
         </is>
       </c>
     </row>
@@ -42993,7 +42993,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-09 · PTT 1006 법인 승인 완료 · QA Final Live Check(게시 직전)</t>
+          <t>예상 2026-10-09 · PTT 1007 Publishing Approve 1 · QA Final Live Check 5(게시 직전)</t>
         </is>
       </c>
     </row>
@@ -43101,7 +43101,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-23 · 10/02→10/23 조정(PTT 1006 Create Request)</t>
+          <t>예상 2026-10-23 · 10/02→10/23 조정(PTT 1007 Create Request)</t>
         </is>
       </c>
     </row>
@@ -43157,7 +43157,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-16 · 10/05→10/16 조정(PTT 1006 Client Review)</t>
+          <t>예상 2026-10-16 · 10/05→10/16 조정(PTT 1007 Client Review)</t>
         </is>
       </c>
     </row>
@@ -43507,7 +43507,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-16 · 10/02→10/16 조정(PTT 1006 New Request)</t>
+          <t>예상 2026-10-16 · 10/02→10/16 조정(PTT 1007 New Request)</t>
         </is>
       </c>
     </row>
@@ -43693,7 +43693,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>GNB 수정 게시(07-27) · PTT 1006 Closed 6 · QA Final Live Check 1(완료 임박)</t>
+          <t>GNB 수정 게시(07-27) · PTT 1007 Closed 7 · QA Final Live Check 1(완료 임박)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): GNB EG 2개국 취소, ZA 완료(10/07), KZ·HK 게시 진행 비고 반영
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -42838,20 +42838,16 @@
       </c>
       <c r="D21" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E21" s="123" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E21" s="123" t="n"/>
       <c r="F21" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-23 · 10/02→10/23 조정 · 9/30 무응답 시 취소 기한 경과, 취소 여부 확인 필요</t>
+          <t>LDM 무응답으로 법인 취소(2026-10-08)</t>
         </is>
       </c>
     </row>
@@ -42868,20 +42864,16 @@
       </c>
       <c r="D22" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E22" s="123" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
+          <t>취소</t>
+        </is>
+      </c>
+      <c r="E22" s="123" t="n"/>
       <c r="F22" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-23 · 10/02→10/23 조정 · 9/30 무응답 시 취소 기한 경과, 취소 여부 확인 필요</t>
+          <t>LDM 무응답으로 법인 취소(2026-10-08)</t>
         </is>
       </c>
     </row>
@@ -42963,7 +42955,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-09 · 법인 승인 완료 · 게시 직전</t>
+          <t>예상 2026-10-09 · 법인 승인 완료 · 게시 진행 중</t>
         </is>
       </c>
     </row>
@@ -42993,7 +42985,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-09 · 법인 승인 완료 · 게시 직전</t>
+          <t>예상 2026-10-09 · 법인 승인 완료 · 게시 진행 중</t>
         </is>
       </c>
     </row>
@@ -43157,7 +43149,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>예상 2026-10-16 · 10/05→10/16 조정</t>
+          <t>예상 2026-10-16 · 10/05→10/16 조정 · 법인 승인 완료, 게시 진행 중</t>
         </is>
       </c>
     </row>
@@ -43684,16 +43676,20 @@
       </c>
       <c r="D52" s="264" t="inlineStr">
         <is>
-          <t>작업중</t>
-        </is>
-      </c>
-      <c r="E52" s="123" t="inlineStr"/>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E52" s="123" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="F52" s="123" t="n">
         <v>1</v>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>GNB 수정 게시(07-27) · 완료 임박(최종 게시 점검 중)</t>
+          <t>GNB 수정 게시(07-27) · 전체 게시 완료(10-07)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): UltraGear Buying Guide 2차 대상을 요청서 65개 사이트로 확대
Co-Authored-By: Grok 4.7 <noreply@x.ai>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -638,7 +638,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="68" fillId="0" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="297">
+  <cellXfs count="298">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1224,6 +1224,7 @@
     </xf>
     <xf numFmtId="0" fontId="71" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="70" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -40585,7 +40586,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -40611,7 +40612,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>금주 신규 등록 · 1차(W22) 44개국 + 기존 라이브 6곳(AE-en·BE-nl·DE·UK·SG·MX) = 50개 사이트 · 담당 정알찬 책임</t>
+          <t>요청서 Target List 65개 사이트 · 기존 50에 15개국 추가(AR·BG·CH-fr·CL·HR·LEVANT×2·LK·NP·RO·SK·TN·UZ×2·VN) · 담당 정알찬 책임</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -40625,6 +40626,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -40726,14 +40728,10 @@
     <row r="11">
       <c r="B11" s="261" t="inlineStr">
         <is>
-          <t>BD-en</t>
-        </is>
-      </c>
-      <c r="C11" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/bd/ultragear-gaming-buying-guide</t>
-        </is>
-      </c>
+          <t>AR-es</t>
+        </is>
+      </c>
+      <c r="C11" s="290" t="n"/>
       <c r="D11" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40743,17 +40741,21 @@
       <c r="F11" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="0" t="n"/>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="261" t="inlineStr">
         <is>
-          <t>BE-fr</t>
+          <t>BD-en</t>
         </is>
       </c>
       <c r="C12" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/be_fr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/bd/ultragear-gaming-buying-guide</t>
         </is>
       </c>
       <c r="D12" s="265" t="inlineStr">
@@ -40770,12 +40772,12 @@
     <row r="13">
       <c r="B13" s="261" t="inlineStr">
         <is>
-          <t>BE-nl</t>
+          <t>BE-fr</t>
         </is>
       </c>
       <c r="C13" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/be/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/be_fr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D13" s="265" t="inlineStr">
@@ -40787,19 +40789,19 @@
       <c r="F13" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="0" t="inlineStr">
-        <is>
-          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
-        </is>
-      </c>
+      <c r="G13" s="0" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="261" t="inlineStr">
         <is>
-          <t>BR-pt</t>
-        </is>
-      </c>
-      <c r="C14" s="290" t="n"/>
+          <t>BE-nl</t>
+        </is>
+      </c>
+      <c r="C14" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/be/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
       <c r="D14" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40811,21 +40813,17 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>신규 제작(1차 미게시)</t>
+          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="261" t="inlineStr">
         <is>
-          <t>CA-en</t>
-        </is>
-      </c>
-      <c r="C15" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>BG-bg</t>
+        </is>
+      </c>
+      <c r="C15" s="290" t="n"/>
       <c r="D15" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40835,19 +40833,19 @@
       <c r="F15" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="0" t="n"/>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="261" t="inlineStr">
         <is>
-          <t>CA-fr</t>
-        </is>
-      </c>
-      <c r="C16" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_fr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>BR-pt</t>
+        </is>
+      </c>
+      <c r="C16" s="290" t="n"/>
       <c r="D16" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40857,17 +40855,21 @@
       <c r="F16" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="0" t="n"/>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>신규 제작(1차 미게시)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="261" t="inlineStr">
         <is>
-          <t>CAC-es</t>
+          <t>CA-en</t>
         </is>
       </c>
       <c r="C17" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/cac/computacion/ultragear-buying-guide</t>
+          <t>https://www.lg.com/ca_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D17" s="265" t="inlineStr">
@@ -40884,10 +40886,14 @@
     <row r="18">
       <c r="B18" s="261" t="inlineStr">
         <is>
-          <t>CN-zh</t>
-        </is>
-      </c>
-      <c r="C18" s="290" t="n"/>
+          <t>CA-fr</t>
+        </is>
+      </c>
+      <c r="C18" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
       <c r="D18" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40897,19 +40903,19 @@
       <c r="F18" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="0" t="inlineStr">
-        <is>
-          <t>신규 제작(1차 미게시)</t>
-        </is>
-      </c>
+      <c r="G18" s="0" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="261" t="inlineStr">
         <is>
-          <t>CO-es</t>
-        </is>
-      </c>
-      <c r="C19" s="290" t="n"/>
+          <t>CAC-es</t>
+        </is>
+      </c>
+      <c r="C19" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cac/computacion/ultragear-buying-guide</t>
+        </is>
+      </c>
       <c r="D19" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40919,23 +40925,15 @@
       <c r="F19" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="0" t="inlineStr">
-        <is>
-          <t>신규 제작(1차 미게시)</t>
-        </is>
-      </c>
+      <c r="G19" s="0" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="261" t="inlineStr">
         <is>
-          <t>CZ-cz</t>
-        </is>
-      </c>
-      <c r="C20" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/cz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>CH-fr</t>
+        </is>
+      </c>
+      <c r="C20" s="290" t="n"/>
       <c r="D20" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40945,19 +40943,19 @@
       <c r="F20" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="0" t="n"/>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="261" t="inlineStr">
         <is>
-          <t>DE-de</t>
-        </is>
-      </c>
-      <c r="C21" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/de/buying-guides/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>CL-es</t>
+        </is>
+      </c>
+      <c r="C21" s="290" t="n"/>
       <c r="D21" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40969,21 +40967,17 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
+          <t>요청서 Target List 추가</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="261" t="inlineStr">
         <is>
-          <t>DK-da</t>
-        </is>
-      </c>
-      <c r="C22" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/dk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>CN-zh</t>
+        </is>
+      </c>
+      <c r="C22" s="290" t="n"/>
       <c r="D22" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -40993,19 +40987,19 @@
       <c r="F22" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="0" t="n"/>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>신규 제작(1차 미게시)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="261" t="inlineStr">
         <is>
-          <t>EC-es</t>
-        </is>
-      </c>
-      <c r="C23" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ec/computacion/ultragear-buying-guide</t>
-        </is>
-      </c>
+          <t>CO-es</t>
+        </is>
+      </c>
+      <c r="C23" s="290" t="n"/>
       <c r="D23" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41015,17 +41009,21 @@
       <c r="F23" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="0" t="n"/>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>신규 제작(1차 미게시)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="261" t="inlineStr">
         <is>
-          <t>EE-ee</t>
+          <t>CZ-cz</t>
         </is>
       </c>
       <c r="C24" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/ee/it-seadmed/buying-guide/ultragear-mangumonitorid</t>
+          <t>https://www.lg.com/cz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D24" s="265" t="inlineStr">
@@ -41042,12 +41040,12 @@
     <row r="25">
       <c r="B25" s="261" t="inlineStr">
         <is>
-          <t>ES-es</t>
+          <t>DE-de</t>
         </is>
       </c>
       <c r="C25" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/es/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/de/buying-guides/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D25" s="265" t="inlineStr">
@@ -41059,17 +41057,21 @@
       <c r="F25" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="0" t="n"/>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="261" t="inlineStr">
         <is>
-          <t>FI-fi</t>
+          <t>DK-da</t>
         </is>
       </c>
       <c r="C26" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fi/it-tuotteet/ultragear-buying-guide</t>
+          <t>https://www.lg.com/dk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D26" s="265" t="inlineStr">
@@ -41086,12 +41088,12 @@
     <row r="27">
       <c r="B27" s="261" t="inlineStr">
         <is>
-          <t>FR-fr</t>
+          <t>EC-es</t>
         </is>
       </c>
       <c r="C27" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/fr/moniteurs/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/ec/computacion/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D27" s="265" t="inlineStr">
@@ -41108,10 +41110,14 @@
     <row r="28">
       <c r="B28" s="261" t="inlineStr">
         <is>
-          <t>GR-gr</t>
-        </is>
-      </c>
-      <c r="C28" s="290" t="n"/>
+          <t>EE-ee</t>
+        </is>
+      </c>
+      <c r="C28" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ee/it-seadmed/buying-guide/ultragear-mangumonitorid</t>
+        </is>
+      </c>
       <c r="D28" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41121,21 +41127,17 @@
       <c r="F28" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G28" s="0" t="inlineStr">
-        <is>
-          <t>신규 제작(1차 미게시)</t>
-        </is>
-      </c>
+      <c r="G28" s="0" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="261" t="inlineStr">
         <is>
-          <t>HK-en</t>
+          <t>ES-es</t>
         </is>
       </c>
       <c r="C29" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/es/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D29" s="265" t="inlineStr">
@@ -41152,12 +41154,12 @@
     <row r="30">
       <c r="B30" s="261" t="inlineStr">
         <is>
-          <t>HK-zh</t>
+          <t>FI-fi</t>
         </is>
       </c>
       <c r="C30" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/fi/it-tuotteet/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D30" s="265" t="inlineStr">
@@ -41174,12 +41176,12 @@
     <row r="31">
       <c r="B31" s="261" t="inlineStr">
         <is>
-          <t>HU-hu</t>
+          <t>FR-fr</t>
         </is>
       </c>
       <c r="C31" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/hu/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/fr/moniteurs/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D31" s="265" t="inlineStr">
@@ -41196,14 +41198,10 @@
     <row r="32">
       <c r="B32" s="261" t="inlineStr">
         <is>
-          <t>ID-id</t>
-        </is>
-      </c>
-      <c r="C32" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/id/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>GR-gr</t>
+        </is>
+      </c>
+      <c r="C32" s="290" t="n"/>
       <c r="D32" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41213,17 +41211,21 @@
       <c r="F32" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G32" s="0" t="n"/>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>신규 제작(1차 미게시)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="261" t="inlineStr">
         <is>
-          <t>IL-he</t>
+          <t>HK-en</t>
         </is>
       </c>
       <c r="C33" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/il/monitors/ultragear-buying-guide</t>
+          <t>https://www.lg.com/hk_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D33" s="265" t="inlineStr">
@@ -41240,12 +41242,12 @@
     <row r="34">
       <c r="B34" s="261" t="inlineStr">
         <is>
-          <t>IN-en</t>
+          <t>HK-zh</t>
         </is>
       </c>
       <c r="C34" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/in/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/hk/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D34" s="265" t="inlineStr">
@@ -41262,7 +41264,7 @@
     <row r="35">
       <c r="B35" s="261" t="inlineStr">
         <is>
-          <t>IT-it</t>
+          <t>HR-hr</t>
         </is>
       </c>
       <c r="C35" s="290" t="n"/>
@@ -41277,17 +41279,21 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>신규 제작(1차 미게시)</t>
+          <t>요청서 Target List 추가</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="261" t="inlineStr">
         <is>
-          <t>JP-ja</t>
-        </is>
-      </c>
-      <c r="C36" s="290" t="n"/>
+          <t>HU-hu</t>
+        </is>
+      </c>
+      <c r="C36" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/hu/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
       <c r="D36" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41297,21 +41303,17 @@
       <c r="F36" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G36" s="0" t="inlineStr">
-        <is>
-          <t>신규 제작(1차 미게시)</t>
-        </is>
-      </c>
+      <c r="G36" s="0" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="261" t="inlineStr">
         <is>
-          <t>KZ-ru</t>
+          <t>ID-id</t>
         </is>
       </c>
       <c r="C37" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/kz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/id/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D37" s="265" t="inlineStr">
@@ -41328,12 +41330,12 @@
     <row r="38">
       <c r="B38" s="261" t="inlineStr">
         <is>
-          <t>LT-lt</t>
+          <t>IL-he</t>
         </is>
       </c>
       <c r="C38" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/lt/kompiuterine-technika/buying-guide/ultragear-gaming-monitor</t>
+          <t>https://www.lg.com/il/monitors/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D38" s="265" t="inlineStr">
@@ -41350,12 +41352,12 @@
     <row r="39">
       <c r="B39" s="261" t="inlineStr">
         <is>
-          <t>LV-lv</t>
+          <t>IN-en</t>
         </is>
       </c>
       <c r="C39" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/lv/datortehnika/buying-guide/ultragear-gaming-monitor</t>
+          <t>https://www.lg.com/in/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D39" s="265" t="inlineStr">
@@ -41372,14 +41374,10 @@
     <row r="40">
       <c r="B40" s="261" t="inlineStr">
         <is>
-          <t>MX-es</t>
-        </is>
-      </c>
-      <c r="C40" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/mx/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>IT-it</t>
+        </is>
+      </c>
+      <c r="C40" s="290" t="n"/>
       <c r="D40" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41391,21 +41389,17 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
+          <t>신규 제작(1차 미게시)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="261" t="inlineStr">
         <is>
-          <t>NL-nl</t>
-        </is>
-      </c>
-      <c r="C41" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/nl/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>JP-ja</t>
+        </is>
+      </c>
+      <c r="C41" s="290" t="n"/>
       <c r="D41" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41415,17 +41409,21 @@
       <c r="F41" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G41" s="0" t="n"/>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>신규 제작(1차 미게시)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="261" t="inlineStr">
         <is>
-          <t>NO-no</t>
+          <t>KZ-ru</t>
         </is>
       </c>
       <c r="C42" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/no/it-produkter/ultragear-buying-guide</t>
+          <t>https://www.lg.com/kz/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D42" s="265" t="inlineStr">
@@ -41442,14 +41440,10 @@
     <row r="43">
       <c r="B43" s="261" t="inlineStr">
         <is>
-          <t>PA-es</t>
-        </is>
-      </c>
-      <c r="C43" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/pa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>LEVANT-ar</t>
+        </is>
+      </c>
+      <c r="C43" s="290" t="n"/>
       <c r="D43" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41459,19 +41453,19 @@
       <c r="F43" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G43" s="0" t="n"/>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="261" t="inlineStr">
         <is>
-          <t>PE-es</t>
-        </is>
-      </c>
-      <c r="C44" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/pe/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>LEVANT-en</t>
+        </is>
+      </c>
+      <c r="C44" s="290" t="n"/>
       <c r="D44" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41481,19 +41475,19 @@
       <c r="F44" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G44" s="0" t="n"/>
+      <c r="G44" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="261" t="inlineStr">
         <is>
-          <t>PH-en</t>
-        </is>
-      </c>
-      <c r="C45" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ph/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>LK-en</t>
+        </is>
+      </c>
+      <c r="C45" s="290" t="n"/>
       <c r="D45" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41503,15 +41497,23 @@
       <c r="F45" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G45" s="0" t="n"/>
+      <c r="G45" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="261" t="inlineStr">
         <is>
-          <t>PL-pl</t>
-        </is>
-      </c>
-      <c r="C46" s="290" t="n"/>
+          <t>LT-lt</t>
+        </is>
+      </c>
+      <c r="C46" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lt/kompiuterine-technika/buying-guide/ultragear-gaming-monitor</t>
+        </is>
+      </c>
       <c r="D46" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41521,19 +41523,19 @@
       <c r="F46" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G46" s="0" t="inlineStr">
-        <is>
-          <t>신규 제작(1차 미게시)</t>
-        </is>
-      </c>
+      <c r="G46" s="0" t="n"/>
     </row>
     <row r="47">
       <c r="B47" s="261" t="inlineStr">
         <is>
-          <t>PT-pt</t>
-        </is>
-      </c>
-      <c r="C47" s="290" t="n"/>
+          <t>LV-lv</t>
+        </is>
+      </c>
+      <c r="C47" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/lv/datortehnika/buying-guide/ultragear-gaming-monitor</t>
+        </is>
+      </c>
       <c r="D47" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41543,21 +41545,17 @@
       <c r="F47" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G47" s="0" t="inlineStr">
-        <is>
-          <t>신규 제작(1차 미게시)</t>
-        </is>
-      </c>
+      <c r="G47" s="0" t="n"/>
     </row>
     <row r="48">
       <c r="B48" s="261" t="inlineStr">
         <is>
-          <t>RS-rs</t>
+          <t>MX-es</t>
         </is>
       </c>
       <c r="C48" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/rs/it-proizvodi/ultragear-buying-guide</t>
+          <t>https://www.lg.com/mx/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D48" s="265" t="inlineStr">
@@ -41569,17 +41567,21 @@
       <c r="F48" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G48" s="0" t="n"/>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="261" t="inlineStr">
         <is>
-          <t>SA-ar</t>
+          <t>NL-nl</t>
         </is>
       </c>
       <c r="C49" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/nl/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D49" s="265" t="inlineStr">
@@ -41596,12 +41598,12 @@
     <row r="50">
       <c r="B50" s="261" t="inlineStr">
         <is>
-          <t>SA-en</t>
+          <t>NO-no</t>
         </is>
       </c>
       <c r="C50" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sa_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/no/it-produkter/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D50" s="265" t="inlineStr">
@@ -41618,14 +41620,10 @@
     <row r="51">
       <c r="B51" s="261" t="inlineStr">
         <is>
-          <t>SE-sv</t>
-        </is>
-      </c>
-      <c r="C51" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/se/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>NP-en</t>
+        </is>
+      </c>
+      <c r="C51" s="290" t="n"/>
       <c r="D51" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41635,17 +41633,21 @@
       <c r="F51" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G51" s="0" t="n"/>
+      <c r="G51" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="261" t="inlineStr">
         <is>
-          <t>SG-en</t>
+          <t>PA-es</t>
         </is>
       </c>
       <c r="C52" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/sg/consumer-monitors/featured-page/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/pa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D52" s="265" t="inlineStr">
@@ -41657,21 +41659,17 @@
       <c r="F52" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G52" s="0" t="inlineStr">
-        <is>
-          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
-        </is>
-      </c>
+      <c r="G52" s="0" t="n"/>
     </row>
     <row r="53">
       <c r="B53" s="261" t="inlineStr">
         <is>
-          <t>TH-th</t>
+          <t>PE-es</t>
         </is>
       </c>
       <c r="C53" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/th/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/pe/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D53" s="265" t="inlineStr">
@@ -41688,12 +41686,12 @@
     <row r="54">
       <c r="B54" s="261" t="inlineStr">
         <is>
-          <t>TR-tr</t>
+          <t>PH-en</t>
         </is>
       </c>
       <c r="C54" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/tr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/ph/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
         </is>
       </c>
       <c r="D54" s="265" t="inlineStr">
@@ -41710,14 +41708,10 @@
     <row r="55">
       <c r="B55" s="261" t="inlineStr">
         <is>
-          <t>TW-zh</t>
-        </is>
-      </c>
-      <c r="C55" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/tw/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
-        </is>
-      </c>
+          <t>PL-pl</t>
+        </is>
+      </c>
+      <c r="C55" s="290" t="n"/>
       <c r="D55" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41727,19 +41721,19 @@
       <c r="F55" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G55" s="0" t="n"/>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>신규 제작(1차 미게시)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="261" t="inlineStr">
         <is>
-          <t>UA-uk</t>
-        </is>
-      </c>
-      <c r="C56" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ua/it-products/ultragear-buying-guide</t>
-        </is>
-      </c>
+          <t>PT-pt</t>
+        </is>
+      </c>
+      <c r="C56" s="290" t="n"/>
       <c r="D56" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41749,19 +41743,19 @@
       <c r="F56" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G56" s="0" t="n"/>
+      <c r="G56" s="0" t="inlineStr">
+        <is>
+          <t>신규 제작(1차 미게시)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="261" t="inlineStr">
         <is>
-          <t>UK-en</t>
-        </is>
-      </c>
-      <c r="C57" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/uk/computing/buying-guides/ultragear/</t>
-        </is>
-      </c>
+          <t>RO-ro</t>
+        </is>
+      </c>
+      <c r="C57" s="290" t="n"/>
       <c r="D57" s="265" t="inlineStr">
         <is>
           <t>사전검토</t>
@@ -41773,19 +41767,19 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
+          <t>요청서 Target List 추가</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="261" t="inlineStr">
         <is>
-          <t>ZA-en</t>
+          <t>RS-rs</t>
         </is>
       </c>
       <c r="C58" s="290" t="inlineStr">
         <is>
-          <t>https://www.lg.com/za/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+          <t>https://www.lg.com/rs/it-proizvodi/ultragear-buying-guide</t>
         </is>
       </c>
       <c r="D58" s="265" t="inlineStr">
@@ -41798,51 +41792,389 @@
         <v>1</v>
       </c>
       <c r="G58" s="0" t="n"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="261" t="inlineStr">
+        <is>
+          <t>SA-ar</t>
+        </is>
+      </c>
+      <c r="C59" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D59" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E59" s="123" t="n"/>
+      <c r="F59" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="0" t="n"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="261" t="inlineStr">
+        <is>
+          <t>SA-en</t>
+        </is>
+      </c>
+      <c r="C60" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sa_en/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D60" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E60" s="123" t="n"/>
+      <c r="F60" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="0" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="261" t="inlineStr">
+        <is>
+          <t>SE-sv</t>
+        </is>
+      </c>
+      <c r="C61" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/se/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D61" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E61" s="123" t="n"/>
+      <c r="F61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="0" t="n"/>
+    </row>
+    <row r="62">
+      <c r="B62" s="261" t="inlineStr">
+        <is>
+          <t>SG-en</t>
+        </is>
+      </c>
+      <c r="C62" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/consumer-monitors/featured-page/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D62" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E62" s="123" t="n"/>
+      <c r="F62" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="0" t="inlineStr">
+        <is>
+          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="261" t="inlineStr">
+        <is>
+          <t>SK-sk</t>
+        </is>
+      </c>
+      <c r="C63" s="297" t="n"/>
+      <c r="D63" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E63" s="123" t="n"/>
+      <c r="F63" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="261" t="inlineStr">
+        <is>
+          <t>TH-th</t>
+        </is>
+      </c>
+      <c r="C64" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/th/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D64" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E64" s="123" t="n"/>
+      <c r="F64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="0" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="261" t="inlineStr">
+        <is>
+          <t>TN-fr</t>
+        </is>
+      </c>
+      <c r="C65" s="297" t="n"/>
+      <c r="D65" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E65" s="123" t="n"/>
+      <c r="F65" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="261" t="inlineStr">
+        <is>
+          <t>TR-tr</t>
+        </is>
+      </c>
+      <c r="C66" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tr/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D66" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E66" s="123" t="n"/>
+      <c r="F66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="0" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="261" t="inlineStr">
+        <is>
+          <t>TW-zh</t>
+        </is>
+      </c>
+      <c r="C67" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D67" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E67" s="123" t="n"/>
+      <c r="F67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="0" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="261" t="inlineStr">
+        <is>
+          <t>UA-uk</t>
+        </is>
+      </c>
+      <c r="C68" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ua/it-products/ultragear-buying-guide</t>
+        </is>
+      </c>
+      <c r="D68" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E68" s="123" t="n"/>
+      <c r="F68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="0" t="n"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="261" t="inlineStr">
+        <is>
+          <t>UK-en</t>
+        </is>
+      </c>
+      <c r="C69" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/computing/buying-guides/ultragear/</t>
+        </is>
+      </c>
+      <c r="D69" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E69" s="123" t="n"/>
+      <c r="F69" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
+        <is>
+          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="261" t="inlineStr">
+        <is>
+          <t>UZ-ru</t>
+        </is>
+      </c>
+      <c r="C70" s="297" t="n"/>
+      <c r="D70" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E70" s="123" t="n"/>
+      <c r="F70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="261" t="inlineStr">
+        <is>
+          <t>UZ-uz</t>
+        </is>
+      </c>
+      <c r="C71" s="297" t="n"/>
+      <c r="D71" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E71" s="123" t="n"/>
+      <c r="F71" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="261" t="inlineStr">
+        <is>
+          <t>VN-vi</t>
+        </is>
+      </c>
+      <c r="C72" s="297" t="n"/>
+      <c r="D72" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E72" s="123" t="n"/>
+      <c r="F72" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="0" t="inlineStr">
+        <is>
+          <t>요청서 Target List 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="261" t="inlineStr">
+        <is>
+          <t>ZA-en</t>
+        </is>
+      </c>
+      <c r="C73" s="297" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/za/microsite-article/ms/it/monitor/ultragear-buying-guide/</t>
+        </is>
+      </c>
+      <c r="D73" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E73" s="123" t="n"/>
+      <c r="F73" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="0" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data(it): Windows 11 Home Landing 대상을 요청서 15사이트로 반영
Co-Authored-By: Grok 4.7 <noreply@x.ai>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -14287,7 +14287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14310,7 +14310,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>예정 · 자산 배포 2026-08-09(EN)/2026-09-11(현지화) · 구현 마감 2026-11-15(Jumpstart OEM.com 준수)</t>
+          <t>예정 · 요청서 2026-10-07 기준 15사이트(Global 포함) · Due 2026-10-31 · 담당 정의현 책임</t>
         </is>
       </c>
     </row>
@@ -14351,7 +14351,414 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="B4" s="261" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C4" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D4" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E4" s="123" t="n"/>
+      <c r="F4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="261" t="inlineStr">
+        <is>
+          <t>CA-en</t>
+        </is>
+      </c>
+      <c r="C5" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D5" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E5" s="123" t="n"/>
+      <c r="F5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="261" t="inlineStr">
+        <is>
+          <t>CA-fr</t>
+        </is>
+      </c>
+      <c r="C6" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/page-de-presentation/decouvrez-choisirmc-lg-gram/windows-11/</t>
+        </is>
+      </c>
+      <c r="D6" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E6" s="123" t="n"/>
+      <c r="F6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>Translation FR-CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="261" t="inlineStr">
+        <is>
+          <t>ES-es</t>
+        </is>
+      </c>
+      <c r="C7" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/ordenadores/windows-11/</t>
+        </is>
+      </c>
+      <c r="D7" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E7" s="123" t="n"/>
+      <c r="F7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>Translation ES-ES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="261" t="inlineStr">
+        <is>
+          <t>IT-it</t>
+        </is>
+      </c>
+      <c r="C8" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/windows-11/</t>
+        </is>
+      </c>
+      <c r="D8" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E8" s="123" t="n"/>
+      <c r="F8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(It-LT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="261" t="inlineStr">
+        <is>
+          <t>UK-en</t>
+        </is>
+      </c>
+      <c r="C9" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D9" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E9" s="123" t="n"/>
+      <c r="F9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>Translation EN-GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="261" t="inlineStr">
+        <is>
+          <t>DE-de</t>
+        </is>
+      </c>
+      <c r="C10" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/windows-11/</t>
+        </is>
+      </c>
+      <c r="D10" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E10" s="123" t="n"/>
+      <c r="F10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>Translation DE-DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="261" t="inlineStr">
+        <is>
+          <t>FR-fr</t>
+        </is>
+      </c>
+      <c r="C11" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/pc-portables/windows11/</t>
+        </is>
+      </c>
+      <c r="D11" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E11" s="123" t="n"/>
+      <c r="F11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>Translation FR-FR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="261" t="inlineStr">
+        <is>
+          <t>AU-en</t>
+        </is>
+      </c>
+      <c r="C12" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D12" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E12" s="123" t="n"/>
+      <c r="F12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>Translation EN-GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="261" t="inlineStr">
+        <is>
+          <t>IN-en</t>
+        </is>
+      </c>
+      <c r="C13" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/laptop/windows-11/</t>
+        </is>
+      </c>
+      <c r="D13" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E13" s="123" t="n"/>
+      <c r="F13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="261" t="inlineStr">
+        <is>
+          <t>JP-ja</t>
+        </is>
+      </c>
+      <c r="C14" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/computer-pc/windows11/</t>
+        </is>
+      </c>
+      <c r="D14" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E14" s="123" t="n"/>
+      <c r="F14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>Translation JA-JP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="261" t="inlineStr">
+        <is>
+          <t>CN-zh</t>
+        </is>
+      </c>
+      <c r="C15" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/windows11</t>
+        </is>
+      </c>
+      <c r="D15" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E15" s="123" t="n"/>
+      <c r="F15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(zh-CN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="261" t="inlineStr">
+        <is>
+          <t>SG-en</t>
+        </is>
+      </c>
+      <c r="C16" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D16" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E16" s="123" t="n"/>
+      <c r="F16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="261" t="inlineStr">
+        <is>
+          <t>VN-vi</t>
+        </is>
+      </c>
+      <c r="C17" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/windows-11/</t>
+        </is>
+      </c>
+      <c r="D17" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E17" s="123" t="n"/>
+      <c r="F17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(vi-VN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="261" t="inlineStr">
+        <is>
+          <t>TW-zh</t>
+        </is>
+      </c>
+      <c r="C18" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D18" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E18" s="123" t="n"/>
+      <c r="F18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(zh-TW)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId15"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -40626,7 +41033,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>

</xml_diff>

<commit_message>
data(it): Windows 11 Home Landing을 W41로 옮긴다
Co-Authored-By: Grok 4.7 <noreply@x.ai>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -20,15 +20,15 @@
     <sheet name="W30 - SmartMonitor ScreenShare" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="W30 - UltraGear 1000Hz FAQ" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Windows 11 Landing" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="W31 - PDP Gallery Win11 Pro" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="W31 - Smart Monitor Multi AI" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="W32 - UltraGear 27GX704A" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="W32 - Digital Trends Award 삭제" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="W32 - UltraGear PDP 5모델" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="W32 - UltraFine PDP MIC 삭제" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="W38 - gram pro gallery" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="W41 - UltraGear Buying Guide 2차" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="W31 - PDP Gallery Win11 Pro" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="W31 - Smart Monitor Multi AI" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="W32 - UltraGear 27GX704A" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="W32 - Digital Trends Award 삭제" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="W32 - UltraGear PDP 5모델" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="W32 - UltraFine PDP MIC 삭제" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="W38 - gram pro gallery" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="W41 - UltraGear Buying Guide 2차" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="W41 - Windows 11 Landing" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14287,488 +14287,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="0" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" s="0" t="inlineStr">
-        <is>
-          <t>GR26-MS-IT Windows 11 Home Landing Page 업데이트</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t>이번주 추가</t>
-        </is>
-      </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t>예정 · 요청서 2026-10-07 기준 15사이트(Global 포함) · Due 2026-10-31 · 담당 정의현 책임</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0" t="inlineStr">
-        <is>
-          <t>Head</t>
-        </is>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="C3" s="0" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D3" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E3" s="0" t="inlineStr">
-        <is>
-          <t>완료일</t>
-        </is>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
-        <is>
-          <t>Page#</t>
-        </is>
-      </c>
-      <c r="G3" s="0" t="inlineStr">
-        <is>
-          <t>Remark</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="261" t="inlineStr">
-        <is>
-          <t>GLOBAL : GLOBAL (en)</t>
-        </is>
-      </c>
-      <c r="C4" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/global/laptops/windows-11/</t>
-        </is>
-      </c>
-      <c r="D4" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E4" s="123" t="n"/>
-      <c r="F4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="0" t="inlineStr">
-        <is>
-          <t>MS 참고본(English)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="261" t="inlineStr">
-        <is>
-          <t>CA-en</t>
-        </is>
-      </c>
-      <c r="C5" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/laptops/windows-11/</t>
-        </is>
-      </c>
-      <c r="D5" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E5" s="123" t="n"/>
-      <c r="F5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="0" t="inlineStr">
-        <is>
-          <t>MS 참고본(English)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="261" t="inlineStr">
-        <is>
-          <t>CA-fr</t>
-        </is>
-      </c>
-      <c r="C6" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_fr/page-de-presentation/decouvrez-choisirmc-lg-gram/windows-11/</t>
-        </is>
-      </c>
-      <c r="D6" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E6" s="123" t="n"/>
-      <c r="F6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="0" t="inlineStr">
-        <is>
-          <t>Translation FR-CA</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="261" t="inlineStr">
-        <is>
-          <t>ES-es</t>
-        </is>
-      </c>
-      <c r="C7" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/es/ordenadores/windows-11/</t>
-        </is>
-      </c>
-      <c r="D7" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E7" s="123" t="n"/>
-      <c r="F7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="0" t="inlineStr">
-        <is>
-          <t>Translation ES-ES</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="261" t="inlineStr">
-        <is>
-          <t>IT-it</t>
-        </is>
-      </c>
-      <c r="C8" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/it/notebook/windows-11/</t>
-        </is>
-      </c>
-      <c r="D8" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E8" s="123" t="n"/>
-      <c r="F8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="0" t="inlineStr">
-        <is>
-          <t>MS 참고본(It-LT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="261" t="inlineStr">
-        <is>
-          <t>UK-en</t>
-        </is>
-      </c>
-      <c r="C9" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/uk/laptops/windows-11/</t>
-        </is>
-      </c>
-      <c r="D9" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E9" s="123" t="n"/>
-      <c r="F9" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="0" t="inlineStr">
-        <is>
-          <t>Translation EN-GB</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="261" t="inlineStr">
-        <is>
-          <t>DE-de</t>
-        </is>
-      </c>
-      <c r="C10" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/de/notebooks/windows-11/</t>
-        </is>
-      </c>
-      <c r="D10" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E10" s="123" t="n"/>
-      <c r="F10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="0" t="inlineStr">
-        <is>
-          <t>Translation DE-DE</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="261" t="inlineStr">
-        <is>
-          <t>FR-fr</t>
-        </is>
-      </c>
-      <c r="C11" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/fr/pc-portables/windows11/</t>
-        </is>
-      </c>
-      <c r="D11" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E11" s="123" t="n"/>
-      <c r="F11" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="0" t="inlineStr">
-        <is>
-          <t>Translation FR-FR</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="261" t="inlineStr">
-        <is>
-          <t>AU-en</t>
-        </is>
-      </c>
-      <c r="C12" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/au/laptops/windows-11/</t>
-        </is>
-      </c>
-      <c r="D12" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E12" s="123" t="n"/>
-      <c r="F12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="0" t="inlineStr">
-        <is>
-          <t>Translation EN-GB</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="261" t="inlineStr">
-        <is>
-          <t>IN-en</t>
-        </is>
-      </c>
-      <c r="C13" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/in/laptop/windows-11/</t>
-        </is>
-      </c>
-      <c r="D13" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E13" s="123" t="n"/>
-      <c r="F13" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="0" t="inlineStr">
-        <is>
-          <t>MS 참고본(English)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="261" t="inlineStr">
-        <is>
-          <t>JP-ja</t>
-        </is>
-      </c>
-      <c r="C14" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/jp/computer-pc/windows11/</t>
-        </is>
-      </c>
-      <c r="D14" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E14" s="123" t="n"/>
-      <c r="F14" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="0" t="inlineStr">
-        <is>
-          <t>Translation JA-JP</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="261" t="inlineStr">
-        <is>
-          <t>CN-zh</t>
-        </is>
-      </c>
-      <c r="C15" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/cn/notebooks/windows11</t>
-        </is>
-      </c>
-      <c r="D15" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E15" s="123" t="n"/>
-      <c r="F15" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="0" t="inlineStr">
-        <is>
-          <t>MS 참고본(zh-CN)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="261" t="inlineStr">
-        <is>
-          <t>SG-en</t>
-        </is>
-      </c>
-      <c r="C16" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/sg/laptops/windows-11/</t>
-        </is>
-      </c>
-      <c r="D16" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E16" s="123" t="n"/>
-      <c r="F16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="0" t="inlineStr">
-        <is>
-          <t>MS 참고본(English)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="261" t="inlineStr">
-        <is>
-          <t>VN-vi</t>
-        </is>
-      </c>
-      <c r="C17" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/vn/laptop-lg-gram/windows-11/</t>
-        </is>
-      </c>
-      <c r="D17" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E17" s="123" t="n"/>
-      <c r="F17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="0" t="inlineStr">
-        <is>
-          <t>MS 참고본(vi-VN)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="261" t="inlineStr">
-        <is>
-          <t>TW-zh</t>
-        </is>
-      </c>
-      <c r="C18" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/tw/laptops/windows-11/</t>
-        </is>
-      </c>
-      <c r="D18" s="265" t="inlineStr">
-        <is>
-          <t>사전검토</t>
-        </is>
-      </c>
-      <c r="E18" s="123" t="n"/>
-      <c r="F18" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="0" t="inlineStr">
-        <is>
-          <t>MS 참고본(zh-TW)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId15"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -17289,967 +16807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AP16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="8.130000000000001" customWidth="1" style="203" min="1" max="1"/>
-    <col width="49.63" customWidth="1" style="203" min="4" max="4"/>
-    <col width="13" customWidth="1" style="203" min="39" max="39"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="35" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" s="36" t="inlineStr">
-        <is>
-          <t>GR26-W16-MS-IT-PC Copilot+ Filter Creation</t>
-        </is>
-      </c>
-      <c r="C1" s="37" t="n"/>
-      <c r="D1" s="37" t="n"/>
-      <c r="E1" s="37" t="n"/>
-      <c r="K1" s="37" t="n"/>
-      <c r="L1" s="37" t="n"/>
-      <c r="M1" s="37" t="n"/>
-      <c r="N1" s="37" t="n"/>
-      <c r="O1" s="37" t="n"/>
-      <c r="P1" s="37" t="n"/>
-      <c r="Q1" s="37" t="n"/>
-      <c r="R1" s="37" t="n"/>
-      <c r="S1" s="37" t="n"/>
-      <c r="T1" s="37" t="n"/>
-      <c r="U1" s="37" t="n"/>
-      <c r="V1" s="37" t="n"/>
-      <c r="W1" s="37" t="n"/>
-      <c r="X1" s="37" t="n"/>
-      <c r="Y1" s="37" t="n"/>
-      <c r="Z1" s="37" t="n"/>
-      <c r="AA1" s="37" t="n"/>
-      <c r="AB1" s="37" t="n"/>
-      <c r="AC1" s="37" t="n"/>
-      <c r="AD1" s="37" t="n"/>
-      <c r="AE1" s="37" t="n"/>
-      <c r="AF1" s="37" t="n"/>
-      <c r="AG1" s="37" t="n"/>
-      <c r="AH1" s="38" t="n"/>
-      <c r="AI1" s="38" t="n"/>
-      <c r="AJ1" s="38" t="n"/>
-      <c r="AK1" s="38" t="n"/>
-      <c r="AL1" s="38" t="n"/>
-      <c r="AM1" s="38" t="n"/>
-      <c r="AN1" s="39" t="n"/>
-      <c r="AO1" s="39" t="n"/>
-      <c r="AP1" s="39" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="40" t="inlineStr">
-        <is>
-          <t>이번주 추가</t>
-        </is>
-      </c>
-      <c r="B2" s="41" t="inlineStr">
-        <is>
-          <t>GLOBAL : 작업중 → 완료</t>
-        </is>
-      </c>
-      <c r="C2" s="37" t="n"/>
-      <c r="D2" s="37" t="n"/>
-      <c r="E2" s="37" t="n"/>
-      <c r="K2" s="37" t="n"/>
-      <c r="L2" s="37" t="n"/>
-      <c r="M2" s="37" t="n"/>
-      <c r="N2" s="37" t="n"/>
-      <c r="O2" s="37" t="n"/>
-      <c r="P2" s="37" t="n"/>
-      <c r="Q2" s="37" t="n"/>
-      <c r="R2" s="37" t="n"/>
-      <c r="S2" s="37" t="n"/>
-      <c r="T2" s="37" t="n"/>
-      <c r="U2" s="37" t="n"/>
-      <c r="V2" s="37" t="n"/>
-      <c r="W2" s="37" t="n"/>
-      <c r="X2" s="37" t="n"/>
-      <c r="Y2" s="37" t="n"/>
-      <c r="Z2" s="37" t="n"/>
-      <c r="AA2" s="37" t="n"/>
-      <c r="AB2" s="37" t="n"/>
-      <c r="AC2" s="37" t="n"/>
-      <c r="AD2" s="37" t="n"/>
-      <c r="AE2" s="37" t="n"/>
-      <c r="AF2" s="37" t="n"/>
-      <c r="AG2" s="37" t="n"/>
-      <c r="AH2" s="38" t="n"/>
-      <c r="AI2" s="38" t="n"/>
-      <c r="AJ2" s="38" t="n"/>
-      <c r="AK2" s="38" t="n"/>
-      <c r="AL2" s="38" t="n"/>
-      <c r="AM2" s="38" t="n"/>
-      <c r="AN2" s="39" t="n"/>
-      <c r="AO2" s="39" t="n"/>
-      <c r="AP2" s="39" t="n"/>
-    </row>
-    <row r="3" ht="42.75" customHeight="1" s="203">
-      <c r="D3" s="37" t="n"/>
-      <c r="E3" s="37" t="n"/>
-      <c r="K3" s="37" t="n"/>
-      <c r="L3" s="37" t="n"/>
-      <c r="M3" s="37" t="n"/>
-      <c r="N3" s="37" t="n"/>
-      <c r="O3" s="37" t="n"/>
-      <c r="P3" s="37" t="n"/>
-      <c r="Q3" s="37" t="n"/>
-      <c r="R3" s="37" t="n"/>
-      <c r="S3" s="37" t="n"/>
-      <c r="T3" s="37" t="n"/>
-      <c r="U3" s="37" t="n"/>
-      <c r="V3" s="37" t="n"/>
-      <c r="W3" s="37" t="n"/>
-      <c r="X3" s="37" t="n"/>
-      <c r="Y3" s="37" t="n"/>
-      <c r="Z3" s="37" t="n"/>
-      <c r="AA3" s="37" t="n"/>
-      <c r="AB3" s="37" t="n"/>
-      <c r="AC3" s="37" t="n"/>
-      <c r="AD3" s="37" t="n"/>
-      <c r="AE3" s="37" t="n"/>
-      <c r="AF3" s="37" t="n"/>
-      <c r="AG3" s="37" t="n"/>
-      <c r="AH3" s="38" t="n"/>
-      <c r="AI3" s="38" t="n"/>
-      <c r="AJ3" s="38" t="n"/>
-      <c r="AK3" s="38" t="n"/>
-      <c r="AL3" s="38" t="n"/>
-      <c r="AM3" s="38" t="n"/>
-      <c r="AN3" s="39" t="n"/>
-      <c r="AO3" s="39" t="n"/>
-      <c r="AP3" s="39" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="42" t="n"/>
-      <c r="B4" s="37" t="n"/>
-      <c r="C4" s="37" t="n"/>
-      <c r="D4" s="37" t="n"/>
-      <c r="E4" s="37" t="n"/>
-      <c r="F4" s="37" t="n"/>
-      <c r="G4" s="37" t="n"/>
-      <c r="H4" s="37" t="n"/>
-      <c r="I4" s="37" t="n"/>
-      <c r="J4" s="37" t="n"/>
-      <c r="K4" s="37" t="n"/>
-      <c r="L4" s="37" t="n"/>
-      <c r="M4" s="37" t="n"/>
-      <c r="N4" s="37" t="n"/>
-      <c r="O4" s="37" t="n"/>
-      <c r="P4" s="37" t="n"/>
-      <c r="Q4" s="37" t="n"/>
-      <c r="R4" s="37" t="n"/>
-      <c r="S4" s="37" t="n"/>
-      <c r="T4" s="37" t="n"/>
-      <c r="U4" s="37" t="n"/>
-      <c r="V4" s="37" t="n"/>
-      <c r="W4" s="37" t="n"/>
-      <c r="X4" s="37" t="n"/>
-      <c r="Y4" s="37" t="n"/>
-      <c r="Z4" s="37" t="n"/>
-      <c r="AA4" s="37" t="n"/>
-      <c r="AB4" s="37" t="n"/>
-      <c r="AC4" s="37" t="n"/>
-      <c r="AD4" s="37" t="n"/>
-      <c r="AE4" s="37" t="n"/>
-      <c r="AF4" s="37" t="n"/>
-      <c r="AG4" s="37" t="n"/>
-      <c r="AH4" s="38" t="n"/>
-      <c r="AI4" s="38" t="n"/>
-      <c r="AJ4" s="38" t="n"/>
-      <c r="AK4" s="38" t="n"/>
-      <c r="AL4" s="38" t="n"/>
-      <c r="AM4" s="38" t="n"/>
-      <c r="AN4" s="39" t="n"/>
-      <c r="AO4" s="39" t="n"/>
-      <c r="AP4" s="39" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="280" t="inlineStr">
-        <is>
-          <t>Head</t>
-        </is>
-      </c>
-      <c r="B5" s="219" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="C5" s="219" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D5" s="219" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E5" s="219" t="inlineStr">
-        <is>
-          <t>완료일</t>
-        </is>
-      </c>
-      <c r="F5" s="219" t="inlineStr">
-        <is>
-          <t>Page#</t>
-        </is>
-      </c>
-      <c r="G5" s="219" t="inlineStr">
-        <is>
-          <t>Remark</t>
-        </is>
-      </c>
-      <c r="H5" s="219" t="n"/>
-      <c r="I5" s="219" t="n"/>
-      <c r="J5" s="283" t="n"/>
-      <c r="K5" s="219" t="n"/>
-      <c r="L5" s="219" t="n"/>
-      <c r="M5" s="219" t="n"/>
-      <c r="N5" s="219" t="n"/>
-      <c r="O5" s="219" t="n"/>
-      <c r="P5" s="219" t="n"/>
-      <c r="Q5" s="219" t="n"/>
-      <c r="R5" s="219" t="n"/>
-      <c r="S5" s="219" t="n"/>
-      <c r="T5" s="283" t="n"/>
-      <c r="U5" s="283" t="n"/>
-      <c r="V5" s="283" t="n"/>
-      <c r="W5" s="219" t="n"/>
-      <c r="X5" s="219" t="n"/>
-      <c r="Y5" s="219" t="n"/>
-      <c r="Z5" s="219" t="n"/>
-      <c r="AA5" s="219" t="n"/>
-      <c r="AB5" s="219" t="n"/>
-      <c r="AC5" s="283" t="n"/>
-      <c r="AD5" s="283" t="n"/>
-      <c r="AE5" s="219" t="n"/>
-      <c r="AF5" s="219" t="n"/>
-      <c r="AG5" s="219" t="n"/>
-      <c r="AH5" s="283" t="n"/>
-      <c r="AI5" s="283" t="n"/>
-      <c r="AJ5" s="283" t="n"/>
-      <c r="AK5" s="283" t="n"/>
-      <c r="AL5" s="283" t="n"/>
-      <c r="AM5" s="283" t="n"/>
-      <c r="AN5" s="55" t="n"/>
-      <c r="AO5" s="55" t="n"/>
-      <c r="AP5" s="55" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="220" t="n"/>
-      <c r="B6" s="113" t="inlineStr">
-        <is>
-          <t>AU : AU (en)</t>
-        </is>
-      </c>
-      <c r="C6" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/au/laptops/gram/16z90tl-g-au88a/</t>
-        </is>
-      </c>
-      <c r="D6" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E6" s="223" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="F6" s="224" t="n">
-        <v>4</v>
-      </c>
-      <c r="G6" s="225" t="inlineStr"/>
-      <c r="H6" s="224" t="inlineStr"/>
-      <c r="I6" s="225" t="inlineStr"/>
-      <c r="J6" s="224" t="inlineStr"/>
-      <c r="K6" s="226" t="inlineStr"/>
-      <c r="L6" s="226" t="n"/>
-      <c r="M6" s="226" t="inlineStr"/>
-      <c r="N6" s="226" t="inlineStr"/>
-      <c r="O6" s="227" t="inlineStr"/>
-      <c r="P6" s="113" t="inlineStr"/>
-      <c r="Q6" s="113" t="inlineStr"/>
-      <c r="R6" s="226" t="inlineStr"/>
-      <c r="S6" s="228" t="n"/>
-      <c r="T6" s="228" t="n"/>
-      <c r="U6" s="228" t="n"/>
-      <c r="V6" s="228" t="n"/>
-      <c r="W6" s="228" t="inlineStr"/>
-      <c r="X6" s="228" t="n"/>
-      <c r="Y6" s="228" t="n"/>
-      <c r="Z6" s="228" t="n"/>
-      <c r="AA6" s="228" t="inlineStr"/>
-      <c r="AB6" s="228" t="inlineStr"/>
-      <c r="AC6" s="228" t="inlineStr"/>
-      <c r="AD6" s="228" t="inlineStr"/>
-      <c r="AE6" s="228" t="inlineStr"/>
-      <c r="AF6" s="229" t="inlineStr"/>
-      <c r="AG6" s="230" t="inlineStr"/>
-      <c r="AH6" s="55" t="inlineStr"/>
-      <c r="AI6" s="55" t="inlineStr"/>
-      <c r="AJ6" s="55" t="inlineStr"/>
-      <c r="AK6" s="55" t="n"/>
-      <c r="AL6" s="55" t="n"/>
-      <c r="AM6" s="55" t="n"/>
-      <c r="AN6" s="55" t="inlineStr"/>
-      <c r="AO6" s="55" t="inlineStr"/>
-      <c r="AP6" s="55" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="220" t="n"/>
-      <c r="B7" s="113" t="inlineStr">
-        <is>
-          <t>CA_EN : CA (en)</t>
-        </is>
-      </c>
-      <c r="C7" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/ca_en/laptops/gram/17z90tl-g-au78a9/</t>
-        </is>
-      </c>
-      <c r="D7" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E7" s="223" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F7" s="224" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="225" t="inlineStr"/>
-      <c r="H7" s="224" t="inlineStr"/>
-      <c r="I7" s="225" t="inlineStr"/>
-      <c r="J7" s="224" t="inlineStr"/>
-      <c r="K7" s="226" t="inlineStr"/>
-      <c r="L7" s="226" t="inlineStr"/>
-      <c r="M7" s="226" t="inlineStr"/>
-      <c r="N7" s="226" t="inlineStr"/>
-      <c r="O7" s="227" t="inlineStr"/>
-      <c r="P7" s="113" t="inlineStr"/>
-      <c r="Q7" s="113" t="inlineStr"/>
-      <c r="R7" s="226" t="inlineStr"/>
-      <c r="S7" s="228" t="inlineStr"/>
-      <c r="T7" s="228" t="inlineStr"/>
-      <c r="U7" s="228" t="inlineStr"/>
-      <c r="V7" s="228" t="inlineStr"/>
-      <c r="W7" s="228" t="inlineStr"/>
-      <c r="X7" s="228" t="inlineStr"/>
-      <c r="Y7" s="228" t="inlineStr"/>
-      <c r="Z7" s="228" t="inlineStr"/>
-      <c r="AA7" s="228" t="inlineStr"/>
-      <c r="AB7" s="228" t="inlineStr"/>
-      <c r="AC7" s="228" t="inlineStr"/>
-      <c r="AD7" s="228" t="inlineStr"/>
-      <c r="AE7" s="228" t="inlineStr"/>
-      <c r="AF7" s="229" t="inlineStr"/>
-      <c r="AG7" s="230" t="inlineStr"/>
-      <c r="AH7" s="55" t="inlineStr"/>
-      <c r="AI7" s="55" t="inlineStr"/>
-      <c r="AJ7" s="55" t="inlineStr"/>
-      <c r="AK7" s="55" t="inlineStr"/>
-      <c r="AL7" s="55" t="inlineStr"/>
-      <c r="AM7" s="55" t="inlineStr"/>
-      <c r="AN7" s="55" t="inlineStr"/>
-      <c r="AO7" s="55" t="inlineStr"/>
-      <c r="AP7" s="55" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="220" t="n"/>
-      <c r="B8" s="113" t="inlineStr">
-        <is>
-          <t>DE : DE (de)</t>
-        </is>
-      </c>
-      <c r="C8" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/de/notebooks/gram-pro/16z90ts-g-au89g/</t>
-        </is>
-      </c>
-      <c r="D8" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E8" s="231" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F8" s="232" t="n">
-        <v>8</v>
-      </c>
-      <c r="G8" s="225" t="inlineStr"/>
-      <c r="H8" s="225" t="inlineStr"/>
-      <c r="I8" s="224" t="inlineStr"/>
-      <c r="J8" s="224" t="inlineStr"/>
-      <c r="K8" s="228" t="inlineStr"/>
-      <c r="L8" s="228" t="inlineStr"/>
-      <c r="M8" s="228" t="inlineStr"/>
-      <c r="N8" s="228" t="inlineStr"/>
-      <c r="O8" s="229" t="inlineStr"/>
-      <c r="P8" s="113" t="inlineStr"/>
-      <c r="Q8" s="113" t="inlineStr"/>
-      <c r="R8" s="226" t="inlineStr"/>
-      <c r="S8" s="228" t="inlineStr"/>
-      <c r="T8" s="228" t="inlineStr"/>
-      <c r="U8" s="228" t="inlineStr"/>
-      <c r="V8" s="228" t="inlineStr"/>
-      <c r="W8" s="228" t="inlineStr"/>
-      <c r="X8" s="228" t="inlineStr"/>
-      <c r="Y8" s="228" t="inlineStr"/>
-      <c r="Z8" s="228" t="inlineStr"/>
-      <c r="AA8" s="228" t="inlineStr"/>
-      <c r="AB8" s="228" t="inlineStr"/>
-      <c r="AC8" s="228" t="inlineStr"/>
-      <c r="AD8" s="228" t="inlineStr"/>
-      <c r="AE8" s="228" t="inlineStr"/>
-      <c r="AF8" s="229" t="inlineStr"/>
-      <c r="AG8" s="230" t="inlineStr"/>
-      <c r="AH8" s="55" t="inlineStr"/>
-      <c r="AI8" s="55" t="inlineStr"/>
-      <c r="AJ8" s="55" t="inlineStr"/>
-      <c r="AK8" s="55" t="inlineStr"/>
-      <c r="AL8" s="55" t="inlineStr"/>
-      <c r="AM8" s="55" t="inlineStr"/>
-      <c r="AN8" s="55" t="inlineStr"/>
-      <c r="AO8" s="55" t="inlineStr"/>
-      <c r="AP8" s="55" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="220" t="n"/>
-      <c r="B9" s="113" t="inlineStr">
-        <is>
-          <t>ES : ES (es)</t>
-        </is>
-      </c>
-      <c r="C9" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/es/portatiles/gram/16z90ts-g-au99b/</t>
-        </is>
-      </c>
-      <c r="D9" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E9" s="231" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F9" s="232" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="225" t="inlineStr"/>
-      <c r="H9" s="225" t="inlineStr"/>
-      <c r="I9" s="225" t="inlineStr"/>
-      <c r="J9" s="224" t="inlineStr"/>
-      <c r="K9" s="228" t="inlineStr"/>
-      <c r="L9" s="228" t="inlineStr"/>
-      <c r="M9" s="228" t="inlineStr"/>
-      <c r="N9" s="228" t="inlineStr"/>
-      <c r="O9" s="229" t="inlineStr"/>
-      <c r="P9" s="113" t="inlineStr"/>
-      <c r="Q9" s="113" t="inlineStr"/>
-      <c r="R9" s="226" t="inlineStr"/>
-      <c r="S9" s="228" t="inlineStr"/>
-      <c r="T9" s="228" t="inlineStr"/>
-      <c r="U9" s="228" t="inlineStr"/>
-      <c r="V9" s="228" t="inlineStr"/>
-      <c r="W9" s="228" t="inlineStr"/>
-      <c r="X9" s="228" t="inlineStr"/>
-      <c r="Y9" s="228" t="inlineStr"/>
-      <c r="Z9" s="228" t="inlineStr"/>
-      <c r="AA9" s="228" t="inlineStr"/>
-      <c r="AB9" s="228" t="inlineStr"/>
-      <c r="AC9" s="228" t="inlineStr"/>
-      <c r="AD9" s="228" t="inlineStr"/>
-      <c r="AE9" s="228" t="inlineStr"/>
-      <c r="AF9" s="229" t="inlineStr"/>
-      <c r="AG9" s="230" t="inlineStr"/>
-      <c r="AH9" s="55" t="inlineStr"/>
-      <c r="AI9" s="55" t="inlineStr"/>
-      <c r="AJ9" s="55" t="inlineStr"/>
-      <c r="AK9" s="55" t="inlineStr"/>
-      <c r="AL9" s="55" t="inlineStr"/>
-      <c r="AM9" s="55" t="inlineStr"/>
-      <c r="AN9" s="55" t="inlineStr"/>
-      <c r="AO9" s="55" t="inlineStr"/>
-      <c r="AP9" s="55" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="220" t="n"/>
-      <c r="B10" s="113" t="inlineStr">
-        <is>
-          <t>FR : FR (fr)</t>
-        </is>
-      </c>
-      <c r="C10" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/fr/pc-portables/gram/lg-15z80t-g-as55f/</t>
-        </is>
-      </c>
-      <c r="D10" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E10" s="231" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F10" s="225" t="n">
-        <v>14</v>
-      </c>
-      <c r="G10" s="225" t="inlineStr"/>
-      <c r="H10" s="225" t="inlineStr"/>
-      <c r="I10" s="225" t="inlineStr"/>
-      <c r="J10" s="224" t="inlineStr"/>
-      <c r="K10" s="228" t="inlineStr"/>
-      <c r="L10" s="228" t="inlineStr"/>
-      <c r="M10" s="228" t="inlineStr"/>
-      <c r="N10" s="228" t="inlineStr"/>
-      <c r="O10" s="229" t="inlineStr"/>
-      <c r="P10" s="113" t="inlineStr"/>
-      <c r="Q10" s="113" t="inlineStr"/>
-      <c r="R10" s="226" t="inlineStr"/>
-      <c r="S10" s="228" t="inlineStr"/>
-      <c r="T10" s="228" t="inlineStr"/>
-      <c r="U10" s="228" t="inlineStr"/>
-      <c r="V10" s="228" t="inlineStr"/>
-      <c r="W10" s="228" t="inlineStr"/>
-      <c r="X10" s="228" t="inlineStr"/>
-      <c r="Y10" s="228" t="inlineStr"/>
-      <c r="Z10" s="228" t="inlineStr"/>
-      <c r="AA10" s="228" t="inlineStr"/>
-      <c r="AB10" s="228" t="inlineStr"/>
-      <c r="AC10" s="228" t="inlineStr"/>
-      <c r="AD10" s="228" t="inlineStr"/>
-      <c r="AE10" s="228" t="inlineStr"/>
-      <c r="AF10" s="229" t="inlineStr"/>
-      <c r="AG10" s="230" t="inlineStr"/>
-      <c r="AH10" s="55" t="inlineStr"/>
-      <c r="AI10" s="55" t="inlineStr"/>
-      <c r="AJ10" s="55" t="inlineStr"/>
-      <c r="AK10" s="55" t="inlineStr"/>
-      <c r="AL10" s="55" t="inlineStr"/>
-      <c r="AM10" s="55" t="inlineStr"/>
-      <c r="AN10" s="55" t="inlineStr"/>
-      <c r="AO10" s="55" t="inlineStr"/>
-      <c r="AP10" s="55" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="220" t="n"/>
-      <c r="B11" s="113" t="inlineStr">
-        <is>
-          <t>GLOBAL : GLOBAL (en)</t>
-        </is>
-      </c>
-      <c r="C11" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/16z90ts/</t>
-        </is>
-      </c>
-      <c r="D11" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E11" s="231" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F11" s="225" t="n">
-        <v>4</v>
-      </c>
-      <c r="G11" s="225" t="inlineStr"/>
-      <c r="H11" s="224" t="inlineStr"/>
-      <c r="I11" s="224" t="inlineStr"/>
-      <c r="J11" s="224" t="inlineStr"/>
-      <c r="K11" s="228" t="inlineStr"/>
-      <c r="L11" s="228" t="inlineStr"/>
-      <c r="M11" s="228" t="inlineStr"/>
-      <c r="N11" s="228" t="inlineStr"/>
-      <c r="O11" s="229" t="inlineStr"/>
-      <c r="P11" s="113" t="inlineStr"/>
-      <c r="Q11" s="113" t="inlineStr"/>
-      <c r="R11" s="226" t="inlineStr"/>
-      <c r="S11" s="228" t="inlineStr"/>
-      <c r="T11" s="228" t="inlineStr"/>
-      <c r="U11" s="228" t="inlineStr"/>
-      <c r="V11" s="228" t="inlineStr"/>
-      <c r="W11" s="228" t="inlineStr"/>
-      <c r="X11" s="228" t="inlineStr"/>
-      <c r="Y11" s="228" t="inlineStr"/>
-      <c r="Z11" s="228" t="inlineStr"/>
-      <c r="AA11" s="228" t="inlineStr"/>
-      <c r="AB11" s="228" t="inlineStr"/>
-      <c r="AC11" s="228" t="inlineStr"/>
-      <c r="AD11" s="228" t="inlineStr"/>
-      <c r="AE11" s="228" t="inlineStr"/>
-      <c r="AF11" s="229" t="inlineStr"/>
-      <c r="AG11" s="230" t="inlineStr"/>
-      <c r="AH11" s="55" t="inlineStr"/>
-      <c r="AI11" s="55" t="inlineStr"/>
-      <c r="AJ11" s="55" t="inlineStr"/>
-      <c r="AK11" s="55" t="inlineStr"/>
-      <c r="AL11" s="55" t="inlineStr"/>
-      <c r="AM11" s="55" t="inlineStr"/>
-      <c r="AN11" s="55" t="inlineStr"/>
-      <c r="AO11" s="55" t="inlineStr"/>
-      <c r="AP11" s="55" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="220" t="n"/>
-      <c r="B12" s="113" t="inlineStr">
-        <is>
-          <t>IT : IT (it)</t>
-        </is>
-      </c>
-      <c r="C12" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/it/notebook/gram/17z90tl-g/</t>
-        </is>
-      </c>
-      <c r="D12" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E12" s="231" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F12" s="232" t="n">
-        <v>7</v>
-      </c>
-      <c r="G12" s="225" t="inlineStr"/>
-      <c r="H12" s="224" t="inlineStr"/>
-      <c r="I12" s="225" t="inlineStr"/>
-      <c r="J12" s="224" t="inlineStr"/>
-      <c r="K12" s="228" t="inlineStr"/>
-      <c r="L12" s="228" t="inlineStr"/>
-      <c r="M12" s="228" t="inlineStr"/>
-      <c r="N12" s="228" t="inlineStr"/>
-      <c r="O12" s="229" t="inlineStr"/>
-      <c r="P12" s="113" t="inlineStr"/>
-      <c r="Q12" s="113" t="inlineStr"/>
-      <c r="R12" s="226" t="inlineStr"/>
-      <c r="S12" s="228" t="inlineStr"/>
-      <c r="T12" s="228" t="inlineStr"/>
-      <c r="U12" s="228" t="inlineStr"/>
-      <c r="V12" s="228" t="inlineStr"/>
-      <c r="W12" s="228" t="inlineStr"/>
-      <c r="X12" s="228" t="inlineStr"/>
-      <c r="Y12" s="228" t="inlineStr"/>
-      <c r="Z12" s="228" t="inlineStr"/>
-      <c r="AA12" s="228" t="inlineStr"/>
-      <c r="AB12" s="228" t="inlineStr"/>
-      <c r="AC12" s="228" t="inlineStr"/>
-      <c r="AD12" s="228" t="inlineStr"/>
-      <c r="AE12" s="228" t="inlineStr"/>
-      <c r="AF12" s="229" t="inlineStr"/>
-      <c r="AG12" s="230" t="inlineStr"/>
-      <c r="AH12" s="55" t="inlineStr"/>
-      <c r="AI12" s="55" t="inlineStr"/>
-      <c r="AJ12" s="55" t="inlineStr"/>
-      <c r="AK12" s="55" t="inlineStr"/>
-      <c r="AL12" s="55" t="inlineStr"/>
-      <c r="AM12" s="55" t="inlineStr"/>
-      <c r="AN12" s="55" t="inlineStr"/>
-      <c r="AO12" s="55" t="inlineStr"/>
-      <c r="AP12" s="55" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="220" t="n"/>
-      <c r="B13" s="113" t="inlineStr">
-        <is>
-          <t>JP : JP (ja)</t>
-        </is>
-      </c>
-      <c r="C13" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/jp/mobile-pc/gram/16z90ts-gu86j/</t>
-        </is>
-      </c>
-      <c r="D13" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E13" s="234" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F13" s="232" t="n">
-        <v>27</v>
-      </c>
-      <c r="G13" s="225" t="inlineStr"/>
-      <c r="H13" s="225" t="inlineStr"/>
-      <c r="I13" s="225" t="inlineStr"/>
-      <c r="J13" s="224" t="inlineStr"/>
-      <c r="K13" s="228" t="inlineStr"/>
-      <c r="L13" s="228" t="inlineStr"/>
-      <c r="M13" s="228" t="inlineStr"/>
-      <c r="N13" s="228" t="inlineStr"/>
-      <c r="O13" s="229" t="inlineStr"/>
-      <c r="P13" s="113" t="inlineStr"/>
-      <c r="Q13" s="113" t="inlineStr"/>
-      <c r="R13" s="226" t="inlineStr"/>
-      <c r="S13" s="228" t="inlineStr"/>
-      <c r="T13" s="228" t="inlineStr"/>
-      <c r="U13" s="228" t="inlineStr"/>
-      <c r="V13" s="228" t="inlineStr"/>
-      <c r="W13" s="228" t="inlineStr"/>
-      <c r="X13" s="228" t="inlineStr"/>
-      <c r="Y13" s="228" t="inlineStr"/>
-      <c r="Z13" s="228" t="inlineStr"/>
-      <c r="AA13" s="228" t="inlineStr"/>
-      <c r="AB13" s="228" t="inlineStr"/>
-      <c r="AC13" s="228" t="inlineStr"/>
-      <c r="AD13" s="228" t="inlineStr"/>
-      <c r="AE13" s="228" t="inlineStr"/>
-      <c r="AF13" s="229" t="inlineStr"/>
-      <c r="AG13" s="230" t="inlineStr"/>
-      <c r="AH13" s="55" t="inlineStr"/>
-      <c r="AI13" s="55" t="inlineStr"/>
-      <c r="AJ13" s="55" t="inlineStr"/>
-      <c r="AK13" s="55" t="inlineStr"/>
-      <c r="AL13" s="55" t="inlineStr"/>
-      <c r="AM13" s="55" t="inlineStr"/>
-      <c r="AN13" s="55" t="inlineStr"/>
-      <c r="AO13" s="55" t="inlineStr"/>
-      <c r="AP13" s="55" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="220" t="n"/>
-      <c r="B14" s="113" t="inlineStr">
-        <is>
-          <t>SG : SG (en)</t>
-        </is>
-      </c>
-      <c r="C14" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90tl-g-az88a3/</t>
-        </is>
-      </c>
-      <c r="D14" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E14" s="231" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F14" s="225" t="n">
-        <v>13</v>
-      </c>
-      <c r="G14" s="225" t="inlineStr"/>
-      <c r="H14" s="225" t="inlineStr"/>
-      <c r="I14" s="225" t="inlineStr"/>
-      <c r="J14" s="224" t="inlineStr"/>
-      <c r="K14" s="228" t="inlineStr"/>
-      <c r="L14" s="228" t="inlineStr"/>
-      <c r="M14" s="228" t="inlineStr"/>
-      <c r="N14" s="228" t="inlineStr"/>
-      <c r="O14" s="229" t="inlineStr"/>
-      <c r="P14" s="113" t="inlineStr"/>
-      <c r="Q14" s="113" t="inlineStr"/>
-      <c r="R14" s="226" t="inlineStr"/>
-      <c r="S14" s="228" t="inlineStr"/>
-      <c r="T14" s="228" t="inlineStr"/>
-      <c r="U14" s="228" t="inlineStr"/>
-      <c r="V14" s="228" t="inlineStr"/>
-      <c r="W14" s="228" t="inlineStr"/>
-      <c r="X14" s="228" t="inlineStr"/>
-      <c r="Y14" s="228" t="inlineStr"/>
-      <c r="Z14" s="228" t="inlineStr"/>
-      <c r="AA14" s="228" t="inlineStr"/>
-      <c r="AB14" s="228" t="inlineStr"/>
-      <c r="AC14" s="228" t="inlineStr"/>
-      <c r="AD14" s="228" t="inlineStr"/>
-      <c r="AE14" s="228" t="inlineStr"/>
-      <c r="AF14" s="229" t="inlineStr"/>
-      <c r="AG14" s="230" t="inlineStr"/>
-      <c r="AH14" s="55" t="inlineStr"/>
-      <c r="AI14" s="55" t="inlineStr"/>
-      <c r="AJ14" s="55" t="inlineStr"/>
-      <c r="AK14" s="55" t="inlineStr"/>
-      <c r="AL14" s="55" t="inlineStr"/>
-      <c r="AM14" s="55" t="inlineStr"/>
-      <c r="AN14" s="55" t="inlineStr"/>
-      <c r="AO14" s="55" t="inlineStr"/>
-      <c r="AP14" s="55" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="220" t="n"/>
-      <c r="B15" s="113" t="inlineStr">
-        <is>
-          <t>TW : TW (zh)</t>
-        </is>
-      </c>
-      <c r="C15" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/tw/laptops/gram-pro/16z90ts-g-au79c2/</t>
-        </is>
-      </c>
-      <c r="D15" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E15" s="231" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F15" s="232" t="n">
-        <v>18</v>
-      </c>
-      <c r="G15" s="225" t="inlineStr"/>
-      <c r="H15" s="225" t="inlineStr"/>
-      <c r="I15" s="225" t="inlineStr"/>
-      <c r="J15" s="224" t="inlineStr"/>
-      <c r="K15" s="228" t="inlineStr"/>
-      <c r="L15" s="228" t="inlineStr"/>
-      <c r="M15" s="228" t="inlineStr"/>
-      <c r="N15" s="228" t="inlineStr"/>
-      <c r="O15" s="229" t="inlineStr"/>
-      <c r="P15" s="113" t="inlineStr"/>
-      <c r="Q15" s="113" t="inlineStr"/>
-      <c r="R15" s="226" t="inlineStr"/>
-      <c r="S15" s="235" t="inlineStr"/>
-      <c r="T15" s="235" t="inlineStr"/>
-      <c r="U15" s="235" t="inlineStr"/>
-      <c r="V15" s="235" t="inlineStr"/>
-      <c r="W15" s="235" t="inlineStr"/>
-      <c r="X15" s="235" t="inlineStr"/>
-      <c r="Y15" s="235" t="inlineStr"/>
-      <c r="Z15" s="235" t="inlineStr"/>
-      <c r="AA15" s="235" t="inlineStr"/>
-      <c r="AB15" s="235" t="inlineStr"/>
-      <c r="AC15" s="235" t="inlineStr"/>
-      <c r="AD15" s="235" t="inlineStr"/>
-      <c r="AE15" s="235" t="inlineStr"/>
-      <c r="AF15" s="236" t="inlineStr"/>
-      <c r="AG15" s="230" t="inlineStr"/>
-      <c r="AH15" s="55" t="inlineStr"/>
-      <c r="AI15" s="55" t="inlineStr"/>
-      <c r="AJ15" s="55" t="inlineStr"/>
-      <c r="AK15" s="55" t="inlineStr"/>
-      <c r="AL15" s="55" t="inlineStr"/>
-      <c r="AM15" s="55" t="inlineStr"/>
-      <c r="AN15" s="55" t="inlineStr"/>
-      <c r="AO15" s="55" t="inlineStr"/>
-      <c r="AP15" s="55" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="220" t="n"/>
-      <c r="B16" s="113" t="inlineStr">
-        <is>
-          <t>UK : GB (en)</t>
-        </is>
-      </c>
-      <c r="C16" s="290" t="inlineStr">
-        <is>
-          <t>https://www.lg.com/uk/laptops/gram-pro/16z90ts-g-au89a1/</t>
-        </is>
-      </c>
-      <c r="D16" s="222" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="E16" s="228" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F16" s="225" t="n">
-        <v>8</v>
-      </c>
-      <c r="G16" s="228" t="inlineStr"/>
-      <c r="H16" s="228" t="inlineStr"/>
-      <c r="I16" s="228" t="inlineStr"/>
-      <c r="J16" s="228" t="inlineStr"/>
-      <c r="K16" s="228" t="inlineStr"/>
-      <c r="L16" s="228" t="inlineStr"/>
-      <c r="M16" s="228" t="inlineStr"/>
-      <c r="N16" s="228" t="inlineStr"/>
-      <c r="O16" s="229" t="inlineStr"/>
-      <c r="P16" s="113" t="inlineStr"/>
-      <c r="Q16" s="113" t="inlineStr"/>
-      <c r="R16" s="226" t="inlineStr"/>
-      <c r="S16" s="237" t="n"/>
-      <c r="T16" s="223" t="n"/>
-      <c r="U16" s="223" t="n"/>
-      <c r="V16" s="223" t="n"/>
-      <c r="W16" s="226" t="inlineStr"/>
-      <c r="X16" s="226" t="inlineStr"/>
-      <c r="Y16" s="226" t="inlineStr"/>
-      <c r="Z16" s="226" t="inlineStr"/>
-      <c r="AA16" s="226" t="inlineStr"/>
-      <c r="AB16" s="226" t="inlineStr"/>
-      <c r="AC16" s="226" t="inlineStr"/>
-      <c r="AD16" s="226" t="inlineStr"/>
-      <c r="AE16" s="226" t="inlineStr"/>
-      <c r="AF16" s="227" t="inlineStr"/>
-      <c r="AG16" s="230" t="inlineStr"/>
-      <c r="AH16" s="55" t="inlineStr"/>
-      <c r="AI16" s="55" t="inlineStr"/>
-      <c r="AJ16" s="55" t="inlineStr"/>
-      <c r="AK16" s="55" t="inlineStr"/>
-      <c r="AL16" s="55" t="inlineStr"/>
-      <c r="AM16" s="55" t="inlineStr"/>
-      <c r="AN16" s="55" t="inlineStr"/>
-      <c r="AO16" s="55" t="inlineStr"/>
-      <c r="AP16" s="55" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId11"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20054,7 +18612,967 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AP16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="8.130000000000001" customWidth="1" style="203" min="1" max="1"/>
+    <col width="49.63" customWidth="1" style="203" min="4" max="4"/>
+    <col width="13" customWidth="1" style="203" min="39" max="39"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="36" t="inlineStr">
+        <is>
+          <t>GR26-W16-MS-IT-PC Copilot+ Filter Creation</t>
+        </is>
+      </c>
+      <c r="C1" s="37" t="n"/>
+      <c r="D1" s="37" t="n"/>
+      <c r="E1" s="37" t="n"/>
+      <c r="K1" s="37" t="n"/>
+      <c r="L1" s="37" t="n"/>
+      <c r="M1" s="37" t="n"/>
+      <c r="N1" s="37" t="n"/>
+      <c r="O1" s="37" t="n"/>
+      <c r="P1" s="37" t="n"/>
+      <c r="Q1" s="37" t="n"/>
+      <c r="R1" s="37" t="n"/>
+      <c r="S1" s="37" t="n"/>
+      <c r="T1" s="37" t="n"/>
+      <c r="U1" s="37" t="n"/>
+      <c r="V1" s="37" t="n"/>
+      <c r="W1" s="37" t="n"/>
+      <c r="X1" s="37" t="n"/>
+      <c r="Y1" s="37" t="n"/>
+      <c r="Z1" s="37" t="n"/>
+      <c r="AA1" s="37" t="n"/>
+      <c r="AB1" s="37" t="n"/>
+      <c r="AC1" s="37" t="n"/>
+      <c r="AD1" s="37" t="n"/>
+      <c r="AE1" s="37" t="n"/>
+      <c r="AF1" s="37" t="n"/>
+      <c r="AG1" s="37" t="n"/>
+      <c r="AH1" s="38" t="n"/>
+      <c r="AI1" s="38" t="n"/>
+      <c r="AJ1" s="38" t="n"/>
+      <c r="AK1" s="38" t="n"/>
+      <c r="AL1" s="38" t="n"/>
+      <c r="AM1" s="38" t="n"/>
+      <c r="AN1" s="39" t="n"/>
+      <c r="AO1" s="39" t="n"/>
+      <c r="AP1" s="39" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" s="41" t="inlineStr">
+        <is>
+          <t>GLOBAL : 작업중 → 완료</t>
+        </is>
+      </c>
+      <c r="C2" s="37" t="n"/>
+      <c r="D2" s="37" t="n"/>
+      <c r="E2" s="37" t="n"/>
+      <c r="K2" s="37" t="n"/>
+      <c r="L2" s="37" t="n"/>
+      <c r="M2" s="37" t="n"/>
+      <c r="N2" s="37" t="n"/>
+      <c r="O2" s="37" t="n"/>
+      <c r="P2" s="37" t="n"/>
+      <c r="Q2" s="37" t="n"/>
+      <c r="R2" s="37" t="n"/>
+      <c r="S2" s="37" t="n"/>
+      <c r="T2" s="37" t="n"/>
+      <c r="U2" s="37" t="n"/>
+      <c r="V2" s="37" t="n"/>
+      <c r="W2" s="37" t="n"/>
+      <c r="X2" s="37" t="n"/>
+      <c r="Y2" s="37" t="n"/>
+      <c r="Z2" s="37" t="n"/>
+      <c r="AA2" s="37" t="n"/>
+      <c r="AB2" s="37" t="n"/>
+      <c r="AC2" s="37" t="n"/>
+      <c r="AD2" s="37" t="n"/>
+      <c r="AE2" s="37" t="n"/>
+      <c r="AF2" s="37" t="n"/>
+      <c r="AG2" s="37" t="n"/>
+      <c r="AH2" s="38" t="n"/>
+      <c r="AI2" s="38" t="n"/>
+      <c r="AJ2" s="38" t="n"/>
+      <c r="AK2" s="38" t="n"/>
+      <c r="AL2" s="38" t="n"/>
+      <c r="AM2" s="38" t="n"/>
+      <c r="AN2" s="39" t="n"/>
+      <c r="AO2" s="39" t="n"/>
+      <c r="AP2" s="39" t="n"/>
+    </row>
+    <row r="3" ht="42.75" customHeight="1" s="203">
+      <c r="D3" s="37" t="n"/>
+      <c r="E3" s="37" t="n"/>
+      <c r="K3" s="37" t="n"/>
+      <c r="L3" s="37" t="n"/>
+      <c r="M3" s="37" t="n"/>
+      <c r="N3" s="37" t="n"/>
+      <c r="O3" s="37" t="n"/>
+      <c r="P3" s="37" t="n"/>
+      <c r="Q3" s="37" t="n"/>
+      <c r="R3" s="37" t="n"/>
+      <c r="S3" s="37" t="n"/>
+      <c r="T3" s="37" t="n"/>
+      <c r="U3" s="37" t="n"/>
+      <c r="V3" s="37" t="n"/>
+      <c r="W3" s="37" t="n"/>
+      <c r="X3" s="37" t="n"/>
+      <c r="Y3" s="37" t="n"/>
+      <c r="Z3" s="37" t="n"/>
+      <c r="AA3" s="37" t="n"/>
+      <c r="AB3" s="37" t="n"/>
+      <c r="AC3" s="37" t="n"/>
+      <c r="AD3" s="37" t="n"/>
+      <c r="AE3" s="37" t="n"/>
+      <c r="AF3" s="37" t="n"/>
+      <c r="AG3" s="37" t="n"/>
+      <c r="AH3" s="38" t="n"/>
+      <c r="AI3" s="38" t="n"/>
+      <c r="AJ3" s="38" t="n"/>
+      <c r="AK3" s="38" t="n"/>
+      <c r="AL3" s="38" t="n"/>
+      <c r="AM3" s="38" t="n"/>
+      <c r="AN3" s="39" t="n"/>
+      <c r="AO3" s="39" t="n"/>
+      <c r="AP3" s="39" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="42" t="n"/>
+      <c r="B4" s="37" t="n"/>
+      <c r="C4" s="37" t="n"/>
+      <c r="D4" s="37" t="n"/>
+      <c r="E4" s="37" t="n"/>
+      <c r="F4" s="37" t="n"/>
+      <c r="G4" s="37" t="n"/>
+      <c r="H4" s="37" t="n"/>
+      <c r="I4" s="37" t="n"/>
+      <c r="J4" s="37" t="n"/>
+      <c r="K4" s="37" t="n"/>
+      <c r="L4" s="37" t="n"/>
+      <c r="M4" s="37" t="n"/>
+      <c r="N4" s="37" t="n"/>
+      <c r="O4" s="37" t="n"/>
+      <c r="P4" s="37" t="n"/>
+      <c r="Q4" s="37" t="n"/>
+      <c r="R4" s="37" t="n"/>
+      <c r="S4" s="37" t="n"/>
+      <c r="T4" s="37" t="n"/>
+      <c r="U4" s="37" t="n"/>
+      <c r="V4" s="37" t="n"/>
+      <c r="W4" s="37" t="n"/>
+      <c r="X4" s="37" t="n"/>
+      <c r="Y4" s="37" t="n"/>
+      <c r="Z4" s="37" t="n"/>
+      <c r="AA4" s="37" t="n"/>
+      <c r="AB4" s="37" t="n"/>
+      <c r="AC4" s="37" t="n"/>
+      <c r="AD4" s="37" t="n"/>
+      <c r="AE4" s="37" t="n"/>
+      <c r="AF4" s="37" t="n"/>
+      <c r="AG4" s="37" t="n"/>
+      <c r="AH4" s="38" t="n"/>
+      <c r="AI4" s="38" t="n"/>
+      <c r="AJ4" s="38" t="n"/>
+      <c r="AK4" s="38" t="n"/>
+      <c r="AL4" s="38" t="n"/>
+      <c r="AM4" s="38" t="n"/>
+      <c r="AN4" s="39" t="n"/>
+      <c r="AO4" s="39" t="n"/>
+      <c r="AP4" s="39" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="280" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B5" s="219" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C5" s="219" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D5" s="219" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E5" s="219" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F5" s="219" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G5" s="219" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+      <c r="H5" s="219" t="n"/>
+      <c r="I5" s="219" t="n"/>
+      <c r="J5" s="283" t="n"/>
+      <c r="K5" s="219" t="n"/>
+      <c r="L5" s="219" t="n"/>
+      <c r="M5" s="219" t="n"/>
+      <c r="N5" s="219" t="n"/>
+      <c r="O5" s="219" t="n"/>
+      <c r="P5" s="219" t="n"/>
+      <c r="Q5" s="219" t="n"/>
+      <c r="R5" s="219" t="n"/>
+      <c r="S5" s="219" t="n"/>
+      <c r="T5" s="283" t="n"/>
+      <c r="U5" s="283" t="n"/>
+      <c r="V5" s="283" t="n"/>
+      <c r="W5" s="219" t="n"/>
+      <c r="X5" s="219" t="n"/>
+      <c r="Y5" s="219" t="n"/>
+      <c r="Z5" s="219" t="n"/>
+      <c r="AA5" s="219" t="n"/>
+      <c r="AB5" s="219" t="n"/>
+      <c r="AC5" s="283" t="n"/>
+      <c r="AD5" s="283" t="n"/>
+      <c r="AE5" s="219" t="n"/>
+      <c r="AF5" s="219" t="n"/>
+      <c r="AG5" s="219" t="n"/>
+      <c r="AH5" s="283" t="n"/>
+      <c r="AI5" s="283" t="n"/>
+      <c r="AJ5" s="283" t="n"/>
+      <c r="AK5" s="283" t="n"/>
+      <c r="AL5" s="283" t="n"/>
+      <c r="AM5" s="283" t="n"/>
+      <c r="AN5" s="55" t="n"/>
+      <c r="AO5" s="55" t="n"/>
+      <c r="AP5" s="55" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="220" t="n"/>
+      <c r="B6" s="113" t="inlineStr">
+        <is>
+          <t>AU : AU (en)</t>
+        </is>
+      </c>
+      <c r="C6" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/gram/16z90tl-g-au88a/</t>
+        </is>
+      </c>
+      <c r="D6" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E6" s="223" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="F6" s="224" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="225" t="inlineStr"/>
+      <c r="H6" s="224" t="inlineStr"/>
+      <c r="I6" s="225" t="inlineStr"/>
+      <c r="J6" s="224" t="inlineStr"/>
+      <c r="K6" s="226" t="inlineStr"/>
+      <c r="L6" s="226" t="n"/>
+      <c r="M6" s="226" t="inlineStr"/>
+      <c r="N6" s="226" t="inlineStr"/>
+      <c r="O6" s="227" t="inlineStr"/>
+      <c r="P6" s="113" t="inlineStr"/>
+      <c r="Q6" s="113" t="inlineStr"/>
+      <c r="R6" s="226" t="inlineStr"/>
+      <c r="S6" s="228" t="n"/>
+      <c r="T6" s="228" t="n"/>
+      <c r="U6" s="228" t="n"/>
+      <c r="V6" s="228" t="n"/>
+      <c r="W6" s="228" t="inlineStr"/>
+      <c r="X6" s="228" t="n"/>
+      <c r="Y6" s="228" t="n"/>
+      <c r="Z6" s="228" t="n"/>
+      <c r="AA6" s="228" t="inlineStr"/>
+      <c r="AB6" s="228" t="inlineStr"/>
+      <c r="AC6" s="228" t="inlineStr"/>
+      <c r="AD6" s="228" t="inlineStr"/>
+      <c r="AE6" s="228" t="inlineStr"/>
+      <c r="AF6" s="229" t="inlineStr"/>
+      <c r="AG6" s="230" t="inlineStr"/>
+      <c r="AH6" s="55" t="inlineStr"/>
+      <c r="AI6" s="55" t="inlineStr"/>
+      <c r="AJ6" s="55" t="inlineStr"/>
+      <c r="AK6" s="55" t="n"/>
+      <c r="AL6" s="55" t="n"/>
+      <c r="AM6" s="55" t="n"/>
+      <c r="AN6" s="55" t="inlineStr"/>
+      <c r="AO6" s="55" t="inlineStr"/>
+      <c r="AP6" s="55" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="220" t="n"/>
+      <c r="B7" s="113" t="inlineStr">
+        <is>
+          <t>CA_EN : CA (en)</t>
+        </is>
+      </c>
+      <c r="C7" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/gram/17z90tl-g-au78a9/</t>
+        </is>
+      </c>
+      <c r="D7" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E7" s="223" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F7" s="224" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="225" t="inlineStr"/>
+      <c r="H7" s="224" t="inlineStr"/>
+      <c r="I7" s="225" t="inlineStr"/>
+      <c r="J7" s="224" t="inlineStr"/>
+      <c r="K7" s="226" t="inlineStr"/>
+      <c r="L7" s="226" t="inlineStr"/>
+      <c r="M7" s="226" t="inlineStr"/>
+      <c r="N7" s="226" t="inlineStr"/>
+      <c r="O7" s="227" t="inlineStr"/>
+      <c r="P7" s="113" t="inlineStr"/>
+      <c r="Q7" s="113" t="inlineStr"/>
+      <c r="R7" s="226" t="inlineStr"/>
+      <c r="S7" s="228" t="inlineStr"/>
+      <c r="T7" s="228" t="inlineStr"/>
+      <c r="U7" s="228" t="inlineStr"/>
+      <c r="V7" s="228" t="inlineStr"/>
+      <c r="W7" s="228" t="inlineStr"/>
+      <c r="X7" s="228" t="inlineStr"/>
+      <c r="Y7" s="228" t="inlineStr"/>
+      <c r="Z7" s="228" t="inlineStr"/>
+      <c r="AA7" s="228" t="inlineStr"/>
+      <c r="AB7" s="228" t="inlineStr"/>
+      <c r="AC7" s="228" t="inlineStr"/>
+      <c r="AD7" s="228" t="inlineStr"/>
+      <c r="AE7" s="228" t="inlineStr"/>
+      <c r="AF7" s="229" t="inlineStr"/>
+      <c r="AG7" s="230" t="inlineStr"/>
+      <c r="AH7" s="55" t="inlineStr"/>
+      <c r="AI7" s="55" t="inlineStr"/>
+      <c r="AJ7" s="55" t="inlineStr"/>
+      <c r="AK7" s="55" t="inlineStr"/>
+      <c r="AL7" s="55" t="inlineStr"/>
+      <c r="AM7" s="55" t="inlineStr"/>
+      <c r="AN7" s="55" t="inlineStr"/>
+      <c r="AO7" s="55" t="inlineStr"/>
+      <c r="AP7" s="55" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="220" t="n"/>
+      <c r="B8" s="113" t="inlineStr">
+        <is>
+          <t>DE : DE (de)</t>
+        </is>
+      </c>
+      <c r="C8" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/gram-pro/16z90ts-g-au89g/</t>
+        </is>
+      </c>
+      <c r="D8" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E8" s="231" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F8" s="232" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" s="225" t="inlineStr"/>
+      <c r="H8" s="225" t="inlineStr"/>
+      <c r="I8" s="224" t="inlineStr"/>
+      <c r="J8" s="224" t="inlineStr"/>
+      <c r="K8" s="228" t="inlineStr"/>
+      <c r="L8" s="228" t="inlineStr"/>
+      <c r="M8" s="228" t="inlineStr"/>
+      <c r="N8" s="228" t="inlineStr"/>
+      <c r="O8" s="229" t="inlineStr"/>
+      <c r="P8" s="113" t="inlineStr"/>
+      <c r="Q8" s="113" t="inlineStr"/>
+      <c r="R8" s="226" t="inlineStr"/>
+      <c r="S8" s="228" t="inlineStr"/>
+      <c r="T8" s="228" t="inlineStr"/>
+      <c r="U8" s="228" t="inlineStr"/>
+      <c r="V8" s="228" t="inlineStr"/>
+      <c r="W8" s="228" t="inlineStr"/>
+      <c r="X8" s="228" t="inlineStr"/>
+      <c r="Y8" s="228" t="inlineStr"/>
+      <c r="Z8" s="228" t="inlineStr"/>
+      <c r="AA8" s="228" t="inlineStr"/>
+      <c r="AB8" s="228" t="inlineStr"/>
+      <c r="AC8" s="228" t="inlineStr"/>
+      <c r="AD8" s="228" t="inlineStr"/>
+      <c r="AE8" s="228" t="inlineStr"/>
+      <c r="AF8" s="229" t="inlineStr"/>
+      <c r="AG8" s="230" t="inlineStr"/>
+      <c r="AH8" s="55" t="inlineStr"/>
+      <c r="AI8" s="55" t="inlineStr"/>
+      <c r="AJ8" s="55" t="inlineStr"/>
+      <c r="AK8" s="55" t="inlineStr"/>
+      <c r="AL8" s="55" t="inlineStr"/>
+      <c r="AM8" s="55" t="inlineStr"/>
+      <c r="AN8" s="55" t="inlineStr"/>
+      <c r="AO8" s="55" t="inlineStr"/>
+      <c r="AP8" s="55" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="220" t="n"/>
+      <c r="B9" s="113" t="inlineStr">
+        <is>
+          <t>ES : ES (es)</t>
+        </is>
+      </c>
+      <c r="C9" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/portatiles/gram/16z90ts-g-au99b/</t>
+        </is>
+      </c>
+      <c r="D9" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E9" s="231" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F9" s="232" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="225" t="inlineStr"/>
+      <c r="H9" s="225" t="inlineStr"/>
+      <c r="I9" s="225" t="inlineStr"/>
+      <c r="J9" s="224" t="inlineStr"/>
+      <c r="K9" s="228" t="inlineStr"/>
+      <c r="L9" s="228" t="inlineStr"/>
+      <c r="M9" s="228" t="inlineStr"/>
+      <c r="N9" s="228" t="inlineStr"/>
+      <c r="O9" s="229" t="inlineStr"/>
+      <c r="P9" s="113" t="inlineStr"/>
+      <c r="Q9" s="113" t="inlineStr"/>
+      <c r="R9" s="226" t="inlineStr"/>
+      <c r="S9" s="228" t="inlineStr"/>
+      <c r="T9" s="228" t="inlineStr"/>
+      <c r="U9" s="228" t="inlineStr"/>
+      <c r="V9" s="228" t="inlineStr"/>
+      <c r="W9" s="228" t="inlineStr"/>
+      <c r="X9" s="228" t="inlineStr"/>
+      <c r="Y9" s="228" t="inlineStr"/>
+      <c r="Z9" s="228" t="inlineStr"/>
+      <c r="AA9" s="228" t="inlineStr"/>
+      <c r="AB9" s="228" t="inlineStr"/>
+      <c r="AC9" s="228" t="inlineStr"/>
+      <c r="AD9" s="228" t="inlineStr"/>
+      <c r="AE9" s="228" t="inlineStr"/>
+      <c r="AF9" s="229" t="inlineStr"/>
+      <c r="AG9" s="230" t="inlineStr"/>
+      <c r="AH9" s="55" t="inlineStr"/>
+      <c r="AI9" s="55" t="inlineStr"/>
+      <c r="AJ9" s="55" t="inlineStr"/>
+      <c r="AK9" s="55" t="inlineStr"/>
+      <c r="AL9" s="55" t="inlineStr"/>
+      <c r="AM9" s="55" t="inlineStr"/>
+      <c r="AN9" s="55" t="inlineStr"/>
+      <c r="AO9" s="55" t="inlineStr"/>
+      <c r="AP9" s="55" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="220" t="n"/>
+      <c r="B10" s="113" t="inlineStr">
+        <is>
+          <t>FR : FR (fr)</t>
+        </is>
+      </c>
+      <c r="C10" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/pc-portables/gram/lg-15z80t-g-as55f/</t>
+        </is>
+      </c>
+      <c r="D10" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E10" s="231" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F10" s="225" t="n">
+        <v>14</v>
+      </c>
+      <c r="G10" s="225" t="inlineStr"/>
+      <c r="H10" s="225" t="inlineStr"/>
+      <c r="I10" s="225" t="inlineStr"/>
+      <c r="J10" s="224" t="inlineStr"/>
+      <c r="K10" s="228" t="inlineStr"/>
+      <c r="L10" s="228" t="inlineStr"/>
+      <c r="M10" s="228" t="inlineStr"/>
+      <c r="N10" s="228" t="inlineStr"/>
+      <c r="O10" s="229" t="inlineStr"/>
+      <c r="P10" s="113" t="inlineStr"/>
+      <c r="Q10" s="113" t="inlineStr"/>
+      <c r="R10" s="226" t="inlineStr"/>
+      <c r="S10" s="228" t="inlineStr"/>
+      <c r="T10" s="228" t="inlineStr"/>
+      <c r="U10" s="228" t="inlineStr"/>
+      <c r="V10" s="228" t="inlineStr"/>
+      <c r="W10" s="228" t="inlineStr"/>
+      <c r="X10" s="228" t="inlineStr"/>
+      <c r="Y10" s="228" t="inlineStr"/>
+      <c r="Z10" s="228" t="inlineStr"/>
+      <c r="AA10" s="228" t="inlineStr"/>
+      <c r="AB10" s="228" t="inlineStr"/>
+      <c r="AC10" s="228" t="inlineStr"/>
+      <c r="AD10" s="228" t="inlineStr"/>
+      <c r="AE10" s="228" t="inlineStr"/>
+      <c r="AF10" s="229" t="inlineStr"/>
+      <c r="AG10" s="230" t="inlineStr"/>
+      <c r="AH10" s="55" t="inlineStr"/>
+      <c r="AI10" s="55" t="inlineStr"/>
+      <c r="AJ10" s="55" t="inlineStr"/>
+      <c r="AK10" s="55" t="inlineStr"/>
+      <c r="AL10" s="55" t="inlineStr"/>
+      <c r="AM10" s="55" t="inlineStr"/>
+      <c r="AN10" s="55" t="inlineStr"/>
+      <c r="AO10" s="55" t="inlineStr"/>
+      <c r="AP10" s="55" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="220" t="n"/>
+      <c r="B11" s="113" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C11" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/business/monitors-pcs/laptops/gram-pro/16z90ts/</t>
+        </is>
+      </c>
+      <c r="D11" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E11" s="231" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F11" s="225" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="225" t="inlineStr"/>
+      <c r="H11" s="224" t="inlineStr"/>
+      <c r="I11" s="224" t="inlineStr"/>
+      <c r="J11" s="224" t="inlineStr"/>
+      <c r="K11" s="228" t="inlineStr"/>
+      <c r="L11" s="228" t="inlineStr"/>
+      <c r="M11" s="228" t="inlineStr"/>
+      <c r="N11" s="228" t="inlineStr"/>
+      <c r="O11" s="229" t="inlineStr"/>
+      <c r="P11" s="113" t="inlineStr"/>
+      <c r="Q11" s="113" t="inlineStr"/>
+      <c r="R11" s="226" t="inlineStr"/>
+      <c r="S11" s="228" t="inlineStr"/>
+      <c r="T11" s="228" t="inlineStr"/>
+      <c r="U11" s="228" t="inlineStr"/>
+      <c r="V11" s="228" t="inlineStr"/>
+      <c r="W11" s="228" t="inlineStr"/>
+      <c r="X11" s="228" t="inlineStr"/>
+      <c r="Y11" s="228" t="inlineStr"/>
+      <c r="Z11" s="228" t="inlineStr"/>
+      <c r="AA11" s="228" t="inlineStr"/>
+      <c r="AB11" s="228" t="inlineStr"/>
+      <c r="AC11" s="228" t="inlineStr"/>
+      <c r="AD11" s="228" t="inlineStr"/>
+      <c r="AE11" s="228" t="inlineStr"/>
+      <c r="AF11" s="229" t="inlineStr"/>
+      <c r="AG11" s="230" t="inlineStr"/>
+      <c r="AH11" s="55" t="inlineStr"/>
+      <c r="AI11" s="55" t="inlineStr"/>
+      <c r="AJ11" s="55" t="inlineStr"/>
+      <c r="AK11" s="55" t="inlineStr"/>
+      <c r="AL11" s="55" t="inlineStr"/>
+      <c r="AM11" s="55" t="inlineStr"/>
+      <c r="AN11" s="55" t="inlineStr"/>
+      <c r="AO11" s="55" t="inlineStr"/>
+      <c r="AP11" s="55" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="220" t="n"/>
+      <c r="B12" s="113" t="inlineStr">
+        <is>
+          <t>IT : IT (it)</t>
+        </is>
+      </c>
+      <c r="C12" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/gram/17z90tl-g/</t>
+        </is>
+      </c>
+      <c r="D12" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E12" s="231" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F12" s="232" t="n">
+        <v>7</v>
+      </c>
+      <c r="G12" s="225" t="inlineStr"/>
+      <c r="H12" s="224" t="inlineStr"/>
+      <c r="I12" s="225" t="inlineStr"/>
+      <c r="J12" s="224" t="inlineStr"/>
+      <c r="K12" s="228" t="inlineStr"/>
+      <c r="L12" s="228" t="inlineStr"/>
+      <c r="M12" s="228" t="inlineStr"/>
+      <c r="N12" s="228" t="inlineStr"/>
+      <c r="O12" s="229" t="inlineStr"/>
+      <c r="P12" s="113" t="inlineStr"/>
+      <c r="Q12" s="113" t="inlineStr"/>
+      <c r="R12" s="226" t="inlineStr"/>
+      <c r="S12" s="228" t="inlineStr"/>
+      <c r="T12" s="228" t="inlineStr"/>
+      <c r="U12" s="228" t="inlineStr"/>
+      <c r="V12" s="228" t="inlineStr"/>
+      <c r="W12" s="228" t="inlineStr"/>
+      <c r="X12" s="228" t="inlineStr"/>
+      <c r="Y12" s="228" t="inlineStr"/>
+      <c r="Z12" s="228" t="inlineStr"/>
+      <c r="AA12" s="228" t="inlineStr"/>
+      <c r="AB12" s="228" t="inlineStr"/>
+      <c r="AC12" s="228" t="inlineStr"/>
+      <c r="AD12" s="228" t="inlineStr"/>
+      <c r="AE12" s="228" t="inlineStr"/>
+      <c r="AF12" s="229" t="inlineStr"/>
+      <c r="AG12" s="230" t="inlineStr"/>
+      <c r="AH12" s="55" t="inlineStr"/>
+      <c r="AI12" s="55" t="inlineStr"/>
+      <c r="AJ12" s="55" t="inlineStr"/>
+      <c r="AK12" s="55" t="inlineStr"/>
+      <c r="AL12" s="55" t="inlineStr"/>
+      <c r="AM12" s="55" t="inlineStr"/>
+      <c r="AN12" s="55" t="inlineStr"/>
+      <c r="AO12" s="55" t="inlineStr"/>
+      <c r="AP12" s="55" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="220" t="n"/>
+      <c r="B13" s="113" t="inlineStr">
+        <is>
+          <t>JP : JP (ja)</t>
+        </is>
+      </c>
+      <c r="C13" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/mobile-pc/gram/16z90ts-gu86j/</t>
+        </is>
+      </c>
+      <c r="D13" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E13" s="234" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F13" s="232" t="n">
+        <v>27</v>
+      </c>
+      <c r="G13" s="225" t="inlineStr"/>
+      <c r="H13" s="225" t="inlineStr"/>
+      <c r="I13" s="225" t="inlineStr"/>
+      <c r="J13" s="224" t="inlineStr"/>
+      <c r="K13" s="228" t="inlineStr"/>
+      <c r="L13" s="228" t="inlineStr"/>
+      <c r="M13" s="228" t="inlineStr"/>
+      <c r="N13" s="228" t="inlineStr"/>
+      <c r="O13" s="229" t="inlineStr"/>
+      <c r="P13" s="113" t="inlineStr"/>
+      <c r="Q13" s="113" t="inlineStr"/>
+      <c r="R13" s="226" t="inlineStr"/>
+      <c r="S13" s="228" t="inlineStr"/>
+      <c r="T13" s="228" t="inlineStr"/>
+      <c r="U13" s="228" t="inlineStr"/>
+      <c r="V13" s="228" t="inlineStr"/>
+      <c r="W13" s="228" t="inlineStr"/>
+      <c r="X13" s="228" t="inlineStr"/>
+      <c r="Y13" s="228" t="inlineStr"/>
+      <c r="Z13" s="228" t="inlineStr"/>
+      <c r="AA13" s="228" t="inlineStr"/>
+      <c r="AB13" s="228" t="inlineStr"/>
+      <c r="AC13" s="228" t="inlineStr"/>
+      <c r="AD13" s="228" t="inlineStr"/>
+      <c r="AE13" s="228" t="inlineStr"/>
+      <c r="AF13" s="229" t="inlineStr"/>
+      <c r="AG13" s="230" t="inlineStr"/>
+      <c r="AH13" s="55" t="inlineStr"/>
+      <c r="AI13" s="55" t="inlineStr"/>
+      <c r="AJ13" s="55" t="inlineStr"/>
+      <c r="AK13" s="55" t="inlineStr"/>
+      <c r="AL13" s="55" t="inlineStr"/>
+      <c r="AM13" s="55" t="inlineStr"/>
+      <c r="AN13" s="55" t="inlineStr"/>
+      <c r="AO13" s="55" t="inlineStr"/>
+      <c r="AP13" s="55" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="220" t="n"/>
+      <c r="B14" s="113" t="inlineStr">
+        <is>
+          <t>SG : SG (en)</t>
+        </is>
+      </c>
+      <c r="C14" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/business/it-products/lg-gram/16z90tl-g-az88a3/</t>
+        </is>
+      </c>
+      <c r="D14" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E14" s="231" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F14" s="225" t="n">
+        <v>13</v>
+      </c>
+      <c r="G14" s="225" t="inlineStr"/>
+      <c r="H14" s="225" t="inlineStr"/>
+      <c r="I14" s="225" t="inlineStr"/>
+      <c r="J14" s="224" t="inlineStr"/>
+      <c r="K14" s="228" t="inlineStr"/>
+      <c r="L14" s="228" t="inlineStr"/>
+      <c r="M14" s="228" t="inlineStr"/>
+      <c r="N14" s="228" t="inlineStr"/>
+      <c r="O14" s="229" t="inlineStr"/>
+      <c r="P14" s="113" t="inlineStr"/>
+      <c r="Q14" s="113" t="inlineStr"/>
+      <c r="R14" s="226" t="inlineStr"/>
+      <c r="S14" s="228" t="inlineStr"/>
+      <c r="T14" s="228" t="inlineStr"/>
+      <c r="U14" s="228" t="inlineStr"/>
+      <c r="V14" s="228" t="inlineStr"/>
+      <c r="W14" s="228" t="inlineStr"/>
+      <c r="X14" s="228" t="inlineStr"/>
+      <c r="Y14" s="228" t="inlineStr"/>
+      <c r="Z14" s="228" t="inlineStr"/>
+      <c r="AA14" s="228" t="inlineStr"/>
+      <c r="AB14" s="228" t="inlineStr"/>
+      <c r="AC14" s="228" t="inlineStr"/>
+      <c r="AD14" s="228" t="inlineStr"/>
+      <c r="AE14" s="228" t="inlineStr"/>
+      <c r="AF14" s="229" t="inlineStr"/>
+      <c r="AG14" s="230" t="inlineStr"/>
+      <c r="AH14" s="55" t="inlineStr"/>
+      <c r="AI14" s="55" t="inlineStr"/>
+      <c r="AJ14" s="55" t="inlineStr"/>
+      <c r="AK14" s="55" t="inlineStr"/>
+      <c r="AL14" s="55" t="inlineStr"/>
+      <c r="AM14" s="55" t="inlineStr"/>
+      <c r="AN14" s="55" t="inlineStr"/>
+      <c r="AO14" s="55" t="inlineStr"/>
+      <c r="AP14" s="55" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="220" t="n"/>
+      <c r="B15" s="113" t="inlineStr">
+        <is>
+          <t>TW : TW (zh)</t>
+        </is>
+      </c>
+      <c r="C15" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/gram-pro/16z90ts-g-au79c2/</t>
+        </is>
+      </c>
+      <c r="D15" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E15" s="231" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F15" s="232" t="n">
+        <v>18</v>
+      </c>
+      <c r="G15" s="225" t="inlineStr"/>
+      <c r="H15" s="225" t="inlineStr"/>
+      <c r="I15" s="225" t="inlineStr"/>
+      <c r="J15" s="224" t="inlineStr"/>
+      <c r="K15" s="228" t="inlineStr"/>
+      <c r="L15" s="228" t="inlineStr"/>
+      <c r="M15" s="228" t="inlineStr"/>
+      <c r="N15" s="228" t="inlineStr"/>
+      <c r="O15" s="229" t="inlineStr"/>
+      <c r="P15" s="113" t="inlineStr"/>
+      <c r="Q15" s="113" t="inlineStr"/>
+      <c r="R15" s="226" t="inlineStr"/>
+      <c r="S15" s="235" t="inlineStr"/>
+      <c r="T15" s="235" t="inlineStr"/>
+      <c r="U15" s="235" t="inlineStr"/>
+      <c r="V15" s="235" t="inlineStr"/>
+      <c r="W15" s="235" t="inlineStr"/>
+      <c r="X15" s="235" t="inlineStr"/>
+      <c r="Y15" s="235" t="inlineStr"/>
+      <c r="Z15" s="235" t="inlineStr"/>
+      <c r="AA15" s="235" t="inlineStr"/>
+      <c r="AB15" s="235" t="inlineStr"/>
+      <c r="AC15" s="235" t="inlineStr"/>
+      <c r="AD15" s="235" t="inlineStr"/>
+      <c r="AE15" s="235" t="inlineStr"/>
+      <c r="AF15" s="236" t="inlineStr"/>
+      <c r="AG15" s="230" t="inlineStr"/>
+      <c r="AH15" s="55" t="inlineStr"/>
+      <c r="AI15" s="55" t="inlineStr"/>
+      <c r="AJ15" s="55" t="inlineStr"/>
+      <c r="AK15" s="55" t="inlineStr"/>
+      <c r="AL15" s="55" t="inlineStr"/>
+      <c r="AM15" s="55" t="inlineStr"/>
+      <c r="AN15" s="55" t="inlineStr"/>
+      <c r="AO15" s="55" t="inlineStr"/>
+      <c r="AP15" s="55" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="220" t="n"/>
+      <c r="B16" s="113" t="inlineStr">
+        <is>
+          <t>UK : GB (en)</t>
+        </is>
+      </c>
+      <c r="C16" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/laptops/gram-pro/16z90ts-g-au89a1/</t>
+        </is>
+      </c>
+      <c r="D16" s="222" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="E16" s="228" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F16" s="225" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="228" t="inlineStr"/>
+      <c r="H16" s="228" t="inlineStr"/>
+      <c r="I16" s="228" t="inlineStr"/>
+      <c r="J16" s="228" t="inlineStr"/>
+      <c r="K16" s="228" t="inlineStr"/>
+      <c r="L16" s="228" t="inlineStr"/>
+      <c r="M16" s="228" t="inlineStr"/>
+      <c r="N16" s="228" t="inlineStr"/>
+      <c r="O16" s="229" t="inlineStr"/>
+      <c r="P16" s="113" t="inlineStr"/>
+      <c r="Q16" s="113" t="inlineStr"/>
+      <c r="R16" s="226" t="inlineStr"/>
+      <c r="S16" s="237" t="n"/>
+      <c r="T16" s="223" t="n"/>
+      <c r="U16" s="223" t="n"/>
+      <c r="V16" s="223" t="n"/>
+      <c r="W16" s="226" t="inlineStr"/>
+      <c r="X16" s="226" t="inlineStr"/>
+      <c r="Y16" s="226" t="inlineStr"/>
+      <c r="Z16" s="226" t="inlineStr"/>
+      <c r="AA16" s="226" t="inlineStr"/>
+      <c r="AB16" s="226" t="inlineStr"/>
+      <c r="AC16" s="226" t="inlineStr"/>
+      <c r="AD16" s="226" t="inlineStr"/>
+      <c r="AE16" s="226" t="inlineStr"/>
+      <c r="AF16" s="227" t="inlineStr"/>
+      <c r="AG16" s="230" t="inlineStr"/>
+      <c r="AH16" s="55" t="inlineStr"/>
+      <c r="AI16" s="55" t="inlineStr"/>
+      <c r="AJ16" s="55" t="inlineStr"/>
+      <c r="AK16" s="55" t="inlineStr"/>
+      <c r="AL16" s="55" t="inlineStr"/>
+      <c r="AM16" s="55" t="inlineStr"/>
+      <c r="AN16" s="55" t="inlineStr"/>
+      <c r="AO16" s="55" t="inlineStr"/>
+      <c r="AP16" s="55" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId11"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21763,7 +21281,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -35483,7 +35001,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -38168,7 +37686,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40002,7 +39520,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40987,7 +40505,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -42581,6 +42099,489 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId42"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>GR26-W41-MS-IT Windows 11 Home Landing Page 업데이트</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>이번주 추가</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>예정 · 요청서 2026-10-07 기준 15사이트(Global 포함) · Due 2026-10-31 · 담당 정의현 책임</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Page#</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="261" t="inlineStr">
+        <is>
+          <t>GLOBAL : GLOBAL (en)</t>
+        </is>
+      </c>
+      <c r="C4" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/global/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D4" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E4" s="123" t="n"/>
+      <c r="F4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="261" t="inlineStr">
+        <is>
+          <t>CA-en</t>
+        </is>
+      </c>
+      <c r="C5" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_en/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D5" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E5" s="123" t="n"/>
+      <c r="F5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="261" t="inlineStr">
+        <is>
+          <t>CA-fr</t>
+        </is>
+      </c>
+      <c r="C6" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/ca_fr/page-de-presentation/decouvrez-choisirmc-lg-gram/windows-11/</t>
+        </is>
+      </c>
+      <c r="D6" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E6" s="123" t="n"/>
+      <c r="F6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>Translation FR-CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="261" t="inlineStr">
+        <is>
+          <t>ES-es</t>
+        </is>
+      </c>
+      <c r="C7" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/es/ordenadores/windows-11/</t>
+        </is>
+      </c>
+      <c r="D7" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E7" s="123" t="n"/>
+      <c r="F7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>Translation ES-ES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="261" t="inlineStr">
+        <is>
+          <t>IT-it</t>
+        </is>
+      </c>
+      <c r="C8" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/it/notebook/windows-11/</t>
+        </is>
+      </c>
+      <c r="D8" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E8" s="123" t="n"/>
+      <c r="F8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(It-LT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="261" t="inlineStr">
+        <is>
+          <t>UK-en</t>
+        </is>
+      </c>
+      <c r="C9" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/uk/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D9" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E9" s="123" t="n"/>
+      <c r="F9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>Translation EN-GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="261" t="inlineStr">
+        <is>
+          <t>DE-de</t>
+        </is>
+      </c>
+      <c r="C10" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/de/notebooks/windows-11/</t>
+        </is>
+      </c>
+      <c r="D10" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E10" s="123" t="n"/>
+      <c r="F10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>Translation DE-DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="261" t="inlineStr">
+        <is>
+          <t>FR-fr</t>
+        </is>
+      </c>
+      <c r="C11" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/fr/pc-portables/windows11/</t>
+        </is>
+      </c>
+      <c r="D11" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E11" s="123" t="n"/>
+      <c r="F11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>Translation FR-FR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="261" t="inlineStr">
+        <is>
+          <t>AU-en</t>
+        </is>
+      </c>
+      <c r="C12" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/au/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D12" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E12" s="123" t="n"/>
+      <c r="F12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>Translation EN-GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="261" t="inlineStr">
+        <is>
+          <t>IN-en</t>
+        </is>
+      </c>
+      <c r="C13" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/in/laptop/windows-11/</t>
+        </is>
+      </c>
+      <c r="D13" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E13" s="123" t="n"/>
+      <c r="F13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="261" t="inlineStr">
+        <is>
+          <t>JP-ja</t>
+        </is>
+      </c>
+      <c r="C14" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/jp/computer-pc/windows11/</t>
+        </is>
+      </c>
+      <c r="D14" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E14" s="123" t="n"/>
+      <c r="F14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>Translation JA-JP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="261" t="inlineStr">
+        <is>
+          <t>CN-zh</t>
+        </is>
+      </c>
+      <c r="C15" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/cn/notebooks/windows11</t>
+        </is>
+      </c>
+      <c r="D15" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E15" s="123" t="n"/>
+      <c r="F15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(zh-CN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="261" t="inlineStr">
+        <is>
+          <t>SG-en</t>
+        </is>
+      </c>
+      <c r="C16" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/sg/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D16" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E16" s="123" t="n"/>
+      <c r="F16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="261" t="inlineStr">
+        <is>
+          <t>VN-vi</t>
+        </is>
+      </c>
+      <c r="C17" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/vn/laptop-lg-gram/windows-11/</t>
+        </is>
+      </c>
+      <c r="D17" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E17" s="123" t="n"/>
+      <c r="F17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(vi-VN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="261" t="inlineStr">
+        <is>
+          <t>TW-zh</t>
+        </is>
+      </c>
+      <c r="C18" s="290" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/tw/laptops/windows-11/</t>
+        </is>
+      </c>
+      <c r="D18" s="265" t="inlineStr">
+        <is>
+          <t>사전검토</t>
+        </is>
+      </c>
+      <c r="E18" s="123" t="n"/>
+      <c r="F18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>MS 참고본(zh-TW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data(it): Buying Guide 2차 UK는 로컬 드리븐 Client Review로 표시한다.
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -40537,7 +40537,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>사전검토 64 · 취소 1(UK, 로컬 WR2338674EL과 중복) · 15개국 추가</t>
+          <t>사전검토 64 · 법인리뷰 1(UK, 로컬 드리븐) · 15개국 추가</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -40551,7 +40551,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -41971,7 +41970,7 @@
       </c>
       <c r="D69" s="265" t="inlineStr">
         <is>
-          <t>취소</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E69" s="123" t="n"/>
@@ -41980,7 +41979,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함 · 로컬 WR2338674EL과 중복이라 취소</t>
+          <t>1차 대상 외 기존 라이브(10/06 실측) · 2차 포함 · 로컬 드리븐 · WR2338674EL(LGCOMUK-3928)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): Buying Guide 2차를 10/14 Raw 기준으로 맞춘다.
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -40537,7 +40537,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>사전검토 59 · 작업중 2(EE·LT) · 법인리뷰 3(UK·LV·CA-fr) · 완료 1(CA-en) · 15개국 추가</t>
+          <t>10/14 기준 · 사전검토 59 · 법인리뷰 5(UK·EE·LT·LV·CA-fr) · 완료 1(CA-en) · 15개국 추가</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -41052,7 +41052,7 @@
       </c>
       <c r="D28" s="265" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E28" s="123" t="n"/>
@@ -41061,7 +41061,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · 허브만 · WR2341063AK(LGCOMEE-557)</t>
+          <t>로컬 드리븐 · WR2341063AK(LGCOMEE-557)</t>
         </is>
       </c>
     </row>
@@ -41173,7 +41173,11 @@
       <c r="F33" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="0" t="n"/>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>접수됨, 착수 전</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="261" t="inlineStr">
@@ -41283,7 +41287,11 @@
       <c r="F38" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G38" s="0" t="n"/>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>접수됨, 착수 전</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="261" t="inlineStr">
@@ -41305,7 +41313,11 @@
       <c r="F39" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G39" s="0" t="n"/>
+      <c r="G39" s="0" t="inlineStr">
+        <is>
+          <t>접수됨, 착수 전</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="261" t="inlineStr">
@@ -41371,7 +41383,11 @@
       <c r="F42" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G42" s="0" t="n"/>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>접수됨, 착수 전</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="261" t="inlineStr">
@@ -41452,7 +41468,7 @@
       </c>
       <c r="D46" s="265" t="inlineStr">
         <is>
-          <t>작업중</t>
+          <t>법인리뷰</t>
         </is>
       </c>
       <c r="E46" s="123" t="n"/>
@@ -41487,7 +41503,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · 허브만 · WR2341048AK(LGCOMLV-634)</t>
+          <t>로컬 드리븐 · WR2341048AK(LGCOMLV-634)</t>
         </is>
       </c>
     </row>
@@ -41753,7 +41769,11 @@
       <c r="F59" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G59" s="0" t="n"/>
+      <c r="G59" s="0" t="inlineStr">
+        <is>
+          <t>접수됨, 착수 전</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="261" t="inlineStr">
@@ -41775,7 +41795,11 @@
       <c r="F60" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G60" s="0" t="n"/>
+      <c r="G60" s="0" t="inlineStr">
+        <is>
+          <t>접수됨, 착수 전</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="261" t="inlineStr">
@@ -41883,7 +41907,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>페이지 없음 · 접수됨, 착수 전</t>
         </is>
       </c>
     </row>
@@ -41955,7 +41979,11 @@
       <c r="F68" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G68" s="0" t="n"/>
+      <c r="G68" s="0" t="inlineStr">
+        <is>
+          <t>LDM 확인 대기</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="261" t="inlineStr">
@@ -41979,7 +42007,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · WR2338674EL(LGCOMUK-3928)</t>
+          <t>로컬 드리븐 · WR2338674EL(LGCOMUK-3928) · 글로벌 건 취소</t>
         </is>
       </c>
     </row>
@@ -42001,7 +42029,7 @@
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>페이지 없음 · 접수됨, 착수 전</t>
         </is>
       </c>
     </row>
@@ -42023,7 +42051,7 @@
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>페이지 없음 · 접수됨, 착수 전</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(it): UltraGear Buying Guide 2차 LDM 승인 16건 작업중 전환
10/12 법인 LDM 승인 요청에 회신한 CZ·RO·HU·HR·RS·BG·TR·DE·ES·PA·CAC·EC·BR·GR·VN·ZA를
사전검토에서 작업중으로 옮긴다. UK·CA는 이미 법인리뷰·완료라 상태는 두고 비고만 단다.
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -1,35 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="W16 - CineBeam S PDP Video Upda" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="W16 - Copilot+ Filter Creation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="W16 - Microsoft PDP Gallery Car" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="W17 - GNB Structure" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="W18 - FAQ Request (UltraGear PL" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="W18 - UltraGear OLED FAQ Update" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="W22 - UltraGear Buying Guide" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="W23 - 27GM950B-B 갤러리 이미지 교체" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="W23 - 39GX950B 이미지 수정 2차" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="W23 - 52G930B Feature 수정 건" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="W23 - UL인증 feature 삭제 1차" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="W25 - Copilot+ Hero Banner" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="W28 - AI Upscaling Disclaimer" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="W28 - UL Verified Eye Comfort" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="W30 - SmartMonitor ScreenShare" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="W30 - UltraGear 1000Hz FAQ" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="W31 - PDP Gallery Win11 Pro" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="W31 - Smart Monitor Multi AI" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="W32 - UltraGear 27GX704A" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="W32 - Digital Trends Award 삭제" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="W32 - UltraGear PDP 5모델" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="W32 - UltraFine PDP MIC 삭제" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="W38 - gram pro gallery" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="W41 - UltraGear Buying Guide 2차" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="W41 - Windows 11 Landing" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="W41 - IT B2B TCO Mark" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W16 - CineBeam S PDP Video Upda" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W16 - Copilot+ Filter Creation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W16 - Microsoft PDP Gallery Car" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W17 - GNB Structure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W18 - FAQ Request (UltraGear PL" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W18 - UltraGear OLED FAQ Update" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W22 - UltraGear Buying Guide" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W23 - 27GM950B-B 갤러리 이미지 교체" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W23 - 39GX950B 이미지 수정 2차" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W23 - 52G930B Feature 수정 건" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W23 - UL인증 feature 삭제 1차" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W25 - Copilot+ Hero Banner" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W28 - AI Upscaling Disclaimer" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W28 - UL Verified Eye Comfort" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W30 - SmartMonitor ScreenShare" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W30 - UltraGear 1000Hz FAQ" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W31 - gram Secure Lock" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W31 - PDP Gallery Win11 Pro" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W31 - Smart Monitor Multi AI" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W32 - UltraGear 27GX704A" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W32 - Digital Trends Award 삭제" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W32 - UltraGear PDP 5모델" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W32 - UltraFine PDP MIC 삭제" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W38 - gram pro gallery" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W41 - UltraGear Buying Guide 2차" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W41 - Windows 11 Landing" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W41 - IT B2B TCO Mark" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'W41 - IT B2B TCO Mark'!$A$3:$G$232</definedName>
@@ -40546,7 +40546,7 @@
       </c>
       <c r="B2" s="163" t="inlineStr">
         <is>
-          <t>10/15 기준 · 사전검토 59 · 법인리뷰 5(UK·EE·LT·LV·CA-fr) · 완료 1(CA-en) · 15개국 추가</t>
+          <t>10/20 기준 · 10/12 법인 LDM 승인 요청 → 16건 승인 회신(CZ·RO·HU·HR·RS·BG·TR·DE·UK·ES·CA·PA/CAC/EC·BR·GR·VN·ZA) · 작업중 16 · 사전검토 43 · 법인리뷰 5(UK·EE·LT·LV·CA-fr) · 완료 1(CA-en)</t>
         </is>
       </c>
       <c r="C2" s="164" t="n"/>
@@ -40759,7 +40759,7 @@
       <c r="C15" s="290" t="n"/>
       <c r="D15" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E15" s="123" t="n"/>
@@ -40768,7 +40768,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>10/12 LDM 승인 · 페이지 없음</t>
         </is>
       </c>
     </row>
@@ -40781,7 +40781,7 @@
       <c r="C16" s="290" t="n"/>
       <c r="D16" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E16" s="123" t="n"/>
@@ -40790,7 +40790,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>10/12 LDM 승인 · 페이지 없음</t>
         </is>
       </c>
     </row>
@@ -40820,7 +40820,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · WR2340922BH(LGCOMCI-5144)</t>
+          <t>10/12 LDM 승인 · 로컬 드리븐 · WR2340922BH(LGCOMCI-5144)</t>
         </is>
       </c>
     </row>
@@ -40846,7 +40846,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · WR2340921BH(LGCOMCI-5144)</t>
+          <t>10/12 LDM 승인 · 로컬 드리븐 · WR2340921BH(LGCOMCI-5144)</t>
         </is>
       </c>
     </row>
@@ -40863,14 +40863,18 @@
       </c>
       <c r="D19" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E19" s="123" t="n"/>
       <c r="F19" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="0" t="n"/>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>10/12 LDM 승인</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="261" t="inlineStr">
@@ -40973,7 +40977,7 @@
       </c>
       <c r="D24" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E24" s="123" t="n"/>
@@ -40982,7 +40986,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>접수됨, 착수 전</t>
+          <t>10/12 LDM 승인</t>
         </is>
       </c>
     </row>
@@ -40999,14 +41003,18 @@
       </c>
       <c r="D25" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E25" s="123" t="n"/>
       <c r="F25" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="0" t="n"/>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>10/12 LDM 승인</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="261" t="inlineStr">
@@ -41043,14 +41051,18 @@
       </c>
       <c r="D27" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E27" s="123" t="n"/>
       <c r="F27" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="0" t="n"/>
+      <c r="G27" s="0" t="inlineStr">
+        <is>
+          <t>10/12 LDM 승인</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="261" t="inlineStr">
@@ -41091,14 +41103,18 @@
       </c>
       <c r="D29" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E29" s="123" t="n"/>
       <c r="F29" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="0" t="n"/>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>10/12 LDM 승인</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="261" t="inlineStr">
@@ -41153,7 +41169,7 @@
       <c r="C32" s="290" t="n"/>
       <c r="D32" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E32" s="123" t="n"/>
@@ -41162,7 +41178,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>10/12 LDM 승인 · 페이지 없음</t>
         </is>
       </c>
     </row>
@@ -41223,7 +41239,7 @@
       <c r="C35" s="290" t="n"/>
       <c r="D35" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E35" s="123" t="n"/>
@@ -41232,7 +41248,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>10/12 LDM 승인 · 페이지 없음</t>
         </is>
       </c>
     </row>
@@ -41249,14 +41265,18 @@
       </c>
       <c r="D36" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E36" s="123" t="n"/>
       <c r="F36" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G36" s="0" t="n"/>
+      <c r="G36" s="0" t="inlineStr">
+        <is>
+          <t>10/12 LDM 승인</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="261" t="inlineStr">
@@ -41621,14 +41641,18 @@
       </c>
       <c r="D52" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E52" s="123" t="n"/>
       <c r="F52" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G52" s="0" t="n"/>
+      <c r="G52" s="0" t="inlineStr">
+        <is>
+          <t>10/12 LDM 승인</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="261" t="inlineStr">
@@ -41727,7 +41751,7 @@
       <c r="C57" s="290" t="n"/>
       <c r="D57" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E57" s="123" t="n"/>
@@ -41736,7 +41760,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>10/12 LDM 승인 · 페이지 없음</t>
         </is>
       </c>
     </row>
@@ -41753,14 +41777,18 @@
       </c>
       <c r="D58" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E58" s="123" t="n"/>
       <c r="F58" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G58" s="0" t="n"/>
+      <c r="G58" s="0" t="inlineStr">
+        <is>
+          <t>10/12 LDM 승인</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="261" t="inlineStr">
@@ -41945,7 +41973,7 @@
       </c>
       <c r="D66" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E66" s="123" t="n"/>
@@ -41954,7 +41982,7 @@
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>접수됨, 착수 전</t>
+          <t>10/12 LDM 승인</t>
         </is>
       </c>
     </row>
@@ -42028,7 +42056,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · WR2338674EL(LGCOMUK-3928) · 글로벌 건 취소</t>
+          <t>10/12 LDM 승인 · 로컬 드리븐 · WR2338674EL(LGCOMUK-3928) · 글로벌 건 취소</t>
         </is>
       </c>
     </row>
@@ -42085,7 +42113,7 @@
       <c r="C72" s="297" t="n"/>
       <c r="D72" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E72" s="123" t="n"/>
@@ -42094,7 +42122,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>페이지 없음</t>
+          <t>10/12 LDM 승인 · 페이지 없음</t>
         </is>
       </c>
     </row>
@@ -42111,14 +42139,18 @@
       </c>
       <c r="D73" s="265" t="inlineStr">
         <is>
-          <t>사전검토</t>
+          <t>작업중</t>
         </is>
       </c>
       <c r="E73" s="123" t="n"/>
       <c r="F73" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G73" s="0" t="n"/>
+      <c r="G73" s="0" t="inlineStr">
+        <is>
+          <t>10/12 LDM 승인</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
data(it): UltraGear Buying Guide 2차 비고에서 PTT ID 삭제
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -3009,6 +3009,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -3597,6 +3598,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -5587,6 +5589,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -7516,6 +7519,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -40560,6 +40564,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -40820,7 +40825,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>10/12 LDM 승인 · 로컬 드리븐 · WR2340922BH(LGCOMCI-5144)</t>
+          <t>10/12 LDM 승인 · 로컬 드리븐</t>
         </is>
       </c>
     </row>
@@ -40846,7 +40851,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>10/12 LDM 승인 · 로컬 드리븐 · WR2340921BH(LGCOMCI-5144)</t>
+          <t>10/12 LDM 승인 · 로컬 드리븐</t>
         </is>
       </c>
     </row>
@@ -41086,7 +41091,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · WR2341063AK(LGCOMEE-557)</t>
+          <t>로컬 드리븐</t>
         </is>
       </c>
     </row>
@@ -41510,7 +41515,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · WR2341062AK(LGCOMLT-527)</t>
+          <t>로컬 드리븐</t>
         </is>
       </c>
     </row>
@@ -41536,7 +41541,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>로컬 드리븐 · WR2341048AK(LGCOMLV-634)</t>
+          <t>로컬 드리븐</t>
         </is>
       </c>
     </row>
@@ -42056,7 +42061,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>10/12 LDM 승인 · 로컬 드리븐 · WR2338674EL(LGCOMUK-3928)</t>
+          <t>10/12 LDM 승인 · 로컬 드리븐</t>
         </is>
       </c>
     </row>
@@ -48801,6 +48806,7 @@
       <c r="G5" s="127" t="n"/>
     </row>
     <row r="6" ht="40.5" customHeight="1" s="203"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
@@ -50592,6 +50598,10 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -52046,6 +52056,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -53309,6 +53320,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -53871,6 +53883,7 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>

</xml_diff>

<commit_message>
data(it): GNB 지난 예정일 9건을 10/23으로, URL Library를 10월 20일 CMS로 맞춘다.
- W17 GNB Structure: 작업중·법인리뷰인데 예정일이 지난 DK·HK·HK_EN·KZ·MY·PL·PT·SE·SG를 2026-10-23으로
- W22 시트 제목 오타 Bying → Buying (gr-titles 매핑 포함)
- url-library.json: cms_merged_view_20261020_160355 기준(모델 2,051 · URL 27,973)
</commit_message>
<xml_diff>
--- a/it/Global Request.xlsx
+++ b/it/Global Request.xlsx
@@ -3009,7 +3009,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -3598,7 +3597,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -5589,7 +5587,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -7519,7 +7516,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>
@@ -40564,7 +40560,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -48806,7 +48801,6 @@
       <c r="G5" s="127" t="n"/>
     </row>
     <row r="6" ht="40.5" customHeight="1" s="203"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
@@ -49683,7 +49677,7 @@
       </c>
       <c r="E20" s="123" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F20" s="123" t="n">
@@ -49813,7 +49807,7 @@
       </c>
       <c r="E25" s="123" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F25" s="123" t="n">
@@ -49839,7 +49833,7 @@
       </c>
       <c r="E26" s="123" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F26" s="123" t="n">
@@ -49983,7 +49977,7 @@
       </c>
       <c r="E32" s="123" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F32" s="123" t="n">
@@ -50061,7 +50055,7 @@
       </c>
       <c r="E35" s="123" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F35" s="123" t="n">
@@ -50209,7 +50203,7 @@
       </c>
       <c r="E41" s="123" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F41" s="123" t="n">
@@ -50235,7 +50229,7 @@
       </c>
       <c r="E42" s="123" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F42" s="123" t="n">
@@ -50309,7 +50303,7 @@
       </c>
       <c r="E45" s="123" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F45" s="123" t="n">
@@ -50335,7 +50329,7 @@
       </c>
       <c r="E46" s="123" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F46" s="123" t="n">
@@ -50598,10 +50592,6 @@
       <c r="F3" s="131" t="n"/>
       <c r="G3" s="127" t="n"/>
     </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="266" t="inlineStr">
         <is>
@@ -52027,7 +52017,7 @@
       </c>
       <c r="B1" s="163" t="inlineStr">
         <is>
-          <t>GR26-W22-MS-IT UltraGear Bying Guide</t>
+          <t>GR26-W22-MS-IT UltraGear Buying Guide</t>
         </is>
       </c>
       <c r="C1" s="164" t="n"/>
@@ -52056,7 +52046,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -53320,7 +53309,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="127" t="n"/>
       <c r="B5" s="127" t="n"/>
@@ -53883,7 +53871,6 @@
       <c r="D3" s="164" t="n"/>
       <c r="E3" s="165" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="E5" s="127" t="n"/>
     </row>

</xml_diff>